<commit_message>
evaluasi llm as a judge
</commit_message>
<xml_diff>
--- a/data/eval_outputs/evaluation_report.xlsx
+++ b/data/eval_outputs/evaluation_report.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD21"/>
+  <dimension ref="A1:AE21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,115 +457,120 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>llm_judge_score</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>semantic_similarity</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>keyword_coverage</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>keyword_hits</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>keyword_missing</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>retrieval_citation_coverage</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>retrieval_citation_hit</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>retrieval_law_hit</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>retrieval_article_hit</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>answer_citation_hit</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>expected_article_rank</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>expected_law_rank</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>article_mrr</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>law_mrr</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>precision_at_3</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>article_hit_at_3</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>article_hit_at_8</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>answer_word_count</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>answer_length_score</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>latency_seconds</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>model_id</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>top1_reference</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>retrieved_references_text</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>retrieved_references_json</t>
         </is>
@@ -607,7 +612,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.9184461808204651</v>
+        <v>0.9298496687412263</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -615,24 +620,24 @@
         </is>
       </c>
       <c r="H2" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="I2" t="n">
         <v>0.7656644582748413</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>0.8333333333333334</v>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>PKWT; uang kompensasi; 1 bulan upah; proporsional; masa kerja dibagi 12</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>berakhir</t>
         </is>
       </c>
-      <c r="L2" t="n">
-        <v>1</v>
-      </c>
       <c r="M2" t="n">
         <v>1</v>
       </c>
@@ -667,30 +672,33 @@
         <v>1</v>
       </c>
       <c r="X2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y2" t="n">
         <v>155</v>
       </c>
-      <c r="Y2" t="n">
-        <v>1</v>
-      </c>
       <c r="Z2" t="n">
-        <v>44.66412854194641</v>
-      </c>
-      <c r="AA2" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>43.90230417251587</v>
+      </c>
+      <c r="AB2" t="inlineStr">
         <is>
           <t>Qwen/Qwen3.5-9B</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
+      <c r="AC2" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 15 | PP Nomor 35 Tahun 2021.pdf | Pasal 15</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AD2" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 15 | PP Nomor 35 Tahun 2021.pdf | Pasal 15 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 17 | PP Nomor 35 Tahun 2021.pdf | Pasal 17 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 16 | PP Nomor 35 Tahun 2021.pdf | Pasal 16 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 64 | PP Nomor 35 Tahun 2021.pdf | Pasal 64 || Peraturan Pemerintah No. 6 Tahun 2025, Pasal 19 | pp_Nomor_6_Tahun_2025.pdf | Pasal 19 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 1 bagian 1 | PP Nomor 35 Tahun 2021.pdf | Pasal 1 || Peraturan Menteri Ketenagakerjaan No. 28 Tahun 2014, Pasal 1 bagian 1 | permen_Nomor_28_Tahun_2014.pdf | Pasal 1 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 54 | PP Nomor 35 Tahun 2021.pdf | Pasal 54</t>
         </is>
       </c>
-      <c r="AD2" t="inlineStr">
+      <c r="AE2" t="inlineStr">
         <is>
           <t>[{"rank": 1, "chunk_id": "174a6caf0ddd3791ff66aa1e4b6d8417fc84c2e2", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 15 | PP Nomor 35 Tahun 2021.pdf | Pasal 15", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 15", "rrf_score": 0.029508196721311476, "rerank_score": 0.9833083152770996, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB II - Perjanjian Kerja Waktu Tertentu Bagian Ketiga - Pemberian Uang Kompensasi Pasal 15 (1) Pengusaha wajib memberikan uang kompensasi kepada Pekerja/Buruh yang hubungan kerjanya berdasarkan PKWT. (2) Pemberian uang kompensasi dilaksanakan pada saat berakhirnya PKWT. (3) Uang kompensasi sebagaimana dimaksud pada ayat (1) diberikan kepada Pek"}, {"rank": 2, "chunk_id": "beda60ec5197e979747c00fcdea85f8aa67e0f9f", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 17 | PP Nomor 35 Tahun 2021.pdf | Pasal 17", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 17", "rrf_score": 0.02818070818070818, "rerank_score": 0.9380102753639221, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB II - Perjanjian Kerja Waktu Tertentu Bagian Ketiga - Pemberian Uang Kompensasi Pasal 17 Dalam hal salah satu pihak mengakhiri Hubungan Kerja sebelum berakhirnya jangka waktu yang ditetapkan dalam PKWT, Pengusaha wajib memberikan uang kompensasi sebagaimana dimaksud dalam Pasal 15 ayat (1) yang besarannya dihitung berdasarkan jangka waktu PKW"}, {"rank": 3, "chunk_id": "4162f26e429b0da776807f7a3ebfb05bdb999784", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 16 | PP Nomor 35 Tahun 2021.pdf | Pasal 16", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 16", "rrf_score": 0.029032258064516127, "rerank_score": 0.917829692363739, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB II - Perjanjian Kerja Waktu Tertentu Bagian Ketiga - Pemberian Uang Kompensasi Pasal 16 (1) Besaran uang kompensasi diberikan sesuai dengan ketentuan sebagai berikut: a. PKWT selama 12 (dua belas) bulan secara terus menerus, diberikan sebesar 1 (satu) bulan Upah; b. PKWT selama 1 (satu) bulan atau lebih tetapi kurang dari 12 (dwa belas) bula"}, {"rank": 4, "chunk_id": "404c9b5be45bdd40314d1f6629cc3a4054075dd3", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 64 | PP Nomor 35 Tahun 2021.pdf | Pasal 64", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 64", "rrf_score": 0.026226012793176972, "rerank_score": 0.7856653332710266, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 BAB IX - Ketentuan Penutup Pasal 64 Pada saat Peraturan Pemerintah ini mulai berlaku a. uang kompensasi untuk PKWT yang jangka waktunya belum berakhir diberikan sesuai dengan ketentuan dalam Peraturan Pemerintah ini; dan b. besaran uang kompensasi sebagaimana dimaksud pada huruf a dihitung berdasarkan masa kerja Pekerja/Buruh yang perhitungannya dimulai sejak tanggal diundangkan Undang-Undang Nomor 11 Tahun 2020 TENTANG Cipta Kerja."}, {"rank": 5, "chunk_id": "728a3b4794695ee074f9dde293c7fb15c9692c3c", "reference": "Peraturan Pemerintah No. 6 Tahun 2025, Pasal 19 | pp_Nomor_6_Tahun_2025.pdf | Pasal 19", "source_file": "pp_Nomor_6_Tahun_2025.pdf", "pasal_id": "Pasal 19", "rrf_score": 0.024624624624624628, "rerank_score": 0.732478678226471, "text_preview": "Peraturan Pemerintah No. 6 Tahun 2025 Pasal 19 SITASI: Peraturan Pemerintah No. 6 Tahun 2025, Pasal 19 Ayat (1) Cukup jelas. Ayat (2) Yang dimaksud dengan \"bersedia untuk bekerja kembali\" yaitu bekerja sebagai pekerja penerima upah atau berusaha mandiri atau wirausaha. Ayat (3) Makna 24 (dua puluh empat) bulan dalam ketentuan Pasal 19 ayat (3) adalah bulan kalender, bukan bulan masa iur dan bukan bulan masa kepesertaan dalam program BPJS Ketenagakerjaan. Syarat masa iur 12 (dua belas) bulan dima"}, {"rank": 6, "chunk_id": "ef31e26ce2dd832602d5bb45532dde7319c92704", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 1 bagian 1 | PP Nomor 35 Tahun 2021.pdf | Pasal 1", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 1", "rrf_score": 0.010126582278481013, "rerank_score": 0.6283866763114929, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB I - Ketentuan Umum Pasal 1 bagian 1 Hubungan Kerja adalah hubungan antara Pengusaha 1 dengan Pekerja/Buruh berdasarkan Perjanjian Kerja, yang mempunyai unsur pekerjaan, Upah, dan perintah. 2 Pekerja/Buruh adalah setiap orang yang bekerja dengan menerima Upah atau imbalan dalam bentuk lain. 3 Pengusaha adalah: a. orang perseorangan, persekutu"}, {"rank": 7, "chunk_id": "f22a2c245e8ebfca109c15a979624ac02005ab52", "reference": "Peraturan Menteri Ketenagakerjaan No. 28 Tahun 2014, Pasal 1 bagian 1 | permen_Nomor_28_Tahun_2014.pdf | Pasal 1", "source_file": "permen_Nomor_28_Tahun_2014.pdf", "pasal_id": "Pasal 1", "rrf_score": 0.019874274661508706, "rerank_score": 0.5727373361587524, "text_preview": "Peraturan Menteri Ketenagakerjaan No. 28 Tahun 2014 tentang TATA CARA PEMBUATAN DAN PENGESAHAN PERATURAN PERUSAHAAN SERTA PEMBUATAN DAN PENDAFTARAN PERJANJIAN KERJA BERSAMA BAB I - Ketentuan Umum Pasal 1 bagian 1 1. Peraturan Perusahaan yang selanjutnya disingkat PP adalah peraturan yang dibuat secara tertulis oleh pengusaha yang memuat syarat-syarat kerja dan tata tertib perusahaan. 2. Perjanjian Kerja Bersama yang selanjutnya disingkat PKB adalah perjanjian yang merupakan hasil perundingan ant"}, {"rank": 8, "chunk_id": "8b27dbefd4415136637241a90d1b04a057678314", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 54 | PP Nomor 35 Tahun 2021.pdf | Pasal 54", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 54", "rrf_score": 0.02315648982315649, "rerank_score": 0.48618438839912415, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kedua - Hak Akibat Pemutusan Hubungan Kerja Pasal 54 (1) Pengusaha dapat melakukan Pemutusan Hubungan Kerja terhadap Pekerja/Buruh karena alasan Pekerja/Buruh tidak dapat melakukan pekerjaan selama 6 (enam) bulan akibat ditahan pihak yang berwajib karena diduga melakukan tindak pidana sebagaimana dimaksud "}]</t>
         </is>
@@ -730,7 +738,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.9612854552268981</v>
+        <v>0.9736037194728853</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -738,20 +746,20 @@
         </is>
       </c>
       <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="n">
         <v>0.8240247964859009</v>
       </c>
-      <c r="I3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J3" t="inlineStr">
+      <c r="J3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" t="inlineStr">
         <is>
           <t>PKWT; masa percobaan; tidak boleh; batal demi hukum; masa kerja tetap dihitung</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="n">
-        <v>1</v>
-      </c>
+      <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
         <v>1</v>
       </c>
@@ -786,30 +794,33 @@
         <v>1</v>
       </c>
       <c r="X3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y3" t="n">
         <v>148</v>
       </c>
-      <c r="Y3" t="n">
-        <v>1</v>
-      </c>
       <c r="Z3" t="n">
-        <v>43.45739126205444</v>
-      </c>
-      <c r="AA3" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>43.17098212242126</v>
+      </c>
+      <c r="AB3" t="inlineStr">
         <is>
           <t>Qwen/Qwen3.5-9B</t>
         </is>
       </c>
-      <c r="AB3" t="inlineStr">
+      <c r="AC3" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 12 | PP Nomor 35 Tahun 2021.pdf | Pasal 12</t>
         </is>
       </c>
-      <c r="AC3" t="inlineStr">
+      <c r="AD3" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 12 | PP Nomor 35 Tahun 2021.pdf | Pasal 12 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 9 | PP Nomor 35 Tahun 2021.pdf | Pasal 9 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 5 | PP Nomor 35 Tahun 2021.pdf | Pasal 5 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 1 bagian 1 | PP Nomor 35 Tahun 2021.pdf | Pasal 1 || Undang-Undang No. 13 Tahun 2003, Pasal 58 | UU_Nomor_13_Tahun_2003.pdf | Pasal 58 || Peraturan Pemerintah No. 6 Tahun 2025, Pasal 19 | pp_Nomor_6_Tahun_2025.pdf | Pasal 19 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 8 | PP Nomor 35 Tahun 2021.pdf | Pasal 8 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 1 | PP Nomor 35 Tahun 2021.pdf | Pasal 1</t>
         </is>
       </c>
-      <c r="AD3" t="inlineStr">
+      <c r="AE3" t="inlineStr">
         <is>
           <t>[{"rank": 1, "chunk_id": "ae15dffc34bf49f464cbeefc253595637b2dc66b", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 12 | PP Nomor 35 Tahun 2021.pdf | Pasal 12", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 12", "rrf_score": 0.029508196721311476, "rerank_score": 0.9751182794570923, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB II - Perjanjian Kerja Waktu Tertentu Bagian Kedua - Pelaksanaan Perjanjian Kerja Waktu Tertentu Pasal 12 (1) PKWT tidak dapat mensyaratkan adanya masa percobaan kerja. (2) Dalam hal disyaratkan masa percobaan kerja, masa percobaan kerja yang disyaratkan tersebut batal demi hukum dan masa kerja tetap dihitung."}, {"rank": 2, "chunk_id": "f7929ba6d33c6ef53a454e08ee67b33bdbf1f821", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 9 | PP Nomor 35 Tahun 2021.pdf | Pasal 9", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 9", "rrf_score": 0.027692307692307693, "rerank_score": 0.46758273243904114, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB II - Perjanjian Kerja Waktu Tertentu Bagian Kedua - Pelaksanaan Perjanjian Kerja Waktu Tertentu Pasal 9 (1) PKWT berdasarkan selesainya suatu pekerjaan tertentu sebagaimana dimaksud dalam Pasal 5 ayat (21didasarkan atas kesepakatan para pihak yang dituangkan dalam Perjanjian Kerja. (2) Kesepakatan para pihak sebagaimana dimaksud pada ayat (1"}, {"rank": 3, "chunk_id": "b9e022bdc1ce11e24d99e1801f0e6f5d4cad4178", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 5 | PP Nomor 35 Tahun 2021.pdf | Pasal 5", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 5", "rrf_score": 0.026745718050065877, "rerank_score": 0.44956785440444946, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB II - Perjanjian Kerja Waktu Tertentu Bagian Kedua - Pelaksanaan Perjanjian Kerja Waktu Tertentu Pasal 5 (1) PKWT berdasarkan jangka waktu sebagaimana dimaksud dalam Pasal 4 ayat (1) huruf a dibuat untuk pekerjaan tertentu yaitu: a. pekerjaan yang diperkirakan penyelesaiannya dalam waktu yang tidak terlalu lama; b. pekerjaan yang bersifat mus"}, {"rank": 4, "chunk_id": "ef31e26ce2dd832602d5bb45532dde7319c92704", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 1 bagian 1 | PP Nomor 35 Tahun 2021.pdf | Pasal 1", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 1", "rrf_score": 0.008888888888888889, "rerank_score": 0.2854800224304199, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB I - Ketentuan Umum Pasal 1 bagian 1 Hubungan Kerja adalah hubungan antara Pengusaha 1 dengan Pekerja/Buruh berdasarkan Perjanjian Kerja, yang mempunyai unsur pekerjaan, Upah, dan perintah. 2 Pekerja/Buruh adalah setiap orang yang bekerja dengan menerima Upah atau imbalan dalam bentuk lain. 3 Pengusaha adalah: a. orang perseorangan, persekutu"}, {"rank": 5, "chunk_id": "104ebafcafe91c1c6554400a9481a2ebb7454e90", "reference": "Undang-Undang No. 13 Tahun 2003, Pasal 58 | UU_Nomor_13_Tahun_2003.pdf | Pasal 58", "source_file": "UU_Nomor_13_Tahun_2003.pdf", "pasal_id": "Pasal 58", "rrf_score": 0.026470588235294117, "rerank_score": 0.2199932336807251, "text_preview": "Undang-Undang No. 13 Tahun 2003 tentang KETENAGAKERJAAN BAB IX - Hubungan Kerja Pasal 58 (1) Perjanjian kerja untuk waktu tertentu tidak dapat mensyaratkan adanya masa percobaan kerja. (2) Dalam hal disyaratkan masa percobaan kerja dalam perjanjian kerja sebagaimana dimaksud dalam ayat (1), masa percobaan kerja yang disyaratkan batal demi hukum."}, {"rank": 6, "chunk_id": "728a3b4794695ee074f9dde293c7fb15c9692c3c", "reference": "Peraturan Pemerintah No. 6 Tahun 2025, Pasal 19 | pp_Nomor_6_Tahun_2025.pdf | Pasal 19", "source_file": "pp_Nomor_6_Tahun_2025.pdf", "pasal_id": "Pasal 19", "rrf_score": 0.021924735980960883, "rerank_score": 0.2118273675441742, "text_preview": "Peraturan Pemerintah No. 6 Tahun 2025 Pasal 19 SITASI: Peraturan Pemerintah No. 6 Tahun 2025, Pasal 19 Ayat (1) Cukup jelas. Ayat (2) Yang dimaksud dengan \"bersedia untuk bekerja kembali\" yaitu bekerja sebagai pekerja penerima upah atau berusaha mandiri atau wirausaha. Ayat (3) Makna 24 (dua puluh empat) bulan dalam ketentuan Pasal 19 ayat (3) adalah bulan kalender, bukan bulan masa iur dan bukan bulan masa kepesertaan dalam program BPJS Ketenagakerjaan. Syarat masa iur 12 (dua belas) bulan dima"}, {"rank": 7, "chunk_id": "d09ac5ae28956298a98a70ced4c841956ab85b9e", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 8 | PP Nomor 35 Tahun 2021.pdf | Pasal 8", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 8", "rrf_score": 0.0283234126984127, "rerank_score": 0.1933976262807846, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB II - Perjanjian Kerja Waktu Tertentu Bagian Kedua - Pelaksanaan Perjanjian Kerja Waktu Tertentu Pasal 8 (1) PKWT berdasarkan jangka waktu sebagaimana dimaksud dalam Pasal 5 ayat (1) dapat dibuat untuk paling lama 5 (lima) tahun. (2) Dalam hal jangka waktu PKWT sebagaimana dimaksud pada ayat (1) akan berakhir dan pekerjaan yang dilaksanakan b"}, {"rank": 8, "chunk_id": "8877ce6af30ffbbf7b922de381b1b7929324f379", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 1 | PP Nomor 35 Tahun 2021.pdf | Pasal 1", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 1", "rrf_score": 0.018773738469886055, "rerank_score": 0.18537476658821106, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 BAB I - Ketentuan Umum Pasal 1 Pekerja/Buruh dengan Pengusaha untuk mengadakan Hubungan Kerja dalam waktu tertentu atau untuk pekerjaan tertentu. 1. Perjanjian Kerja Waktu Tertentu (PKWT) yang selanjutnya disingkat PKWT adalah Perjanjian Kerja antara Pekerja/Buruh dengan Pengusaha untuk mengadakan Hubungan Kerja yang bersifat tetap. 12. Peraturan Perusahaan adalah peraturan yang dibuat secara tertulis oleh Pengusaha yang memuat syarat-syarat kerja dan tata "}]</t>
         </is>
@@ -848,7 +859,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.9334691190719605</v>
+        <v>0.8766834902763367</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -856,20 +867,20 @@
         </is>
       </c>
       <c r="H4" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I4" t="n">
         <v>0.8112232685089111</v>
       </c>
-      <c r="I4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" t="inlineStr">
+      <c r="J4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" t="inlineStr">
         <is>
           <t>PKWT; jangka waktu; paling lama 5 tahun; perpanjangan</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="n">
-        <v>1</v>
-      </c>
+      <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
         <v>1</v>
       </c>
@@ -883,17 +894,17 @@
         <v>1</v>
       </c>
       <c r="Q4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R4" t="n">
         <v>2</v>
       </c>
-      <c r="R4" t="n">
-        <v>1</v>
-      </c>
       <c r="S4" t="n">
+        <v>1</v>
+      </c>
+      <c r="T4" t="n">
         <v>0.5</v>
       </c>
-      <c r="T4" t="n">
-        <v>1</v>
-      </c>
       <c r="U4" t="n">
         <v>1</v>
       </c>
@@ -904,30 +915,33 @@
         <v>1</v>
       </c>
       <c r="X4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y4" t="n">
         <v>174</v>
       </c>
-      <c r="Y4" t="n">
-        <v>1</v>
-      </c>
       <c r="Z4" t="n">
-        <v>46.90166258811951</v>
-      </c>
-      <c r="AA4" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>46.29595255851746</v>
+      </c>
+      <c r="AB4" t="inlineStr">
         <is>
           <t>Qwen/Qwen3.5-9B</t>
         </is>
       </c>
-      <c r="AB4" t="inlineStr">
+      <c r="AC4" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 9 | PP Nomor 35 Tahun 2021.pdf | Pasal 9</t>
         </is>
       </c>
-      <c r="AC4" t="inlineStr">
+      <c r="AD4" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 9 | PP Nomor 35 Tahun 2021.pdf | Pasal 9 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 8 | PP Nomor 35 Tahun 2021.pdf | Pasal 8 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 5 | PP Nomor 35 Tahun 2021.pdf | Pasal 5 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 15 | PP Nomor 35 Tahun 2021.pdf | Pasal 15 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 4 | PP Nomor 35 Tahun 2021.pdf | Pasal 4 || Undang-Undang No. 13 Tahun 2003, Pasal 59 | UU_Nomor_13_Tahun_2003.pdf | Pasal 59 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 6 | PP Nomor 35 Tahun 2021.pdf | Pasal 6 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 16 | PP Nomor 35 Tahun 2021.pdf | Pasal 16</t>
         </is>
       </c>
-      <c r="AD4" t="inlineStr">
+      <c r="AE4" t="inlineStr">
         <is>
           <t>[{"rank": 1, "chunk_id": "f7929ba6d33c6ef53a454e08ee67b33bdbf1f821", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 9 | PP Nomor 35 Tahun 2021.pdf | Pasal 9", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 9", "rrf_score": 0.02909185532136352, "rerank_score": 0.9868289828300476, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB II - Perjanjian Kerja Waktu Tertentu Bagian Kedua - Pelaksanaan Perjanjian Kerja Waktu Tertentu Pasal 9 (1) PKWT berdasarkan selesainya suatu pekerjaan tertentu sebagaimana dimaksud dalam Pasal 5 ayat (21didasarkan atas kesepakatan para pihak yang dituangkan dalam Perjanjian Kerja. (2) Kesepakatan para pihak sebagaimana dimaksud pada ayat (1"}, {"rank": 2, "chunk_id": "d09ac5ae28956298a98a70ced4c841956ab85b9e", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 8 | PP Nomor 35 Tahun 2021.pdf | Pasal 8", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 8", "rrf_score": 0.02924378635642517, "rerank_score": 0.9814056754112244, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB II - Perjanjian Kerja Waktu Tertentu Bagian Kedua - Pelaksanaan Perjanjian Kerja Waktu Tertentu Pasal 8 (1) PKWT berdasarkan jangka waktu sebagaimana dimaksud dalam Pasal 5 ayat (1) dapat dibuat untuk paling lama 5 (lima) tahun. (2) Dalam hal jangka waktu PKWT sebagaimana dimaksud pada ayat (1) akan berakhir dan pekerjaan yang dilaksanakan b"}, {"rank": 3, "chunk_id": "b9e022bdc1ce11e24d99e1801f0e6f5d4cad4178", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 5 | PP Nomor 35 Tahun 2021.pdf | Pasal 5", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 5", "rrf_score": 0.028373015873015873, "rerank_score": 0.958801805973053, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB II - Perjanjian Kerja Waktu Tertentu Bagian Kedua - Pelaksanaan Perjanjian Kerja Waktu Tertentu Pasal 5 (1) PKWT berdasarkan jangka waktu sebagaimana dimaksud dalam Pasal 4 ayat (1) huruf a dibuat untuk pekerjaan tertentu yaitu: a. pekerjaan yang diperkirakan penyelesaiannya dalam waktu yang tidak terlalu lama; b. pekerjaan yang bersifat mus"}, {"rank": 4, "chunk_id": "174a6caf0ddd3791ff66aa1e4b6d8417fc84c2e2", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 15 | PP Nomor 35 Tahun 2021.pdf | Pasal 15", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 15", "rrf_score": 0.028054740957966763, "rerank_score": 0.8483312129974365, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB II - Perjanjian Kerja Waktu Tertentu Bagian Ketiga - Pemberian Uang Kompensasi Pasal 15 (1) Pengusaha wajib memberikan uang kompensasi kepada Pekerja/Buruh yang hubungan kerjanya berdasarkan PKWT. (2) Pemberian uang kompensasi dilaksanakan pada saat berakhirnya PKWT. (3) Uang kompensasi sebagaimana dimaksud pada ayat (1) diberikan kepada Pek"}, {"rank": 5, "chunk_id": "6b65a49c782cb46e0d40e99d6b7ad5a438010754", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 4 | PP Nomor 35 Tahun 2021.pdf | Pasal 4", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 4", "rrf_score": 0.026353944562899786, "rerank_score": 0.82743901014328, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB II - Perjanjian Kerja Waktu Tertentu Bagian Kedua - Pelaksanaan Perjanjian Kerja Waktu Tertentu Pasal 4 (1) PKWT didasarkan atas: a. jangka waktu; atau b. selesainya suatu pekerjaan tertentu. (2) PKWT tidak dapat diadakan untuk pekerjaan yang bersifat tetap."}, {"rank": 6, "chunk_id": "d411f4006ff6fe710baf2f6a92225aba7719b315", "reference": "Undang-Undang No. 13 Tahun 2003, Pasal 59 | UU_Nomor_13_Tahun_2003.pdf | Pasal 59", "source_file": "UU_Nomor_13_Tahun_2003.pdf", "pasal_id": "Pasal 59", "rrf_score": 0.026800445930880712, "rerank_score": 0.8211844563484192, "text_preview": "Undang-Undang No. 13 Tahun 2003 tentang KETENAGAKERJAAN BAB IX - Hubungan Kerja Pasal 59 (1) Perjanjian kerja untuk waktu tertentu hanya dapat dibuat untuk pekerjaan tertentu yang menurut jenis dan sifat atau kegiatan pekerjaannya akan selesai dalam waktu tertentu, yaitu: a. pekerjaan yang sekali selesai atau yang sementara sifatnya; b. pekerjaaan yang diperkirakan penyelesaiannya dalam waktu yang tidak terlalu lama dan paling lama 3 (tiga) tahun; c. pekerjaan yang bersifat musiman; atau d. peke"}, {"rank": 7, "chunk_id": "ad00015531626c854f9d37a83cd11551bf6cd7c4", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 6 | PP Nomor 35 Tahun 2021.pdf | Pasal 6", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 6", "rrf_score": 0.02245315698315226, "rerank_score": 0.7358750700950623, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB II - Perjanjian Kerja Waktu Tertentu Bagian Kedua - Pelaksanaan Perjanjian Kerja Waktu Tertentu Pasal 6 Pekerjaan yang diperkirakan penyelesaiannya dalam waktu yang tidak terlalu lama sebagaimana dimaksud dalam Pasal 5 ayat (1) huruf a dilaksanakan paling lama 5 (lima) tahun."}, {"rank": 8, "chunk_id": "4162f26e429b0da776807f7a3ebfb05bdb999784", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 16 | PP Nomor 35 Tahun 2021.pdf | Pasal 16", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 16", "rrf_score": 0.02697881828316611, "rerank_score": 0.7334725260734558, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB II - Perjanjian Kerja Waktu Tertentu Bagian Ketiga - Pemberian Uang Kompensasi Pasal 16 (1) Besaran uang kompensasi diberikan sesuai dengan ketentuan sebagai berikut: a. PKWT selama 12 (dua belas) bulan secara terus menerus, diberikan sebesar 1 (satu) bulan Upah; b. PKWT selama 1 (satu) bulan atau lebih tetapi kurang dari 12 (dwa belas) bula"}]</t>
         </is>
@@ -961,7 +975,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.8937286732991535</v>
+        <v>0.9232998530069988</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -969,24 +983,24 @@
         </is>
       </c>
       <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" t="n">
         <v>0.7108879089355469</v>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
         <v>0.8</v>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>harian; kurang dari 21 hari; 21 hari atau lebih; 3 bulan berturut-turut</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>menjadi PKWTT</t>
         </is>
       </c>
-      <c r="L5" t="n">
-        <v>1</v>
-      </c>
       <c r="M5" t="n">
         <v>1</v>
       </c>
@@ -1012,39 +1026,42 @@
         <v>1</v>
       </c>
       <c r="U5" t="n">
+        <v>1</v>
+      </c>
+      <c r="V5" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="V5" t="n">
-        <v>1</v>
-      </c>
       <c r="W5" t="n">
         <v>1</v>
       </c>
       <c r="X5" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y5" t="n">
         <v>54</v>
       </c>
-      <c r="Y5" t="n">
-        <v>1</v>
-      </c>
       <c r="Z5" t="n">
-        <v>16.92839670181274</v>
-      </c>
-      <c r="AA5" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>16.77782320976257</v>
+      </c>
+      <c r="AB5" t="inlineStr">
         <is>
           <t>Qwen/Qwen3.5-9B</t>
         </is>
       </c>
-      <c r="AB5" t="inlineStr">
+      <c r="AC5" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 10 | PP Nomor 35 Tahun 2021.pdf | Pasal 10</t>
         </is>
       </c>
-      <c r="AC5" t="inlineStr">
+      <c r="AD5" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 10 | PP Nomor 35 Tahun 2021.pdf | Pasal 10 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 1 bagian 1 | PP Nomor 35 Tahun 2021.pdf | Pasal 1 || Peraturan Menteri Ketenagakerjaan No. 1 Tahun 2020, Keempat bagian 3 | PERMEN_Nomor_1_Tahun_2020.pdf | Keempat || Peraturan Pemerintah No. 6 Tahun 2025, Pasal 19 | pp_Nomor_6_Tahun_2025.pdf | Pasal 19 || Peraturan Menteri Ketenagakerjaan No. 28 Tahun 2014, Pasal 1 bagian 1 | permen_Nomor_28_Tahun_2014.pdf | Pasal 1 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 1 | PP Nomor 35 Tahun 2021.pdf | Pasal 1 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 15 | PP Nomor 35 Tahun 2021.pdf | Pasal 15 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 9 | PP Nomor 35 Tahun 2021.pdf | Pasal 9</t>
         </is>
       </c>
-      <c r="AD5" t="inlineStr">
+      <c r="AE5" t="inlineStr">
         <is>
           <t>[{"rank": 1, "chunk_id": "a47f933de3e7e9ec242f902100bc4e305976febf", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 10 | PP Nomor 35 Tahun 2021.pdf | Pasal 10", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 10", "rrf_score": 0.029508196721311476, "rerank_score": 0.9731410145759583, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB II - Perjanjian Kerja Waktu Tertentu Bagian Kedua - Pelaksanaan Perjanjian Kerja Waktu Tertentu Pasal 10 (1) PKWT yang dapat dilaksanakan terhadap pekerjaan tertentu lainnya yang jenis dan sifat atau kegiatannya bersifat tidak tetap sebagaimana dimaksud dalam Pasal 5 ayat (3) berupa pekerjaan tertentu yang berubah-ubah dalam hal waktu dan vo"}, {"rank": 2, "chunk_id": "ef31e26ce2dd832602d5bb45532dde7319c92704", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 1 bagian 1 | PP Nomor 35 Tahun 2021.pdf | Pasal 1", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 1", "rrf_score": 0.02043135735503035, "rerank_score": 0.814124345779419, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB I - Ketentuan Umum Pasal 1 bagian 1 Hubungan Kerja adalah hubungan antara Pengusaha 1 dengan Pekerja/Buruh berdasarkan Perjanjian Kerja, yang mempunyai unsur pekerjaan, Upah, dan perintah. 2 Pekerja/Buruh adalah setiap orang yang bekerja dengan menerima Upah atau imbalan dalam bentuk lain. 3 Pengusaha adalah: a. orang perseorangan, persekutu"}, {"rank": 3, "chunk_id": "6ce8716ce9d3903e756486287fa88ad52cd701e5", "reference": "Peraturan Menteri Ketenagakerjaan No. 1 Tahun 2020, Keempat bagian 3 | PERMEN_Nomor_1_Tahun_2020.pdf | Keempat", "source_file": "PERMEN_Nomor_1_Tahun_2020.pdf", "pasal_id": "Keempat", "rrf_score": 0.009090909090909092, "rerank_score": 0.7579032182693481, "text_preview": "Peraturan Menteri Ketenagakerjaan No. 1 Tahun 2020 tentang PERUBAHAN ATAS PERATURAN MENTERI KETENAGAKERJAAN NOMOR 33 TAHUN 2016 TENTANG TATA CARA PENGAWASAN KETENAGAKERJAAN Keempat bagian 3 PELARANGAN PROSES PEKERJAAN Nomor: Pada hari ini tanggal bulan tahun berdasarkan hasil pemeriksaan dan/atau pengujian terhadap objek K3 telah dilaksanakan penghentian/pelarangan proses pekerjaan atas: Nama Objek K3 Lokasi Penghentian/pelarangan proses pekerjaan disaksikan oleh: Nama: , alamat: pekerjaan: , se"}, {"rank": 4, "chunk_id": "728a3b4794695ee074f9dde293c7fb15c9692c3c", "reference": "Peraturan Pemerintah No. 6 Tahun 2025, Pasal 19 | pp_Nomor_6_Tahun_2025.pdf | Pasal 19", "source_file": "pp_Nomor_6_Tahun_2025.pdf", "pasal_id": "Pasal 19", "rrf_score": 0.026134453781512607, "rerank_score": 0.7320820689201355, "text_preview": "Peraturan Pemerintah No. 6 Tahun 2025 Pasal 19 SITASI: Peraturan Pemerintah No. 6 Tahun 2025, Pasal 19 Ayat (1) Cukup jelas. Ayat (2) Yang dimaksud dengan \"bersedia untuk bekerja kembali\" yaitu bekerja sebagai pekerja penerima upah atau berusaha mandiri atau wirausaha. Ayat (3) Makna 24 (dua puluh empat) bulan dalam ketentuan Pasal 19 ayat (3) adalah bulan kalender, bukan bulan masa iur dan bukan bulan masa kepesertaan dalam program BPJS Ketenagakerjaan. Syarat masa iur 12 (dua belas) bulan dima"}, {"rank": 5, "chunk_id": "f22a2c245e8ebfca109c15a979624ac02005ab52", "reference": "Peraturan Menteri Ketenagakerjaan No. 28 Tahun 2014, Pasal 1 bagian 1 | permen_Nomor_28_Tahun_2014.pdf | Pasal 1", "source_file": "permen_Nomor_28_Tahun_2014.pdf", "pasal_id": "Pasal 1", "rrf_score": 0.012658227848101266, "rerank_score": 0.6797122359275818, "text_preview": "Peraturan Menteri Ketenagakerjaan No. 28 Tahun 2014 tentang TATA CARA PEMBUATAN DAN PENGESAHAN PERATURAN PERUSAHAAN SERTA PEMBUATAN DAN PENDAFTARAN PERJANJIAN KERJA BERSAMA BAB I - Ketentuan Umum Pasal 1 bagian 1 1. Peraturan Perusahaan yang selanjutnya disingkat PP adalah peraturan yang dibuat secara tertulis oleh pengusaha yang memuat syarat-syarat kerja dan tata tertib perusahaan. 2. Perjanjian Kerja Bersama yang selanjutnya disingkat PKB adalah perjanjian yang merupakan hasil perundingan ant"}, {"rank": 6, "chunk_id": "8877ce6af30ffbbf7b922de381b1b7929324f379", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 1 | PP Nomor 35 Tahun 2021.pdf | Pasal 1", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 1", "rrf_score": 0.0125, "rerank_score": 0.6604538559913635, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 BAB I - Ketentuan Umum Pasal 1 Pekerja/Buruh dengan Pengusaha untuk mengadakan Hubungan Kerja dalam waktu tertentu atau untuk pekerjaan tertentu. 1. Perjanjian Kerja Waktu Tertentu (PKWT) yang selanjutnya disingkat PKWT adalah Perjanjian Kerja antara Pekerja/Buruh dengan Pengusaha untuk mengadakan Hubungan Kerja yang bersifat tetap. 12. Peraturan Perusahaan adalah peraturan yang dibuat secara tertulis oleh Pengusaha yang memuat syarat-syarat kerja dan tata "}, {"rank": 7, "chunk_id": "174a6caf0ddd3791ff66aa1e4b6d8417fc84c2e2", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 15 | PP Nomor 35 Tahun 2021.pdf | Pasal 15", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 15", "rrf_score": 0.028287841191066997, "rerank_score": 0.6388614773750305, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB II - Perjanjian Kerja Waktu Tertentu Bagian Ketiga - Pemberian Uang Kompensasi Pasal 15 (1) Pengusaha wajib memberikan uang kompensasi kepada Pekerja/Buruh yang hubungan kerjanya berdasarkan PKWT. (2) Pemberian uang kompensasi dilaksanakan pada saat berakhirnya PKWT. (3) Uang kompensasi sebagaimana dimaksud pada ayat (1) diberikan kepada Pek"}, {"rank": 8, "chunk_id": "f7929ba6d33c6ef53a454e08ee67b33bdbf1f821", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 9 | PP Nomor 35 Tahun 2021.pdf | Pasal 9", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 9", "rrf_score": 0.027219202898550725, "rerank_score": 0.5656158924102783, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB II - Perjanjian Kerja Waktu Tertentu Bagian Kedua - Pelaksanaan Perjanjian Kerja Waktu Tertentu Pasal 9 (1) PKWT berdasarkan selesainya suatu pekerjaan tertentu sebagaimana dimaksud dalam Pasal 5 ayat (21didasarkan atas kesepakatan para pihak yang dituangkan dalam Perjanjian Kerja. (2) Kesepakatan para pihak sebagaimana dimaksud pada ayat (1"}]</t>
         </is>
@@ -1078,32 +1095,32 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.7275232021013894</v>
+        <v>0.5961143044630687</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>fair</t>
         </is>
       </c>
       <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
         <v>0.6629842519760132</v>
       </c>
-      <c r="I6" t="n">
+      <c r="J6" t="n">
         <v>0.5</v>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>tertulis; bahasa Indonesia; bahasa asing</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>huruf latin; penafsiran; bahasa Indonesia berlaku</t>
         </is>
       </c>
-      <c r="L6" t="n">
-        <v>1</v>
-      </c>
       <c r="M6" t="n">
         <v>1</v>
       </c>
@@ -1117,51 +1134,54 @@
         <v>1</v>
       </c>
       <c r="Q6" t="n">
+        <v>1</v>
+      </c>
+      <c r="R6" t="n">
         <v>6</v>
       </c>
-      <c r="R6" t="n">
-        <v>1</v>
-      </c>
       <c r="S6" t="n">
+        <v>1</v>
+      </c>
+      <c r="T6" t="n">
         <v>0.1666666666666667</v>
       </c>
-      <c r="T6" t="n">
-        <v>1</v>
-      </c>
       <c r="U6" t="n">
+        <v>1</v>
+      </c>
+      <c r="V6" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="V6" t="n">
+      <c r="W6" t="n">
         <v>0</v>
       </c>
-      <c r="W6" t="n">
-        <v>1</v>
-      </c>
       <c r="X6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y6" t="n">
         <v>93</v>
       </c>
-      <c r="Y6" t="n">
-        <v>1</v>
-      </c>
       <c r="Z6" t="n">
-        <v>23.39311671257019</v>
-      </c>
-      <c r="AA6" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>23.19345831871033</v>
+      </c>
+      <c r="AB6" t="inlineStr">
         <is>
           <t>Qwen/Qwen3.5-9B</t>
         </is>
       </c>
-      <c r="AB6" t="inlineStr">
+      <c r="AC6" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 1 | PP Nomor 35 Tahun 2021.pdf | Pasal 1</t>
         </is>
       </c>
-      <c r="AC6" t="inlineStr">
+      <c r="AD6" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 1 | PP Nomor 35 Tahun 2021.pdf | Pasal 1 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 1 bagian 1 | PP Nomor 35 Tahun 2021.pdf | Pasal 1 || Peraturan Menteri Ketenagakerjaan No. 28 Tahun 2014, Pasal 1 bagian 1 | permen_Nomor_28_Tahun_2014.pdf | Pasal 1 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 18 | PP Nomor 35 Tahun 2021.pdf | Pasal 18 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 5 | PP Nomor 35 Tahun 2021.pdf | Pasal 5 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 13 | PP Nomor 35 Tahun 2021.pdf | Pasal 13 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 8 | PP Nomor 35 Tahun 2021.pdf | Pasal 8 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 15 | PP Nomor 35 Tahun 2021.pdf | Pasal 15</t>
         </is>
       </c>
-      <c r="AD6" t="inlineStr">
+      <c r="AE6" t="inlineStr">
         <is>
           <t>[{"rank": 1, "chunk_id": "8877ce6af30ffbbf7b922de381b1b7929324f379", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 1 | PP Nomor 35 Tahun 2021.pdf | Pasal 1", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 1", "rrf_score": 0.024211089320734534, "rerank_score": 0.3187059462070465, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 BAB I - Ketentuan Umum Pasal 1 Pekerja/Buruh dengan Pengusaha untuk mengadakan Hubungan Kerja dalam waktu tertentu atau untuk pekerjaan tertentu. 1. Perjanjian Kerja Waktu Tertentu (PKWT) yang selanjutnya disingkat PKWT adalah Perjanjian Kerja antara Pekerja/Buruh dengan Pengusaha untuk mengadakan Hubungan Kerja yang bersifat tetap. 12. Peraturan Perusahaan adalah peraturan yang dibuat secara tertulis oleh Pengusaha yang memuat syarat-syarat kerja dan tata "}, {"rank": 2, "chunk_id": "ef31e26ce2dd832602d5bb45532dde7319c92704", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 1 bagian 1 | PP Nomor 35 Tahun 2021.pdf | Pasal 1", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 1", "rrf_score": 0.010666666666666668, "rerank_score": 0.2704562246799469, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB I - Ketentuan Umum Pasal 1 bagian 1 Hubungan Kerja adalah hubungan antara Pengusaha 1 dengan Pekerja/Buruh berdasarkan Perjanjian Kerja, yang mempunyai unsur pekerjaan, Upah, dan perintah. 2 Pekerja/Buruh adalah setiap orang yang bekerja dengan menerima Upah atau imbalan dalam bentuk lain. 3 Pengusaha adalah: a. orang perseorangan, persekutu"}, {"rank": 3, "chunk_id": "f22a2c245e8ebfca109c15a979624ac02005ab52", "reference": "Peraturan Menteri Ketenagakerjaan No. 28 Tahun 2014, Pasal 1 bagian 1 | permen_Nomor_28_Tahun_2014.pdf | Pasal 1", "source_file": "permen_Nomor_28_Tahun_2014.pdf", "pasal_id": "Pasal 1", "rrf_score": 0.022576610381488428, "rerank_score": 0.2700200080871582, "text_preview": "Peraturan Menteri Ketenagakerjaan No. 28 Tahun 2014 tentang TATA CARA PEMBUATAN DAN PENGESAHAN PERATURAN PERUSAHAAN SERTA PEMBUATAN DAN PENDAFTARAN PERJANJIAN KERJA BERSAMA BAB I - Ketentuan Umum Pasal 1 bagian 1 1. Peraturan Perusahaan yang selanjutnya disingkat PP adalah peraturan yang dibuat secara tertulis oleh pengusaha yang memuat syarat-syarat kerja dan tata tertib perusahaan. 2. Perjanjian Kerja Bersama yang selanjutnya disingkat PKB adalah perjanjian yang merupakan hasil perundingan ant"}, {"rank": 4, "chunk_id": "f5ad73d152f752d54b479ccee3129c79c165136f", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 18 | PP Nomor 35 Tahun 2021.pdf | Pasal 18", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 18", "rrf_score": 0.02745920745920746, "rerank_score": 0.19767683744430542, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB III - Alih Daya Pasal 18 (1) Hubungan Kerja antara Perusahaan Alih Daya dengan Pekerja/Buruh yang dipekerjakan, didasarkan pada PKWT atau PKWTT. (2) PKWT atau PKWTT sebagaimana dimaksud pada ayat (1) harus dibuat secara tertulis. (3) Pelindungan Pekerja/Buruh, Upah, kesejahteraan, syarat kerja, dan perselisihan yang timbul dilaksanakan sesua"}, {"rank": 5, "chunk_id": "b9e022bdc1ce11e24d99e1801f0e6f5d4cad4178", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 5 | PP Nomor 35 Tahun 2021.pdf | Pasal 5", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 5", "rrf_score": 0.027813314380478557, "rerank_score": 0.1353786587715149, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB II - Perjanjian Kerja Waktu Tertentu Bagian Kedua - Pelaksanaan Perjanjian Kerja Waktu Tertentu Pasal 5 (1) PKWT berdasarkan jangka waktu sebagaimana dimaksud dalam Pasal 4 ayat (1) huruf a dibuat untuk pekerjaan tertentu yaitu: a. pekerjaan yang diperkirakan penyelesaiannya dalam waktu yang tidak terlalu lama; b. pekerjaan yang bersifat mus"}, {"rank": 6, "chunk_id": "f26c1f86b5008c251c1cf8a9613adbccd3284d8a", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 13 | PP Nomor 35 Tahun 2021.pdf | Pasal 13", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 13", "rrf_score": 0.025156494522691704, "rerank_score": 0.11836402118206024, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB II - Perjanjian Kerja Waktu Tertentu Bagian Kedua - Pelaksanaan Perjanjian Kerja Waktu Tertentu Pasal 13 PKWT paling sedikit memuat: a. nama, alamat Perusahaan, dan jenis usaha; b. nama, jenis kelamin, umur, dan alamat Pekerja/Buruh; c. jabatan atau jenis pekerjaan; d. tempat pekerjaan; e. besaran dan cara pembayaran Upah; f. hak dan kewajib"}, {"rank": 7, "chunk_id": "d09ac5ae28956298a98a70ced4c841956ab85b9e", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 8 | PP Nomor 35 Tahun 2021.pdf | Pasal 8", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 8", "rrf_score": 0.02852822580645161, "rerank_score": 0.09228933602571487, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB II - Perjanjian Kerja Waktu Tertentu Bagian Kedua - Pelaksanaan Perjanjian Kerja Waktu Tertentu Pasal 8 (1) PKWT berdasarkan jangka waktu sebagaimana dimaksud dalam Pasal 5 ayat (1) dapat dibuat untuk paling lama 5 (lima) tahun. (2) Dalam hal jangka waktu PKWT sebagaimana dimaksud pada ayat (1) akan berakhir dan pekerjaan yang dilaksanakan b"}, {"rank": 8, "chunk_id": "174a6caf0ddd3791ff66aa1e4b6d8417fc84c2e2", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 15 | PP Nomor 35 Tahun 2021.pdf | Pasal 15", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 15", "rrf_score": 0.029508196721311476, "rerank_score": 0.08778513967990875, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB II - Perjanjian Kerja Waktu Tertentu Bagian Ketiga - Pemberian Uang Kompensasi Pasal 15 (1) Pengusaha wajib memberikan uang kompensasi kepada Pekerja/Buruh yang hubungan kerjanya berdasarkan PKWT. (2) Pemberian uang kompensasi dilaksanakan pada saat berakhirnya PKWT. (3) Uang kompensasi sebagaimana dimaksud pada ayat (1) diberikan kepada Pek"}]</t>
         </is>
@@ -1197,7 +1217,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.9080977408091228</v>
+        <v>0.9297636111577352</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1205,20 +1225,20 @@
         </is>
       </c>
       <c r="H7" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="I7" t="n">
         <v>0.6428685188293457</v>
       </c>
-      <c r="I7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J7" t="inlineStr">
+      <c r="J7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" t="inlineStr">
         <is>
           <t>alih daya; badan hukum; perizinan berusaha; pemerintah pusat</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="n">
-        <v>1</v>
-      </c>
+      <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
         <v>1</v>
       </c>
@@ -1244,39 +1264,42 @@
         <v>1</v>
       </c>
       <c r="U7" t="n">
+        <v>1</v>
+      </c>
+      <c r="V7" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="V7" t="n">
-        <v>1</v>
-      </c>
       <c r="W7" t="n">
         <v>1</v>
       </c>
       <c r="X7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y7" t="n">
         <v>96</v>
       </c>
-      <c r="Y7" t="n">
-        <v>1</v>
-      </c>
       <c r="Z7" t="n">
-        <v>26.97086453437805</v>
-      </c>
-      <c r="AA7" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>27.51719379425049</v>
+      </c>
+      <c r="AB7" t="inlineStr">
         <is>
           <t>Qwen/Qwen3.5-9B</t>
         </is>
       </c>
-      <c r="AB7" t="inlineStr">
+      <c r="AC7" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 20 | PP Nomor 35 Tahun 2021.pdf | Pasal 20</t>
         </is>
       </c>
-      <c r="AC7" t="inlineStr">
+      <c r="AD7" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 20 | PP Nomor 35 Tahun 2021.pdf | Pasal 20 || Peraturan Menteri Ketenagakerjaan No. 7 Tahun 2026, Pasal 1 | permen_Nomor_7_Tahun_2026.pdf | Pasal 1 || Peraturan Menteri Ketenagakerjaan No. 7 Tahun 2026, Pasal 6 | permen_Nomor_7_Tahun_2026.pdf | Pasal 6 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 19 | PP Nomor 35 Tahun 2021.pdf | Pasal 19 || Peraturan Menteri Ketenagakerjaan No. 7 Tahun 2026, Pasal 4 | permen_Nomor_7_Tahun_2026.pdf | Pasal 4 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 1 | PP Nomor 35 Tahun 2021.pdf | Pasal 1 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 18 | PP Nomor 35 Tahun 2021.pdf | Pasal 18 || Peraturan Menteri Ketenagakerjaan No. 14 Tahun 2025, Pasal 5 | permen_Nomor_14_Tahun_2025.pdf | Pasal 5</t>
         </is>
       </c>
-      <c r="AD7" t="inlineStr">
+      <c r="AE7" t="inlineStr">
         <is>
           <t>[{"rank": 1, "chunk_id": "cb6e1dcf7fc13ca9cef282aec4e001fcaaae01a5", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 20 | PP Nomor 35 Tahun 2021.pdf | Pasal 20", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 20", "rrf_score": 0.028827444956477214, "rerank_score": 0.9584782123565674, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB III - Alih Daya Pasal 20 (1) Perusahaan Alih Daya harus berbentuk badan hukum dan wajib memenuhi perizinan berusaha yang diterbitkan oleh Pemerintah Pusat. (2) Syarat dan tata cara memperoleh perizinan berusaha dilaksanakan sesuai dengan ketentuan peraturan perundang-undangan mengenai norma, standar, prosedur, dan kriteria perrzinan berusaha"}, {"rank": 2, "chunk_id": "5df82deda8c676f6a34692c30c6a9fb736eef61e", "reference": "Peraturan Menteri Ketenagakerjaan No. 7 Tahun 2026, Pasal 1 | permen_Nomor_7_Tahun_2026.pdf | Pasal 1", "source_file": "permen_Nomor_7_Tahun_2026.pdf", "pasal_id": "Pasal 1", "rrf_score": 0.027188940092165898, "rerank_score": 0.9281668663024902, "text_preview": "Peraturan Menteri Ketenagakerjaan No. 7 Tahun 2026 tentang PEKERJAAN ALIH DAYA BAB I - Ketentuan Umum Pasal 1 1. Perusahaan adalah: a. setiap bentuk usaha yang berbadan hukum atau tidak, milik orang perseorangan, milik persekutuan, atau milik badan hukum, baik milik swasta maupun milik negara yang mempekerjakan pekerja/buruh dengan membayar upah atau imbalan dalam bentuk lain; b. usaha-usaha sosial dan usaha-usaha lain yang mempunyai pengurus dan mempekerjakan orang lain dengan membayar upah ata"}, {"rank": 3, "chunk_id": "18929ea2de6a962f9bbd6310ad35b936b34774f8", "reference": "Peraturan Menteri Ketenagakerjaan No. 7 Tahun 2026, Pasal 6 | permen_Nomor_7_Tahun_2026.pdf | Pasal 6", "source_file": "permen_Nomor_7_Tahun_2026.pdf", "pasal_id": "Pasal 6", "rrf_score": 0.02889344262295082, "rerank_score": 0.8871814012527466, "text_preview": "Peraturan Menteri Ketenagakerjaan No. 7 Tahun 2026 tentang PEKERJAAN ALIH DAYA BAB IV - Kewajiban Perusahaan Alih Daya Pasal 6 Perusahaan Alih Daya wajib memenuhi kewajiban sebagai pemegang perizinan berusaha bidang alih daya, yaitu: a. menerapkan standar keselamatan, kesehatan kerja, dan lingkungan; b. mencatatkan Perjanjian Alih Daya kepada Dinas; dan c. menjalankan kegiatan usaha paling lambat 1 (satu) tahun sejak perizinan berusaha diterbitkan."}, {"rank": 4, "chunk_id": "c37e9169eb345e26aee3a24bff36c8e486e2de6e", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 19 | PP Nomor 35 Tahun 2021.pdf | Pasal 19", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 19", "rrf_score": 0.027746212121212123, "rerank_score": 0.7376814484596252, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB III - Alih Daya Pasal 19 (1) Dalam hal Perusahaan Alih Daya mempekerjakan Pekerja/Buruh berdasarkan PKWT maka Perjanjian Kerja tersebut harus mensyaratkan pengalihan pelindungan hak bagi Pekerja/Buruh apabila terjadi pergantian Perusahaan Alih Daya dan sepanjang obyek pekerjaannya tetap ada. (2) Persyaratan... -t4- (2) Persyaratan pengalihan"}, {"rank": 5, "chunk_id": "33d126d9fe0c20600a194b2aef3e072aea252734", "reference": "Peraturan Menteri Ketenagakerjaan No. 7 Tahun 2026, Pasal 4 | permen_Nomor_7_Tahun_2026.pdf | Pasal 4", "source_file": "permen_Nomor_7_Tahun_2026.pdf", "pasal_id": "Pasal 4", "rrf_score": 0.02818070818070818, "rerank_score": 0.7321521043777466, "text_preview": "Peraturan Menteri Ketenagakerjaan No. 7 Tahun 2026 tentang PEKERJAAN ALIH DAYA BAB III - Perjanjian Alih Daya Pasal 4 (1) Perjanjian Alih Daya sebagaimana dimaksud dalam Pasal 2 paling sedikit memuat: a. pekerjaan yang dialihdayakan kepada Perusahaan Alih Daya; b. jangka waktu Perjanjian Alih Daya; c. lokasi pelaksanaan pekerjaan; d. jumlah pekerja/buruh alih daya; e. pelindungan dan hak pekerja/buruh alih daya paling sedikit meliputi upah, upah kerja lembur, waktu kerja dan waktu istirahat, cut"}, {"rank": 6, "chunk_id": "8877ce6af30ffbbf7b922de381b1b7929324f379", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 1 | PP Nomor 35 Tahun 2021.pdf | Pasal 1", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 1", "rrf_score": 0.010526315789473684, "rerank_score": 0.6110467910766602, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 BAB I - Ketentuan Umum Pasal 1 Pekerja/Buruh dengan Pengusaha untuk mengadakan Hubungan Kerja dalam waktu tertentu atau untuk pekerjaan tertentu. 1. Perjanjian Kerja Waktu Tertentu (PKWT) yang selanjutnya disingkat PKWT adalah Perjanjian Kerja antara Pekerja/Buruh dengan Pengusaha untuk mengadakan Hubungan Kerja yang bersifat tetap. 12. Peraturan Perusahaan adalah peraturan yang dibuat secara tertulis oleh Pengusaha yang memuat syarat-syarat kerja dan tata "}, {"rank": 7, "chunk_id": "f5ad73d152f752d54b479ccee3129c79c165136f", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 18 | PP Nomor 35 Tahun 2021.pdf | Pasal 18", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 18", "rrf_score": 0.028266269249875808, "rerank_score": 0.5461682677268982, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB III - Alih Daya Pasal 18 (1) Hubungan Kerja antara Perusahaan Alih Daya dengan Pekerja/Buruh yang dipekerjakan, didasarkan pada PKWT atau PKWTT. (2) PKWT atau PKWTT sebagaimana dimaksud pada ayat (1) harus dibuat secara tertulis. (3) Pelindungan Pekerja/Buruh, Upah, kesejahteraan, syarat kerja, dan perselisihan yang timbul dilaksanakan sesua"}, {"rank": 8, "chunk_id": "10dba7781414caf1ba9e5430f212979f8dc9f0fb", "reference": "Peraturan Menteri Ketenagakerjaan No. 14 Tahun 2025, Pasal 5 | permen_Nomor_14_Tahun_2025.pdf | Pasal 5", "source_file": "permen_Nomor_14_Tahun_2025.pdf", "pasal_id": "Pasal 5", "rrf_score": 0.027149321266968326, "rerank_score": 0.48328155279159546, "text_preview": "Peraturan Menteri Ketenagakerjaan No. 14 Tahun 2025 tentang STANDAR KEGIATAN USAHA DAN STANDAR PRODUK/JASA PADA PENYELENGGARAAN PERIZINAN BERUSAHA BERBASIS RISIKO SEKTOR KETENAGAKERJAAN BAB II - Standar Kegiatan Usaha Dan Pasal 5 Kewajiban PB sektor ketenagakerjaan untuk kegiatan usaha alih daya yang memiliki risiko rendah, meliputi: a. menerapkan standar Keselamatan, Kesehatan Kerja, dan Lingkungan; b. mencatatkan perjanjian alih daya kepada instansi yang berwenang; c. menjalankan kegiatan usah"}]</t>
         </is>
@@ -1313,7 +1336,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.8945549503962199</v>
+        <v>0.9159844358762106</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1321,24 +1344,24 @@
         </is>
       </c>
       <c r="H8" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="I8" t="n">
         <v>0.7176740169525146</v>
       </c>
-      <c r="I8" t="n">
+      <c r="J8" t="n">
         <v>0.8333333333333334</v>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>alih daya; upah; kesejahteraan; syarat kerja; tanggung jawab perusahaan alih daya</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>perlindungan pekerja</t>
         </is>
       </c>
-      <c r="L8" t="n">
-        <v>1</v>
-      </c>
       <c r="M8" t="n">
         <v>1</v>
       </c>
@@ -1364,39 +1387,42 @@
         <v>1</v>
       </c>
       <c r="U8" t="n">
+        <v>1</v>
+      </c>
+      <c r="V8" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="V8" t="n">
-        <v>1</v>
-      </c>
       <c r="W8" t="n">
         <v>1</v>
       </c>
       <c r="X8" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y8" t="n">
         <v>124</v>
       </c>
-      <c r="Y8" t="n">
-        <v>1</v>
-      </c>
       <c r="Z8" t="n">
-        <v>34.48432445526123</v>
-      </c>
-      <c r="AA8" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>34.01590514183044</v>
+      </c>
+      <c r="AB8" t="inlineStr">
         <is>
           <t>Qwen/Qwen3.5-9B</t>
         </is>
       </c>
-      <c r="AB8" t="inlineStr">
+      <c r="AC8" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 18 | PP Nomor 35 Tahun 2021.pdf | Pasal 18</t>
         </is>
       </c>
-      <c r="AC8" t="inlineStr">
+      <c r="AD8" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 18 | PP Nomor 35 Tahun 2021.pdf | Pasal 18 || Peraturan Menteri Ketenagakerjaan No. 7 Tahun 2026, Pasal 4 | permen_Nomor_7_Tahun_2026.pdf | Pasal 4 || Undang-Undang No. 13 Tahun 2003, Pasal 66 | UU_Nomor_13_Tahun_2003.pdf | Pasal 66 || Undang-Undang No. 2 Tahun 2004, Pasal 1 bagian 1 | UU_Nomor_2_Tahun_2004_2.pdf | Pasal 1 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 1 bagian 1 | PP Nomor 35 Tahun 2021.pdf | Pasal 1 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 19 | PP Nomor 35 Tahun 2021.pdf | Pasal 19 || Undang-Undang No. 13 Tahun 2003, Pasal 1 | UU_Nomor_13_Tahun_2003.pdf | Pasal 1 || Undang-Undang No. 2 Tahun 2004, Pasal 1 bagian 2 | UU_Nomor_2_Tahun_2004_2.pdf | Pasal 1</t>
         </is>
       </c>
-      <c r="AD8" t="inlineStr">
+      <c r="AE8" t="inlineStr">
         <is>
           <t>[{"rank": 1, "chunk_id": "f5ad73d152f752d54b479ccee3129c79c165136f", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 18 | PP Nomor 35 Tahun 2021.pdf | Pasal 18", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 18", "rrf_score": 0.02924378635642517, "rerank_score": 0.9980210065841675, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB III - Alih Daya Pasal 18 (1) Hubungan Kerja antara Perusahaan Alih Daya dengan Pekerja/Buruh yang dipekerjakan, didasarkan pada PKWT atau PKWTT. (2) PKWT atau PKWTT sebagaimana dimaksud pada ayat (1) harus dibuat secara tertulis. (3) Pelindungan Pekerja/Buruh, Upah, kesejahteraan, syarat kerja, dan perselisihan yang timbul dilaksanakan sesua"}, {"rank": 2, "chunk_id": "33d126d9fe0c20600a194b2aef3e072aea252734", "reference": "Peraturan Menteri Ketenagakerjaan No. 7 Tahun 2026, Pasal 4 | permen_Nomor_7_Tahun_2026.pdf | Pasal 4", "source_file": "permen_Nomor_7_Tahun_2026.pdf", "pasal_id": "Pasal 4", "rrf_score": 0.02909185532136352, "rerank_score": 0.9759954810142517, "text_preview": "Peraturan Menteri Ketenagakerjaan No. 7 Tahun 2026 tentang PEKERJAAN ALIH DAYA BAB III - Perjanjian Alih Daya Pasal 4 (1) Perjanjian Alih Daya sebagaimana dimaksud dalam Pasal 2 paling sedikit memuat: a. pekerjaan yang dialihdayakan kepada Perusahaan Alih Daya; b. jangka waktu Perjanjian Alih Daya; c. lokasi pelaksanaan pekerjaan; d. jumlah pekerja/buruh alih daya; e. pelindungan dan hak pekerja/buruh alih daya paling sedikit meliputi upah, upah kerja lembur, waktu kerja dan waktu istirahat, cut"}, {"rank": 3, "chunk_id": "163fa4795c1e6b8c793f23e2ff566653eb57477d", "reference": "Undang-Undang No. 13 Tahun 2003, Pasal 66 | UU_Nomor_13_Tahun_2003.pdf | Pasal 66", "source_file": "UU_Nomor_13_Tahun_2003.pdf", "pasal_id": "Pasal 66", "rrf_score": 0.025723738626964435, "rerank_score": 0.964897871017456, "text_preview": "Undang-Undang No. 13 Tahun 2003 tentang KETENAGAKERJAAN BAB IX - Hubungan Kerja Pasal 66 (1) Pekerja/buruh dari perusahaan penyedia jasa pekerja/buruh tidak boleh digunakan oleh pemberi kerja untuk melaksanakan kegiatan pokok atau kegiatan yang berhubungan langsung dengan proses produksi, kecuali untuk kegiatan jasa penunjang atau kegiatan yang tidak berhubungan langsung dengan proses produksi. (2) Penyedia jasa pekerja/buruh untuk kegiatan jasa penunjang atau kegiatan yang tidak berhubungan lan"}, {"rank": 4, "chunk_id": "781d93e40123c33a1aa29554645d31ec5b4263cb", "reference": "Undang-Undang No. 2 Tahun 2004, Pasal 1 bagian 1 | UU_Nomor_2_Tahun_2004_2.pdf | Pasal 1", "source_file": "UU_Nomor_2_Tahun_2004_2.pdf", "pasal_id": "Pasal 1", "rrf_score": 0.012121212121212121, "rerank_score": 0.9368283152580261, "text_preview": "Undang-Undang No. 2 Tahun 2004 tentang PENYELESAIAN PERSELISIHAN HUBUNGAN INDUSTRIAL BAB I - Ketentuan Umum Pasal 1 bagian 1 1. Perselisihan Hubungan Industrial adalah perbedaan pendapat yang mengakibatkan pertentangan antara pengusaha atau gabungan pengusaha dengan pekerja/ buruh atau serikat pekerja/serikat buruh karena adanya perselisihan mengenai hak, perselisihan kepentingan, perselisihan pemutusan hubungan kerja dan perselisihan antar serikat pekerja/serikat buruh dalam satu perusahaan. 2."}, {"rank": 5, "chunk_id": "ef31e26ce2dd832602d5bb45532dde7319c92704", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 1 bagian 1 | PP Nomor 35 Tahun 2021.pdf | Pasal 1", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 1", "rrf_score": 0.0125, "rerank_score": 0.9364674687385559, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB I - Ketentuan Umum Pasal 1 bagian 1 Hubungan Kerja adalah hubungan antara Pengusaha 1 dengan Pekerja/Buruh berdasarkan Perjanjian Kerja, yang mempunyai unsur pekerjaan, Upah, dan perintah. 2 Pekerja/Buruh adalah setiap orang yang bekerja dengan menerima Upah atau imbalan dalam bentuk lain. 3 Pengusaha adalah: a. orang perseorangan, persekutu"}, {"rank": 6, "chunk_id": "c37e9169eb345e26aee3a24bff36c8e486e2de6e", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 19 | PP Nomor 35 Tahun 2021.pdf | Pasal 19", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 19", "rrf_score": 0.02447516641065028, "rerank_score": 0.9330078959465027, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB III - Alih Daya Pasal 19 (1) Dalam hal Perusahaan Alih Daya mempekerjakan Pekerja/Buruh berdasarkan PKWT maka Perjanjian Kerja tersebut harus mensyaratkan pengalihan pelindungan hak bagi Pekerja/Buruh apabila terjadi pergantian Perusahaan Alih Daya dan sepanjang obyek pekerjaannya tetap ada. (2) Persyaratan... -t4- (2) Persyaratan pengalihan"}, {"rank": 7, "chunk_id": "9b2208c51b01b038d49bc5e27a9be763c2bd1fd8", "reference": "Undang-Undang No. 13 Tahun 2003, Pasal 1 | UU_Nomor_13_Tahun_2003.pdf | Pasal 1", "source_file": "UU_Nomor_13_Tahun_2003.pdf", "pasal_id": "Pasal 1", "rrf_score": 0.011594202898550725, "rerank_score": 0.9108238220214844, "text_preview": "Undang-Undang No. 13 Tahun 2003 BAB I - Ketentuan Umum Pasal 1 sesuai dengan kebutuhannya. 13. Tenaga kerja asing adalah warga negara asing pemegang visa dengan maksud bekerja di wilayah Indonesia. 14. Perjanjian kerja adalah perjanjian antara pekerja/buruh dengan pengusaha atau pemberi kerja yang memuat syarat-syarat kerja, hak, dan kewajiban para pihak. 15. Hubungan kerja adalah hubungan antara pengusaha dengan pekerja/buruh berdasarkan perjanjian kerja, yang mempunyai unsur pekerjaan, upah, d"}, {"rank": 8, "chunk_id": "97d2043680990b91762b13e1e71f9b6c4f093646", "reference": "Undang-Undang No. 2 Tahun 2004, Pasal 1 bagian 2 | UU_Nomor_2_Tahun_2004_2.pdf | Pasal 1", "source_file": "UU_Nomor_2_Tahun_2004_2.pdf", "pasal_id": "Pasal 1", "rrf_score": 0.008, "rerank_score": 0.7387803196907043, "text_preview": "Undang-Undang No. 2 Tahun 2004 tentang PENYELESAIAN PERSELISIHAN HUBUNGAN INDUSTRIAL BAB I - Ketentuan Umum Pasal 1 bagian 2 pemutusan hubungan kerja, dan perselisihan antar serikat pekerja/serikat buruh hanya dalam satu perusahaan melalui musyawarah yang ditengahi oleh seorang atau lebih mediator yang netral . 12. Mediator Hubungan Industrial yang selanjutnya disebut mediator adalah pegawai instansi pemerintah yang bertanggung jawab di bidang ketenagakerjaan yang memenuhi syarat-syarat sebagai "}]</t>
         </is>
@@ -1431,7 +1457,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.968933048248291</v>
+        <v>0.9788179874420168</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1439,20 +1465,20 @@
         </is>
       </c>
       <c r="H9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" t="n">
         <v>0.8587865829467773</v>
       </c>
-      <c r="I9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J9" t="inlineStr">
+      <c r="J9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" t="inlineStr">
         <is>
           <t>7 jam sehari; 40 jam seminggu; 6 hari kerja; 8 jam sehari; 5 hari kerja</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="n">
-        <v>1</v>
-      </c>
+      <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
         <v>1</v>
       </c>
@@ -1487,30 +1513,33 @@
         <v>1</v>
       </c>
       <c r="X9" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y9" t="n">
         <v>56</v>
       </c>
-      <c r="Y9" t="n">
-        <v>1</v>
-      </c>
       <c r="Z9" t="n">
-        <v>16.45044612884521</v>
-      </c>
-      <c r="AA9" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>16.22343039512634</v>
+      </c>
+      <c r="AB9" t="inlineStr">
         <is>
           <t>Qwen/Qwen3.5-9B</t>
         </is>
       </c>
-      <c r="AB9" t="inlineStr">
+      <c r="AC9" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 21 | PP Nomor 35 Tahun 2021.pdf | Pasal 21</t>
         </is>
       </c>
-      <c r="AC9" t="inlineStr">
+      <c r="AD9" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 21 | PP Nomor 35 Tahun 2021.pdf | Pasal 21 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 1 bagian 1 | PP Nomor 35 Tahun 2021.pdf | Pasal 1 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 31 | PP Nomor 35 Tahun 2021.pdf | Pasal 31 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 33 | PP Nomor 35 Tahun 2021.pdf | Pasal 33 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 26 | PP Nomor 35 Tahun 2021.pdf | Pasal 26 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 23 | PP Nomor 35 Tahun 2021.pdf | Pasal 23 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 51 | PP Nomor 35 Tahun 2021.pdf | Pasal 51 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 25 | PP Nomor 35 Tahun 2021.pdf | Pasal 25</t>
         </is>
       </c>
-      <c r="AD9" t="inlineStr">
+      <c r="AE9" t="inlineStr">
         <is>
           <t>[{"rank": 1, "chunk_id": "a26e961461e6e8119de5fce3346cb284238e41aa", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 21 | PP Nomor 35 Tahun 2021.pdf | Pasal 21", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 21", "rrf_score": 0.027233065442020664, "rerank_score": 0.9900931715965271, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB IV - Waktu Kerja Dan Waktu Istirahat Bagian Kesatu - Umum Pasal 21 (1) Setiap Pengusaha wajib melaksanakan ketentuan waktu kerja. (2) Waktu kerja sebagaimana dimaksud pada ayat (1) meliputi: a. 7 (tujuh) jam 1 (satu) hari dan 40 (empat puluh) jam 1 (satu) minggu untuk 6 (enam) hari kerja dalam 1 (satu) minggu; atau ... b.8(delapan) b. 8 (del"}, {"rank": 2, "chunk_id": "ef31e26ce2dd832602d5bb45532dde7319c92704", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 1 bagian 1 | PP Nomor 35 Tahun 2021.pdf | Pasal 1", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 1", "rrf_score": 0.02202029380584583, "rerank_score": 0.9810625910758972, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB I - Ketentuan Umum Pasal 1 bagian 1 Hubungan Kerja adalah hubungan antara Pengusaha 1 dengan Pekerja/Buruh berdasarkan Perjanjian Kerja, yang mempunyai unsur pekerjaan, Upah, dan perintah. 2 Pekerja/Buruh adalah setiap orang yang bekerja dengan menerima Upah atau imbalan dalam bentuk lain. 3 Pengusaha adalah: a. orang perseorangan, persekutu"}, {"rank": 3, "chunk_id": "492115371e1d77b17f8ffafd13c1273f574afe86", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 31 | PP Nomor 35 Tahun 2021.pdf | Pasal 31", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 31", "rrf_score": 0.0125, "rerank_score": 0.9635045528411865, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 BAB IV - Waktu Kerja Dan Waktu Istirahat Bagian Keempat - Upah Kerja Lembur Pasal 31 (1) Perusahaan yang mempekerjakan Pekerja/Buruh melebihi waktu kerja sebagaimana dimaksud dalam Pasal 2l ayat (2) wajib membayar Upah Kerja Lembur dengan ketentuan: a.untuk... REPUBLIK INDONESIA -L9a. untuk ja- kerja lembur pertama sebesar 1,5 (satu koma lima) kali Upah sejam; dan b. untuk setiap ja- kerja lembur berikutnya, sebesar 2 (dua) kali Upah sejam. (2) Perusahaan y"}, {"rank": 4, "chunk_id": "0b3b32e95a4a332bf8b376851b0d5b0b6df7f250", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 33 | PP Nomor 35 Tahun 2021.pdf | Pasal 33", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 33", "rrf_score": 0.02270891581236409, "rerank_score": 0.9559402465820312, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB IV - Waktu Kerja Dan Waktu Istirahat Bagian Keempat - Upah Kerja Lembur Pasal 33 (1) Dalam hal Upah Pekerja/Buruh dibayar secara harian maka penghitungan besarnya Upah sebulan dilaksanakan dengan ketentuan : a. Upah sehari dikalikan 25 (dua puluh lima), bagi Pekerja/Buruh yang bekerja 6 (enam) hari kerja dalam 1 (satu) minggu; atau b. Upah s"}, {"rank": 5, "chunk_id": "6d31a9753078e43bb8b72d5e97cdaf16f4dd0caa", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 26 | PP Nomor 35 Tahun 2021.pdf | Pasal 26", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 26", "rrf_score": 0.027204253433761632, "rerank_score": 0.8358643651008606, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB IV - Waktu Kerja Dan Waktu Istirahat Bagian Kedua - Waktu Kerja Pada Sektor Usaha Atau Pekerjaan Tertentu Pasal 26 (1) Waktu Kerja Lembur hanya dapat dilakukan paling lama 4 (empat)jam dalam 1 (satu) hari dan 18 (delapan belas) jam dalam 1 (satu) minggu. (2) Ketentuan Waktu Kerja Lembur sebagaimana dimaksud pada ayat (1) tidak termasuk kerja"}, {"rank": 6, "chunk_id": "0498210c60df95bb270e456136a10c70a25f53fc", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 23 | PP Nomor 35 Tahun 2021.pdf | Pasal 23", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 23", "rrf_score": 0.023795079204583756, "rerank_score": 0.8067201972007751, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB IV - Waktu Kerja Dan Waktu Istirahat Bagian Kedua - Waktu Kerja Pada Sektor Usaha Atau Pekerjaan Tertentu Pasal 23 (1) Perusahaan pada sektor usaha atau pekerjaan tertentu dapat menerapkan waktu kerja yang kurang atau lebih dari ketentuan sebagaimana dimaksud dalam Pasal 21 ayat (21. (2) Perusahaan pada sektor usaha atau pekerjaan tertentu y"}, {"rank": 7, "chunk_id": "9883382497b3ac0974b8583c8ade65b7174eaa8a", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 51 | PP Nomor 35 Tahun 2021.pdf | Pasal 51", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 51", "rrf_score": 0.01953216374269006, "rerank_score": 0.6944249868392944, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kedua - Hak Akibat Pemutusan Hubungan Kerja Pasal 51 Pengusaha dapat melakukan Pemutusan Hubungan Kerja terhadap Pekerja/Buruh karena alasan Pekerja/Buruh mangkir selama 5 (lima) hari kerja atau lebih berturut-turut tanpa keterangan secara tertulis yang dilengkapi dengan bukti yang sah dan telah dipanggil "}, {"rank": 8, "chunk_id": "c90e53303d2c82df649198dc556971a9b2c099d5", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 25 | PP Nomor 35 Tahun 2021.pdf | Pasal 25", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 25", "rrf_score": 0.02575158227848101, "rerank_score": 0.6750662326812744, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB IV - Waktu Kerja Dan Waktu Istirahat Bagian Kedua - Waktu Kerja Pada Sektor Usaha Atau Pekerjaan Tertentu Pasal 25 (1) Pelaksanaan waktu kerja dan jam kerja bagi Pekerja/Buruh yang dipekerjakan pada sektor usaha atau pekerjaan tertentu yang menerapkan waktu kerja kurang dari ketentuan sebagaimana dimaksud dalam Pasal 2l ayat (21, diatur dala"}]</t>
         </is>
@@ -1546,7 +1575,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.7567363161132449</v>
+        <v>0.7361297393412818</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1554,24 +1583,24 @@
         </is>
       </c>
       <c r="H10" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I10" t="n">
         <v>0.8011823892593384</v>
       </c>
-      <c r="I10" t="n">
+      <c r="J10" t="n">
         <v>0.5</v>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>persetujuan pekerja; melebihi waktu kerja</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>lembur; perintah kerja lembur</t>
         </is>
       </c>
-      <c r="L10" t="n">
-        <v>1</v>
-      </c>
       <c r="M10" t="n">
         <v>1</v>
       </c>
@@ -1585,51 +1614,54 @@
         <v>1</v>
       </c>
       <c r="Q10" t="n">
+        <v>1</v>
+      </c>
+      <c r="R10" t="n">
         <v>7</v>
       </c>
-      <c r="R10" t="n">
+      <c r="S10" t="n">
         <v>2</v>
       </c>
-      <c r="S10" t="n">
+      <c r="T10" t="n">
         <v>0.1428571428571428</v>
       </c>
-      <c r="T10" t="n">
+      <c r="U10" t="n">
         <v>0.5</v>
       </c>
-      <c r="U10" t="n">
+      <c r="V10" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="V10" t="n">
+      <c r="W10" t="n">
         <v>0</v>
       </c>
-      <c r="W10" t="n">
-        <v>1</v>
-      </c>
       <c r="X10" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y10" t="n">
         <v>72</v>
       </c>
-      <c r="Y10" t="n">
-        <v>1</v>
-      </c>
       <c r="Z10" t="n">
-        <v>21.14453887939453</v>
-      </c>
-      <c r="AA10" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>20.82744526863098</v>
+      </c>
+      <c r="AB10" t="inlineStr">
         <is>
           <t>Qwen/Qwen3.5-9B</t>
         </is>
       </c>
-      <c r="AB10" t="inlineStr">
+      <c r="AC10" t="inlineStr">
         <is>
           <t>Undang-Undang No. 13 Tahun 2003, Pasal 78 | UU_Nomor_13_Tahun_2003.pdf | Pasal 78</t>
         </is>
       </c>
-      <c r="AC10" t="inlineStr">
+      <c r="AD10" t="inlineStr">
         <is>
           <t>Undang-Undang No. 13 Tahun 2003, Pasal 78 | UU_Nomor_13_Tahun_2003.pdf | Pasal 78 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 27 | PP Nomor 35 Tahun 2021.pdf | Pasal 27 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 1 bagian 1 | PP Nomor 35 Tahun 2021.pdf | Pasal 1 || Undang-Undang No. 13 Tahun 2003, Pasal 76 | UU_Nomor_13_Tahun_2003.pdf | Pasal 76 || Undang-Undang No. 13 Tahun 2003, Pasal 85 | UU_Nomor_13_Tahun_2003.pdf | Pasal 85 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 31 | PP Nomor 35 Tahun 2021.pdf | Pasal 31 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 28 | PP Nomor 35 Tahun 2021.pdf | Pasal 28 || Undang-Undang No. 13 Tahun 2003, Pasal 71 | UU_Nomor_13_Tahun_2003.pdf | Pasal 71</t>
         </is>
       </c>
-      <c r="AD10" t="inlineStr">
+      <c r="AE10" t="inlineStr">
         <is>
           <t>[{"rank": 1, "chunk_id": "e4b526d9a4e019074799ac0cbfcf97f73efc2948", "reference": "Undang-Undang No. 13 Tahun 2003, Pasal 78 | UU_Nomor_13_Tahun_2003.pdf | Pasal 78", "source_file": "UU_Nomor_13_Tahun_2003.pdf", "pasal_id": "Pasal 78", "rrf_score": 0.029508196721311476, "rerank_score": 0.9835985898971558, "text_preview": "Undang-Undang No. 13 Tahun 2003 tentang KETENAGAKERJAAN BAB X - Perlindungan, Pengupahan, Bagian Kesatu - Perlindungan Paragraf 4 - Waktu Kerja Pasal 78 (1) Pengusaha yang mempekerjakan pekerja/buruh melebihi waktu kerja sebagaimana dimaksud dalam Pasal 77 ayat (2) harus memenuhi syarat: a. ada persetujuan pekerja/buruh yang bersangkutan; dan b. waktu kerja lembur hanya dapat dilakukan paling banyak 3 (tiga) jam dalam 1 (satu) hari dan 14 (empat belas) jam dalam 1 (satu) minggu. (2) Pengusaha ya"}, {"rank": 2, "chunk_id": "b9209bf7a1c7bbebaeb65a2e30ee401466e736f9", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 27 | PP Nomor 35 Tahun 2021.pdf | Pasal 27", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 27", "rrf_score": 0.024140279196458975, "rerank_score": 0.8479360938072205, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB IV - Waktu Kerja Dan Waktu Istirahat Bagian Kedua - Waktu Kerja Pada Sektor Usaha Atau Pekerjaan Tertentu Pasal 27 (1) Pengusaha yang mempekerjakan Pekerja/Buruh melebihi waktu kerja sebagaimana dimaksud dalam Pasal 2l ayat (2), wajib membayar Upah Kerja Lembur. (2) Kewajiban membayar Upah Kerja Lembur dikecualikan bagi Pekerja/Buruh dalam g"}, {"rank": 3, "chunk_id": "ef31e26ce2dd832602d5bb45532dde7319c92704", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 1 bagian 1 | PP Nomor 35 Tahun 2021.pdf | Pasal 1", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 1", "rrf_score": 0.024965920155793575, "rerank_score": 0.5778697729110718, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB I - Ketentuan Umum Pasal 1 bagian 1 Hubungan Kerja adalah hubungan antara Pengusaha 1 dengan Pekerja/Buruh berdasarkan Perjanjian Kerja, yang mempunyai unsur pekerjaan, Upah, dan perintah. 2 Pekerja/Buruh adalah setiap orang yang bekerja dengan menerima Upah atau imbalan dalam bentuk lain. 3 Pengusaha adalah: a. orang perseorangan, persekutu"}, {"rank": 4, "chunk_id": "d6916991ef6895835aca7e9537047b42b65e91be", "reference": "Undang-Undang No. 13 Tahun 2003, Pasal 76 | UU_Nomor_13_Tahun_2003.pdf | Pasal 76", "source_file": "UU_Nomor_13_Tahun_2003.pdf", "pasal_id": "Pasal 76", "rrf_score": 0.011111111111111112, "rerank_score": 0.5664456486701965, "text_preview": "Undang-Undang No. 13 Tahun 2003 tentang KETENAGAKERJAAN BAB X - Perlindungan, Pengupahan, Bagian Kesatu - Perlindungan Paragraf 3 - Perempuan Pasal 76 (1) Pekerja/buruh perempuan yang berumur kurang dari 18 (delapan belas) tahun dilarang dipekerjakan antara pukul 23.00 s.d. 07.00. (2) Pengusaha dilarang mempekerjakan pekerja/buruh perempuan hamil yang menurut keterangan dokter berbahaya bagi kesehatan dan keselamatan kandungannya maupun dirinya apabila bekerja antara pukul 23.00 s.d. pukul 07.00"}, {"rank": 5, "chunk_id": "df6a00e38ac0410976b3943e0b52a76bd00423d3", "reference": "Undang-Undang No. 13 Tahun 2003, Pasal 85 | UU_Nomor_13_Tahun_2003.pdf | Pasal 85", "source_file": "UU_Nomor_13_Tahun_2003.pdf", "pasal_id": "Pasal 85", "rrf_score": 0.01891595347816546, "rerank_score": 0.5377025604248047, "text_preview": "Undang-Undang No. 13 Tahun 2003 tentang KETENAGAKERJAAN BAB X - Perlindungan, Pengupahan, Bagian Kesatu - Perlindungan Paragraf 4 - Waktu Kerja Pasal 85 (1) Pekerja/buruh tidak wajib bekerja pada hari-hari libur resmi. (2) Pengusaha dapat mempekerjakan pekerja/buruh untuk bekerja pada hari-hari libur resmi apabila jenis dan sifat pekerjaan tersebut harus dilaksanakan atau dijalankan secara terus-menerus atau pada keadaan lain berdasarkan kesepakatan antara pekerja/buruh dengan pengusaha. (3) Pen"}, {"rank": 6, "chunk_id": "492115371e1d77b17f8ffafd13c1273f574afe86", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 31 | PP Nomor 35 Tahun 2021.pdf | Pasal 31", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 31", "rrf_score": 0.023429541595925297, "rerank_score": 0.48880690336227417, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 BAB IV - Waktu Kerja Dan Waktu Istirahat Bagian Keempat - Upah Kerja Lembur Pasal 31 (1) Perusahaan yang mempekerjakan Pekerja/Buruh melebihi waktu kerja sebagaimana dimaksud dalam Pasal 2l ayat (2) wajib membayar Upah Kerja Lembur dengan ketentuan: a.untuk... REPUBLIK INDONESIA -L9a. untuk ja- kerja lembur pertama sebesar 1,5 (satu koma lima) kali Upah sejam; dan b. untuk setiap ja- kerja lembur berikutnya, sebesar 2 (dua) kali Upah sejam. (2) Perusahaan y"}, {"rank": 7, "chunk_id": "6d5ca945a606951f3c4ddc676a841934a255f78c", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 28 | PP Nomor 35 Tahun 2021.pdf | Pasal 28", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 28", "rrf_score": 0.028827444956477214, "rerank_score": 0.2691859006881714, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB IV - Waktu Kerja Dan Waktu Istirahat Bagian Kedua - Waktu Kerja Pada Sektor Usaha Atau Pekerjaan Tertentu Pasal 28 (1) Untuk melaksanakan Waktu Kerja Lembur harus ada perintah dari Pengusaha dan persetujuan dari Pekerja/Buruh yang bersangkutan secara tertulis dan/atau melalui media digital. (2) Perintah REPUBLIK INDONESI,A. (2) Perintah dan "}, {"rank": 8, "chunk_id": "cc06182a37d69c9772c0e38079e20b75682ee3f3", "reference": "Undang-Undang No. 13 Tahun 2003, Pasal 71 | UU_Nomor_13_Tahun_2003.pdf | Pasal 71", "source_file": "UU_Nomor_13_Tahun_2003.pdf", "pasal_id": "Pasal 71", "rrf_score": 0.008791208791208791, "rerank_score": 0.2443213164806366, "text_preview": "Undang-Undang No. 13 Tahun 2003 tentang KETENAGAKERJAAN BAB X - Perlindungan, Pengupahan, Bagian Kesatu - Perlindungan Paragraf 2 - Anak Pasal 71 (1) Anak dapat melakukan pekerjaan untuk mengembangkan bakat dan minatnya. (2) Pengusaha yang mempekerjakan anak sebagaimana dimaksud dalam ayat (1) wajib memenuhi syarat : a. di bawah pengawasan langsung dari orang tua atau wali; b. waktu kerja paling lama 3 (tiga) jam sehari; dan c. kondisi dan lingkungan kerja tidak mengganggu perkembangan fisik, me"}]</t>
         </is>
@@ -1667,7 +1699,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0.8573137124379475</v>
+        <v>0.8868805615107219</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1675,24 +1707,24 @@
         </is>
       </c>
       <c r="H11" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="I11" t="n">
         <v>0.7680926322937012</v>
       </c>
-      <c r="I11" t="n">
+      <c r="J11" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>surat peringatan pertama; kedua; ketiga; uang penggantian hak</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>setengah kali pesangon; satu kali uang penghargaan masa kerja</t>
         </is>
       </c>
-      <c r="L11" t="n">
-        <v>1</v>
-      </c>
       <c r="M11" t="n">
         <v>1</v>
       </c>
@@ -1706,51 +1738,54 @@
         <v>1</v>
       </c>
       <c r="Q11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R11" t="n">
         <v>2</v>
       </c>
       <c r="S11" t="n">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="T11" t="n">
         <v>0.5</v>
       </c>
       <c r="U11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="V11" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="V11" t="n">
-        <v>1</v>
-      </c>
       <c r="W11" t="n">
         <v>1</v>
       </c>
       <c r="X11" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y11" t="n">
         <v>165</v>
       </c>
-      <c r="Y11" t="n">
-        <v>1</v>
-      </c>
       <c r="Z11" t="n">
-        <v>45.17784094810486</v>
-      </c>
-      <c r="AA11" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>44.57093548774719</v>
+      </c>
+      <c r="AB11" t="inlineStr">
         <is>
           <t>Qwen/Qwen3.5-9B</t>
         </is>
       </c>
-      <c r="AB11" t="inlineStr">
+      <c r="AC11" t="inlineStr">
         <is>
           <t>Undang-Undang No. 13 Tahun 2003, Pasal 161 | UU_Nomor_13_Tahun_2003.pdf | Pasal 161</t>
         </is>
       </c>
-      <c r="AC11" t="inlineStr">
+      <c r="AD11" t="inlineStr">
         <is>
           <t>Undang-Undang No. 13 Tahun 2003, Pasal 161 | UU_Nomor_13_Tahun_2003.pdf | Pasal 161 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 52 | PP Nomor 35 Tahun 2021.pdf | Pasal 52 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 36 | PP Nomor 35 Tahun 2021.pdf | Pasal 36 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 50 | PP Nomor 35 Tahun 2021.pdf | Pasal 50 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 51 | PP Nomor 35 Tahun 2021.pdf | Pasal 51 || Undang-Undang No. 13 Tahun 2003, Pasal 168 | UU_Nomor_13_Tahun_2003.pdf | Pasal 168 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 45 | PP Nomor 35 Tahun 2021.pdf | Pasal 45 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 54 | PP Nomor 35 Tahun 2021.pdf | Pasal 54</t>
         </is>
       </c>
-      <c r="AD11" t="inlineStr">
+      <c r="AE11" t="inlineStr">
         <is>
           <t>[{"rank": 1, "chunk_id": "56805803f10f2865010ad9be0e01a7a31f697222", "reference": "Undang-Undang No. 13 Tahun 2003, Pasal 161 | UU_Nomor_13_Tahun_2003.pdf | Pasal 161", "source_file": "UU_Nomor_13_Tahun_2003.pdf", "pasal_id": "Pasal 161", "rrf_score": 0.029296668429402435, "rerank_score": 0.9730236530303955, "text_preview": "Undang-Undang No. 13 Tahun 2003 tentang KETENAGAKERJAAN BAB XII - Pemutusan Hubungan Kerja Pasal 161 (1) Dalam hal pekerja/buruh melakukan pelanggaran ketentuan yang diatur dalam perjanjian kerja, peraturan perusahaan atau perjanjian kerja bersama, pengusaha dapat melakukan pemutusan hubungan kerja, setelah kepada pekerja/buruh yang bersangkutan diberikan surat peringatan pertama, kedua, dan ketiga secara berturutturut. (2) Surat peringatan sebagaimana dimaksud dalam ayat (1) masing-masing berla"}, {"rank": 2, "chunk_id": "6342df2412f32ef274fc7204bb3dba645ea81370", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 52 | PP Nomor 35 Tahun 2021.pdf | Pasal 52", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 52", "rrf_score": 0.02924378635642517, "rerank_score": 0.9546220898628235, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kedua - Hak Akibat Pemutusan Hubungan Kerja Pasal 52 (1) Pengusaha dapat melakukan Pemutusan Hubungan Kerja terhadap Pekerja/Buruh karena alasan Pekerja/Buruh melakukan pelanggaran ketentuan yang diatur dalam Perjanjian Kerja, Peraturan Perusahaan, atau Perjanjian Kerja Bersama dan sebelumnya telah diberik"}, {"rank": 3, "chunk_id": "654617c9d52f8988bd188f0984852fd554a2cc5b", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 36 | PP Nomor 35 Tahun 2021.pdf | Pasal 36", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 36", "rrf_score": 0.011764705882352941, "rerank_score": 0.8047511577606201, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kesatu - Tata Cara Pemutusan Hubungan Kerja Pasal 36 Pemutusan Hubungan Kerja dapat terjadi karena alasan: a. Perusahaan melakukan penggabungan, peleburan, pengambilalihan, atau pemisahan Perusahaan dan Pekerja/Buruh tidak bersedia melanjutkan Hubungan Kerja atau Pengusaha tidak bersedia menerima Pekerja/B"}, {"rank": 4, "chunk_id": "061320f3b82f07db7ec06e98be7998663c14fa6c", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 50 | PP Nomor 35 Tahun 2021.pdf | Pasal 50", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 50", "rrf_score": 0.021115593267492003, "rerank_score": 0.1765781193971634, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kedua - Hak Akibat Pemutusan Hubungan Kerja Pasal 50 Pekerja/Buruh yang mengundurkan diri atas kemauan sendiri dan memenuhi syarat sebagaimana dimaksud dalam Pasal 36 huruf i, berhak atas: a. uang penggantian hak sesuai ketentuan Pasal 40 ayat (4); dan b. uang pisah yang besarannya diatur dalam Perjanjian "}, {"rank": 5, "chunk_id": "9883382497b3ac0974b8583c8ade65b7174eaa8a", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 51 | PP Nomor 35 Tahun 2021.pdf | Pasal 51", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 51", "rrf_score": 0.021924735980960883, "rerank_score": 0.1656203418970108, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kedua - Hak Akibat Pemutusan Hubungan Kerja Pasal 51 Pengusaha dapat melakukan Pemutusan Hubungan Kerja terhadap Pekerja/Buruh karena alasan Pekerja/Buruh mangkir selama 5 (lima) hari kerja atau lebih berturut-turut tanpa keterangan secara tertulis yang dilengkapi dengan bukti yang sah dan telah dipanggil "}, {"rank": 6, "chunk_id": "742e4669283c3b5296fba9dea7c1aa1d945da69e", "reference": "Undang-Undang No. 13 Tahun 2003, Pasal 168 | UU_Nomor_13_Tahun_2003.pdf | Pasal 168", "source_file": "UU_Nomor_13_Tahun_2003.pdf", "pasal_id": "Pasal 168", "rrf_score": 0.019403335682405452, "rerank_score": 0.15252389013767242, "text_preview": "Undang-Undang No. 13 Tahun 2003 tentang KETENAGAKERJAAN BAB XII - Pemutusan Hubungan Kerja Pasal 168 (1) Pekerja/buruh yang mangkir selama 5 (lima) hari kerja atau lebih berturut-turut tanpa keterangan secara tertulis yang dilengkapi dengan bukti yang sah dan telah dipanggil oleh pengusaha 2 (dua) kali secara patut dan tertulis dapat diputus hubungan kerjanya karena dikualifikasikan mengundurkan diri. (2) Keterangan tertulis dengan bukti yang sah sebagaimana dimaksud dalam ayat (1) harus diserah"}, {"rank": 7, "chunk_id": "23a99bc4b93e65bb80ee6bb331325d405dfbad40", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 45 | PP Nomor 35 Tahun 2021.pdf | Pasal 45", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 45", "rrf_score": 0.025483091787439613, "rerank_score": 0.14205528795719147, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kedua - Hak Akibat Pemutusan Hubungan Kerja Pasal 45 (1) Pengusaha dapat melakukan Pemutusan Hubungan Kerja terhadap Pekerja/Buruh karena alasan Perusahaan tutup yang disebabkan keadaan memaksa (force majeure) maka Pekerja/ Buruh berhak atas: a. uang pesangon sebesar 0,5 (nol koma lima) kali ketentuan Pasa"}, {"rank": 8, "chunk_id": "8b27dbefd4415136637241a90d1b04a057678314", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 54 | PP Nomor 35 Tahun 2021.pdf | Pasal 54", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 54", "rrf_score": 0.02546333601933924, "rerank_score": 0.13816599547863007, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kedua - Hak Akibat Pemutusan Hubungan Kerja Pasal 54 (1) Pengusaha dapat melakukan Pemutusan Hubungan Kerja terhadap Pekerja/Buruh karena alasan Pekerja/Buruh tidak dapat melakukan pekerjaan selama 6 (enam) bulan akibat ditahan pihak yang berwajib karena diduga melakukan tindak pidana sebagaimana dimaksud "}]</t>
         </is>
@@ -1787,7 +1822,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.8771370995839437</v>
+        <v>0.8965328709284466</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -1795,24 +1830,24 @@
         </is>
       </c>
       <c r="H12" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="I12" t="n">
         <v>0.7991080284118652</v>
       </c>
-      <c r="I12" t="n">
+      <c r="J12" t="n">
         <v>0.6</v>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>pelanggaran bersifat mendesak; uang penggantian hak; uang pisah</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>tidak pesangon; tidak UPMK</t>
         </is>
       </c>
-      <c r="L12" t="n">
-        <v>1</v>
-      </c>
       <c r="M12" t="n">
         <v>1</v>
       </c>
@@ -1838,39 +1873,42 @@
         <v>1</v>
       </c>
       <c r="U12" t="n">
+        <v>1</v>
+      </c>
+      <c r="V12" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="V12" t="n">
-        <v>1</v>
-      </c>
       <c r="W12" t="n">
         <v>1</v>
       </c>
       <c r="X12" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y12" t="n">
         <v>109</v>
       </c>
-      <c r="Y12" t="n">
-        <v>1</v>
-      </c>
       <c r="Z12" t="n">
-        <v>29.19733381271362</v>
-      </c>
-      <c r="AA12" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>28.02168560028076</v>
+      </c>
+      <c r="AB12" t="inlineStr">
         <is>
           <t>Qwen/Qwen3.5-9B</t>
         </is>
       </c>
-      <c r="AB12" t="inlineStr">
+      <c r="AC12" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 52 | PP Nomor 35 Tahun 2021.pdf | Pasal 52</t>
         </is>
       </c>
-      <c r="AC12" t="inlineStr">
+      <c r="AD12" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 52 | PP Nomor 35 Tahun 2021.pdf | Pasal 52 || Undang-Undang No. 13 Tahun 2003, Pasal 161 | UU_Nomor_13_Tahun_2003.pdf | Pasal 161 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 45 | PP Nomor 35 Tahun 2021.pdf | Pasal 45 || Undang-Undang No. 13 Tahun 2003, Pasal 169 | UU_Nomor_13_Tahun_2003.pdf | Pasal 169 || Undang-Undang No. 13 Tahun 2003, Pasal 167 | UU_Nomor_13_Tahun_2003.pdf | Pasal 167 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 40 | PP Nomor 35 Tahun 2021.pdf | Pasal 40 || Undang-Undang No. 13 Tahun 2003, Pasal 156 bagian 1 | UU_Nomor_13_Tahun_2003.pdf | Pasal 156 || Undang-Undang No. 13 Tahun 2003, Pasal 164 | UU_Nomor_13_Tahun_2003.pdf | Pasal 164</t>
         </is>
       </c>
-      <c r="AD12" t="inlineStr">
+      <c r="AE12" t="inlineStr">
         <is>
           <t>[{"rank": 1, "chunk_id": "6342df2412f32ef274fc7204bb3dba645ea81370", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 52 | PP Nomor 35 Tahun 2021.pdf | Pasal 52", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 52", "rrf_score": 0.027400468384074943, "rerank_score": 0.6312013864517212, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kedua - Hak Akibat Pemutusan Hubungan Kerja Pasal 52 (1) Pengusaha dapat melakukan Pemutusan Hubungan Kerja terhadap Pekerja/Buruh karena alasan Pekerja/Buruh melakukan pelanggaran ketentuan yang diatur dalam Perjanjian Kerja, Peraturan Perusahaan, atau Perjanjian Kerja Bersama dan sebelumnya telah diberik"}, {"rank": 2, "chunk_id": "56805803f10f2865010ad9be0e01a7a31f697222", "reference": "Undang-Undang No. 13 Tahun 2003, Pasal 161 | UU_Nomor_13_Tahun_2003.pdf | Pasal 161", "source_file": "UU_Nomor_13_Tahun_2003.pdf", "pasal_id": "Pasal 161", "rrf_score": 0.023333333333333334, "rerank_score": 0.38430875539779663, "text_preview": "Undang-Undang No. 13 Tahun 2003 tentang KETENAGAKERJAAN BAB XII - Pemutusan Hubungan Kerja Pasal 161 (1) Dalam hal pekerja/buruh melakukan pelanggaran ketentuan yang diatur dalam perjanjian kerja, peraturan perusahaan atau perjanjian kerja bersama, pengusaha dapat melakukan pemutusan hubungan kerja, setelah kepada pekerja/buruh yang bersangkutan diberikan surat peringatan pertama, kedua, dan ketiga secara berturutturut. (2) Surat peringatan sebagaimana dimaksud dalam ayat (1) masing-masing berla"}, {"rank": 3, "chunk_id": "23a99bc4b93e65bb80ee6bb331325d405dfbad40", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 45 | PP Nomor 35 Tahun 2021.pdf | Pasal 45", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 45", "rrf_score": 0.027565298507462685, "rerank_score": 0.23186923563480377, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kedua - Hak Akibat Pemutusan Hubungan Kerja Pasal 45 (1) Pengusaha dapat melakukan Pemutusan Hubungan Kerja terhadap Pekerja/Buruh karena alasan Perusahaan tutup yang disebabkan keadaan memaksa (force majeure) maka Pekerja/ Buruh berhak atas: a. uang pesangon sebesar 0,5 (nol koma lima) kali ketentuan Pasa"}, {"rank": 4, "chunk_id": "ddfb9a681bf272ac21c601e8f021b39cfd17f422", "reference": "Undang-Undang No. 13 Tahun 2003, Pasal 169 | UU_Nomor_13_Tahun_2003.pdf | Pasal 169", "source_file": "UU_Nomor_13_Tahun_2003.pdf", "pasal_id": "Pasal 169", "rrf_score": 0.02614954018392643, "rerank_score": 0.13950569927692413, "text_preview": "Undang-Undang No. 13 Tahun 2003 tentang KETENAGAKERJAAN BAB XII - Pemutusan Hubungan Kerja Pasal 169 (1) Pekerja/buruh dapat mengajukan permohonan pemutusan hubungan kerja kepada lembaga penyelesaian perselisihan hubungan industrial dalam hal pengusaha melakukan perbuatan sebagai berikut: a. menganiaya, menghina secara kasar atau mengancam pekerja/buruh; b. membujuk dan/atau menyuruh pekerja/buruh untuk melakukan perbuatan yang bertentangan dengan peraturan perundang-undangan; c. tidak membayar "}, {"rank": 5, "chunk_id": "08ea06839a7fb3d99ba9057f0a553fe364102048", "reference": "Undang-Undang No. 13 Tahun 2003, Pasal 167 | UU_Nomor_13_Tahun_2003.pdf | Pasal 167", "source_file": "UU_Nomor_13_Tahun_2003.pdf", "pasal_id": "Pasal 167", "rrf_score": 0.029032258064516127, "rerank_score": 0.11569511145353317, "text_preview": "Undang-Undang No. 13 Tahun 2003 tentang KETENAGAKERJAAN BAB XII - Pemutusan Hubungan Kerja Pasal 167 (1) Pengusaha dapat melakukan pemutusan hubungan kerja terhadap pekerja/buruh karena memasuki usia pensiun dan apabila pengusaha telah mengikutkan pekerja/buruh pada program pensiun yang iurannya dibayar penuh oleh pengusaha, maka pekerja/buruh tidak berhak mendapatkan uang pesangon sesuai ketentuan Pasal 156 ayat (2), uang penghargaan masa kerja sesuai ketentuan Pasal 156 ayat (3), tetapi tetap "}, {"rank": 6, "chunk_id": "7569131d663a780a3e49ce577028fe7f37551d85", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 40 | PP Nomor 35 Tahun 2021.pdf | Pasal 40", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 40", "rrf_score": 0.019191919191919194, "rerank_score": 0.10963747650384903, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kedua - Hak Akibat Pemutusan Hubungan Kerja Pasal 40 (1) Dalam hal terjadi Pemutusan Hubungan Kerja, Pengusaha wajib membayar uang pesangon dan/atau uang penghargaan masa kerja, dan uang penggantian hak yang seharusnya diterima. (2) Uang pesangon sebagaimana dimaksud pada ayat (1) diberikan dengan ketentua"}, {"rank": 7, "chunk_id": "10ddefacf628bfa3cb659991d3fbc835ec08a706", "reference": "Undang-Undang No. 13 Tahun 2003, Pasal 156 bagian 1 | UU_Nomor_13_Tahun_2003.pdf | Pasal 156", "source_file": "UU_Nomor_13_Tahun_2003.pdf", "pasal_id": "Pasal 156", "rrf_score": 0.019411764705882354, "rerank_score": 0.104617178440094, "text_preview": "Undang-Undang No. 13 Tahun 2003 tentang KETENAGAKERJAAN BAB XII - Pemutusan Hubungan Kerja Pasal 156 bagian 1 (1) Dalam hal terjadi pemutusan hubungan kerja, pengusaha diwajibkan membayar uang pesangon dan atau uang penghargaan masa kerja dan uang penggantian hak yang seharusnya diterima. (2) Perhitungan uang pesangon sebagaimana dimaksud dalam ayat (1) paling sedikit sebagai berikut: a. masa kerja kurang dari 1 (satu) tahun, 1 (satu) bulan upah; b. masa kerja 1 (satu) tahun atau lebih tetapi ku"}, {"rank": 8, "chunk_id": "44c28f65920d24abed71f425276323d906b10da6", "reference": "Undang-Undang No. 13 Tahun 2003, Pasal 164 | UU_Nomor_13_Tahun_2003.pdf | Pasal 164", "source_file": "UU_Nomor_13_Tahun_2003.pdf", "pasal_id": "Pasal 164", "rrf_score": 0.025664786462530217, "rerank_score": 0.10385588556528091, "text_preview": "Undang-Undang No. 13 Tahun 2003 tentang KETENAGAKERJAAN BAB XII - Pemutusan Hubungan Kerja Pasal 164 (1) Pengusaha dapat melakukan pemutusan hubungan kerja terhadap pekerja/buruh karena perusahaan tutup yang disebabkan perusahaan mengalami kerugian secara terus menerus selama 2 (dua) tahun, atau keadaan memaksa (force majeur), dengan ketentuan pekerja/buruh berhak atas uang pesangon sebesar 1 (satu) kali ketentuan Pasal 156 ayat (2) uang penghargaan masa kerja sebesar 1 (satu) kali ketentuan Pas"}]</t>
         </is>
@@ -1912,7 +1950,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0.9104557331403096</v>
+        <v>0.9322046665350597</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1920,20 +1958,20 @@
         </is>
       </c>
       <c r="H13" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="I13" t="n">
         <v>0.7369199991226196</v>
       </c>
-      <c r="I13" t="n">
-        <v>1</v>
-      </c>
-      <c r="J13" t="inlineStr">
+      <c r="J13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" t="inlineStr">
         <is>
           <t>mengundurkan diri; uang penggantian hak; uang pisah; syarat pengunduran diri</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="n">
-        <v>1</v>
-      </c>
+      <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
         <v>1</v>
       </c>
@@ -1947,51 +1985,54 @@
         <v>1</v>
       </c>
       <c r="Q13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R13" t="n">
         <v>2</v>
       </c>
       <c r="S13" t="n">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="T13" t="n">
         <v>0.5</v>
       </c>
       <c r="U13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="V13" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="V13" t="n">
-        <v>1</v>
-      </c>
       <c r="W13" t="n">
         <v>1</v>
       </c>
       <c r="X13" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y13" t="n">
         <v>137</v>
       </c>
-      <c r="Y13" t="n">
-        <v>1</v>
-      </c>
       <c r="Z13" t="n">
-        <v>41.86613035202026</v>
-      </c>
-      <c r="AA13" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>40.18789720535278</v>
+      </c>
+      <c r="AB13" t="inlineStr">
         <is>
           <t>Qwen/Qwen3.5-9B</t>
         </is>
       </c>
-      <c r="AB13" t="inlineStr">
+      <c r="AC13" t="inlineStr">
         <is>
           <t>Undang-Undang No. 13 Tahun 2003, Pasal 162 | UU_Nomor_13_Tahun_2003.pdf | Pasal 162</t>
         </is>
       </c>
-      <c r="AC13" t="inlineStr">
+      <c r="AD13" t="inlineStr">
         <is>
           <t>Undang-Undang No. 13 Tahun 2003, Pasal 162 | UU_Nomor_13_Tahun_2003.pdf | Pasal 162 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 50 | PP Nomor 35 Tahun 2021.pdf | Pasal 50 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 36 | PP Nomor 35 Tahun 2021.pdf | Pasal 36 || Undang-Undang No. 13 Tahun 2003, Pasal 154 | UU_Nomor_13_Tahun_2003.pdf | Pasal 154 || Undang-Undang No. 13 Tahun 2003, Pasal 168 | UU_Nomor_13_Tahun_2003.pdf | Pasal 168 || Peraturan Pemerintah No. 6 Tahun 2025, Pasal 20 | pp_Nomor_6_Tahun_2025.pdf | Pasal 20 || Undang-Undang No. 13 Tahun 2003, Pasal 156 bagian 1 | UU_Nomor_13_Tahun_2003.pdf | Pasal 156 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 42 | PP Nomor 35 Tahun 2021.pdf | Pasal 42</t>
         </is>
       </c>
-      <c r="AD13" t="inlineStr">
+      <c r="AE13" t="inlineStr">
         <is>
           <t>[{"rank": 1, "chunk_id": "64f86f0da5e7e99fa0691f872a31c758edcdeb6b", "reference": "Undang-Undang No. 13 Tahun 2003, Pasal 162 | UU_Nomor_13_Tahun_2003.pdf | Pasal 162", "source_file": "UU_Nomor_13_Tahun_2003.pdf", "pasal_id": "Pasal 162", "rrf_score": 0.029508196721311476, "rerank_score": 0.997239351272583, "text_preview": "Undang-Undang No. 13 Tahun 2003 tentang KETENAGAKERJAAN BAB XII - Pemutusan Hubungan Kerja Pasal 162 (1) Pekerja/buruh yang mengundurkan diri atas kemauan sendiri, memperoleh uang penggantian hak sesuai ketentuan Pasal 156 ayat (4). (2) Bagi pekerja/buruh yang mengundurkan diri atas kemauan sendiri, yang tugas dan fungsinya tidak mewakili kepentingan pengusaha secara langsung, selain menerima uang penggantian hak sesuai ketentuan Pasal 156 ayat (4) diberikan uang pisah yang besarnya dan pelaksan"}, {"rank": 2, "chunk_id": "061320f3b82f07db7ec06e98be7998663c14fa6c", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 50 | PP Nomor 35 Tahun 2021.pdf | Pasal 50", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 50", "rrf_score": 0.029032258064516127, "rerank_score": 0.9924665093421936, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kedua - Hak Akibat Pemutusan Hubungan Kerja Pasal 50 Pekerja/Buruh yang mengundurkan diri atas kemauan sendiri dan memenuhi syarat sebagaimana dimaksud dalam Pasal 36 huruf i, berhak atas: a. uang penggantian hak sesuai ketentuan Pasal 40 ayat (4); dan b. uang pisah yang besarannya diatur dalam Perjanjian "}, {"rank": 3, "chunk_id": "654617c9d52f8988bd188f0984852fd554a2cc5b", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 36 | PP Nomor 35 Tahun 2021.pdf | Pasal 36", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 36", "rrf_score": 0.02268665757988793, "rerank_score": 0.9553349614143372, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kesatu - Tata Cara Pemutusan Hubungan Kerja Pasal 36 Pemutusan Hubungan Kerja dapat terjadi karena alasan: a. Perusahaan melakukan penggabungan, peleburan, pengambilalihan, atau pemisahan Perusahaan dan Pekerja/Buruh tidak bersedia melanjutkan Hubungan Kerja atau Pengusaha tidak bersedia menerima Pekerja/B"}, {"rank": 4, "chunk_id": "e8434f50402f7a88d30b4e4ed82a53bd37c99f5b", "reference": "Undang-Undang No. 13 Tahun 2003, Pasal 154 | UU_Nomor_13_Tahun_2003.pdf | Pasal 154", "source_file": "UU_Nomor_13_Tahun_2003.pdf", "pasal_id": "Pasal 154", "rrf_score": 0.018390086431323546, "rerank_score": 0.8889303207397461, "text_preview": "Undang-Undang No. 13 Tahun 2003 tentang KETENAGAKERJAAN BAB XII - Pemutusan Hubungan Kerja Pasal 154 Penetapan sebagaimana dimaksud dalam Pasal 151 ayat (3) tidak diperlukan dalam hal: a. pekerja/buruh masih dalam masa percobaan kerja, bilamana telah dipersyaratkan secara tertulis sebelumnya; b. pekerja/buruh mengajukan permintaan pengunduran diri, secara tertulis atas kemauan sendiri tanpa ada indikasi adanya tekanan/intimidasi dari pengusaha, berakhirnya hubungan kerja sesuai dengan perjanjian"}, {"rank": 5, "chunk_id": "742e4669283c3b5296fba9dea7c1aa1d945da69e", "reference": "Undang-Undang No. 13 Tahun 2003, Pasal 168 | UU_Nomor_13_Tahun_2003.pdf | Pasal 168", "source_file": "UU_Nomor_13_Tahun_2003.pdf", "pasal_id": "Pasal 168", "rrf_score": 0.023284477015323116, "rerank_score": 0.521122932434082, "text_preview": "Undang-Undang No. 13 Tahun 2003 tentang KETENAGAKERJAAN BAB XII - Pemutusan Hubungan Kerja Pasal 168 (1) Pekerja/buruh yang mangkir selama 5 (lima) hari kerja atau lebih berturut-turut tanpa keterangan secara tertulis yang dilengkapi dengan bukti yang sah dan telah dipanggil oleh pengusaha 2 (dua) kali secara patut dan tertulis dapat diputus hubungan kerjanya karena dikualifikasikan mengundurkan diri. (2) Keterangan tertulis dengan bukti yang sah sebagaimana dimaksud dalam ayat (1) harus diserah"}, {"rank": 6, "chunk_id": "836e50474c243289962bb54904baa614bdd1e723", "reference": "Peraturan Pemerintah No. 6 Tahun 2025, Pasal 20 | pp_Nomor_6_Tahun_2025.pdf | Pasal 20", "source_file": "pp_Nomor_6_Tahun_2025.pdf", "pasal_id": "Pasal 20", "rrf_score": 0.011904761904761904, "rerank_score": 0.08169704675674438, "text_preview": "Peraturan Pemerintah No. 6 Tahun 2025 tentang PERUBAHAN ATAS PERATURAN PEMERINTAH NOMOR 37 TAHUN 2021 TENTANG PENYELENGGARAAN PROGRAM JAMINAN KEHII,ANGAN PEKER^'AAN DENGAN RAHMATTUHAN YANG MAHA ESA Pasal 20 (1) Manfaat JKP bagi Peserta yang mengalami Pemutusan Hubungan Kerja dikecualikan untuk alasan Pemutusan Hubungan Kerja karena: a. mengundurkan diri; b. cacat total tetap; c. pensiun; atau d. meninggal dunia. (2) Manfaat JKP bagi Peserta yang hubungan kerjanya berdasarkan perjanjian kerja wak"}, {"rank": 7, "chunk_id": "10ddefacf628bfa3cb659991d3fbc835ec08a706", "reference": "Undang-Undang No. 13 Tahun 2003, Pasal 156 bagian 1 | UU_Nomor_13_Tahun_2003.pdf | Pasal 156", "source_file": "UU_Nomor_13_Tahun_2003.pdf", "pasal_id": "Pasal 156", "rrf_score": 0.009195402298850575, "rerank_score": 0.06713631004095078, "text_preview": "Undang-Undang No. 13 Tahun 2003 tentang KETENAGAKERJAAN BAB XII - Pemutusan Hubungan Kerja Pasal 156 bagian 1 (1) Dalam hal terjadi pemutusan hubungan kerja, pengusaha diwajibkan membayar uang pesangon dan atau uang penghargaan masa kerja dan uang penggantian hak yang seharusnya diterima. (2) Perhitungan uang pesangon sebagaimana dimaksud dalam ayat (1) paling sedikit sebagai berikut: a. masa kerja kurang dari 1 (satu) tahun, 1 (satu) bulan upah; b. masa kerja 1 (satu) tahun atau lebih tetapi ku"}, {"rank": 8, "chunk_id": "c8c7b415c1c9e9d6c21b81c62e1d51830a98ad7e", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 42 | PP Nomor 35 Tahun 2021.pdf | Pasal 42", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 42", "rrf_score": 0.027746212121212123, "rerank_score": 0.06097463145852089, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kedua - Hak Akibat Pemutusan Hubungan Kerja Pasal 42 (1) Pengusaha dapat melakukan Pemutusan Hubungan Kerja terhadap Pekerja/Buruh karena alasan pengambilalihan Perusahaan maka Pekerja/Buruh berhak atas: a. uang pesangon sebesar 1 (satu) kali ketentuan Pasal 40 ayat (2); b. uang penghargaan masa kerja sebe"}]</t>
         </is>
@@ -2027,7 +2068,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.7981231532778058</v>
+        <v>0.8188177343777249</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -2035,24 +2076,24 @@
         </is>
       </c>
       <c r="H14" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="I14" t="n">
         <v>0.6635468006134033</v>
       </c>
-      <c r="I14" t="n">
+      <c r="J14" t="n">
         <v>0.4285714285714285</v>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>uang penggantian hak; cuti tahunan; ongkos pulang</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>pekerja dan keluarga; perjanjian kerja; peraturan perusahaan; PKB</t>
         </is>
       </c>
-      <c r="L14" t="n">
-        <v>1</v>
-      </c>
       <c r="M14" t="n">
         <v>1</v>
       </c>
@@ -2066,17 +2107,17 @@
         <v>1</v>
       </c>
       <c r="Q14" t="n">
+        <v>1</v>
+      </c>
+      <c r="R14" t="n">
         <v>2</v>
       </c>
-      <c r="R14" t="n">
-        <v>1</v>
-      </c>
       <c r="S14" t="n">
+        <v>1</v>
+      </c>
+      <c r="T14" t="n">
         <v>0.5</v>
       </c>
-      <c r="T14" t="n">
-        <v>1</v>
-      </c>
       <c r="U14" t="n">
         <v>1</v>
       </c>
@@ -2087,30 +2128,33 @@
         <v>1</v>
       </c>
       <c r="X14" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y14" t="n">
         <v>48</v>
       </c>
-      <c r="Y14" t="n">
-        <v>1</v>
-      </c>
       <c r="Z14" t="n">
-        <v>14.76256394386292</v>
-      </c>
-      <c r="AA14" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>14.29284286499023</v>
+      </c>
+      <c r="AB14" t="inlineStr">
         <is>
           <t>Qwen/Qwen3.5-9B</t>
         </is>
       </c>
-      <c r="AB14" t="inlineStr">
+      <c r="AC14" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 59 | PP Nomor 35 Tahun 2021.pdf | Pasal 59</t>
         </is>
       </c>
-      <c r="AC14" t="inlineStr">
+      <c r="AD14" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 59 | PP Nomor 35 Tahun 2021.pdf | Pasal 59 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 40 | PP Nomor 35 Tahun 2021.pdf | Pasal 40 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 41 | PP Nomor 35 Tahun 2021.pdf | Pasal 41 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 55 | PP Nomor 35 Tahun 2021.pdf | Pasal 55 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 42 | PP Nomor 35 Tahun 2021.pdf | Pasal 42 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 52 | PP Nomor 35 Tahun 2021.pdf | Pasal 52 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 44 | PP Nomor 35 Tahun 2021.pdf | Pasal 44 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 45 | PP Nomor 35 Tahun 2021.pdf | Pasal 45</t>
         </is>
       </c>
-      <c r="AD14" t="inlineStr">
+      <c r="AE14" t="inlineStr">
         <is>
           <t>[{"rank": 1, "chunk_id": "ddcf2188fefefcf797f175b43802b7a4db23b8e7", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 59 | PP Nomor 35 Tahun 2021.pdf | Pasal 59", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 59", "rrf_score": 0.025890238793464602, "rerank_score": 0.9561264514923096, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kedua - Hak Akibat Pemutusan Hubungan Kerja Pasal 59 Pengusaha pada usaha mikro dan usaha kecil wajib membayar uang pesangon, uang penghargaan masa kerja, uang penggantian hak, dan/atau uang pisah bagi Pekerja/Buruh yang mengalami Pemutusan Hubungan Kerja dengan besaran ditentukan berdasarkan kesepakatan a"}, {"rank": 2, "chunk_id": "7569131d663a780a3e49ce577028fe7f37551d85", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 40 | PP Nomor 35 Tahun 2021.pdf | Pasal 40", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 40", "rrf_score": 0.02159090909090909, "rerank_score": 0.9533262848854065, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kedua - Hak Akibat Pemutusan Hubungan Kerja Pasal 40 (1) Dalam hal terjadi Pemutusan Hubungan Kerja, Pengusaha wajib membayar uang pesangon dan/atau uang penghargaan masa kerja, dan uang penggantian hak yang seharusnya diterima. (2) Uang pesangon sebagaimana dimaksud pada ayat (1) diberikan dengan ketentua"}, {"rank": 3, "chunk_id": "c076389031da5a571c5a93f23505037c3c38d4f9", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 41 | PP Nomor 35 Tahun 2021.pdf | Pasal 41", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 41", "rrf_score": 0.025511197663096397, "rerank_score": 0.9324071407318115, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kedua - Hak Akibat Pemutusan Hubungan Kerja Pasal 41 Pengusaha dapat melakukan Pemutusan Hubungan Kerja terhadap Pekerja/Buruh karena alasan Perusahaan melakukan penggabungan, peleburan atau pemisahan Perusahaan dan Pekerja/Buruh tidak bersedia melanjutkan Hubungan Kerja atau Pengusaha tidak bersedia mener"}, {"rank": 4, "chunk_id": "1dc2206e35ec15f2cde1330cd0fef80d176febb7", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 55 | PP Nomor 35 Tahun 2021.pdf | Pasal 55", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 55", "rrf_score": 0.025592039800995024, "rerank_score": 0.9212700724601746, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kedua - Hak Akibat Pemutusan Hubungan Kerja Pasal 55 (1) Pengusaha dapat melakukan Pemutusan Hubungan Kerja terhadap Pekerja/Buruh karena alasan Pekerja/Buruh mengalami sakit berkepanjangan atau cacat akibat kecelakaan kerja dan tidak dapat melakukan pekerjaannya setelah melampaui batas 12 (dua belas) bula"}, {"rank": 5, "chunk_id": "c8c7b415c1c9e9d6c21b81c62e1d51830a98ad7e", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 42 | PP Nomor 35 Tahun 2021.pdf | Pasal 42", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 42", "rrf_score": 0.028629032258064516, "rerank_score": 0.9201177954673767, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kedua - Hak Akibat Pemutusan Hubungan Kerja Pasal 42 (1) Pengusaha dapat melakukan Pemutusan Hubungan Kerja terhadap Pekerja/Buruh karena alasan pengambilalihan Perusahaan maka Pekerja/Buruh berhak atas: a. uang pesangon sebesar 1 (satu) kali ketentuan Pasal 40 ayat (2); b. uang penghargaan masa kerja sebe"}, {"rank": 6, "chunk_id": "6342df2412f32ef274fc7204bb3dba645ea81370", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 52 | PP Nomor 35 Tahun 2021.pdf | Pasal 52", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 52", "rrf_score": 0.028739754098360656, "rerank_score": 0.9130414128303528, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kedua - Hak Akibat Pemutusan Hubungan Kerja Pasal 52 (1) Pengusaha dapat melakukan Pemutusan Hubungan Kerja terhadap Pekerja/Buruh karena alasan Pekerja/Buruh melakukan pelanggaran ketentuan yang diatur dalam Perjanjian Kerja, Peraturan Perusahaan, atau Perjanjian Kerja Bersama dan sebelumnya telah diberik"}, {"rank": 7, "chunk_id": "e70e201c90bd3b227a16e495b2d9f76b2bf5d86a", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 44 | PP Nomor 35 Tahun 2021.pdf | Pasal 44", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 44", "rrf_score": 0.026024805549716208, "rerank_score": 0.908123791217804, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kedua - Hak Akibat Pemutusan Hubungan Kerja Pasal 44 (1) Pengusaha dapat melakukan Pemutusan Hubungan Kerja terhadap Pekerja/Buruh karena alasan Perusahaan tutup yang disebabkan Perusahaan mengalami kerugian secara terus menerus selama 2 (dua) tahun atau mengalami kerugian tidak secara terus menerus selama"}, {"rank": 8, "chunk_id": "23a99bc4b93e65bb80ee6bb331325d405dfbad40", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 45 | PP Nomor 35 Tahun 2021.pdf | Pasal 45", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 45", "rrf_score": 0.026916221033868093, "rerank_score": 0.9059479832649231, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kedua - Hak Akibat Pemutusan Hubungan Kerja Pasal 45 (1) Pengusaha dapat melakukan Pemutusan Hubungan Kerja terhadap Pekerja/Buruh karena alasan Perusahaan tutup yang disebabkan keadaan memaksa (force majeure) maka Pekerja/ Buruh berhak atas: a. uang pesangon sebesar 0,5 (nol koma lima) kali ketentuan Pasa"}]</t>
         </is>
@@ -2148,28 +2192,28 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.8237053708235423</v>
+        <v>0.8664051770766577</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>excellent</t>
         </is>
       </c>
       <c r="H15" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="I15" t="n">
         <v>0.7138122916221619</v>
       </c>
-      <c r="I15" t="n">
-        <v>1</v>
-      </c>
-      <c r="J15" t="inlineStr">
+      <c r="J15" t="n">
+        <v>1</v>
+      </c>
+      <c r="K15" t="inlineStr">
         <is>
           <t>PHK; uang pesangon; uang penghargaan masa kerja; uang penggantian hak</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="n">
-        <v>1</v>
-      </c>
+      <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
         <v>1</v>
       </c>
@@ -2183,51 +2227,54 @@
         <v>1</v>
       </c>
       <c r="Q15" t="n">
+        <v>1</v>
+      </c>
+      <c r="R15" t="n">
         <v>5</v>
       </c>
-      <c r="R15" t="n">
-        <v>1</v>
-      </c>
       <c r="S15" t="n">
+        <v>1</v>
+      </c>
+      <c r="T15" t="n">
         <v>0.2</v>
       </c>
-      <c r="T15" t="n">
-        <v>1</v>
-      </c>
       <c r="U15" t="n">
+        <v>1</v>
+      </c>
+      <c r="V15" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="V15" t="n">
+      <c r="W15" t="n">
         <v>0</v>
       </c>
-      <c r="W15" t="n">
-        <v>1</v>
-      </c>
       <c r="X15" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y15" t="n">
         <v>91</v>
       </c>
-      <c r="Y15" t="n">
-        <v>1</v>
-      </c>
       <c r="Z15" t="n">
-        <v>26.5613157749176</v>
-      </c>
-      <c r="AA15" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>25.62117075920105</v>
+      </c>
+      <c r="AB15" t="inlineStr">
         <is>
           <t>Qwen/Qwen3.5-9B</t>
         </is>
       </c>
-      <c r="AB15" t="inlineStr">
+      <c r="AC15" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 59 | PP Nomor 35 Tahun 2021.pdf | Pasal 59</t>
         </is>
       </c>
-      <c r="AC15" t="inlineStr">
+      <c r="AD15" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 59 | PP Nomor 35 Tahun 2021.pdf | Pasal 59 || Undang-Undang No. 13 Tahun 2003, Pasal 156 bagian 1 | UU_Nomor_13_Tahun_2003.pdf | Pasal 156 || Peraturan Pemerintah No. 6 Tahun 2025, Pasal 39 | pp_Nomor_6_Tahun_2025.pdf | Pasal 39 || Peraturan Pemerintah No. 37 Tahun 2021, Pasal 39 | pp_Nomor_37_Tahun_2021.pdf | Pasal 39 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 40 | PP Nomor 35 Tahun 2021.pdf | Pasal 40 || Peraturan Pemerintah No. 37 Tahun 2021, Pasal 23 | pp_Nomor_37_Tahun_2021.pdf | Pasal 23 || Undang-Undang No. 13 Tahun 2003, Pasal 160 | UU_Nomor_13_Tahun_2003.pdf | Pasal 160 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 15 | PP Nomor 35 Tahun 2021.pdf | Pasal 15</t>
         </is>
       </c>
-      <c r="AD15" t="inlineStr">
+      <c r="AE15" t="inlineStr">
         <is>
           <t>[{"rank": 1, "chunk_id": "ddcf2188fefefcf797f175b43802b7a4db23b8e7", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 59 | PP Nomor 35 Tahun 2021.pdf | Pasal 59", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 59", "rrf_score": 0.02760910815939279, "rerank_score": 0.3221922516822815, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kedua - Hak Akibat Pemutusan Hubungan Kerja Pasal 59 Pengusaha pada usaha mikro dan usaha kecil wajib membayar uang pesangon, uang penghargaan masa kerja, uang penggantian hak, dan/atau uang pisah bagi Pekerja/Buruh yang mengalami Pemutusan Hubungan Kerja dengan besaran ditentukan berdasarkan kesepakatan a"}, {"rank": 2, "chunk_id": "10ddefacf628bfa3cb659991d3fbc835ec08a706", "reference": "Undang-Undang No. 13 Tahun 2003, Pasal 156 bagian 1 | UU_Nomor_13_Tahun_2003.pdf | Pasal 156", "source_file": "UU_Nomor_13_Tahun_2003.pdf", "pasal_id": "Pasal 156", "rrf_score": 0.019960474308300398, "rerank_score": 0.19961249828338623, "text_preview": "Undang-Undang No. 13 Tahun 2003 tentang KETENAGAKERJAAN BAB XII - Pemutusan Hubungan Kerja Pasal 156 bagian 1 (1) Dalam hal terjadi pemutusan hubungan kerja, pengusaha diwajibkan membayar uang pesangon dan atau uang penghargaan masa kerja dan uang penggantian hak yang seharusnya diterima. (2) Perhitungan uang pesangon sebagaimana dimaksud dalam ayat (1) paling sedikit sebagai berikut: a. masa kerja kurang dari 1 (satu) tahun, 1 (satu) bulan upah; b. masa kerja 1 (satu) tahun atau lebih tetapi ku"}, {"rank": 3, "chunk_id": "c71be547c408e39e856c688425e62c2347f0906c", "reference": "Peraturan Pemerintah No. 6 Tahun 2025, Pasal 39 | pp_Nomor_6_Tahun_2025.pdf | Pasal 39", "source_file": "pp_Nomor_6_Tahun_2025.pdf", "pasal_id": "Pasal 39", "rrf_score": 0.02185363014695184, "rerank_score": 0.1822463721036911, "text_preview": "Peraturan Pemerintah No. 6 Tahun 2025 tentang PERUBAHAN ATAS PERATURAN PEMERINTAH NOMOR 37 TAHUN 2021 TENTANG PENYELENGGARAAN PROGRAM JAMINAN KEHII,ANGAN PEKER^'AAN DENGAN RAHMATTUHAN YANG MAHA ESA Pasal 39 (1) Pengusaha yang menunggak iuran JKK sebagai sumber pendanaan program JKP sampai dengan 3 (tiga) bulan berturut-turut dan terjadi Pemutusan Hubungan Kerja, BPJS aan wajib membayar manfaat uang tunai sebagaimana dimaksud dalam Pasal 2L ayat (l) kepada Peserta. (2) Dalam hal BPJS Ketenagakerj"}, {"rank": 4, "chunk_id": "8aebe00f4ad742289af63d2dddd6c3641ce7afe2", "reference": "Peraturan Pemerintah No. 37 Tahun 2021, Pasal 39 | pp_Nomor_37_Tahun_2021.pdf | Pasal 39", "source_file": "pp_Nomor_37_Tahun_2021.pdf", "pasal_id": "Pasal 39", "rrf_score": 0.021018062397372743, "rerank_score": 0.17606434226036072, "text_preview": "Peraturan Pemerintah No. 37 Tahun 2021 BAB IV - Manfaat Jkp Bagian Kelima - Pelaksanaan Pemberian Manfaat Jkp Pasal 39 (1) Pengusaha yang menunggak iuran JKK dan JKM sebagai sumber pendanaan program JKP sampai dengan 3 (tiga) bulan berturut-turut dan terjadi Pemutusan Hubungan Kerja, BPJS Ketenagakerjaan wajib membayar manfaat uang tunai sebagaimana dimaksud dalam Pasal 21 ayat (1) kepada Peserta. (2) Dalam hal BPJS Ketenagakerjaan telah membayar manfaat uang tunai sebagaimana dimaksud pada ayat"}, {"rank": 5, "chunk_id": "7569131d663a780a3e49ce577028fe7f37551d85", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 40 | PP Nomor 35 Tahun 2021.pdf | Pasal 40", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 40", "rrf_score": 0.019415204678362573, "rerank_score": 0.17473100125789642, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kedua - Hak Akibat Pemutusan Hubungan Kerja Pasal 40 (1) Dalam hal terjadi Pemutusan Hubungan Kerja, Pengusaha wajib membayar uang pesangon dan/atau uang penghargaan masa kerja, dan uang penggantian hak yang seharusnya diterima. (2) Uang pesangon sebagaimana dimaksud pada ayat (1) diberikan dengan ketentua"}, {"rank": 6, "chunk_id": "063fb560ce3a91e5756e672020d6a9d3d321327b", "reference": "Peraturan Pemerintah No. 37 Tahun 2021, Pasal 23 | pp_Nomor_37_Tahun_2021.pdf | Pasal 23", "source_file": "pp_Nomor_37_Tahun_2021.pdf", "pasal_id": "Pasal 23", "rrf_score": 0.008333333333333333, "rerank_score": 0.12891577184200287, "text_preview": "Peraturan Pemerintah No. 37 Tahun 2021 tentang PENYELENGGARAAN PROGRAM JAMINAN KEHILANGAN PEKERJAAN BAB IV - Manfaat Jkp Bagian Kedua - Manfaat Uang Tunai Pasal 23 Dalam hal terjadi Pemutusan Hubungan Kerja dan Upah Pekerja/Buruh yang dilaporkan sebagaimana dimaksud dalam Pasal 21 ayat (2) tidak sesuai dengan Upah yang sebenarnya sehingga terdapat kekurangan pembayaran manfaat uang tunai, Pengusaha wajib membayar kekurangan manfaat uang tunai kepada Pekerja/Buruh secara sekaligus."}, {"rank": 7, "chunk_id": "2ee414f451ad7408ffb3226061cabf75b0f93434", "reference": "Undang-Undang No. 13 Tahun 2003, Pasal 160 | UU_Nomor_13_Tahun_2003.pdf | Pasal 160", "source_file": "UU_Nomor_13_Tahun_2003.pdf", "pasal_id": "Pasal 160", "rrf_score": 0.02177943821779438, "rerank_score": 0.07957401871681213, "text_preview": "Undang-Undang No. 13 Tahun 2003 tentang KETENAGAKERJAAN BAB XII - Pemutusan Hubungan Kerja Pasal 160 (1) Dalam hal pekerja/buruh ditahan pihak yang berwajib karena diduga melakukan tindak pidana bukan atas pengaduan pengusaha, maka pengusaha tidak wajib membayar upah tetapi wajib memberikan bantuan kepada keluarga pekerja/buruh yang menjadi tanggungannya dengan ketentuan sebagai berikut: a. untuk 1 (satu) orang tanggungan : 25% (dua puluh lima perseratus) dari upah; b. untuk 2 (dua) orang tanggu"}, {"rank": 8, "chunk_id": "174a6caf0ddd3791ff66aa1e4b6d8417fc84c2e2", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 15 | PP Nomor 35 Tahun 2021.pdf | Pasal 15", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 15", "rrf_score": 0.022136311569301258, "rerank_score": 0.05389653146266937, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB II - Perjanjian Kerja Waktu Tertentu Bagian Ketiga - Pemberian Uang Kompensasi Pasal 15 (1) Pengusaha wajib memberikan uang kompensasi kepada Pekerja/Buruh yang hubungan kerjanya berdasarkan PKWT. (2) Pemberian uang kompensasi dilaksanakan pada saat berakhirnya PKWT. (3) Uang kompensasi sebagaimana dimaksud pada ayat (1) diberikan kepada Pek"}]</t>
         </is>
@@ -2264,7 +2311,7 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.7950715150833129</v>
+        <v>0.8424351239204406</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -2272,24 +2319,24 @@
         </is>
       </c>
       <c r="H16" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="I16" t="n">
         <v>0.7662341594696045</v>
       </c>
-      <c r="I16" t="n">
+      <c r="J16" t="n">
         <v>0.8</v>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>dasar perhitungan; upah pokok; pesangon; uang penghargaan masa kerja</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>tunjangan tetap</t>
         </is>
       </c>
-      <c r="L16" t="n">
-        <v>1</v>
-      </c>
       <c r="M16" t="n">
         <v>1</v>
       </c>
@@ -2303,51 +2350,54 @@
         <v>1</v>
       </c>
       <c r="Q16" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="R16" t="n">
         <v>4</v>
       </c>
       <c r="S16" t="n">
-        <v>0.25</v>
+        <v>4</v>
       </c>
       <c r="T16" t="n">
         <v>0.25</v>
       </c>
       <c r="U16" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="V16" t="n">
         <v>0</v>
       </c>
       <c r="W16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X16" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y16" t="n">
         <v>140</v>
       </c>
-      <c r="Y16" t="n">
-        <v>1</v>
-      </c>
       <c r="Z16" t="n">
-        <v>39.15322971343994</v>
-      </c>
-      <c r="AA16" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>38.46526765823364</v>
+      </c>
+      <c r="AB16" t="inlineStr">
         <is>
           <t>Qwen/Qwen3.5-9B</t>
         </is>
       </c>
-      <c r="AB16" t="inlineStr">
+      <c r="AC16" t="inlineStr">
         <is>
           <t>Undang-Undang No. 13 Tahun 2003, Pasal 157 | UU_Nomor_13_Tahun_2003.pdf | Pasal 157</t>
         </is>
       </c>
-      <c r="AC16" t="inlineStr">
+      <c r="AD16" t="inlineStr">
         <is>
           <t>Undang-Undang No. 13 Tahun 2003, Pasal 157 | UU_Nomor_13_Tahun_2003.pdf | Pasal 157 || Undang-Undang No. 13 Tahun 2003, Pasal 156 bagian 1 | UU_Nomor_13_Tahun_2003.pdf | Pasal 156 || Undang-Undang No. 13 Tahun 2003, Pasal 156 bagian 2 | UU_Nomor_13_Tahun_2003.pdf | Pasal 156 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 40 | PP Nomor 35 Tahun 2021.pdf | Pasal 40 || Undang-Undang No. 13 Tahun 2003, Pasal 166 | UU_Nomor_13_Tahun_2003.pdf | Pasal 166 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 57 | PP Nomor 35 Tahun 2021.pdf | Pasal 57 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 58 | PP Nomor 35 Tahun 2021.pdf | Pasal 58 || Undang-Undang No. 13 Tahun 2003, Pasal 167 | UU_Nomor_13_Tahun_2003.pdf | Pasal 167</t>
         </is>
       </c>
-      <c r="AD16" t="inlineStr">
+      <c r="AE16" t="inlineStr">
         <is>
           <t>[{"rank": 1, "chunk_id": "48a260baf6a30616c5ff8addfedfdcae60e937c7", "reference": "Undang-Undang No. 13 Tahun 2003, Pasal 157 | UU_Nomor_13_Tahun_2003.pdf | Pasal 157", "source_file": "UU_Nomor_13_Tahun_2003.pdf", "pasal_id": "Pasal 157", "rrf_score": 0.029508196721311476, "rerank_score": 0.9962732791900635, "text_preview": "Undang-Undang No. 13 Tahun 2003 tentang KETENAGAKERJAAN BAB XII - Pemutusan Hubungan Kerja Pasal 157 (1) Komponen upah yang digunakan sebagai dasar perhitungan uang pesangon, uang penghargaan masa kerja, dan uang pengganti hak yang seharusnya diterima yang tertunda, terdiri atas: a. upah pokok; b. segala macam bentuk tunjangan yang bersifat tetap yang diberikan kepada pekerja/buruh dan keluarganya, termasuk harga pembelian dari catu yang diberikan kepada pekerja/buruh secara cuma-cuma, yang apab"}, {"rank": 2, "chunk_id": "10ddefacf628bfa3cb659991d3fbc835ec08a706", "reference": "Undang-Undang No. 13 Tahun 2003, Pasal 156 bagian 1 | UU_Nomor_13_Tahun_2003.pdf | Pasal 156", "source_file": "UU_Nomor_13_Tahun_2003.pdf", "pasal_id": "Pasal 156", "rrf_score": 0.027623785832741055, "rerank_score": 0.959564745426178, "text_preview": "Undang-Undang No. 13 Tahun 2003 tentang KETENAGAKERJAAN BAB XII - Pemutusan Hubungan Kerja Pasal 156 bagian 1 (1) Dalam hal terjadi pemutusan hubungan kerja, pengusaha diwajibkan membayar uang pesangon dan atau uang penghargaan masa kerja dan uang penggantian hak yang seharusnya diterima. (2) Perhitungan uang pesangon sebagaimana dimaksud dalam ayat (1) paling sedikit sebagai berikut: a. masa kerja kurang dari 1 (satu) tahun, 1 (satu) bulan upah; b. masa kerja 1 (satu) tahun atau lebih tetapi ku"}, {"rank": 3, "chunk_id": "2ef4995a3a222d631872d03bde4069f1cd1e47b5", "reference": "Undang-Undang No. 13 Tahun 2003, Pasal 156 bagian 2 | UU_Nomor_13_Tahun_2003.pdf | Pasal 156", "source_file": "UU_Nomor_13_Tahun_2003.pdf", "pasal_id": "Pasal 156", "rrf_score": 0.0261986301369863, "rerank_score": 0.7986147403717041, "text_preview": "Undang-Undang No. 13 Tahun 2003 tentang KETENAGAKERJAAN BAB XII - Pemutusan Hubungan Kerja Pasal 156 bagian 2 cuti tahunan yang belum diambil dan belum gugur; b. biaya atau ongkos pulang untuk pekerja/buruh dan keluarganya ketempat dimana pekerja/buruh diterima bekerja; c. penggantian perumahan serta pengobatan dan perawatan ditetapkan 15% (lima belas perseratus) dari uang pesangon dan/atau uang penghargaan masa kerja bagi yang memenuhi syarat; d. hal-hal lain yang ditetapkan dalam perjanjian ke"}, {"rank": 4, "chunk_id": "7569131d663a780a3e49ce577028fe7f37551d85", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 40 | PP Nomor 35 Tahun 2021.pdf | Pasal 40", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 40", "rrf_score": 0.024761904761904763, "rerank_score": 0.7985117435455322, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kedua - Hak Akibat Pemutusan Hubungan Kerja Pasal 40 (1) Dalam hal terjadi Pemutusan Hubungan Kerja, Pengusaha wajib membayar uang pesangon dan/atau uang penghargaan masa kerja, dan uang penggantian hak yang seharusnya diterima. (2) Uang pesangon sebagaimana dimaksud pada ayat (1) diberikan dengan ketentua"}, {"rank": 5, "chunk_id": "80a194af4a93207d167a6ec372101429ebb925ee", "reference": "Undang-Undang No. 13 Tahun 2003, Pasal 166 | UU_Nomor_13_Tahun_2003.pdf | Pasal 166", "source_file": "UU_Nomor_13_Tahun_2003.pdf", "pasal_id": "Pasal 166", "rrf_score": 0.02325895875591616, "rerank_score": 0.6796290278434753, "text_preview": "Undang-Undang No. 13 Tahun 2003 tentang KETENAGAKERJAAN BAB XII - Pemutusan Hubungan Kerja Pasal 166 Dalam hal hubungan kerja berakhir karena pekerja/buruh meninggal dunia, kepada ahli warisnya diberikan sejumlah uang yang besar perhitungannya sama dengan perhitungan 2 (dua) kali uang pesangon sesuai ketentuan Pasal 156 ayat (2), 1 (satu) kali uang penghargaan masa kerja sesuai ketentuan Pasal 156 ayat (3), dan uang penggantian hak sesuai ketentuan Pasal 156 ayat (4)."}, {"rank": 6, "chunk_id": "7d733971c854e864c59f9195c4d3c51f402684bb", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 57 | PP Nomor 35 Tahun 2021.pdf | Pasal 57", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 57", "rrf_score": 0.02285900358189515, "rerank_score": 0.6579893231391907, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kedua - Hak Akibat Pemutusan Hubungan Kerja Pasal 57 Pemutusan Hubungan Kerja karena alasan Pekerja/Buruh meninggal dunia maka kepada ahli warisnya diberikan sejumlah uang yang perhitungannya sama dengan: a uang pesangon sebesar 2 (dua) kali ketentuan Pasal 40 ayat (2)'., b uang penghargaan masa kerja sebe"}, {"rank": 7, "chunk_id": "12a004202107792a2c123a234712587d60267092", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 58 | PP Nomor 35 Tahun 2021.pdf | Pasal 58", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 58", "rrf_score": 0.025128205128205128, "rerank_score": 0.6209962964057922, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kedua - Hak Akibat Pemutusan Hubungan Kerja Pasal 58 (1) Pengusaha yang mengikutsertakan Pekerja/Buruh dalam program pensiun sesuai dengan ketentuan peraturan perundang-undangan di bidang dana pensiun, iuran yang dibayar oleh Pengusaha dapat diperhitungkan sebagai bagian dari pemenuhan kewajiban Pengusaha "}, {"rank": 8, "chunk_id": "08ea06839a7fb3d99ba9057f0a553fe364102048", "reference": "Undang-Undang No. 13 Tahun 2003, Pasal 167 | UU_Nomor_13_Tahun_2003.pdf | Pasal 167", "source_file": "UU_Nomor_13_Tahun_2003.pdf", "pasal_id": "Pasal 167", "rrf_score": 0.027140621506818688, "rerank_score": 0.5375155806541443, "text_preview": "Undang-Undang No. 13 Tahun 2003 tentang KETENAGAKERJAAN BAB XII - Pemutusan Hubungan Kerja Pasal 167 (1) Pengusaha dapat melakukan pemutusan hubungan kerja terhadap pekerja/buruh karena memasuki usia pensiun dan apabila pengusaha telah mengikutkan pekerja/buruh pada program pensiun yang iurannya dibayar penuh oleh pengusaha, maka pekerja/buruh tidak berhak mendapatkan uang pesangon sesuai ketentuan Pasal 156 ayat (2), uang penghargaan masa kerja sesuai ketentuan Pasal 156 ayat (3), tetapi tetap "}]</t>
         </is>
@@ -2393,7 +2443,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0.7315822368939717</v>
+        <v>0.7477272827307383</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -2401,27 +2451,27 @@
         </is>
       </c>
       <c r="H17" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="I17" t="n">
         <v>0.788404107093811</v>
       </c>
-      <c r="I17" t="n">
+      <c r="J17" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>perundingan; SP1; SP2; SP3; uang penggantian hak; bipartit; 30 hari kerja; mediasi</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>mencegah PHK; setengah kali pesangon; satu kali UPMK; Pengadilan Hubungan Industrial</t>
         </is>
       </c>
-      <c r="L17" t="n">
+      <c r="M17" t="n">
         <v>0.2</v>
       </c>
-      <c r="M17" t="n">
-        <v>1</v>
-      </c>
       <c r="N17" t="n">
         <v>1</v>
       </c>
@@ -2432,17 +2482,17 @@
         <v>1</v>
       </c>
       <c r="Q17" t="n">
+        <v>1</v>
+      </c>
+      <c r="R17" t="n">
         <v>3</v>
       </c>
-      <c r="R17" t="n">
-        <v>1</v>
-      </c>
       <c r="S17" t="n">
+        <v>1</v>
+      </c>
+      <c r="T17" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="T17" t="n">
-        <v>1</v>
-      </c>
       <c r="U17" t="n">
         <v>1</v>
       </c>
@@ -2453,30 +2503,33 @@
         <v>1</v>
       </c>
       <c r="X17" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y17" t="n">
         <v>236</v>
       </c>
-      <c r="Y17" t="n">
+      <c r="Z17" t="n">
         <v>0.9466666666666667</v>
       </c>
-      <c r="Z17" t="n">
-        <v>67.36106276512146</v>
-      </c>
-      <c r="AA17" t="inlineStr">
+      <c r="AA17" t="n">
+        <v>66.88468241691589</v>
+      </c>
+      <c r="AB17" t="inlineStr">
         <is>
           <t>Qwen/Qwen3.5-9B</t>
         </is>
       </c>
-      <c r="AB17" t="inlineStr">
+      <c r="AC17" t="inlineStr">
         <is>
           <t>Undang-Undang No. 13 Tahun 2003, Pasal 1 | UU_Nomor_13_Tahun_2003.pdf | Pasal 1</t>
         </is>
       </c>
-      <c r="AC17" t="inlineStr">
+      <c r="AD17" t="inlineStr">
         <is>
           <t>Undang-Undang No. 13 Tahun 2003, Pasal 1 | UU_Nomor_13_Tahun_2003.pdf | Pasal 1 || Undang-Undang No. 13 Tahun 2003, Pasal 161 | UU_Nomor_13_Tahun_2003.pdf | Pasal 161 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 52 | PP Nomor 35 Tahun 2021.pdf | Pasal 52 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 36 | PP Nomor 35 Tahun 2021.pdf | Pasal 36 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 39 | PP Nomor 35 Tahun 2021.pdf | Pasal 39 || Undang-Undang No. 13 Tahun 2003, Pasal 164 | UU_Nomor_13_Tahun_2003.pdf | Pasal 164 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 54 | PP Nomor 35 Tahun 2021.pdf | Pasal 54 || Peraturan Pemerintah No. 35 Tahun 2021, Pasal 45 | PP Nomor 35 Tahun 2021.pdf | Pasal 45</t>
         </is>
       </c>
-      <c r="AD17" t="inlineStr">
+      <c r="AE17" t="inlineStr">
         <is>
           <t>[{"rank": 1, "chunk_id": "9b2208c51b01b038d49bc5e27a9be763c2bd1fd8", "reference": "Undang-Undang No. 13 Tahun 2003, Pasal 1 | UU_Nomor_13_Tahun_2003.pdf | Pasal 1", "source_file": "UU_Nomor_13_Tahun_2003.pdf", "pasal_id": "Pasal 1", "rrf_score": 0.00808080808080808, "rerank_score": 0.21186302602291107, "text_preview": "Undang-Undang No. 13 Tahun 2003 BAB I - Ketentuan Umum Pasal 1 sesuai dengan kebutuhannya. 13. Tenaga kerja asing adalah warga negara asing pemegang visa dengan maksud bekerja di wilayah Indonesia. 14. Perjanjian kerja adalah perjanjian antara pekerja/buruh dengan pengusaha atau pemberi kerja yang memuat syarat-syarat kerja, hak, dan kewajiban para pihak. 15. Hubungan kerja adalah hubungan antara pengusaha dengan pekerja/buruh berdasarkan perjanjian kerja, yang mempunyai unsur pekerjaan, upah, d"}, {"rank": 2, "chunk_id": "56805803f10f2865010ad9be0e01a7a31f697222", "reference": "Undang-Undang No. 13 Tahun 2003, Pasal 161 | UU_Nomor_13_Tahun_2003.pdf | Pasal 161", "source_file": "UU_Nomor_13_Tahun_2003.pdf", "pasal_id": "Pasal 161", "rrf_score": 0.024415584415584418, "rerank_score": 0.1963445246219635, "text_preview": "Undang-Undang No. 13 Tahun 2003 tentang KETENAGAKERJAAN BAB XII - Pemutusan Hubungan Kerja Pasal 161 (1) Dalam hal pekerja/buruh melakukan pelanggaran ketentuan yang diatur dalam perjanjian kerja, peraturan perusahaan atau perjanjian kerja bersama, pengusaha dapat melakukan pemutusan hubungan kerja, setelah kepada pekerja/buruh yang bersangkutan diberikan surat peringatan pertama, kedua, dan ketiga secara berturutturut. (2) Surat peringatan sebagaimana dimaksud dalam ayat (1) masing-masing berla"}, {"rank": 3, "chunk_id": "6342df2412f32ef274fc7204bb3dba645ea81370", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 52 | PP Nomor 35 Tahun 2021.pdf | Pasal 52", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 52", "rrf_score": 0.028987769971376528, "rerank_score": 0.15494579076766968, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kedua - Hak Akibat Pemutusan Hubungan Kerja Pasal 52 (1) Pengusaha dapat melakukan Pemutusan Hubungan Kerja terhadap Pekerja/Buruh karena alasan Pekerja/Buruh melakukan pelanggaran ketentuan yang diatur dalam Perjanjian Kerja, Peraturan Perusahaan, atau Perjanjian Kerja Bersama dan sebelumnya telah diberik"}, {"rank": 4, "chunk_id": "654617c9d52f8988bd188f0984852fd554a2cc5b", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 36 | PP Nomor 35 Tahun 2021.pdf | Pasal 36", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 36", "rrf_score": 0.015625, "rerank_score": 0.14743086695671082, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kesatu - Tata Cara Pemutusan Hubungan Kerja Pasal 36 Pemutusan Hubungan Kerja dapat terjadi karena alasan: a. Perusahaan melakukan penggabungan, peleburan, pengambilalihan, atau pemisahan Perusahaan dan Pekerja/Buruh tidak bersedia melanjutkan Hubungan Kerja atau Pengusaha tidak bersedia menerima Pekerja/B"}, {"rank": 5, "chunk_id": "31f731808df438b6b61498cc7fc1927885bc2a53", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 39 | PP Nomor 35 Tahun 2021.pdf | Pasal 39", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 39", "rrf_score": 0.01098901098901099, "rerank_score": 0.11761978268623352, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kesatu - Tata Cara Pemutusan Hubungan Kerja Pasal 39 (1) Pekerja/Buruh yang telah mendapatkan surat pemberitahuan Pemutusan Hubungan Kerja dan menyatakan menolak, harus membuat surat penolakan disertai alasan paling lama 7 (tujuh) hari kerja setelah diterimanya surat pemberitahuan. (2\\ Dalam hal terjadi pe"}, {"rank": 6, "chunk_id": "44c28f65920d24abed71f425276323d906b10da6", "reference": "Undang-Undang No. 13 Tahun 2003, Pasal 164 | UU_Nomor_13_Tahun_2003.pdf | Pasal 164", "source_file": "UU_Nomor_13_Tahun_2003.pdf", "pasal_id": "Pasal 164", "rrf_score": 0.0267921146953405, "rerank_score": 0.09522704035043716, "text_preview": "Undang-Undang No. 13 Tahun 2003 tentang KETENAGAKERJAAN BAB XII - Pemutusan Hubungan Kerja Pasal 164 (1) Pengusaha dapat melakukan pemutusan hubungan kerja terhadap pekerja/buruh karena perusahaan tutup yang disebabkan perusahaan mengalami kerugian secara terus menerus selama 2 (dua) tahun, atau keadaan memaksa (force majeur), dengan ketentuan pekerja/buruh berhak atas uang pesangon sebesar 1 (satu) kali ketentuan Pasal 156 ayat (2) uang penghargaan masa kerja sebesar 1 (satu) kali ketentuan Pas"}, {"rank": 7, "chunk_id": "8b27dbefd4415136637241a90d1b04a057678314", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 54 | PP Nomor 35 Tahun 2021.pdf | Pasal 54", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 54", "rrf_score": 0.027623785832741055, "rerank_score": 0.09364338964223862, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kedua - Hak Akibat Pemutusan Hubungan Kerja Pasal 54 (1) Pengusaha dapat melakukan Pemutusan Hubungan Kerja terhadap Pekerja/Buruh karena alasan Pekerja/Buruh tidak dapat melakukan pekerjaan selama 6 (enam) bulan akibat ditahan pihak yang berwajib karena diduga melakukan tindak pidana sebagaimana dimaksud "}, {"rank": 8, "chunk_id": "23a99bc4b93e65bb80ee6bb331325d405dfbad40", "reference": "Peraturan Pemerintah No. 35 Tahun 2021, Pasal 45 | PP Nomor 35 Tahun 2021.pdf | Pasal 45", "source_file": "PP Nomor 35 Tahun 2021.pdf", "pasal_id": "Pasal 45", "rrf_score": 0.025278219395866455, "rerank_score": 0.09278638660907745, "text_preview": "Peraturan Pemerintah No. 35 Tahun 2021 tentang PERJANJIAN KERJA WAKTU TERTENTU, ALIH DAYA, WAKTU KERJA DAN WAKTU ISTIRAHAT, DAN PEMUTUSAN HUBUNGAN KERJA BAB V - Pemutusan Hubungan Kerja Bagian Kedua - Hak Akibat Pemutusan Hubungan Kerja Pasal 45 (1) Pengusaha dapat melakukan Pemutusan Hubungan Kerja terhadap Pekerja/Buruh karena alasan Perusahaan tutup yang disebabkan keadaan memaksa (force majeure) maka Pekerja/ Buruh berhak atas: a. uang pesangon sebesar 0,5 (nol koma lima) kali ketentuan Pasa"}]</t>
         </is>
@@ -2529,7 +2582,7 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.7096137903531392</v>
+        <v>0.7382594025135041</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -2537,27 +2590,27 @@
         </is>
       </c>
       <c r="H18" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="I18" t="n">
         <v>0.7717293500900269</v>
       </c>
-      <c r="I18" t="n">
+      <c r="J18" t="n">
         <v>0.8333333333333334</v>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>PHK; pesangon; uang penghargaan masa kerja; uang penggantian hak; JKP; uang tunai; 25 persen; 6 bulan; informasi pasar kerja; pelatihan kerja</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>kehilangan pekerjaan; 45 persen</t>
         </is>
       </c>
-      <c r="L18" t="n">
+      <c r="M18" t="n">
         <v>0.4</v>
       </c>
-      <c r="M18" t="n">
-        <v>1</v>
-      </c>
       <c r="N18" t="n">
         <v>1</v>
       </c>
@@ -2568,51 +2621,54 @@
         <v>1</v>
       </c>
       <c r="Q18" t="n">
+        <v>1</v>
+      </c>
+      <c r="R18" t="n">
         <v>4</v>
       </c>
-      <c r="R18" t="n">
-        <v>1</v>
-      </c>
       <c r="S18" t="n">
+        <v>1</v>
+      </c>
+      <c r="T18" t="n">
         <v>0.25</v>
       </c>
-      <c r="T18" t="n">
-        <v>1</v>
-      </c>
       <c r="U18" t="n">
+        <v>1</v>
+      </c>
+      <c r="V18" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="V18" t="n">
+      <c r="W18" t="n">
         <v>0</v>
       </c>
-      <c r="W18" t="n">
-        <v>1</v>
-      </c>
       <c r="X18" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y18" t="n">
         <v>320</v>
       </c>
-      <c r="Y18" t="n">
+      <c r="Z18" t="n">
         <v>0.6666666666666667</v>
       </c>
-      <c r="Z18" t="n">
-        <v>84.05413889884949</v>
-      </c>
-      <c r="AA18" t="inlineStr">
+      <c r="AA18" t="n">
+        <v>83.43450665473938</v>
+      </c>
+      <c r="AB18" t="inlineStr">
         <is>
           <t>Qwen/Qwen3.5-9B</t>
         </is>
       </c>
-      <c r="AB18" t="inlineStr">
+      <c r="AC18" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 37 Tahun 2021, Pasal 1 | pp_Nomor_37_Tahun_2021.pdf | Pasal 1</t>
         </is>
       </c>
-      <c r="AC18" t="inlineStr">
+      <c r="AD18" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 37 Tahun 2021, Pasal 1 | pp_Nomor_37_Tahun_2021.pdf | Pasal 1 || Peraturan Pemerintah No. 6 Tahun 2025, Pasal 19 | pp_Nomor_6_Tahun_2025.pdf | Pasal 19 || Peraturan Menteri Ketenagakerjaan No. 7 Tahun 2025, Pasal 1 | permen_Nomor_7_Tahun_2025.pdf | Pasal 1 || Peraturan Pemerintah No. 37 Tahun 2021, Pasal 37 | pp_Nomor_37_Tahun_2021.pdf | Pasal 37 || Peraturan Pemerintah No. 37 Tahun 2021, Pasal 18 | pp_Nomor_37_Tahun_2021.pdf | Pasal 18 || Peraturan Pemerintah No. 6 Tahun 2025, Pasal 11 | pp_Nomor_6_Tahun_2025.pdf | Pasal 11 || Peraturan Pemerintah No. 37 Tahun 2021, Pasal 23 | pp_Nomor_37_Tahun_2021.pdf | Pasal 23 || Peraturan Pemerintah No. 37 Tahun 2021, Pasal 39 | pp_Nomor_37_Tahun_2021.pdf | Pasal 39</t>
         </is>
       </c>
-      <c r="AD18" t="inlineStr">
+      <c r="AE18" t="inlineStr">
         <is>
           <t>[{"rank": 1, "chunk_id": "1f219f284c4b6a218aa280d19264bb8d1aa59a70", "reference": "Peraturan Pemerintah No. 37 Tahun 2021, Pasal 1 | pp_Nomor_37_Tahun_2021.pdf | Pasal 1", "source_file": "pp_Nomor_37_Tahun_2021.pdf", "pasal_id": "Pasal 1", "rrf_score": 0.024248851184164016, "rerank_score": 0.9317411184310913, "text_preview": "Peraturan Pemerintah No. 37 Tahun 2021 BAB I - Ketentuan Umum Pasal 1 1. Jaminan Kehilangan Pekerjaan (JKP) adalah jaminan sosial yang diberikan kepada Pekerja/Buruh yang mengalami Pemutusan Hubungan Kerja berupa manfaat uang tunai, akses informasi pasar kerja, dan Pelatihan Kerja. 2. Pekerja/Buruh adalah setiap orang yang bekerja dengan menerima Upah atau imbalan dalam bentuk lain. 3. Pengusaha adalah: a. orang perseorangan, persekutuan, atau badan hukum yang menjalankan suatu perusahaan milik "}, {"rank": 2, "chunk_id": "728a3b4794695ee074f9dde293c7fb15c9692c3c", "reference": "Peraturan Pemerintah No. 6 Tahun 2025, Pasal 19 | pp_Nomor_6_Tahun_2025.pdf | Pasal 19", "source_file": "pp_Nomor_6_Tahun_2025.pdf", "pasal_id": "Pasal 19", "rrf_score": 0.010416666666666666, "rerank_score": 0.8088058233261108, "text_preview": "Peraturan Pemerintah No. 6 Tahun 2025 Pasal 19 SITASI: Peraturan Pemerintah No. 6 Tahun 2025, Pasal 19 Ayat (1) Cukup jelas. Ayat (2) Yang dimaksud dengan \"bersedia untuk bekerja kembali\" yaitu bekerja sebagai pekerja penerima upah atau berusaha mandiri atau wirausaha. Ayat (3) Makna 24 (dua puluh empat) bulan dalam ketentuan Pasal 19 ayat (3) adalah bulan kalender, bukan bulan masa iur dan bukan bulan masa kepesertaan dalam program BPJS Ketenagakerjaan. Syarat masa iur 12 (dua belas) bulan dima"}, {"rank": 3, "chunk_id": "21006438477868d89108b8d2438b6d1a55921d45", "reference": "Peraturan Menteri Ketenagakerjaan No. 7 Tahun 2025, Pasal 1 | permen_Nomor_7_Tahun_2025.pdf | Pasal 1", "source_file": "permen_Nomor_7_Tahun_2025.pdf", "pasal_id": "Pasal 1", "rrf_score": 0.008602150537634409, "rerank_score": 0.8024934530258179, "text_preview": "Peraturan Menteri Ketenagakerjaan No. 7 Tahun 2025 Pasal 1 1. Dana Iuran Peserta Program Jaminan Kehilangan Pekerjaan yang selanjutnya disebut Dana Iuran Peserta adalah dana iuran yang dibayar oleh pemerintah dan berasal dari anggaran pendapatan dan belanja negara. 2. Jaminan Kehilangan Pekerjaan yang selanjutnya disingkat JKP adalah jaminan sosial yang diberikan kepada pekerja/buruh yang mengalami pemutusan hubungan kerja berupa manfaat uang tunai, akses informasi pasar kerja, dan pelatihan ker"}, {"rank": 4, "chunk_id": "a4f394255a39720459f89501755ced11fe76c404", "reference": "Peraturan Pemerintah No. 37 Tahun 2021, Pasal 37 | pp_Nomor_37_Tahun_2021.pdf | Pasal 37", "source_file": "pp_Nomor_37_Tahun_2021.pdf", "pasal_id": "Pasal 37", "rrf_score": 0.02732491389207807, "rerank_score": 0.7971068024635315, "text_preview": "Peraturan Pemerintah No. 37 Tahun 2021 tentang PENYELENGGARAAN PROGRAM JAMINAN KEHILANGAN PEKERJAAN BAB IV - Manfaat Jkp Bagian Kelima - Pelaksanaan Pemberian Manfaat Jkp Pasal 37 (1) Dalam hal Pengusaha tidak mengikutsertakan Pekerja/Buruh dalam program JKP dan terjadi Pemutusan Hubungan Kerja, Pengusaha wajib memenuhi hak Pekerja/Buruh berupa: a. manfaat uang tunai dengan perhitungan manfaat sebagaimana dimaksud dalam Pasal 21 ayat (1) yang diberikan secara sekaligus; dan b. manfaat Pelatihan "}, {"rank": 5, "chunk_id": "72f912166cdcaa56ec92455fede7f4dbb2c74ade", "reference": "Peraturan Pemerintah No. 37 Tahun 2021, Pasal 18 | pp_Nomor_37_Tahun_2021.pdf | Pasal 18", "source_file": "pp_Nomor_37_Tahun_2021.pdf", "pasal_id": "Pasal 18", "rrf_score": 0.0125, "rerank_score": 0.6544933319091797, "text_preview": "Peraturan Pemerintah No. 37 Tahun 2021 tentang PENYELENGGARAAN PROGRAM JAMINAN KEHILANGAN PEKERJAAN BAB IV - Manfaat Jkp Bagian Kesatu - Umum Pasal 18 Manfaat JKP berupa: a. uang tunai; b. akses informasi pasar kerja; dan c. Pelatihan Kerja."}, {"rank": 6, "chunk_id": "86fd0ba13a6e9c6bfb479a29d8ea7fd30ca995d2", "reference": "Peraturan Pemerintah No. 6 Tahun 2025, Pasal 11 | pp_Nomor_6_Tahun_2025.pdf | Pasal 11", "source_file": "pp_Nomor_6_Tahun_2025.pdf", "pasal_id": "Pasal 11", "rrf_score": 0.011904761904761904, "rerank_score": 0.6309754848480225, "text_preview": "Peraturan Pemerintah No. 6 Tahun 2025 Pasal 11 Peraturan Pemerintah No. 6 Tahun 2025, Pasal 11 puluh enam ribu dua ratus empat puluh) orang pekerja yang mengalami Pemutusan Hubungan Kerja, hal ini meningkat sebanyak 8.865 (delapan ribu delapan ratus enam puluh lima) orang atau 23,7% (dua puluh tiga koma tujuh persen) dibandingkan bulan Agustus 2023 yaitu sebanyak 37.375 (tiga puluh tujuh ribu tiga ratus tujuh puluh lima) orang. Berdasarkan data pada bulan Agustus 2024, tercatat sebanyak 13,38 (t"}, {"rank": 7, "chunk_id": "063fb560ce3a91e5756e672020d6a9d3d321327b", "reference": "Peraturan Pemerintah No. 37 Tahun 2021, Pasal 23 | pp_Nomor_37_Tahun_2021.pdf | Pasal 23", "source_file": "pp_Nomor_37_Tahun_2021.pdf", "pasal_id": "Pasal 23", "rrf_score": 0.022304603027494596, "rerank_score": 0.56784987449646, "text_preview": "Peraturan Pemerintah No. 37 Tahun 2021 tentang PENYELENGGARAAN PROGRAM JAMINAN KEHILANGAN PEKERJAAN BAB IV - Manfaat Jkp Bagian Kedua - Manfaat Uang Tunai Pasal 23 Dalam hal terjadi Pemutusan Hubungan Kerja dan Upah Pekerja/Buruh yang dilaporkan sebagaimana dimaksud dalam Pasal 21 ayat (2) tidak sesuai dengan Upah yang sebenarnya sehingga terdapat kekurangan pembayaran manfaat uang tunai, Pengusaha wajib membayar kekurangan manfaat uang tunai kepada Pekerja/Buruh secara sekaligus."}, {"rank": 8, "chunk_id": "8aebe00f4ad742289af63d2dddd6c3641ce7afe2", "reference": "Peraturan Pemerintah No. 37 Tahun 2021, Pasal 39 | pp_Nomor_37_Tahun_2021.pdf | Pasal 39", "source_file": "pp_Nomor_37_Tahun_2021.pdf", "pasal_id": "Pasal 39", "rrf_score": 0.028436724565756823, "rerank_score": 0.504087507724762, "text_preview": "Peraturan Pemerintah No. 37 Tahun 2021 BAB IV - Manfaat Jkp Bagian Kelima - Pelaksanaan Pemberian Manfaat Jkp Pasal 39 (1) Pengusaha yang menunggak iuran JKK dan JKM sebagai sumber pendanaan program JKP sampai dengan 3 (tiga) bulan berturut-turut dan terjadi Pemutusan Hubungan Kerja, BPJS Ketenagakerjaan wajib membayar manfaat uang tunai sebagaimana dimaksud dalam Pasal 21 ayat (1) kepada Peserta. (2) Dalam hal BPJS Ketenagakerjaan telah membayar manfaat uang tunai sebagaimana dimaksud pada ayat"}]</t>
         </is>
@@ -2672,35 +2728,35 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>0.8458163170814514</v>
+        <v>0.8650565798282623</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>excellent</t>
         </is>
       </c>
       <c r="H19" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="I19" t="n">
         <v>0.8537105321884155</v>
       </c>
-      <c r="I19" t="n">
+      <c r="J19" t="n">
         <v>0.8333333333333334</v>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>pemagangan; penyandang disabilitas; kebutuhan khusus; K3; uang saku; jaminan sosial; sertifikat; alat pelindung diri; ULD Ketenagakerjaan; alat bantu kerja</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>bimbingan; tenaga pendamping</t>
         </is>
       </c>
-      <c r="L19" t="n">
+      <c r="M19" t="n">
         <v>0.6</v>
       </c>
-      <c r="M19" t="n">
-        <v>1</v>
-      </c>
       <c r="N19" t="n">
         <v>1</v>
       </c>
@@ -2711,17 +2767,17 @@
         <v>1</v>
       </c>
       <c r="Q19" t="n">
+        <v>1</v>
+      </c>
+      <c r="R19" t="n">
         <v>2</v>
       </c>
-      <c r="R19" t="n">
-        <v>1</v>
-      </c>
       <c r="S19" t="n">
+        <v>1</v>
+      </c>
+      <c r="T19" t="n">
         <v>0.5</v>
       </c>
-      <c r="T19" t="n">
-        <v>1</v>
-      </c>
       <c r="U19" t="n">
         <v>1</v>
       </c>
@@ -2732,30 +2788,33 @@
         <v>1</v>
       </c>
       <c r="X19" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y19" t="n">
         <v>310</v>
       </c>
-      <c r="Y19" t="n">
+      <c r="Z19" t="n">
         <v>0.7</v>
       </c>
-      <c r="Z19" t="n">
-        <v>90.21447968482971</v>
-      </c>
-      <c r="AA19" t="inlineStr">
+      <c r="AA19" t="n">
+        <v>88.86415815353394</v>
+      </c>
+      <c r="AB19" t="inlineStr">
         <is>
           <t>Qwen/Qwen3.5-9B</t>
         </is>
       </c>
-      <c r="AB19" t="inlineStr">
+      <c r="AC19" t="inlineStr">
         <is>
           <t>Peraturan Menteri Ketenagakerjaan No. 21 Tahun 2020, Pasal 1 bagian 1 | permen_Nomor_21_Tahun_2020.pdf | Pasal 1</t>
         </is>
       </c>
-      <c r="AC19" t="inlineStr">
+      <c r="AD19" t="inlineStr">
         <is>
           <t>Peraturan Menteri Ketenagakerjaan No. 21 Tahun 2020, Pasal 1 bagian 1 | permen_Nomor_21_Tahun_2020.pdf | Pasal 1 || Peraturan Menteri Ketenagakerjaan No. 6 Tahun 2020, Pasal 24 | Permen_Nomor_6_Tahun_2020.pdf | Pasal 24 || Peraturan Menteri Ketenagakerjaan No. 6 Tahun 2020, Pasal 16 | Permen_Nomor_6_Tahun_2020.pdf | Pasal 16 || Peraturan Menteri Ketenagakerjaan No. 21 Tahun 2020, Pasal 18 | permen_Nomor_21_Tahun_2020.pdf | Pasal 18 || Peraturan Pemerintah No. 60 Tahun 2020, Pasal 1 | PP_Nomor_69_Tahun_2020.pdf | Pasal 1 || Undang-Undang No. 8 Tahun 2016, Pasal 48 | UU_Nomor_8_Tahun_2016.pdf | Pasal 48 || Peraturan Menteri Ketenagakerjaan No. 6 Tahun 2020, Pasal 13 | Permen_Nomor_6_Tahun_2020.pdf | Pasal 13 || Peraturan Menteri Ketenagakerjaan No. PER.08/MEN/V/2008 Tahun 2008, Pasal 21 | PERMEN08v2008.pdf | Pasal 21</t>
         </is>
       </c>
-      <c r="AD19" t="inlineStr">
+      <c r="AE19" t="inlineStr">
         <is>
           <t>[{"rank": 1, "chunk_id": "bb18a659818625baf98b6227e3bad6115c9cd25d", "reference": "Peraturan Menteri Ketenagakerjaan No. 21 Tahun 2020, Pasal 1 bagian 1 | permen_Nomor_21_Tahun_2020.pdf | Pasal 1", "source_file": "permen_Nomor_21_Tahun_2020.pdf", "pasal_id": "Pasal 1", "rrf_score": 0.02538109756097561, "rerank_score": 0.8576989769935608, "text_preview": "Peraturan Menteri Ketenagakerjaan No. 21 Tahun 2020 tentang PEDOMAN PENYELENGGARAAN UNIT LAYANAN DISABILITAS BIDANG KETENAGAKERJAAN BAB I - Ketentuan Umum Pasal 1 bagian 1 1. Penyandang Disabilitas adalah setiap orang yaing mengalami keterbatasan fisik, intelektual, mental, dan/atau sensorik dalam jangka waktu lama yang dalam berinteraksi dengan lingkungan dapat mengalami hambatan dan kesulitan untuk berpartisipasi secara penuh dan efektif dengan warga negara lainnya berdasarkan kesamaan hak. 2."}, {"rank": 2, "chunk_id": "12fd1b0b9319e2d80dcdffbc9db124d93f489134", "reference": "Peraturan Menteri Ketenagakerjaan No. 6 Tahun 2020, Pasal 24 | Permen_Nomor_6_Tahun_2020.pdf | Pasal 24", "source_file": "Permen_Nomor_6_Tahun_2020.pdf", "pasal_id": "Pasal 24", "rrf_score": 0.024509440947797112, "rerank_score": 0.7766537666320801, "text_preview": "Peraturan Menteri Ketenagakerjaan No. 6 Tahun 2020 tentang PENYELENGGARAAN PEMAGANGAN DI DALAM NEGERI BAB V - Penyelenggaraan Pemagangan Pasal 24 Penyelenggaraan Pemagangan bagi peserta Pemagangan penyandang disabilitas dilaksanakan dengan memperhatikan kebutuhan khusus peserta Pemagangan penyandang disabilitas."}, {"rank": 3, "chunk_id": "f49488fdf28fee2e804df7d607c58e82cca9b34e", "reference": "Peraturan Menteri Ketenagakerjaan No. 6 Tahun 2020, Pasal 16 | Permen_Nomor_6_Tahun_2020.pdf | Pasal 16", "source_file": "Permen_Nomor_6_Tahun_2020.pdf", "pasal_id": "Pasal 16", "rrf_score": 0.027404295051353875, "rerank_score": 0.7387272715568542, "text_preview": "Peraturan Menteri Ketenagakerjaan No. 6 Tahun 2020 tentang PENYELENGGARAAN PEMAGANGAN DI DALAM NEGERI BAB IV - Hak Dan Kewajiban Bagian Kedua - Hak Dan Kewajiban Penyelenggara Pemagangan Pasal 16 Penyelenggara Pemagangan mempunyai kewajiban untuk: a. membimbing peserta Pemagangan sesuai dengan program Pemagangan; b. memenuhi hak peserta Pemagangan sesuai dengan Perjanjian Pemagangan; c. menyediakan alat pelindung diri sesuai dengan persyaratan keselamatan dan kesehatan kerja; d. memberikan uang "}, {"rank": 4, "chunk_id": "690e0dd8e4d76fdda1e5c30fe3afe2a9fa1fa0cc", "reference": "Peraturan Menteri Ketenagakerjaan No. 21 Tahun 2020, Pasal 18 | permen_Nomor_21_Tahun_2020.pdf | Pasal 18", "source_file": "permen_Nomor_21_Tahun_2020.pdf", "pasal_id": "Pasal 18", "rrf_score": 0.025588844921801395, "rerank_score": 0.6639803051948547, "text_preview": "Peraturan Menteri Ketenagakerjaan No. 21 Tahun 2020 tentang PEDOMAN PENYELENGGARAAN UNIT LAYANAN DISABILITAS BIDANG KETENAGAKERJAAN BAB V - Tugas Unit Layanan Disabilitas Pasal 18 Tugas ULD Ketenagakerjaan meliputi: a. merencanakan Penghormatan, Pelindungan, dan Pemenuhan hak atas pekerjaan Penyandang Disabilitas; b. memberikan informasi kepada Pemerintah, Pemerintah Daerah, dan perusahaan swasta mengenai proses rekrutmen, penerimaan, Pelatihan Kerja, penempatan kerja, keberlanjutan kerja, dein "}, {"rank": 5, "chunk_id": "770e5427c12db698ce7e15cde191cbd2c1ce8a99", "reference": "Peraturan Pemerintah No. 60 Tahun 2020, Pasal 1 | PP_Nomor_69_Tahun_2020.pdf | Pasal 1", "source_file": "PP_Nomor_69_Tahun_2020.pdf", "pasal_id": "Pasal 1", "rrf_score": 0.011627906976744186, "rerank_score": 0.6457191109657288, "text_preview": "Peraturan Pemerintah No. 60 Tahun 2020 tentang UNIT LAYANAN DISABILITAS BIDANG KETENAGAKERJAAN BAB I - Ketentuan Umum Pasal 1 1. Penghormatan adalah sikap menghargai atau menerima keberadaan Penyandang Disabilitas dengan segala hak yang melekat tanpa berkurang. 2. Pelindungan adalah upaya yang dilakukan secara sadar untuk melindungi, mengayomi, dan memperkuat hak Penyandang Disabilitas. 3. Pemenuhan adalah upaya yang dilakukan untuk memenuhi, melaksanakan, dan mewrrjudkan hak Penyandang Disabili"}, {"rank": 6, "chunk_id": "f78039b2d68d6d28545ec07bef8ba32df042bdb6", "reference": "Undang-Undang No. 8 Tahun 2016, Pasal 48 | UU_Nomor_8_Tahun_2016.pdf | Pasal 48", "source_file": "UU_Nomor_8_Tahun_2016.pdf", "pasal_id": "Pasal 48", "rrf_score": 0.02447411743186391, "rerank_score": 0.6322104334831238, "text_preview": "Undang-Undang No. 8 Tahun 2016 tentang PENYANDANG DISABILITAS BAB IV - Pelaksanaan Penghormatan, Pelindungan, Bagian Keempat - Pekerjaan, Kewirausahaan, Dan Koperasi Pasal 48 Pemberi Kerja dalam penempatan tenaga kerja Penyandang Disabilitas dapat: a. memberikan kesempatan untuk masa orientasi atau adaptasi di awal masa kerja untuk menentukan apa yang diperlukan, termasuk penyelenggaraan pelatihan atau magang; b. menyediakan tempat bekerja yang fleksibel dengan menyesuaikan kepada ragam disabili"}, {"rank": 7, "chunk_id": "fd5819bb26de464c4b83d6e84e0218f5a47cca62", "reference": "Peraturan Menteri Ketenagakerjaan No. 6 Tahun 2020, Pasal 13 | Permen_Nomor_6_Tahun_2020.pdf | Pasal 13", "source_file": "Permen_Nomor_6_Tahun_2020.pdf", "pasal_id": "Pasal 13", "rrf_score": 0.011111111111111112, "rerank_score": 0.562305748462677, "text_preview": "Peraturan Menteri Ketenagakerjaan No. 6 Tahun 2020 tentang PENYELENGGARAAN PEMAGANGAN DI DALAM NEGERI BAB IV - Hak Dan Kewajiban Bagian Kesatu - Hak Dan Kewajiban Peserta Pemagangan Pasal 13 (1) Peserta Pemagangan mempunyai hak untuk: a. memperoleh bimbingan dari Pembimbing Pemagangan atau instruktur; b. memperoleh pemenuhan hak sesuai dengan Perjanjian Pemagangan; c. memperoleh fasilitas keselamatan dan kesehatan kerja selama mengikuti Pemagangan; d. memperoleh uang saku; e. diikutsertakan dala"}, {"rank": 8, "chunk_id": "d6267dba3237dedd186ee1756f2708c1b905367f", "reference": "Peraturan Menteri Ketenagakerjaan No. PER.08/MEN/V/2008 Tahun 2008, Pasal 21 | PERMEN08v2008.pdf | Pasal 21", "source_file": "PERMEN08v2008.pdf", "pasal_id": "Pasal 21", "rrf_score": 0.012121212121212121, "rerank_score": 0.5527804493904114, "text_preview": "Peraturan Menteri Ketenagakerjaan No. PER.08/MEN/V/2008 Tahun 2008 tentang TATA CARA PERIZINAN DAN PENYELENGGARAAN PEMAGANGAN DI LUAR NEGERI MENTERI TENAGA KERJA DAN TRANSMIGRASI REPUBLIK INDONESIA, BAB VI - Hak Dan Kewajiban Pasal 21 (1) Penyelenggara pemagangan di luar negeri berkewajiban untuk : a. menyediakan uang saku dan transport sesuai dengan perjanjian antara peserta pemagangan dengan penyelenggara pemagangan; b. menyediakan fasilitas pelatihan; c. menyediakan instruktur dan tenaga kepe"}]</t>
         </is>
@@ -2808,7 +2867,7 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>0.7225060520416653</v>
+        <v>0.7188415389794571</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -2816,27 +2875,27 @@
         </is>
       </c>
       <c r="H20" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I20" t="n">
         <v>0.664071798324585</v>
       </c>
-      <c r="I20" t="n">
+      <c r="J20" t="n">
         <v>0.4615384615384616</v>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>BP2MI; pekerja migran; permintaan pemberi kerja berbadan hukum; perjanjian tertulis; perjanjian penempatan; perjanjian kerja</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>hak dan kewajiban; mekanisme pelindungan; penyelesaian sengketa; sertifikat kompetensi; paspor; visa kerja; pekerjaan upah perintah</t>
         </is>
       </c>
-      <c r="L20" t="n">
+      <c r="M20" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="M20" t="n">
-        <v>1</v>
-      </c>
       <c r="N20" t="n">
         <v>1</v>
       </c>
@@ -2868,30 +2927,33 @@
         <v>1</v>
       </c>
       <c r="X20" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y20" t="n">
         <v>213</v>
       </c>
-      <c r="Y20" t="n">
-        <v>1</v>
-      </c>
       <c r="Z20" t="n">
-        <v>58.43816423416138</v>
-      </c>
-      <c r="AA20" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>57.62241983413696</v>
+      </c>
+      <c r="AB20" t="inlineStr">
         <is>
           <t>Qwen/Qwen3.5-9B</t>
         </is>
       </c>
-      <c r="AB20" t="inlineStr">
+      <c r="AC20" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 10 Tahun 2020, Pasal 3 | PP_10_2020.pdf | Pasal 3</t>
         </is>
       </c>
-      <c r="AC20" t="inlineStr">
+      <c r="AD20" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 10 Tahun 2020, Pasal 3 | PP_10_2020.pdf | Pasal 3 || Peraturan Pemerintah No. 10 Tahun 2020, Pasal 4 | PP_10_2020.pdf | Pasal 4 || Peraturan Pemerintah No. 10 Tahun 2020, Pasal 7 | PP_10_2020.pdf | Pasal 7 || Peraturan Pemerintah No. 10 Tahun 2020, Pasal 2 | PP_10_2020.pdf | Pasal 2 || Undang-Undang No. 18 Tahun 2017, Pasal 1 bagian 1 | UU_Nomor_18_Tahun_2017.pdf | Pasal 1 || Peraturan Pemerintah No. 10 Tahun 2020, Pasal 1 bagian 1 | PP_10_2020.pdf | Pasal 1 || Undang-Undang No. 18 Tahun 2017, Pasal 50 | UU_Nomor_18_Tahun_2017.pdf | Pasal 50 || Undang-Undang No. 18 Tahun 2017, Pasal 1 | UU_Nomor_18_Tahun_2017.pdf | Pasal 1</t>
         </is>
       </c>
-      <c r="AD20" t="inlineStr">
+      <c r="AE20" t="inlineStr">
         <is>
           <t>[{"rank": 1, "chunk_id": "4e76c5df7ea23fd2d8fc3d87aeb944fb5cbf3eae", "reference": "Peraturan Pemerintah No. 10 Tahun 2020, Pasal 3 | PP_10_2020.pdf | Pasal 3", "source_file": "PP_10_2020.pdf", "pasal_id": "Pasal 3", "rrf_score": 0.025999598151496883, "rerank_score": 0.9922250509262085, "text_preview": "Peraturan Pemerintah No. 10 Tahun 2020 BAB I - Ketentuan Umum Pasal 3 (1) Penempatan Pekerja Migran Indonesia oleh BP2MI sebagaimana dimaksud dalam Pasal 2 dilakukan atas dasar perjanjian secara tertulis antara pemerintah dengan pemerintah negara Pemberi Kerja Pekerja Migran Indonesia atau Pemberi Kerja berbadan hukum di negara tujuan penempatan. (2) Dalam...SK No 022504 A Presiden (2) Dalam hal inisiasi perjanjian secara tertulis sebagaimana dimaksud pada ayat (1) berasal dari kementerian / lem"}, {"rank": 2, "chunk_id": "51d04747a44099003edace7f2adc2257bbecab09", "reference": "Peraturan Pemerintah No. 10 Tahun 2020, Pasal 4 | PP_10_2020.pdf | Pasal 4", "source_file": "PP_10_2020.pdf", "pasal_id": "Pasal 4", "rrf_score": 0.025553319919517103, "rerank_score": 0.9915762543678284, "text_preview": "Peraturan Pemerintah No. 10 Tahun 2020 tentang TATA CARA PENEMPATAN PEKERJA MIGRAN INDONESIA OLEH BADAN PELINDUNGAN PEKERJA MIGRAN INDONESIA BAB I - Ketentuan Umum Pasal 4 (1) Pembuatan perjanjian secara tertulis mengenai penempatan Pekerja Migran Indonesia oleh BP2MI sebagaimana dimaksud dalam Pasal 3 dilakukan sesuai dengan ketentuan peraturan perundangundangan mengenai perjanjian internasional. (2) Pembuatan perjanjian secara tertulis mengenai penempatan Pekerja Migran Indonesia sebagaimana d"}, {"rank": 3, "chunk_id": "28ada90e61611072addfa4b5f92479f0f8cae080", "reference": "Peraturan Pemerintah No. 10 Tahun 2020, Pasal 7 | PP_10_2020.pdf | Pasal 7", "source_file": "PP_10_2020.pdf", "pasal_id": "Pasal 7", "rrf_score": 0.02924378635642517, "rerank_score": 0.9910332560539246, "text_preview": "Peraturan Pemerintah No. 10 Tahun 2020 tentang TATA CARA PENEMPATAN PEKERJA MIGRAN INDONESIA OLEH BADAN PELINDUNGAN PEKERJA MIGRAN INDONESIA BAB II - Pelaksanaan Penempatan Bagian Kesatu - Umum Pasal 7 (1) BP2MI dalam menempatkan Pekerja Migran Indonesia kepada Pemberi Keda berbadan hukum di negara tujuan penempatan harus memiliki surat permintaan Pekerja Migran Indonesia yang telah diverifikasi oleh Atase Ketenagakerjaan. (2) Surat permintaan Pekerja Migran Indonesia sebagaimana dimaksud pada a"}, {"rank": 4, "chunk_id": "78de6cc0563d4f1b608e50465829aa4794b6382c", "reference": "Peraturan Pemerintah No. 10 Tahun 2020, Pasal 2 | PP_10_2020.pdf | Pasal 2", "source_file": "PP_10_2020.pdf", "pasal_id": "Pasal 2", "rrf_score": 0.02735234673253986, "rerank_score": 0.9886372685432434, "text_preview": "Peraturan Pemerintah No. 10 Tahun 2020 tentang TATA CARA PENEMPATAN PEKERJA MIGRAN INDONESIA OLEH BADAN PELINDUNGAN PEKERJA MIGRAN INDONESIA BAB I - Ketentuan Umum Pasal 2 Penempatan Pekerja Migran Indonesia oleh BP2MI didasarkan: a. kebutuhan pemerintah; dan b. permintaan dari pemerintah negara Pemberi Kerja Pekerja Migran Indonesia atau permintaan Pemberi Kerja berbadan hukum di negara tujuan penempatan."}, {"rank": 5, "chunk_id": "cb42273139919fc743f8b722c110ece9769fe1d0", "reference": "Undang-Undang No. 18 Tahun 2017, Pasal 1 bagian 1 | UU_Nomor_18_Tahun_2017.pdf | Pasal 1", "source_file": "UU_Nomor_18_Tahun_2017.pdf", "pasal_id": "Pasal 1", "rrf_score": 0.012903225806451613, "rerank_score": 0.9803598523139954, "text_preview": "Undang-Undang No. 18 Tahun 2017 tentang PELINDUNGAN PEKERJA MIGRAN INDONESIA BAB I - Ketentuan Umum Pasal 1 bagian 1 1. Calon Pekerja Migran Indonesia adalah setiap tenaga kerja Indonesia yang memenuhi syarat sebagai pencari kerja yang akan bekerja di luar negeri dan terdaftar di instansi pemerintah kabupaten/ kota yang bertanggung jawab di bidang ketenagakerjaan. 2. Pekerja Migran Indonesia adalah setiap warga negara Indonesia yang akan, sedang, atau telah melakukan pekerjaan dengan menerima up"}, {"rank": 6, "chunk_id": "6bbbfbf6b4875d9fd7a274e978532c2e337e4e33", "reference": "Peraturan Pemerintah No. 10 Tahun 2020, Pasal 1 bagian 1 | PP_10_2020.pdf | Pasal 1", "source_file": "PP_10_2020.pdf", "pasal_id": "Pasal 1", "rrf_score": 0.012698412698412698, "rerank_score": 0.9780359864234924, "text_preview": "Peraturan Pemerintah No. 10 Tahun 2020 tentang TATA CARA PENEMPATAN PEKERJA MIGRAN INDONESIA OLEH BADAN PELINDUNGAN PEKERJA MIGRAN INDONESIA BAB I - Ketentuan Umum Pasal 1 bagian 1 1. Calon Pekerja Migran Indonesia adalah setiap tenaga kerja Indonesia yang memenuhi syarat sebagai pencari kerja yang akan bekerja di luar negeri dan terdaftar di instansi pemerintah kabupaten/kota yang bertanggung jawab di bidang ketenagakerjaan. 2. Pekerja Migran Indonesia adalah setiap warga negara Indonesia yang "}, {"rank": 7, "chunk_id": "f53887e2623f6ccf9cd08c06697a663768d22953", "reference": "Undang-Undang No. 18 Tahun 2017, Pasal 50 | UU_Nomor_18_Tahun_2017.pdf | Pasal 50", "source_file": "UU_Nomor_18_Tahun_2017.pdf", "pasal_id": "Pasal 50", "rrf_score": 0.020460358056265983, "rerank_score": 0.9764377474784851, "text_preview": "Undang-Undang No. 18 Tahun 2017 tentang PELINDUNGAN PEKERJA MIGRAN INDONESIA BAB VII - Pelaksana Penempatan Pekerja Migran Indonesia Bagian Kesatu - Umum Pasal 50 1) Penempatan Pekerja Migran Indonesia oleh Badan ( sebagaimana dimaksud dalam Pasal 49 huruf a, dilakukan atas dasar perjanjian secara tertulis antara pemerintah dengan pemerintah negara Pemberi Kerja Pekerja Migran Indonesia atau Pemberi Kerja berbadan hukum di negara tujuan penempatan. (2) Ketentuan lebih lanjut mengenai tata cara p"}, {"rank": 8, "chunk_id": "d051de810c5f242f4342877c76c56974c304fb4e", "reference": "Undang-Undang No. 18 Tahun 2017, Pasal 1 | UU_Nomor_18_Tahun_2017.pdf | Pasal 1", "source_file": "UU_Nomor_18_Tahun_2017.pdf", "pasal_id": "Pasal 1", "rrf_score": 0.011594202898550725, "rerank_score": 0.9713289737701416, "text_preview": "Undang-Undang No. 18 Tahun 2017 BAB I - Ketentuan Umum Pasal 1 SITASI: Undang-Undang No. 18 Tahun 2017, Pasal 1 Pekerja Migran Indonesia yang memuat hak dan kewajiban setiap pihak, dalam rangka penempatan Pekerja Migran Indonesia di negara tujuan penempatan sesuai dengan ketentuan peraturan perundang-undangan. 14. Perjanjian Kerja adalah perjanjian tertulis antara Pekerja Migran Indonesia dan Pemberi Kerja yang memuat syarat kerja, hak, dan kewajiban setiap pihak, serta jaminan keamanan dan kese"}]</t>
         </is>
@@ -2935,7 +2997,7 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0.7673922807511829</v>
+        <v>0.7755328321139018</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -2943,27 +3005,27 @@
         </is>
       </c>
       <c r="H21" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="I21" t="n">
         <v>0.7204411029815674</v>
       </c>
-      <c r="I21" t="n">
+      <c r="J21" t="n">
         <v>0.5714285714285714</v>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>narkotika; tempat kerja; kebijakan tertulis; instansi ketenagakerjaan; pemagangan; fasilitas K3; JKK; JKM</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>psikotropika; zat adiktif; konsultasi pekerja; lapor Kepolisian; alat pelindung diri; pemberi kerja wajib membayar hak pekerja</t>
         </is>
       </c>
-      <c r="L21" t="n">
+      <c r="M21" t="n">
         <v>0.4285714285714285</v>
       </c>
-      <c r="M21" t="n">
-        <v>1</v>
-      </c>
       <c r="N21" t="n">
         <v>1</v>
       </c>
@@ -2995,30 +3057,33 @@
         <v>1</v>
       </c>
       <c r="X21" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y21" t="n">
         <v>296</v>
       </c>
-      <c r="Y21" t="n">
+      <c r="Z21" t="n">
         <v>0.7466666666666666</v>
       </c>
-      <c r="Z21" t="n">
-        <v>80.26819157600403</v>
-      </c>
-      <c r="AA21" t="inlineStr">
+      <c r="AA21" t="n">
+        <v>79.33536076545715</v>
+      </c>
+      <c r="AB21" t="inlineStr">
         <is>
           <t>Qwen/Qwen3.5-9B</t>
         </is>
       </c>
-      <c r="AB21" t="inlineStr">
+      <c r="AC21" t="inlineStr">
         <is>
           <t>Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 8 | PER-11-MEN-VI-2005.pdf | Pasal 8</t>
         </is>
       </c>
-      <c r="AC21" t="inlineStr">
+      <c r="AD21" t="inlineStr">
         <is>
           <t>Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 8 | PER-11-MEN-VI-2005.pdf | Pasal 8 || Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 1 | PER-11-MEN-VI-2005.pdf | Pasal 1 || Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 2 | PER-11-MEN-VI-2005.pdf | Pasal 2 || Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 4 | PER-11-MEN-VI-2005.pdf | Pasal 4 || Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 7 | PER-11-MEN-VI-2005.pdf | Pasal 7 || Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 3 | PER-11-MEN-VI-2005.pdf | Pasal 3 || Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 6 | PER-11-MEN-VI-2005.pdf | Pasal 6 || Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 5 | PER-11-MEN-VI-2005.pdf | Pasal 5</t>
         </is>
       </c>
-      <c r="AD21" t="inlineStr">
+      <c r="AE21" t="inlineStr">
         <is>
           <t>[{"rank": 1, "chunk_id": "d4a3cd017d35710822165797f505a97a06c5cdd2", "reference": "Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 8 | PER-11-MEN-VI-2005.pdf | Pasal 8", "source_file": "PER-11-MEN-VI-2005.pdf", "pasal_id": "Pasal 8", "rrf_score": 0.027813314380478557, "rerank_score": 0.9582530856132507, "text_preview": "Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005 tentang PENCEGAHAN DAN PENANGGULANGAN PENYALAHGUNAAN DAN PEREDARAN GELAP NARKOTIKA, PSIKOTROPIKA DAN ZAT ADIKTIF LAINNYA DI TEMPAT KERJA MENTERI TENAGA KERJA DAN TRANSMIGRASI REPUBLIK INDONESIA, Pasal 8 (1) Pengusaha atau pekerja/buruh harus segera melaporkan kepada Kepolisian Negara Republik Indonesia apabila ditemukan seseorang atau lebih memiliki atau mengedarkan narkotika, psikotropika dan zat adiktif lainnya di tempat kerja"}, {"rank": 2, "chunk_id": "19c64543a0069c8ef48fa59e57b8e6db2653935d", "reference": "Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 1 | PER-11-MEN-VI-2005.pdf | Pasal 1", "source_file": "PER-11-MEN-VI-2005.pdf", "pasal_id": "Pasal 1", "rrf_score": 0.027003642987249544, "rerank_score": 0.8955042958259583, "text_preview": "Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005 tentang PENCEGAHAN DAN PENANGGULANGAN PENYALAHGUNAAN DAN PEREDARAN GELAP NARKOTIKA, PSIKOTROPIKA DAN ZAT ADIKTIF LAINNYA DI TEMPAT KERJA MENTERI TENAGA KERJA DAN TRANSMIGRASI REPUBLIK INDONESIA, Pasal 1 1. Narkotika adalah zat atau obat yang berasal dari tanaman atau bukan tanaman, baik sintetis maupun semi sintetis yang dapat menyebabkan penurunan atau perubahan kesadaran, hilangnya rasa, mengurangi sampai menghilangkan rasa ny"}, {"rank": 3, "chunk_id": "ad4032ac90dd8ccb54ede6209a5869243a04add6", "reference": "Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 2 | PER-11-MEN-VI-2005.pdf | Pasal 2", "source_file": "PER-11-MEN-VI-2005.pdf", "pasal_id": "Pasal 2", "rrf_score": 0.029296668429402435, "rerank_score": 0.8940011858940125, "text_preview": "Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005 tentang PENCEGAHAN DAN PENANGGULANGAN PENYALAHGUNAAN DAN PEREDARAN GELAP NARKOTIKA, PSIKOTROPIKA DAN ZAT ADIKTIF LAINNYA DI TEMPAT KERJA MENTERI TENAGA KERJA DAN TRANSMIGRASI REPUBLIK INDONESIA, Pasal 2 (1) Pengusaha wajib melakukan upaya aktif pencegahan dan penanggulangan penyalahgunaan dan peredaran gelap narkotika, psikotropika dan zat adiktif lainnya di tempat kerja. (2) Upaya aktif pencegahan dan penanggulangan penyalahgun"}, {"rank": 4, "chunk_id": "b2e63601c8281e33a6c274f74c566fa718b6b6c6", "reference": "Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 4 | PER-11-MEN-VI-2005.pdf | Pasal 4", "source_file": "PER-11-MEN-VI-2005.pdf", "pasal_id": "Pasal 4", "rrf_score": 0.028436724565756823, "rerank_score": 0.7896694540977478, "text_preview": "Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005 tentang PENCEGAHAN DAN PENANGGULANGAN PENYALAHGUNAAN DAN PEREDARAN GELAP NARKOTIKA, PSIKOTROPIKA DAN ZAT ADIKTIF LAINNYA DI TEMPAT KERJA MENTERI TENAGA KERJA DAN TRANSMIGRASI REPUBLIK INDONESIA, Pasal 4 (1) Proses penetapan kebijakan sebagaimana dimaksud dalam Pasal 2 ayat (2) huruf a, harus melalui konsultasi antara pengusaha dengan pekerja/buruh dan atau serikat pekerja/serikat buruh. (2) Kebijakan sebagaimana dimaksud pada ay"}, {"rank": 5, "chunk_id": "c026e822c01cffb77eda5aae2b83801f86920ce0", "reference": "Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 7 | PER-11-MEN-VI-2005.pdf | Pasal 7", "source_file": "PER-11-MEN-VI-2005.pdf", "pasal_id": "Pasal 7", "rrf_score": 0.02658450704225352, "rerank_score": 0.6980270147323608, "text_preview": "Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005 tentang PENCEGAHAN DAN PENANGGULANGAN PENYALAHGUNAAN DAN PEREDARAN GELAP NARKOTIKA, PSIKOTROPIKA DAN ZAT ADIKTIF LAINNYA DI TEMPAT KERJA MENTERI TENAGA KERJA DAN TRANSMIGRASI REPUBLIK INDONESIA, Pasal 7 (1) Ketentuan lebih lanjut mengenai pekerja/buruh yang membutuhkan perawatan dan atau rehabilitasi akibat penyalahgunaan narkotika, psikotropika dan zat adiktif lainnya sebagaimana dimaksud dalam Pasal 6 diatur dalam Perjanjian K"}, {"rank": 6, "chunk_id": "d1d78ece45f74f9324a7147bc8c062e7ca232584", "reference": "Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 3 | PER-11-MEN-VI-2005.pdf | Pasal 3", "source_file": "PER-11-MEN-VI-2005.pdf", "pasal_id": "Pasal 3", "rrf_score": 0.028083028083028084, "rerank_score": 0.6935468912124634, "text_preview": "Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005 tentang PENCEGAHAN DAN PENANGGULANGAN PENYALAHGUNAAN DAN PEREDARAN GELAP NARKOTIKA, PSIKOTROPIKA DAN ZAT ADIKTIF LAINNYA DI TEMPAT KERJA MENTERI TENAGA KERJA DAN TRANSMIGRASI REPUBLIK INDONESIA, Pasal 3 Dalam melaksanakan upaya pencegahan dan penanggulangan penyalahgunaan dan peredaran gelap narkotika, psikotropika dan zat adiktif lainnya di tempat kerja, pengusaha, pekerja/buruh dan serikat pekerja/serikat buruh dapat berkonsul"}, {"rank": 7, "chunk_id": "71b1d9732eef3b3d2607786e2235231985ec385a", "reference": "Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 6 | PER-11-MEN-VI-2005.pdf | Pasal 6", "source_file": "PER-11-MEN-VI-2005.pdf", "pasal_id": "Pasal 6", "rrf_score": 0.026613965744400527, "rerank_score": 0.5322794914245605, "text_preview": "Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005 tentang PENCEGAHAN DAN PENANGGULANGAN PENYALAHGUNAAN DAN PEREDARAN GELAP NARKOTIKA, PSIKOTROPIKA DAN ZAT ADIKTIF LAINNYA DI TEMPAT KERJA MENTERI TENAGA KERJA DAN TRANSMIGRASI REPUBLIK INDONESIA, Pasal 6 (1) Pengusaha dapat meminta pekerja/buruh yang diduga menyalahgunakan narkotika, psikotropika dan zat adiktif lainnya untuk melakukan tes dengan biaya ditanggung oleh perusahaan. (2) Pelaksanaan tes sebagaimana dimaksud pada ayat"}, {"rank": 8, "chunk_id": "222c468369071cb510fc2fe197df81ab0e884199", "reference": "Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 5 | PER-11-MEN-VI-2005.pdf | Pasal 5", "source_file": "PER-11-MEN-VI-2005.pdf", "pasal_id": "Pasal 5", "rrf_score": 0.02253968253968254, "rerank_score": 0.4955546259880066, "text_preview": "Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005 tentang PENCEGAHAN DAN PENANGGULANGAN PENYALAHGUNAAN DAN PEREDARAN GELAP NARKOTIKA, PSIKOTROPIKA DAN ZAT ADIKTIF LAINNYA DI TEMPAT KERJA MENTERI TENAGA KERJA DAN TRANSMIGRASI REPUBLIK INDONESIA, Pasal 5 (1) Pelaksanaan program sebagaimana dimaksud dalam Pasal 2 ayat (2) huruf b, dilaksanakan dengan cara : a. mengkomunikasikan kebijakan dan program kepada semua pekerja/buruh; b. melaksanakan program penyuluhan, pendidikan dan lat"}]</t>
         </is>
@@ -3035,7 +3100,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3068,55 +3133,55 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>semantic_similarity</t>
+          <t>llm_judge_score</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.7520683497190476</v>
+        <v>0.845</v>
       </c>
       <c r="C2" t="n">
-        <v>0.7659493088722229</v>
+        <v>0.95</v>
       </c>
       <c r="D2" t="n">
-        <v>0.6428685188293457</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>0.8587865829467773</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>keyword_coverage</t>
+          <t>semantic_similarity</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.7664102564102565</v>
+        <v>0.7520683497190476</v>
       </c>
       <c r="C3" t="n">
-        <v>0.8166666666666667</v>
+        <v>0.7659493088722229</v>
       </c>
       <c r="D3" t="n">
-        <v>0.4285714285714285</v>
+        <v>0.6428685188293457</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>0.8587865829467773</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>retrieval_citation_coverage</t>
+          <t>keyword_coverage</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.8480952380952379</v>
+        <v>0.7664102564102565</v>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>0.8166666666666667</v>
       </c>
       <c r="D4" t="n">
-        <v>0.2</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="E4" t="n">
         <v>1</v>
@@ -3125,17 +3190,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>retrieval_article_hit</t>
+          <t>retrieval_citation_coverage</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>0.8480952380952379</v>
       </c>
       <c r="C5" t="n">
         <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -3144,7 +3209,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>retrieval_law_hit</t>
+          <t>retrieval_article_hit</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -3163,7 +3228,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>answer_citation_hit</t>
+          <t>retrieval_law_hit</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -3182,17 +3247,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>article_hit_at_3</t>
+          <t>answer_citation_hit</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="C8" t="n">
         <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
         <v>1</v>
@@ -3201,17 +3266,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>article_mrr</t>
+          <t>article_hit_at_3</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.6421428571428571</v>
+        <v>0.75</v>
       </c>
       <c r="C9" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>0.1428571428571428</v>
+        <v>0</v>
       </c>
       <c r="E9" t="n">
         <v>1</v>
@@ -3220,17 +3285,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>precision_at_3</t>
+          <t>article_mrr</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.7166666666666667</v>
+        <v>0.6421428571428571</v>
       </c>
       <c r="C10" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.5</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>0.1428571428571428</v>
       </c>
       <c r="E10" t="n">
         <v>1</v>
@@ -3239,17 +3304,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>answer_length_score</t>
+          <t>precision_at_3</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.953</v>
+        <v>0.7166666666666667</v>
       </c>
       <c r="C11" t="n">
-        <v>1</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="D11" t="n">
-        <v>0.6666666666666667</v>
+        <v>0</v>
       </c>
       <c r="E11" t="n">
         <v>1</v>
@@ -3258,17 +3323,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>article_hit_at_8</t>
+          <t>answer_length_score</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1</v>
+        <v>0.953</v>
       </c>
       <c r="C12" t="n">
         <v>1</v>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>0.6666666666666667</v>
       </c>
       <c r="E12" t="n">
         <v>1</v>
@@ -3277,17 +3342,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>law_mrr</t>
+          <t>article_hit_at_8</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.8875</v>
+        <v>1</v>
       </c>
       <c r="C13" t="n">
         <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="E13" t="n">
         <v>1</v>
@@ -3296,57 +3361,76 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>overall_score</t>
+          <t>law_mrr</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.8400745973777509</v>
+        <v>0.8875</v>
       </c>
       <c r="C14" t="n">
-        <v>0.8515650147596995</v>
+        <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>0.7096137903531392</v>
+        <v>0.25</v>
       </c>
       <c r="E14" t="n">
-        <v>0.968933048248291</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>latency_seconds</t>
+          <t>overall_score</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>42.57246607542038</v>
+        <v>0.8474470290146338</v>
       </c>
       <c r="C15" t="n">
-        <v>40.5096800327301</v>
+        <v>0.8715443336764972</v>
       </c>
       <c r="D15" t="n">
-        <v>14.76256394386292</v>
+        <v>0.5961143044630687</v>
       </c>
       <c r="E15" t="n">
-        <v>90.21447968482971</v>
+        <v>0.9788179874420168</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>latency_seconds</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>41.96127111911774</v>
+      </c>
+      <c r="C16" t="n">
+        <v>39.32658243179321</v>
+      </c>
+      <c r="D16" t="n">
+        <v>14.29284286499023</v>
+      </c>
+      <c r="E16" t="n">
+        <v>88.86415815353394</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>answer_word_count</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B17" t="n">
         <v>151.85</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C17" t="n">
         <v>138.5</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D17" t="n">
         <v>48</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E17" t="n">
         <v>320</v>
       </c>
     </row>
@@ -3361,7 +3445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3382,30 +3466,35 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>llm_judge_score</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>semantic_similarity</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>keyword_coverage</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>retrieval_citation_coverage</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>retrieval_article_hit</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>answer_citation_hit</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>latency_seconds</t>
         </is>
@@ -3421,17 +3510,17 @@
         <v>2</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9013263456026713</v>
+        <v>0.9228740235169729</v>
       </c>
       <c r="D2" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E2" t="n">
         <v>0.6802712678909302</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>0.9166666666666667</v>
       </c>
-      <c r="F2" t="n">
-        <v>1</v>
-      </c>
       <c r="G2" t="n">
         <v>1</v>
       </c>
@@ -3439,7 +3528,10 @@
         <v>1</v>
       </c>
       <c r="I2" t="n">
-        <v>30.72759449481964</v>
+        <v>1</v>
+      </c>
+      <c r="J2" t="n">
+        <v>30.76654946804047</v>
       </c>
     </row>
     <row r="3">
@@ -3452,25 +3544,28 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>0.8458163170814514</v>
+        <v>0.8650565798282623</v>
       </c>
       <c r="D3" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E3" t="n">
         <v>0.8537105321884155</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>0.8333333333333334</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>0.6</v>
       </c>
-      <c r="G3" t="n">
-        <v>1</v>
-      </c>
       <c r="H3" t="n">
         <v>1</v>
       </c>
       <c r="I3" t="n">
-        <v>90.21447968482971</v>
+        <v>1</v>
+      </c>
+      <c r="J3" t="n">
+        <v>88.86415815353394</v>
       </c>
     </row>
     <row r="4">
@@ -3483,25 +3578,28 @@
         <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>0.7673922807511829</v>
+        <v>0.7755328321139018</v>
       </c>
       <c r="D4" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="E4" t="n">
         <v>0.7204411029815674</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>0.5714285714285714</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>0.4285714285714285</v>
       </c>
-      <c r="G4" t="n">
-        <v>1</v>
-      </c>
       <c r="H4" t="n">
         <v>1</v>
       </c>
       <c r="I4" t="n">
-        <v>80.26819157600403</v>
+        <v>1</v>
+      </c>
+      <c r="J4" t="n">
+        <v>79.33536076545715</v>
       </c>
     </row>
     <row r="5">
@@ -3514,17 +3612,17 @@
         <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>0.7567363161132449</v>
+        <v>0.7361297393412818</v>
       </c>
       <c r="D5" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E5" t="n">
         <v>0.8011823892593384</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>0.5</v>
       </c>
-      <c r="F5" t="n">
-        <v>1</v>
-      </c>
       <c r="G5" t="n">
         <v>1</v>
       </c>
@@ -3532,7 +3630,10 @@
         <v>1</v>
       </c>
       <c r="I5" t="n">
-        <v>21.14453887939453</v>
+        <v>1</v>
+      </c>
+      <c r="J5" t="n">
+        <v>20.82744526863098</v>
       </c>
     </row>
     <row r="6">
@@ -3545,17 +3646,17 @@
         <v>6</v>
       </c>
       <c r="C6" t="n">
-        <v>0.8436344307244769</v>
+        <v>0.873879355724842</v>
       </c>
       <c r="D6" t="n">
+        <v>0.9333333333333332</v>
+      </c>
+      <c r="E6" t="n">
         <v>0.741285651922226</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>0.7492063492063492</v>
       </c>
-      <c r="F6" t="n">
-        <v>1</v>
-      </c>
       <c r="G6" t="n">
         <v>1</v>
       </c>
@@ -3563,7 +3664,10 @@
         <v>1</v>
       </c>
       <c r="I6" t="n">
-        <v>32.78640242417654</v>
+        <v>1</v>
+      </c>
+      <c r="J6" t="n">
+        <v>31.85996659596761</v>
       </c>
     </row>
     <row r="7">
@@ -3576,25 +3680,28 @@
         <v>1</v>
       </c>
       <c r="C7" t="n">
-        <v>0.7096137903531392</v>
+        <v>0.7382594025135041</v>
       </c>
       <c r="D7" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="E7" t="n">
         <v>0.7717293500900269</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>0.8333333333333334</v>
       </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>0.4</v>
       </c>
-      <c r="G7" t="n">
-        <v>1</v>
-      </c>
       <c r="H7" t="n">
         <v>1</v>
       </c>
       <c r="I7" t="n">
-        <v>84.05413889884949</v>
+        <v>1</v>
+      </c>
+      <c r="J7" t="n">
+        <v>83.43450665473938</v>
       </c>
     </row>
     <row r="8">
@@ -3607,25 +3714,28 @@
         <v>1</v>
       </c>
       <c r="C8" t="n">
-        <v>0.7315822368939717</v>
+        <v>0.7477272827307383</v>
       </c>
       <c r="D8" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="E8" t="n">
         <v>0.788404107093811</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="F8" t="n">
+      <c r="G8" t="n">
         <v>0.2</v>
       </c>
-      <c r="G8" t="n">
-        <v>1</v>
-      </c>
       <c r="H8" t="n">
         <v>1</v>
       </c>
       <c r="I8" t="n">
-        <v>67.36106276512146</v>
+        <v>1</v>
+      </c>
+      <c r="J8" t="n">
+        <v>66.88468241691589</v>
       </c>
     </row>
     <row r="9">
@@ -3638,17 +3748,17 @@
         <v>4</v>
       </c>
       <c r="C9" t="n">
-        <v>0.8851809893051783</v>
+        <v>0.8440627957383793</v>
       </c>
       <c r="D9" t="n">
+        <v>0.6375</v>
+      </c>
+      <c r="E9" t="n">
         <v>0.7659741938114166</v>
       </c>
-      <c r="E9" t="n">
+      <c r="F9" t="n">
         <v>0.8333333333333334</v>
       </c>
-      <c r="F9" t="n">
-        <v>1</v>
-      </c>
       <c r="G9" t="n">
         <v>1</v>
       </c>
@@ -3656,7 +3766,10 @@
         <v>1</v>
       </c>
       <c r="I9" t="n">
-        <v>39.60407477617264</v>
+        <v>1</v>
+      </c>
+      <c r="J9" t="n">
+        <v>39.14067429304123</v>
       </c>
     </row>
     <row r="10">
@@ -3669,17 +3782,17 @@
         <v>1</v>
       </c>
       <c r="C10" t="n">
-        <v>0.8937286732991535</v>
+        <v>0.9232998530069988</v>
       </c>
       <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="n">
         <v>0.7108879089355469</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>0.8</v>
       </c>
-      <c r="F10" t="n">
-        <v>1</v>
-      </c>
       <c r="G10" t="n">
         <v>1</v>
       </c>
@@ -3687,7 +3800,10 @@
         <v>1</v>
       </c>
       <c r="I10" t="n">
-        <v>16.92839670181274</v>
+        <v>1</v>
+      </c>
+      <c r="J10" t="n">
+        <v>16.77782320976257</v>
       </c>
     </row>
     <row r="11">
@@ -3700,25 +3816,28 @@
         <v>1</v>
       </c>
       <c r="C11" t="n">
-        <v>0.7225060520416653</v>
+        <v>0.7188415389794571</v>
       </c>
       <c r="D11" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E11" t="n">
         <v>0.664071798324585</v>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>0.4615384615384616</v>
       </c>
-      <c r="F11" t="n">
+      <c r="G11" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="G11" t="n">
-        <v>1</v>
-      </c>
       <c r="H11" t="n">
         <v>1</v>
       </c>
       <c r="I11" t="n">
-        <v>58.43816423416138</v>
+        <v>1</v>
+      </c>
+      <c r="J11" t="n">
+        <v>57.62241983413696</v>
       </c>
     </row>
     <row r="12">
@@ -3731,14 +3850,14 @@
         <v>1</v>
       </c>
       <c r="C12" t="n">
-        <v>0.968933048248291</v>
+        <v>0.9788179874420168</v>
       </c>
       <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
         <v>0.8587865829467773</v>
       </c>
-      <c r="E12" t="n">
-        <v>1</v>
-      </c>
       <c r="F12" t="n">
         <v>1</v>
       </c>
@@ -3749,7 +3868,10 @@
         <v>1</v>
       </c>
       <c r="I12" t="n">
-        <v>16.45044612884521</v>
+        <v>1</v>
+      </c>
+      <c r="J12" t="n">
+        <v>16.22343039512634</v>
       </c>
     </row>
   </sheetData>
@@ -3763,7 +3885,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3799,25 +3921,30 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>llm_judge_score</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>quality_label</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>keyword_missing</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>expected_article_rank</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>expected_law_rank</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>top1_reference</t>
         </is>
@@ -3826,20 +3953,206 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Q05</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>PKWT</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Dalam bentuk bahasa apa PKWT wajib dibuat, terutama ketika pekerjanya warga negara Indonesia?</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Berdasarkan referensi yang tersedia, **tidak ditemukan ketentuan spesifik** mengenai bentuk bahasa (misalnya wajib bahasa Indonesia atau boleh bahasa asing) yang harus digunakan dalam pembuatan Perjanjian Kerja Waktu Tertentu (PKWT), baik untuk pekerja Warga Negara Indonesia maupun lainnya.
+Referensi yang tersedia hanya mengatur bahwa PKWT harus dibuat secara **tertulis** (PP No. 35 Tahun 2021 Pasal 18 ayat 2) dan memuat isi tertentu seperti nama, alamat, jabatan, upah, serta jangka waktu (PP No. 35 Tahun 2021 Pasal 6 dan Pasal 13). Ketentuan mengenai bahasa yang digunakan dalam perjanjian kerja tidak tercantum dalam pasal-pasal yang disediakan.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>PKWT wajib dibuat secara tertulis dengan huruf latin dan menggunakan bahasa Indonesia. Jika dibuat dalam bahasa Indonesia dan bahasa asing lalu terdapat perbedaan penafsiran, naskah bahasa Indonesia yang berlaku.</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>0.5961143044630687</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>fair</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>huruf latin; penafsiran; bahasa Indonesia berlaku</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>6</v>
+      </c>
+      <c r="K2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 1 | PP Nomor 35 Tahun 2021.pdf | Pasal 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Q19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Pekerja migran Indonesia</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Calon pekerja migran akan ditempatkan melalui BP2MI berdasarkan permintaan pemberi kerja berbadan hukum di negara tujuan. Jelaskan dasar penempatannya, isi minimum perjanjian tertulis antar pihak penempatan, dan dokumen/hubungan kerja yang wajib ada bagi pekerja migran.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Berdasarkan referensi yang tersedia, berikut adalah jawaban atas pertanyaan Anda:
+**1. Dasar Penempatan**
+Penempatan Calon Pekerja Migran Indonesia (CPMI) oleh Badan Pelindungan Pekerja Migran Indonesia (BP2MI) didasarkan pada dua hal:
+*   Kebutuhan pemerintah; dan
+*   Permintaan dari pemerintah negara Pemberi Kerja atau permintaan Pemberi Kerja berbadan hukum di negara tujuan penempatan.
+*(Dasar hukum: PP Nomor 10 Tahun 2020 Pasal 2)*
+**2. Isi Minimum Perjanjian Tertulis**
+Perjanjian tertulis antara BP2MI dan CPMI (Perjanjian Penempatan) harus memuat rincian dari surat permintaan yang telah diverifikasi, yaitu:
+*   Identitas pemberi kerja;
+*   Jumlah penempatan;
+*   Jenis pekerjaan;
+*   Upah atau gaji;
+*   Kualifikasi jabatan;
+*   Masa berlaku Perjanjian Kerja;
+*   Fasilitas tempat kerja; dan
+*   Jaminan sosial dan/atau asuransi.
+*(Dasar hukum: PP Nomor 10 Tahun 2020 Pasal 7 ayat 2)*
+**3. Dokumen dan Hubungan Kerja yang Wajib Ada**
+*   **Dokumen Wajib:** CPMI wajib memiliki surat permintaan dari Pemberi Kerja yang telah diverifikasi oleh Atase Ketenagakerjaan (atau pejabat dinas luar negeri jika Atase belum ada).
+*   **Hubungan Kerja:** Terjadi hubungan kerja antara CPMI dengan Pemberi Kerja melalui Perjanjian Kerja yang memuat syarat kerja, hak, kewajiban, serta jaminan keamanan dan keselamatan selama bekerja.
+*(Dasar hukum: PP Nomor 10 Tahun 2020 Pasal 7 ayat 1 &amp; 2; PP Nomor 10 Tahun 2020 Pasal 1 bagian 1 ayat 3 &amp; 5)*</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Penempatan PMI oleh BP2MI dapat didasarkan pada kebutuhan pemerintah atau permintaan dari pemerintah negara pemberi kerja atau pemberi kerja berbadan hukum di negara tujuan. Penempatan itu dilakukan atas dasar perjanjian tertulis. Perjanjian tertulis disusun berdasarkan prinsip persamaan kedudukan, saling menguntungkan, dan memperhatikan hukum nasional serta internasional, dan paling sedikit memuat identitas para pihak, hak dan kewajiban, syarat dan prosedur penempatan, mekanisme pelindungan PMI, pemantauan dan evaluasi, penyelesaian sengketa, perubahan perjanjian, serta jangka waktu dan pengakhiran. Dari sisi calon PMI, dokumen wajib mencakup antara lain sertifikat kompetensi, surat keterangan sehat, paspor, visa kerja, perjanjian penempatan, dan perjanjian kerja. Hubungan kerja dengan pemberi kerja didasarkan pada perjanjian kerja yang memuat unsur pekerjaan, upah, dan perintah, serta terjadi setelah perjanjian kerja disepakati dan ditandatangani.</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>0.7188415389794571</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>hak dan kewajiban; mekanisme pelindungan; penyelesaian sengketa; sertifikat kompetensi; paspor; visa kerja; pekerjaan upah perintah</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Peraturan Pemerintah No. 10 Tahun 2020, Pasal 3 | PP_10_2020.pdf | Pasal 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Q09</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Lembur</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Apa syarat utama yang harus ada sebelum pengusaha mempekerjakan pekerja melebihi waktu kerja normal?</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Sebelum pengusaha mempekerjakan pekerja melebihi waktu kerja normal, syarat utamanya adalah adanya **persetujuan pekerja/buruh yang bersangkutan**.
+Dasar hukumnya adalah:
+*   **PP Nomor 35 Tahun 2021 Pasal 52 ayat 2**: Pengusaha dilarang mempekerjakan pekerja/buruh melebihi waktu kerja sebagaimana dimaksud dalam Pasal 51 ayat (2) kecuali dengan persetujuan pekerja/buruh.
+*   **UU No. 13 Tahun 2003 Pasal 78 ayat (1)**: Pengusaha yang mempekerjakan pekerja/buruh melebihi waktu kerja harus memenuhi syarat adanya persetujuan pekerja/buruh yang bersangkutan.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Pengusaha yang mempekerjakan pekerja melebihi waktu kerja harus memenuhi syarat adanya persetujuan pekerja yang bersangkutan dan adanya perintah kerja lembur dari pengusaha.</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>0.7361297393412818</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>lembur; perintah kerja lembur</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>7</v>
+      </c>
+      <c r="K4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Undang-Undang No. 13 Tahun 2003, Pasal 78 | UU_Nomor_13_Tahun_2003.pdf | Pasal 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>Q17</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>PHK dan Jaminan Kehilangan Pekerjaan</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Seorang pekerja PKWTT terkena PHK dan ingin menuntut hak PHK sekaligus manfaat JKP. Bedakan hak uang dari pengusaha saat PHK dengan manfaat JKP dari program jaminan sosial, termasuk komponen manfaat JKP dan skema uang tunainya.</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Berdasarkan referensi yang tersedia, berikut adalah pembedaan hak uang dari pengusaha saat PHK dengan manfaat JKP dari program jaminan sosial:
 **1. Hak Uang dari Pengusaha (Saat PHK)**
@@ -3864,176 +4177,56 @@
 *   **Hubungan Kedua Hak:** Kedua hak ini dapat dituntut secara bersamaan karena berasal dari sumber yang berbeda (pengusaha vs. jaminan sosial). Namun, jika pekerja tidak memenuhi syarat kepesertaan JKP (misalnya masa iuran belum cukup), maka pekerja hanya berhak atas hak uang dari pengusaha, bukan manfaat JKP.</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Hak uang akibat PHK dari pengusaha mengacu pada kewajiban pembayaran uang pesangon dan/atau uang penghargaan masa kerja serta uang penggantian hak. Itu berbeda dari JKP, karena JKP adalah program yang wajib diikuti oleh pengusaha untuk mempertahankan derajat kehidupan layak saat pekerja kehilangan pekerjaan. Manfaat JKP terdiri dari uang tunai, akses informasi pasar kerja, dan pelatihan kerja. Uang tunai JKP diberikan paling banyak 6 bulan upah: 45% dari upah untuk 3 bulan pertama dan 25% dari upah untuk 3 bulan berikutnya, dengan dasar upah terakhir yang dilaporkan dan batas atas yang berlaku.</t>
         </is>
       </c>
-      <c r="F2" t="n">
-        <v>0.7096137903531392</v>
-      </c>
-      <c r="G2" t="inlineStr">
+      <c r="F5" t="n">
+        <v>0.7382594025135041</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>good</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>kehilangan pekerjaan; 45 persen</t>
         </is>
       </c>
-      <c r="I2" t="n">
+      <c r="J5" t="n">
         <v>4</v>
       </c>
-      <c r="J2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K2" t="inlineStr">
+      <c r="K5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 37 Tahun 2021, Pasal 1 | pp_Nomor_37_Tahun_2021.pdf | Pasal 1</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Q19</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Pekerja migran Indonesia</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Calon pekerja migran akan ditempatkan melalui BP2MI berdasarkan permintaan pemberi kerja berbadan hukum di negara tujuan. Jelaskan dasar penempatannya, isi minimum perjanjian tertulis antar pihak penempatan, dan dokumen/hubungan kerja yang wajib ada bagi pekerja migran.</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Berdasarkan referensi yang tersedia, berikut adalah jawaban atas pertanyaan Anda:
-**1. Dasar Penempatan**
-Penempatan Calon Pekerja Migran Indonesia (CPMI) oleh Badan Pelindungan Pekerja Migran Indonesia (BP2MI) didasarkan pada dua hal:
-*   Kebutuhan pemerintah; dan
-*   Permintaan dari pemerintah negara Pemberi Kerja atau permintaan Pemberi Kerja berbadan hukum di negara tujuan penempatan.
-*(Dasar hukum: PP Nomor 10 Tahun 2020 Pasal 2)*
-**2. Isi Minimum Perjanjian Tertulis**
-Perjanjian tertulis antara BP2MI dan CPMI (Perjanjian Penempatan) harus memuat rincian dari surat permintaan yang telah diverifikasi, yaitu:
-*   Identitas pemberi kerja;
-*   Jumlah penempatan;
-*   Jenis pekerjaan;
-*   Upah atau gaji;
-*   Kualifikasi jabatan;
-*   Masa berlaku Perjanjian Kerja;
-*   Fasilitas tempat kerja; dan
-*   Jaminan sosial dan/atau asuransi.
-*(Dasar hukum: PP Nomor 10 Tahun 2020 Pasal 7 ayat 2)*
-**3. Dokumen dan Hubungan Kerja yang Wajib Ada**
-*   **Dokumen Wajib:** CPMI wajib memiliki surat permintaan dari Pemberi Kerja yang telah diverifikasi oleh Atase Ketenagakerjaan (atau pejabat dinas luar negeri jika Atase belum ada).
-*   **Hubungan Kerja:** Terjadi hubungan kerja antara CPMI dengan Pemberi Kerja melalui Perjanjian Kerja yang memuat syarat kerja, hak, kewajiban, serta jaminan keamanan dan keselamatan selama bekerja.
-*(Dasar hukum: PP Nomor 10 Tahun 2020 Pasal 7 ayat 1 &amp; 2; PP Nomor 10 Tahun 2020 Pasal 1 bagian 1 ayat 3 &amp; 5)*</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Penempatan PMI oleh BP2MI dapat didasarkan pada kebutuhan pemerintah atau permintaan dari pemerintah negara pemberi kerja atau pemberi kerja berbadan hukum di negara tujuan. Penempatan itu dilakukan atas dasar perjanjian tertulis. Perjanjian tertulis disusun berdasarkan prinsip persamaan kedudukan, saling menguntungkan, dan memperhatikan hukum nasional serta internasional, dan paling sedikit memuat identitas para pihak, hak dan kewajiban, syarat dan prosedur penempatan, mekanisme pelindungan PMI, pemantauan dan evaluasi, penyelesaian sengketa, perubahan perjanjian, serta jangka waktu dan pengakhiran. Dari sisi calon PMI, dokumen wajib mencakup antara lain sertifikat kompetensi, surat keterangan sehat, paspor, visa kerja, perjanjian penempatan, dan perjanjian kerja. Hubungan kerja dengan pemberi kerja didasarkan pada perjanjian kerja yang memuat unsur pekerjaan, upah, dan perintah, serta terjadi setelah perjanjian kerja disepakati dan ditandatangani.</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>0.7225060520416653</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>hak dan kewajiban; mekanisme pelindungan; penyelesaian sengketa; sertifikat kompetensi; paspor; visa kerja; pekerjaan upah perintah</t>
-        </is>
-      </c>
-      <c r="I3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Peraturan Pemerintah No. 10 Tahun 2020, Pasal 3 | PP_10_2020.pdf | Pasal 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Q05</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>PKWT</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Dalam bentuk bahasa apa PKWT wajib dibuat, terutama ketika pekerjanya warga negara Indonesia?</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Berdasarkan referensi yang tersedia, **tidak ditemukan ketentuan spesifik** mengenai bentuk bahasa (misalnya wajib bahasa Indonesia atau boleh bahasa asing) yang harus digunakan dalam pembuatan Perjanjian Kerja Waktu Tertentu (PKWT), baik untuk pekerja Warga Negara Indonesia maupun lainnya.
-Referensi yang tersedia hanya mengatur bahwa PKWT harus dibuat secara **tertulis** (PP No. 35 Tahun 2021 Pasal 18 ayat 2) dan memuat isi tertentu seperti nama, alamat, jabatan, upah, serta jangka waktu (PP No. 35 Tahun 2021 Pasal 6 dan Pasal 13). Ketentuan mengenai bahasa yang digunakan dalam perjanjian kerja tidak tercantum dalam pasal-pasal yang disediakan.</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>PKWT wajib dibuat secara tertulis dengan huruf latin dan menggunakan bahasa Indonesia. Jika dibuat dalam bahasa Indonesia dan bahasa asing lalu terdapat perbedaan penafsiran, naskah bahasa Indonesia yang berlaku.</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>0.7275232021013894</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>huruf latin; penafsiran; bahasa Indonesia berlaku</t>
-        </is>
-      </c>
-      <c r="I4" t="n">
-        <v>6</v>
-      </c>
-      <c r="J4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 1 | PP Nomor 35 Tahun 2021.pdf | Pasal 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Q16</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>PHK dan perselisihan hubungan industrial</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Perusahaan ingin mem-PHK pekerja karena pelanggaran aturan perusahaan setelah SP1, SP2, dan SP3, tetapi pekerja menolak. Jelaskan urutan langkah yang tepat: apa yang harus diupayakan sebelum PHK, hak uang apa yang menjadi dasar bila PHK karena pelanggaran berulang, dan ke mana sengketa dibawa jika bipartit/mediasi gagal?</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Berdasarkan referensi yang tersedia, berikut adalah jawaban atas kasus tersebut:
 **1. Langkah yang Harus Diupayakan Sebelum PHK**
@@ -4051,87 +4244,36 @@
 *   **Dasar Hukum:** PP Nomor 35 Tahun 2021 Pasal 39 ayat (2) dan ayat (3).</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Sebelum PHK, para pihak harus mengupayakan agar PHK tidak terjadi dan merundingkan maksud PHK. Untuk pelanggaran ketentuan perjanjian kerja, peraturan perusahaan, atau PKB yang telah didahului SP1, SP2, dan SP3 berturut-turut, dasar haknya adalah 0,5 kali uang pesangon, 1 kali uang penghargaan masa kerja, dan uang penggantian hak. Jika pekerja menolak, perselisihan wajib lebih dulu diupayakan melalui perundingan bipartit paling lama 30 hari kerja. Bila gagal, perselisihan dicatatkan ke instansi ketenagakerjaan dengan bukti bipartit; jika konsiliasi atau mediasi tidak mencapai kesepakatan, salah satu pihak dapat mengajukan gugatan ke Pengadilan Hubungan Industrial.</t>
         </is>
       </c>
-      <c r="F5" t="n">
-        <v>0.7315822368939717</v>
-      </c>
-      <c r="G5" t="inlineStr">
+      <c r="F6" t="n">
+        <v>0.7477272827307383</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>good</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>mencegah PHK; setengah kali pesangon; satu kali UPMK; Pengadilan Hubungan Industrial</t>
         </is>
       </c>
-      <c r="I5" t="n">
+      <c r="J6" t="n">
         <v>3</v>
       </c>
-      <c r="J5" t="n">
-        <v>1</v>
-      </c>
-      <c r="K5" t="inlineStr">
+      <c r="K6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" t="inlineStr">
         <is>
           <t>Undang-Undang No. 13 Tahun 2003, Pasal 1 | UU_Nomor_13_Tahun_2003.pdf | Pasal 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Q09</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Lembur</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Apa syarat utama yang harus ada sebelum pengusaha mempekerjakan pekerja melebihi waktu kerja normal?</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Sebelum pengusaha mempekerjakan pekerja melebihi waktu kerja normal, syarat utamanya adalah adanya **persetujuan pekerja/buruh yang bersangkutan**.
-Dasar hukumnya adalah:
-*   **PP Nomor 35 Tahun 2021 Pasal 52 ayat 2**: Pengusaha dilarang mempekerjakan pekerja/buruh melebihi waktu kerja sebagaimana dimaksud dalam Pasal 51 ayat (2) kecuali dengan persetujuan pekerja/buruh.
-*   **UU No. 13 Tahun 2003 Pasal 78 ayat (1)**: Pengusaha yang mempekerjakan pekerja/buruh melebihi waktu kerja harus memenuhi syarat adanya persetujuan pekerja/buruh yang bersangkutan.</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Pengusaha yang mempekerjakan pekerja melebihi waktu kerja harus memenuhi syarat adanya persetujuan pekerja yang bersangkutan dan adanya perintah kerja lembur dari pengusaha.</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>0.7567363161132449</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>lembur; perintah kerja lembur</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>7</v>
-      </c>
-      <c r="J6" t="n">
-        <v>2</v>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Undang-Undang No. 13 Tahun 2003, Pasal 78 | UU_Nomor_13_Tahun_2003.pdf | Pasal 78</t>
         </is>
       </c>
     </row>
@@ -4173,25 +4315,28 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.7673922807511829</v>
-      </c>
-      <c r="G7" t="inlineStr">
+        <v>0.7755328321139018</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>good</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>psikotropika; zat adiktif; konsultasi pekerja; lapor Kepolisian; alat pelindung diri; pemberi kerja wajib membayar hak pekerja</t>
         </is>
       </c>
-      <c r="I7" t="n">
-        <v>1</v>
-      </c>
       <c r="J7" t="n">
         <v>1</v>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L7" t="inlineStr">
         <is>
           <t>Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 8 | PER-11-MEN-VI-2005.pdf | Pasal 8</t>
         </is>
@@ -4200,20 +4345,77 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>Q13</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>PHK</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Dalam PHK, komponen apa saja yang termasuk uang penggantian hak menurut PP 35 Tahun 2021?</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Menurut **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 40 ayat (4)**, komponen yang termasuk dalam uang penggantian hak adalah:
+1.  **Cuti tahunan** yang belum diambil dan belum gugur.
+2.  **Biaya atau ongkos pulang** untuk Pekerja/Buruh.
+*(Catatan: Referensi yang tersedia tidak menyebutkan komponen lain di luar kedua poin tersebut).*</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Uang penggantian hak meliputi cuti tahunan yang belum diambil dan belum gugur, biaya atau ongkos pulang untuk pekerja dan keluarganya ke tempat pekerja diterima bekerja, serta hal lain yang ditetapkan dalam perjanjian kerja, peraturan perusahaan, atau perjanjian kerja bersama.</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>0.8188177343777249</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>pekerja dan keluarga; perjanjian kerja; peraturan perusahaan; PKB</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 59 | PP Nomor 35 Tahun 2021.pdf | Pasal 59</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>Q15</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>PHK</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Apa dasar perhitungan upah yang digunakan untuk menghitung pesangon dan uang penghargaan masa kerja?</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Dasar perhitungan upah untuk menghitung pesangon dan uang penghargaan masa kerja adalah **upah pokok** serta **segala macam bentuk tunjangan yang bersifat tetap** yang diberikan kepada pekerja/buruh dan keluarganya, termasuk harga pembelian dari catu yang diberikan secara cuma-cuma (jika catu harus dibayar dengan subsidi, maka dihitung sebagai selisih antara harga pembelian dan harga yang dibayar pekerja).
 Aturan ini diatur dalam:
@@ -4222,159 +4424,56 @@
 Selain itu, jika upah dibayarkan secara harian, bulanan, satuan hasil, borongan, atau tergantung cuaca, maka perhitungan upah sebulan disesuaikan dengan ketentuan rata-rata penghasilan selama 12 bulan terakhir atau ketentuan upah minimum yang berlaku (Pasal 157 ayat (2), (3), dan (4) UU No. 13 Tahun 2003 / Pasal 40 ayat (1) PP No. 35 Tahun 2021).</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>Upah yang digunakan sebagai dasar pembayaran uang pesangon dan uang penghargaan masa kerja terdiri atas upah pokok dan tunjangan tetap yang diberikan kepada pekerja dan keluarganya.</t>
         </is>
       </c>
-      <c r="F8" t="n">
-        <v>0.7950715150833129</v>
-      </c>
-      <c r="G8" t="inlineStr">
+      <c r="F9" t="n">
+        <v>0.8424351239204406</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>good</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>tunjangan tetap</t>
         </is>
       </c>
-      <c r="I8" t="n">
+      <c r="J9" t="n">
         <v>4</v>
       </c>
-      <c r="J8" t="n">
+      <c r="K9" t="n">
         <v>4</v>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>Undang-Undang No. 13 Tahun 2003, Pasal 157 | UU_Nomor_13_Tahun_2003.pdf | Pasal 157</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Q13</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>PHK</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Dalam PHK, komponen apa saja yang termasuk uang penggantian hak menurut PP 35 Tahun 2021?</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Menurut **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 40 ayat (4)**, komponen yang termasuk dalam uang penggantian hak adalah:
-1.  **Cuti tahunan** yang belum diambil dan belum gugur.
-2.  **Biaya atau ongkos pulang** untuk Pekerja/Buruh.
-*(Catatan: Referensi yang tersedia tidak menyebutkan komponen lain di luar kedua poin tersebut).*</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Uang penggantian hak meliputi cuti tahunan yang belum diambil dan belum gugur, biaya atau ongkos pulang untuk pekerja dan keluarganya ke tempat pekerja diterima bekerja, serta hal lain yang ditetapkan dalam perjanjian kerja, peraturan perusahaan, atau perjanjian kerja bersama.</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>0.7981231532778058</v>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>pekerja dan keluarga; perjanjian kerja; peraturan perusahaan; PKB</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>2</v>
-      </c>
-      <c r="J9" t="n">
-        <v>1</v>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 59 | PP Nomor 35 Tahun 2021.pdf | Pasal 59</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Q14</t>
+          <t>Q18</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PHK</t>
+          <t>Disabilitas dan pemagangan</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Apa saja komponen uang yang wajib dibayarkan pengusaha ketika terjadi PHK secara umum?</t>
+          <t>Jika pemberi kerja membuka program pemagangan untuk peserta penyandang disabilitas, apa saja kewajiban dan bentuk dukungan yang harus diperhatikan dari sisi hak peserta, kewajiban penyelenggara, kebutuhan khusus peserta, dan peran ULD Ketenagakerjaan?</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
-        <is>
-          <t>Berdasarkan referensi yang tersedia, komponen uang yang wajib dibayarkan pengusaha ketika terjadi Pemutusan Hubungan Kerja (PHK) secara umum adalah:
-1.  **Uang Pesangon**
-2.  **Uang Penghargaan Masa Kerja**
-3.  **Uang Penggantian Hak**
-Dasar hukumnya adalah **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 40 ayat (1)** dan **Undang-Undang Nomor 13 Tahun 2003 Pasal 156 ayat (1)** yang menyatakan bahwa pengusaha wajib membayar ketiga komponen tersebut.
-*Catatan: Untuk usaha mikro dan usaha kecil, pembayaran ketiga komponen tersebut dapat ditentukan berdasarkan kesepakatan antara pengusaha dan pekerja sesuai **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 59**.*</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Ketika terjadi PHK, pengusaha wajib membayar uang pesangon, uang penghargaan masa kerja, dan uang penggantian hak yang seharusnya diterima pekerja. Besaran detailnya bergantung pada alasan PHK dan masa kerja.</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
-        <v>0.8237053708235423</v>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="n">
-        <v>5</v>
-      </c>
-      <c r="J10" t="n">
-        <v>1</v>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 59 | PP Nomor 35 Tahun 2021.pdf | Pasal 59</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Q18</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Disabilitas dan pemagangan</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Jika pemberi kerja membuka program pemagangan untuk peserta penyandang disabilitas, apa saja kewajiban dan bentuk dukungan yang harus diperhatikan dari sisi hak peserta, kewajiban penyelenggara, kebutuhan khusus peserta, dan peran ULD Ketenagakerjaan?</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
         <is>
           <t>Berdasarkan referensi yang tersedia, berikut adalah kewajiban dan bentuk dukungan dalam program pemagangan untuk peserta penyandang disabilitas:
 **1. Kewajiban Penyelenggara Pemagangan (Sesuai Permen No. 6 Tahun 2020 Pasal 16)**
@@ -4406,53 +4505,167 @@
 *   Peraturan Menteri Ketenagakerjaan No. 21 Tahun 2020 Pasal 18.</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Peserta pemagangan berhak memperoleh bimbingan, pemenuhan hak sesuai perjanjian pemagangan, fasilitas K3, uang saku, kepesertaan jaminan sosial, serta sertifikat atau surat keterangan. Penyelenggara wajib membimbing peserta, memenuhi hak peserta, menyediakan alat pelindung diri sesuai K3, memberi uang saku, mengikutsertakan peserta dalam jaminan sosial, mengevaluasi, dan memberikan sertifikat atau surat keterangan. Untuk peserta penyandang disabilitas, penyelenggaraan pemagangan harus memperhatikan kebutuhan khusus peserta. ULD Ketenagakerjaan dapat mendukung melalui tenaga pendamping yang mendampingi tenaga kerja penyandang disabilitas dan pemberi kerja, termasuk penyuluhan, bimbingan jabatan, konsultasi pelatihan/penempatan/pemberdayaan, pemenuhan dan pelindungan hak, serta penyediaan alat bantu kerja.</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>0.8650565798282623</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>excellent</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>bimbingan; tenaga pendamping</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>2</v>
+      </c>
+      <c r="K10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Peraturan Menteri Ketenagakerjaan No. 21 Tahun 2020, Pasal 1 bagian 1 | permen_Nomor_21_Tahun_2020.pdf | Pasal 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Q14</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>PHK</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Apa saja komponen uang yang wajib dibayarkan pengusaha ketika terjadi PHK secara umum?</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Berdasarkan referensi yang tersedia, komponen uang yang wajib dibayarkan pengusaha ketika terjadi Pemutusan Hubungan Kerja (PHK) secara umum adalah:
+1.  **Uang Pesangon**
+2.  **Uang Penghargaan Masa Kerja**
+3.  **Uang Penggantian Hak**
+Dasar hukumnya adalah **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 40 ayat (1)** dan **Undang-Undang Nomor 13 Tahun 2003 Pasal 156 ayat (1)** yang menyatakan bahwa pengusaha wajib membayar ketiga komponen tersebut.
+*Catatan: Untuk usaha mikro dan usaha kecil, pembayaran ketiga komponen tersebut dapat ditentukan berdasarkan kesepakatan antara pengusaha dan pekerja sesuai **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 59**.*</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Peserta pemagangan berhak memperoleh bimbingan, pemenuhan hak sesuai perjanjian pemagangan, fasilitas K3, uang saku, kepesertaan jaminan sosial, serta sertifikat atau surat keterangan. Penyelenggara wajib membimbing peserta, memenuhi hak peserta, menyediakan alat pelindung diri sesuai K3, memberi uang saku, mengikutsertakan peserta dalam jaminan sosial, mengevaluasi, dan memberikan sertifikat atau surat keterangan. Untuk peserta penyandang disabilitas, penyelenggaraan pemagangan harus memperhatikan kebutuhan khusus peserta. ULD Ketenagakerjaan dapat mendukung melalui tenaga pendamping yang mendampingi tenaga kerja penyandang disabilitas dan pemberi kerja, termasuk penyuluhan, bimbingan jabatan, konsultasi pelatihan/penempatan/pemberdayaan, pemenuhan dan pelindungan hak, serta penyediaan alat bantu kerja.</t>
+          <t>Ketika terjadi PHK, pengusaha wajib membayar uang pesangon, uang penghargaan masa kerja, dan uang penggantian hak yang seharusnya diterima pekerja. Besaran detailnya bergantung pada alasan PHK dan masa kerja.</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0.8458163170814514</v>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
+        <v>0.8664051770766577</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.95</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>bimbingan; tenaga pendamping</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>2</v>
-      </c>
+          <t>excellent</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
       <c r="J11" t="n">
-        <v>1</v>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>Peraturan Menteri Ketenagakerjaan No. 21 Tahun 2020, Pasal 1 bagian 1 | permen_Nomor_21_Tahun_2020.pdf | Pasal 1</t>
+        <v>5</v>
+      </c>
+      <c r="K11" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 59 | PP Nomor 35 Tahun 2021.pdf | Pasal 59</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Q03</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>PKWT</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Untuk pekerjaan yang diperkirakan selesai dalam waktu tertentu, berapa batas maksimal jangka waktu PKWT beserta perpanjangannya?</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Batas maksimal jangka waktu Perjanjian Kerja Waktu Tertentu (PKWT) untuk pekerjaan yang diperkirakan selesai dalam waktu tertentu adalah **3 (tiga) tahun**, dengan ketentuan dapat diperpanjang **1 (satu) kali** untuk jangka waktu paling lama **1 (satu) tahun**.
+Dasar hukumnya adalah:
+*   **Pasal 4 ayat (1) huruf a PP Nomor 35 Tahun 2021**: PKWT dapat dibuat untuk pekerjaan yang diperkirakan penyelesaiannya dalam waktu yang tidak terlalu lama.
+*   **Pasal 8 ayat (1) PP Nomor 35 Tahun 2021**: Jangka waktu PKWT berdasarkan jangka waktu dapat dibuat untuk paling lama 5 (lima) tahun.
+*   **Pasal 59 ayat (1) huruf b UU Nomor 13 Tahun 2003**: Pekerjaan yang diperkirakan penyelesaiannya dalam waktu yang tidak terlalu lama paling lama 3 (tiga) tahun.
+*   **Pasal 59 ayat (4) UU Nomor 13 Tahun 2003**: PKWT dapat diperpanjang 1 (satu) kali untuk jangka waktu paling lama 1 (satu) tahun.
+*Catatan: Terdapat perbedaan regulasi antara PP Nomor 35 Tahun 2021 (maksimal 5 tahun) dan UU Nomor 13 Tahun 2003 (maksimal 3 tahun + 1 tahun perpanjangan). Berdasarkan referensi yang diberikan, kedua aturan tersebut berlaku.*</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>PKWT berdasarkan jangka waktu untuk pekerjaan yang diperkirakan selesai dalam waktu tertentu dapat dibuat paling lama 5 tahun termasuk perpanjangannya.</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>0.8766834902763367</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>excellent</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="n">
+        <v>2</v>
+      </c>
+      <c r="K12" t="n">
+        <v>1</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 9 | PP Nomor 35 Tahun 2021.pdf | Pasal 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>Q10</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>PHK</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Jika pekerja melanggar ketentuan perjanjian kerja atau peraturan perusahaan setelah diberi surat peringatan pertama, kedua, dan ketiga, hak PHK apa yang menjadi dasar jawabannya?</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>Berdasarkan referensi yang tersedia, jika pekerja melanggar ketentuan perjanjian kerja atau peraturan perusahaan setelah diberi surat peringatan pertama, kedua, dan ketiga secara berturut-turut, maka pekerja berhak atas:
 1.  **Uang pesangon** sebesar 0,5 kali ketentuan Pasal 40 ayat (2) (sesuai PP No. 35 Tahun 2021 Pasal 52 ayat 1 huruf a).
@@ -4462,53 +4675,56 @@
 *Catatan: Ketentuan ini berlaku untuk Perjanjian Kerja Waktu Tertentu (PKWT). Untuk Perjanjian Kerja Waktu Tidak Tertentu (PKWTT), dasar hukumnya adalah Undang-Undang No. 13 Tahun 2003 Pasal 161 yang memberikan hak atas uang pesangon 1 kali ketentuan Pasal 156 ayat (2), uang penghargaan masa kerja 1 kali ketentuan Pasal 156 ayat (3), dan uang penggantian hak.*</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>Untuk PHK karena pekerja melakukan pelanggaran setelah diberikan surat peringatan pertama, kedua, dan ketiga, pekerja berhak atas uang pesangon sebesar setengah kali ketentuan pesangon, uang penghargaan masa kerja sebesar satu kali ketentuan, dan uang penggantian hak.</t>
         </is>
       </c>
-      <c r="F12" t="n">
-        <v>0.8573137124379475</v>
-      </c>
-      <c r="G12" t="inlineStr">
+      <c r="F13" t="n">
+        <v>0.8868805615107219</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H13" t="inlineStr">
         <is>
           <t>excellent</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>setengah kali pesangon; satu kali uang penghargaan masa kerja</t>
         </is>
       </c>
-      <c r="I12" t="n">
+      <c r="J13" t="n">
         <v>2</v>
       </c>
-      <c r="J12" t="n">
+      <c r="K13" t="n">
         <v>2</v>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>Undang-Undang No. 13 Tahun 2003, Pasal 161 | UU_Nomor_13_Tahun_2003.pdf | Pasal 161</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Q11</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>PHK</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>Jika pekerja di-PHK karena pelanggaran bersifat mendesak, apakah ia tetap mendapat pesangon dan UPMK?</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>Berdasarkan referensi yang tersedia, jika pekerja di-PHK karena pelanggaran bersifat mendesak, ia **tidak berhak** atas uang pesangon dan uang penghargaan masa kerja (UPMK).
 Menurut **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 52 ayat (2)**, dalam hal pengusaha melakukan PHK karena alasan pelanggaran bersifat mendesak, pekerja/buruh hanya berhak atas:
@@ -4517,85 +4733,36 @@
 Sementara itu, hak atas uang pesangon dan UPMK hanya diberikan jika PHK dilakukan karena pelanggaran ketentuan yang telah diberikan surat peringatan pertama, kedua, dan ketiga secara berturut-turut (**PP Nomor 35 Tahun 2021 Pasal 52 ayat (1)**).</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>Jika PHK terjadi karena pekerja melakukan pelanggaran bersifat mendesak yang diatur dalam perjanjian kerja, peraturan perusahaan, atau perjanjian kerja bersama, pekerja berhak atas uang penggantian hak dan uang pisah yang besarannya diatur dalam perjanjian kerja, peraturan perusahaan, atau perjanjian kerja bersama. Ketentuan ini tidak memberikan uang pesangon dan uang penghargaan masa kerja.</t>
         </is>
       </c>
-      <c r="F13" t="n">
-        <v>0.8771370995839437</v>
-      </c>
-      <c r="G13" t="inlineStr">
+      <c r="F14" t="n">
+        <v>0.8965328709284466</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H14" t="inlineStr">
         <is>
           <t>excellent</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>tidak pesangon; tidak UPMK</t>
         </is>
       </c>
-      <c r="I13" t="n">
-        <v>1</v>
-      </c>
-      <c r="J13" t="n">
-        <v>1</v>
-      </c>
-      <c r="K13" t="inlineStr">
+      <c r="J14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L14" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 52 | PP Nomor 35 Tahun 2021.pdf | Pasal 52</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Q04</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>PKWT harian</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Pekerja harian lepas bekerja 23 hari dalam sebulan selama 3 bulan berturut-turut. Bagaimana status hubungan kerjanya menurut aturan PKWT harian?</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Berdasarkan **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 10 ayat (4)**, hubungan kerja pekerja harian tersebut **demi hukum berubah menjadi Perjanjian Kerja Waktu Tidak Tertentu (PKWTT)**.
-Hal ini terjadi karena pekerja telah bekerja selama **23 hari** (melebihi batas 21 hari) dalam **3 bulan berturut-turut**, sehingga Perjanjian Kerja Harian yang semula berlaku menjadi tidak berlaku.</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>PKWT harian hanya dapat dibuat untuk pekerjaan tertentu yang berubah dalam waktu dan volume pekerjaan serta upah berdasarkan kehadiran, dengan ketentuan pekerja bekerja kurang dari 21 hari dalam 1 bulan. Jika pekerja bekerja 21 hari atau lebih selama 3 bulan berturut-turut atau lebih, perjanjian kerja harian menjadi PKWTT.</t>
-        </is>
-      </c>
-      <c r="F14" t="n">
-        <v>0.8937286732991535</v>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>excellent</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>menjadi PKWTT</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>1</v>
-      </c>
-      <c r="J14" t="n">
-        <v>1</v>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 10 | PP Nomor 35 Tahun 2021.pdf | Pasal 10</t>
         </is>
       </c>
     </row>
@@ -4630,25 +4797,28 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.8945549503962199</v>
-      </c>
-      <c r="G15" t="inlineStr">
+        <v>0.9159844358762106</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H15" t="inlineStr">
         <is>
           <t>excellent</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>perlindungan pekerja</t>
         </is>
       </c>
-      <c r="I15" t="n">
-        <v>1</v>
-      </c>
       <c r="J15" t="n">
         <v>1</v>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="K15" t="n">
+        <v>1</v>
+      </c>
+      <c r="L15" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 18 | PP Nomor 35 Tahun 2021.pdf | Pasal 18</t>
         </is>
@@ -4657,20 +4827,75 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>Q04</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>PKWT harian</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Pekerja harian lepas bekerja 23 hari dalam sebulan selama 3 bulan berturut-turut. Bagaimana status hubungan kerjanya menurut aturan PKWT harian?</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Berdasarkan **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 10 ayat (4)**, hubungan kerja pekerja harian tersebut **demi hukum berubah menjadi Perjanjian Kerja Waktu Tidak Tertentu (PKWTT)**.
+Hal ini terjadi karena pekerja telah bekerja selama **23 hari** (melebihi batas 21 hari) dalam **3 bulan berturut-turut**, sehingga Perjanjian Kerja Harian yang semula berlaku menjadi tidak berlaku.</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>PKWT harian hanya dapat dibuat untuk pekerjaan tertentu yang berubah dalam waktu dan volume pekerjaan serta upah berdasarkan kehadiran, dengan ketentuan pekerja bekerja kurang dari 21 hari dalam 1 bulan. Jika pekerja bekerja 21 hari atau lebih selama 3 bulan berturut-turut atau lebih, perjanjian kerja harian menjadi PKWTT.</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>0.9232998530069988</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>excellent</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>menjadi PKWTT</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>1</v>
+      </c>
+      <c r="K16" t="n">
+        <v>1</v>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 10 | PP Nomor 35 Tahun 2021.pdf | Pasal 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>Q06</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Alih daya</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Apa syarat pokok perusahaan alih daya terkait bentuk badan usaha dan perizinan sebelum mempekerjakan pekerja alih daya?</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>Berdasarkan referensi yang tersedia, syarat pokok perusahaan alih daya adalah:
 1.  **Bentuk Badan Usaha:** Perusahaan Alih Daya harus berbentuk **badan hukum** (PP No. 35 Tahun 2021 Pasal 20 ayat 1; PM No. 7 Tahun 2026 Pasal 1 ayat 3).
@@ -4678,49 +4903,115 @@
 3.  **Jangka Waktu Usaha:** Kegiatan usaha harus dijalankan paling lambat **1 (satu) tahun** sejak perizinan berusaha diterbitkan (PM No. 7 Tahun 2026 Pasal 6 ayat c).</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>Perusahaan alih daya wajib berbentuk badan hukum dan wajib memenuhi perizinan berusaha yang diterbitkan oleh pemerintah pusat sesuai ketentuan peraturan perundang-undangan.</t>
         </is>
       </c>
-      <c r="F16" t="n">
-        <v>0.9080977408091228</v>
-      </c>
-      <c r="G16" t="inlineStr">
+      <c r="F17" t="n">
+        <v>0.9297636111577352</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H17" t="inlineStr">
         <is>
           <t>excellent</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="n">
-        <v>1</v>
-      </c>
-      <c r="J16" t="n">
-        <v>1</v>
-      </c>
-      <c r="K16" t="inlineStr">
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K17" t="n">
+        <v>1</v>
+      </c>
+      <c r="L17" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 20 | PP Nomor 35 Tahun 2021.pdf | Pasal 20</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Q01</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>PKWT</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Jika pekerja PKWT bekerja selama 6 bulan lalu kontraknya berakhir sesuai jangka waktu, hak kompensasi apa yang perlu diberikan pengusaha dan bagaimana rumus umumnya?</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Berdasarkan referensi yang tersedia, pengusaha wajib memberikan **Uang Kompensasi** kepada pekerja PKWT yang telah bekerja selama 6 bulan sesuai jangka waktu kontrak.
+**Dasar Hukum:**
+*   **PP Nomor 35 Tahun 2021 Pasal 15 ayat (1):** Pengusaha wajib memberikan uang kompensasi kepada pekerja/buruh yang hubungan kerjanya berdasarkan PKWT.
+*   **PP Nomor 35 Tahun 2021 Pasal 15 ayat (3):** Uang kompensasi diberikan kepada pekerja/buruh yang telah mempunyai masa kerja paling sedikit 1 (satu) bulan secara terus menerus.
+*   **PP Nomor 35 Tahun 2021 Pasal 16 ayat (1) huruf b:** Untuk PKWT selama 1 (satu) bulan atau lebih tetapi kurang dari 12 (dua belas) bulan, dihitung secara proporsional.
+**Rumus Umum:**
+Uang Kompensasi = (Masa Kerja / 12) x 1 Bulan Upah
+*(Di mana "1 Bulan Upah" terdiri dari Upah Pokok dan Tunjangan Tetap sesuai Pasal 16 ayat (2)).*
+**Perhitungan untuk kasus 6 bulan:**
+Uang Kompensasi = (6 / 12) x 1 Bulan Upah = **0,5 (satu setengah) Bulan Upah**.</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Pekerja PKWT berhak memperoleh uang kompensasi saat hubungan kerja berakhir karena jangka waktu selesai. Untuk masa kerja 12 bulan secara terus menerus kompensasinya 1 bulan upah. Untuk masa kerja kurang dari 12 bulan atau lebih dari 12 bulan, nilainya dihitung proporsional berdasarkan masa kerja dibagi 12 dikali 1 bulan upah. Jadi masa kerja 6 bulan dihitung 6 per 12 dikali 1 bulan upah.</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>0.9298496687412263</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>excellent</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>berakhir</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>1</v>
+      </c>
+      <c r="K18" t="n">
+        <v>1</v>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 15 | PP Nomor 35 Tahun 2021.pdf | Pasal 15</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Q12</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>PHK</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>Apa hak pekerja yang mengundurkan diri atas kemauan sendiri dan memenuhi syarat pengunduran diri?</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>Berdasarkan referensi yang tersedia, pekerja yang mengundurkan diri atas kemauan sendiri dan memenuhi syarat berhak atas:
 1.  **Uang Penggantian Hak:** Sesuai ketentuan Pasal 40 ayat (4) PP Nomor 35 Tahun 2021 (merujuk pada hak yang sama dalam Pasal 156 ayat (4) UU No. 13 Tahun 2003).
@@ -4734,142 +5025,32 @@
 3.  Tetap melaksanakan kewajibannya sampai tanggal mulai pengunduran diri.</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>Pekerja yang mengundurkan diri atas kemauan sendiri dan memenuhi syarat berhak atas uang penggantian hak dan uang pisah yang besarannya diatur dalam perjanjian kerja, peraturan perusahaan, atau perjanjian kerja bersama.</t>
         </is>
       </c>
-      <c r="F17" t="n">
-        <v>0.9104557331403096</v>
-      </c>
-      <c r="G17" t="inlineStr">
+      <c r="F19" t="n">
+        <v>0.9322046665350597</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H19" t="inlineStr">
         <is>
           <t>excellent</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="n">
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="n">
         <v>2</v>
       </c>
-      <c r="J17" t="n">
+      <c r="K19" t="n">
         <v>2</v>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>Undang-Undang No. 13 Tahun 2003, Pasal 162 | UU_Nomor_13_Tahun_2003.pdf | Pasal 162</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Q01</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>PKWT</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Jika pekerja PKWT bekerja selama 6 bulan lalu kontraknya berakhir sesuai jangka waktu, hak kompensasi apa yang perlu diberikan pengusaha dan bagaimana rumus umumnya?</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Berdasarkan referensi yang tersedia, pengusaha wajib memberikan **Uang Kompensasi** kepada pekerja PKWT yang telah bekerja selama 6 bulan sesuai jangka waktu kontrak.
-**Dasar Hukum:**
-*   **PP Nomor 35 Tahun 2021 Pasal 15 ayat (1):** Pengusaha wajib memberikan uang kompensasi kepada pekerja/buruh yang hubungan kerjanya berdasarkan PKWT.
-*   **PP Nomor 35 Tahun 2021 Pasal 15 ayat (3):** Uang kompensasi diberikan kepada pekerja/buruh yang telah mempunyai masa kerja paling sedikit 1 (satu) bulan secara terus menerus.
-*   **PP Nomor 35 Tahun 2021 Pasal 16 ayat (1) huruf b:** Untuk PKWT selama 1 (satu) bulan atau lebih tetapi kurang dari 12 (dua belas) bulan, dihitung secara proporsional.
-**Rumus Umum:**
-Uang Kompensasi = (Masa Kerja / 12) x 1 Bulan Upah
-*(Di mana "1 Bulan Upah" terdiri dari Upah Pokok dan Tunjangan Tetap sesuai Pasal 16 ayat (2)).*
-**Perhitungan untuk kasus 6 bulan:**
-Uang Kompensasi = (6 / 12) x 1 Bulan Upah = **0,5 (satu setengah) Bulan Upah**.</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Pekerja PKWT berhak memperoleh uang kompensasi saat hubungan kerja berakhir karena jangka waktu selesai. Untuk masa kerja 12 bulan secara terus menerus kompensasinya 1 bulan upah. Untuk masa kerja kurang dari 12 bulan atau lebih dari 12 bulan, nilainya dihitung proporsional berdasarkan masa kerja dibagi 12 dikali 1 bulan upah. Jadi masa kerja 6 bulan dihitung 6 per 12 dikali 1 bulan upah.</t>
-        </is>
-      </c>
-      <c r="F18" t="n">
-        <v>0.9184461808204651</v>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>excellent</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>berakhir</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>1</v>
-      </c>
-      <c r="J18" t="n">
-        <v>1</v>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 15 | PP Nomor 35 Tahun 2021.pdf | Pasal 15</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Q03</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>PKWT</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Untuk pekerjaan yang diperkirakan selesai dalam waktu tertentu, berapa batas maksimal jangka waktu PKWT beserta perpanjangannya?</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Batas maksimal jangka waktu Perjanjian Kerja Waktu Tertentu (PKWT) untuk pekerjaan yang diperkirakan selesai dalam waktu tertentu adalah **3 (tiga) tahun**, dengan ketentuan dapat diperpanjang **1 (satu) kali** untuk jangka waktu paling lama **1 (satu) tahun**.
-Dasar hukumnya adalah:
-*   **Pasal 4 ayat (1) huruf a PP Nomor 35 Tahun 2021**: PKWT dapat dibuat untuk pekerjaan yang diperkirakan penyelesaiannya dalam waktu yang tidak terlalu lama.
-*   **Pasal 8 ayat (1) PP Nomor 35 Tahun 2021**: Jangka waktu PKWT berdasarkan jangka waktu dapat dibuat untuk paling lama 5 (lima) tahun.
-*   **Pasal 59 ayat (1) huruf b UU Nomor 13 Tahun 2003**: Pekerjaan yang diperkirakan penyelesaiannya dalam waktu yang tidak terlalu lama paling lama 3 (tiga) tahun.
-*   **Pasal 59 ayat (4) UU Nomor 13 Tahun 2003**: PKWT dapat diperpanjang 1 (satu) kali untuk jangka waktu paling lama 1 (satu) tahun.
-*Catatan: Terdapat perbedaan regulasi antara PP Nomor 35 Tahun 2021 (maksimal 5 tahun) dan UU Nomor 13 Tahun 2003 (maksimal 3 tahun + 1 tahun perpanjangan). Berdasarkan referensi yang diberikan, kedua aturan tersebut berlaku.*</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>PKWT berdasarkan jangka waktu untuk pekerjaan yang diperkirakan selesai dalam waktu tertentu dapat dibuat paling lama 5 tahun termasuk perpanjangannya.</t>
-        </is>
-      </c>
-      <c r="F19" t="n">
-        <v>0.9334691190719605</v>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>excellent</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="n">
-        <v>2</v>
-      </c>
-      <c r="J19" t="n">
-        <v>1</v>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 9 | PP Nomor 35 Tahun 2021.pdf | Pasal 9</t>
         </is>
       </c>
     </row>
@@ -4907,21 +5088,24 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>0.9612854552268981</v>
-      </c>
-      <c r="G20" t="inlineStr">
+        <v>0.9736037194728853</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" t="inlineStr">
         <is>
           <t>excellent</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="n">
-        <v>1</v>
-      </c>
+      <c r="I20" t="inlineStr"/>
       <c r="J20" t="n">
         <v>1</v>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="K20" t="n">
+        <v>1</v>
+      </c>
+      <c r="L20" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 12 | PP Nomor 35 Tahun 2021.pdf | Pasal 12</t>
         </is>
@@ -4956,21 +5140,24 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0.968933048248291</v>
-      </c>
-      <c r="G21" t="inlineStr">
+        <v>0.9788179874420168</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" t="inlineStr">
         <is>
           <t>excellent</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="n">
-        <v>1</v>
-      </c>
+      <c r="I21" t="inlineStr"/>
       <c r="J21" t="n">
         <v>1</v>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="K21" t="n">
+        <v>1</v>
+      </c>
+      <c r="L21" t="inlineStr">
         <is>
           <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 21 | PP Nomor 35 Tahun 2021.pdf | Pasal 21</t>
         </is>

</xml_diff>

<commit_message>
evaluate new prompt system
</commit_message>
<xml_diff>
--- a/data/eval_outputs/evaluation_report.xlsx
+++ b/data/eval_outputs/evaluation_report.xlsx
@@ -599,20 +599,15 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Berdasarkan referensi yang tersedia, pengusaha wajib memberikan **Uang Kompensasi** kepada pekerja PKWT yang telah bekerja selama 6 bulan sesuai jangka waktu kontrak.
-**Dasar Hukum:**
-*   **PP Nomor 35 Tahun 2021 Pasal 15 ayat (1):** Pengusaha wajib memberikan uang kompensasi kepada pekerja/buruh yang hubungan kerjanya berdasarkan PKWT.
-*   **PP Nomor 35 Tahun 2021 Pasal 15 ayat (3):** Uang kompensasi diberikan kepada pekerja/buruh yang telah mempunyai masa kerja paling sedikit 1 (satu) bulan secara terus menerus.
-*   **PP Nomor 35 Tahun 2021 Pasal 16 ayat (1) huruf b:** Untuk PKWT selama 1 (satu) bulan atau lebih tetapi kurang dari 12 (dua belas) bulan, dihitung secara proporsional.
-**Rumus Umum:**
-Uang Kompensasi = (Masa Kerja / 12) x 1 Bulan Upah
-*(Di mana "1 Bulan Upah" terdiri dari Upah Pokok dan Tunjangan Tetap sesuai Pasal 16 ayat (2)).*
-**Perhitungan untuk kasus 6 bulan:**
-Uang Kompensasi = (6 / 12) x 1 Bulan Upah = **0,5 (satu setengah) Bulan Upah**.</t>
+          <t>Istilah "kompensasi" dalam konteks pertanyaan Anda merujuk pada Uang Kompensasi sebagaimana diatur dalam Peraturan Pemerintah Nomor 35 Tahun 2021. Berdasarkan dokumen tersebut, jika Perjanjian Kerja Waktu Tertentu (PKWT) berakhir sesuai jangka waktu yang diperjanjikan, pengusaha wajib memberikan Uang Kompensasi kepada pekerja yang telah memiliki masa kerja paling sedikit satu bulan secara terus menerus.
+Sesuai dengan Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 15 ayat (1), (2), dan (4), kewajiban pembayaran Uang Kompensasi berlaku bagi pekerja PKWT yang hubungan kerjanya berakhir pada saat jangka waktu PKWT selesai.
+Untuk kasus pekerja yang bekerja selama 6 bulan, perhitungan besaran Uang Kompensanya diatur dalam Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 16 ayat (1) huruf b. Rumus umum perhitungannya adalah:
+**Masa Kerja (dalam bulan) x 1 (satu) bulan Upah**
+Karena masa kerja 6 bulan berada dalam kategori "satu bulan atau lebih tetapi kurang dari 12 bulan", maka pekerja berhak mendapatkan Uang Kompensasi sebesar 6 bulan upah. Dasar perhitungan upah tersebut terdiri dari Upah Pokok dan Tunjangan Tetap sesuai Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 16 ayat (2).</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.9298496687412263</v>
+        <v>0.8685559225082399</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -620,22 +615,22 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>0.95</v>
+        <v>0.6</v>
       </c>
       <c r="I2" t="n">
-        <v>0.7656644582748413</v>
+        <v>0.8237061500549316</v>
       </c>
       <c r="J2" t="n">
         <v>0.8333333333333334</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>PKWT; uang kompensasi; 1 bulan upah; proporsional; masa kerja dibagi 12</t>
+          <t>PKWT; uang kompensasi; berakhir; 1 bulan upah; masa kerja dibagi 12</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>berakhir</t>
+          <t>proporsional</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -675,13 +670,13 @@
         <v>1</v>
       </c>
       <c r="Y2" t="n">
-        <v>155</v>
+        <v>174</v>
       </c>
       <c r="Z2" t="n">
         <v>1</v>
       </c>
       <c r="AA2" t="n">
-        <v>43.90230417251587</v>
+        <v>45.0612678527832</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
@@ -727,18 +722,13 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Berdasarkan referensi yang tersedia, masa percobaan **tidak boleh** diterapkan kepada pekerja Perjanjian Kerja Waktu Tertentu (PKWT).
-Dasar hukumnya adalah:
-1.  **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 12 ayat (1)**: PKWT tidak dapat mensyaratkan adanya masa percobaan kerja.
-2.  **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 12 ayat (2)**: Dalam hal disyaratkan masa percobaan kerja, maka masa percobaan kerja yang disyaratkan tersebut **batal demi hukum** dan masa kerja tetap dihitung.
-3.  **Undang-Undang Nomor 13 Tahun 2003 Pasal 58 ayat (1)**: Perjanjian kerja untuk waktu tertentu tidak dapat mensyaratkan adanya masa percobaan kerja.
-4.  **Undang-Undang Nomor 13 Tahun 2003 Pasal 58 ayat (2)**: Dalam hal disyaratkan masa percobaan kerja, masa percobaan kerja yang disyaratkan **batal demi hukum**.
-**Kesimpulan:**
-Masa percobaan dalam PKWT adalah **ilegal**. Jika tetap dicantumkan dalam perjanjian, masa percobaan tersebut dianggap tidak berlaku (batal demi hukum), dan masa kerja pekerja dihitung sejak awal perjanjian tanpa pengurangan waktu.</t>
+          <t>Istilah "PKWT" dalam pertanyaan Anda merujuk pada Perjanjian Kerja Waktu Tertentu sebagaimana diatur dalam peraturan perundang-undangan ketenagakerjaan. Berdasarkan regulasi yang berlaku, masa percobaan kerja tidak boleh diterapkan kepada pekerja yang diikat dengan Perjanjian Kerja Waktu Tertentu.
+Hal ini diatur secara tegas dalam Peraturan Pemerintah Nomor 35 Tahun 2021 tentang Perjanjian Kerja Waktu Tertentu, Alih Daya, Waktu Kerja dan Waktu Istirahat, dan Pemutusan Hubungan Kerja Pasal 12 ayat (1) yang menyatakan bahwa PKWT tidak dapat mensyaratkan adanya masa percobaan kerja. Ketentuan yang sama juga terdapat dalam Undang-Undang Nomor 13 Tahun 2003 tentang Ketenagakerjaan Pasal 58 ayat (1).
+Akibat hukum jika pihak pengusaha tetap mencantumkan masa percobaan dalam Perjanjian Kerja Waktu Tertentu adalah masa percobaan kerja tersebut batal demi hukum. Meskipun masa percobaan tersebut dicantumkan, masa kerja pekerja tetap dihitung sejak terjadinya hubungan kerja berdasarkan Perjanjian Kerja Waktu Tertentu tersebut, tanpa adanya pengurangan atau pemotongan masa kerja akibat masa percobaan yang tidak sah. Ketentuan ini ditegaskan kembali dalam Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 12 ayat (2) dan Undang-Undang Nomor 13 Tahun 2003 Pasal 58 ayat (2).</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.9736037194728853</v>
+        <v>0.9286643606424333</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -749,17 +739,21 @@
         <v>1</v>
       </c>
       <c r="I3" t="n">
-        <v>0.8240247964859009</v>
+        <v>0.7244290709495544</v>
       </c>
       <c r="J3" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>PKWT; masa percobaan; tidak boleh; batal demi hukum; masa kerja tetap dihitung</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
+          <t>PKWT; masa percobaan; tidak boleh; batal demi hukum</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>masa kerja tetap dihitung</t>
+        </is>
+      </c>
       <c r="M3" t="n">
         <v>1</v>
       </c>
@@ -797,13 +791,13 @@
         <v>1</v>
       </c>
       <c r="Y3" t="n">
-        <v>148</v>
+        <v>176</v>
       </c>
       <c r="Z3" t="n">
         <v>1</v>
       </c>
       <c r="AA3" t="n">
-        <v>43.17098212242126</v>
+        <v>46.05732297897339</v>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
@@ -849,17 +843,14 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Batas maksimal jangka waktu Perjanjian Kerja Waktu Tertentu (PKWT) untuk pekerjaan yang diperkirakan selesai dalam waktu tertentu adalah **3 (tiga) tahun**, dengan ketentuan dapat diperpanjang **1 (satu) kali** untuk jangka waktu paling lama **1 (satu) tahun**.
-Dasar hukumnya adalah:
-*   **Pasal 4 ayat (1) huruf a PP Nomor 35 Tahun 2021**: PKWT dapat dibuat untuk pekerjaan yang diperkirakan penyelesaiannya dalam waktu yang tidak terlalu lama.
-*   **Pasal 8 ayat (1) PP Nomor 35 Tahun 2021**: Jangka waktu PKWT berdasarkan jangka waktu dapat dibuat untuk paling lama 5 (lima) tahun.
-*   **Pasal 59 ayat (1) huruf b UU Nomor 13 Tahun 2003**: Pekerjaan yang diperkirakan penyelesaiannya dalam waktu yang tidak terlalu lama paling lama 3 (tiga) tahun.
-*   **Pasal 59 ayat (4) UU Nomor 13 Tahun 2003**: PKWT dapat diperpanjang 1 (satu) kali untuk jangka waktu paling lama 1 (satu) tahun.
-*Catatan: Terdapat perbedaan regulasi antara PP Nomor 35 Tahun 2021 (maksimal 5 tahun) dan UU Nomor 13 Tahun 2003 (maksimal 3 tahun + 1 tahun perpanjangan). Berdasarkan referensi yang diberikan, kedua aturan tersebut berlaku.*</t>
+          <t>Berdasarkan konteks pertanyaan mengenai batas maksimal jangka waktu Perjanjian Kerja Waktu Tertentu (PKWT) untuk pekerjaan yang diperkirakan selesai dalam waktu tertentu, terdapat perbedaan ketentuan antara peraturan lama dan peraturan terbaru yang lebih spesifik.
+Istilah "pekerjaan yang diperkirakan selesai dalam waktu tertentu" dalam pertanyaan tersebut merujuk pada "pekerjaan yang diperkirakan penyelesaiannya dalam waktu yang tidak terlalu lama" sebagaimana diatur dalam **Undang-Undang Nomor 13 Tahun 2003 Pasal 59 ayat (1) huruf b**. Berdasarkan aturan lama ini, PKWT untuk jenis pekerjaan tersebut dapat diadakan untuk paling lama 2 (dua) tahun dan hanya boleh diperpanjang 1 (satu) kali untuk jangka waktu paling lama 1 (satu) tahun.
+Namun, **Peraturan Pemerintah Nomor 35 Tahun 2021** merupakan aturan terbaru yang lebih spesifik dan mengoreksi ketentuan lama tersebut. Dalam **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 8 ayat (1)**, dinyatakan secara tegas bahwa PKWT berdasarkan jangka waktu dapat dibuat untuk paling lama 5 (lima) tahun. Ayat (2) dari pasal yang sama mengatur bahwa jika pekerjaan belum selesai saat jangka waktu berakhir, perpanjangan dapat dilakukan dengan kesepakatan, dengan ketentuan jangka waktu keseluruhan PKWT beserta perpanjangannya tidak lebih dari 5 (lima) tahun.
+Oleh karena itu, berdasarkan aturan terbaru yang berlaku, batas maksimal jangka waktu PKWT beserta perpanjangannya untuk pekerjaan yang diperkirakan selesai dalam waktu tertentu adalah 5 (lima) tahun. Ketentuan lama mengenai batas 2 tahun dan perpanjangan 1 tahun yang tercantum dalam **Undang-Undang Nomor 13 Tahun 2003 Pasal 59 ayat (4)** telah digantikan oleh ketentuan baru dalam **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 8 ayat (1) dan ayat (2)**.</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.8766834902763367</v>
+        <v>0.9435577776432038</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -867,10 +858,10 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="I4" t="n">
-        <v>0.8112232685089111</v>
+        <v>0.7303851842880249</v>
       </c>
       <c r="J4" t="n">
         <v>1</v>
@@ -918,13 +909,13 @@
         <v>1</v>
       </c>
       <c r="Y4" t="n">
-        <v>174</v>
+        <v>250</v>
       </c>
       <c r="Z4" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="AA4" t="n">
-        <v>46.29595255851746</v>
+        <v>59.65142798423767</v>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
@@ -970,12 +961,14 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Berdasarkan **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 10 ayat (4)**, hubungan kerja pekerja harian tersebut **demi hukum berubah menjadi Perjanjian Kerja Waktu Tidak Tertentu (PKWTT)**.
-Hal ini terjadi karena pekerja telah bekerja selama **23 hari** (melebihi batas 21 hari) dalam **3 bulan berturut-turut**, sehingga Perjanjian Kerja Harian yang semula berlaku menjadi tidak berlaku.</t>
+          <t>Istilah "pekerja harian lepas" dalam pertanyaan Anda dipetakan ke dalam istilah resmi "Perjanjian Kerja Harian" sebagaimana diatur dalam Peraturan Pemerintah Nomor 35 Tahun 2021.
+Berdasarkan **Peraturan Pemerintah Nomor 35 Tahun 2021 tentang Perjanjian Kerja Waktu Tertentu, Alih Daya, Waktu Kerja dan Waktu Istirahat, dan Pemutusan Hubungan Kerja**, khususnya **Pasal 10 ayat (3)** dan **ayat (4)**, status hubungan kerja Anda berubah secara otomatis.
+Aturan tersebut menyatakan bahwa Perjanjian Kerja Harian hanya berlaku jika pekerja bekerja kurang dari 21 hari dalam satu bulan. Namun, dalam kasus Anda, pekerja telah bekerja selama 23 hari dalam sebulan selama 3 bulan berturut-turut. Oleh karena itu, Perjanjian Kerja Harian menjadi tidak berlaku dan hubungan kerja antara pengusaha dengan pekerja demi hukum berubah menjadi **Perjanjian Kerja Waktu Tidak Tertentu (PKWTT)** berdasarkan **Pasal 10 ayat (4)**.
+Konsekuensi hukumnya adalah hubungan kerja yang semula bersifat harian dan tidak tetap, kini beralih menjadi hubungan kerja yang bersifat tetap (PKWTT) sesuai dengan ketentuan dalam **Pasal 10 ayat (1)** yang menyebutkan bahwa pekerjaan dengan sifat tidak tetap dapat dilakukan dengan Perjanjian Kerja Harian, namun ketentuan pada ayat (4) mengoreksi status tersebut jika batas waktu kerja harian tercapai.</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.9232998530069988</v>
+        <v>0.9059004251162213</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -983,10 +976,10 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="I5" t="n">
-        <v>0.7108879089355469</v>
+        <v>0.6615583896636963</v>
       </c>
       <c r="J5" t="n">
         <v>0.8</v>
@@ -1038,13 +1031,13 @@
         <v>1</v>
       </c>
       <c r="Y5" t="n">
-        <v>54</v>
+        <v>185</v>
       </c>
       <c r="Z5" t="n">
         <v>1</v>
       </c>
       <c r="AA5" t="n">
-        <v>16.77782320976257</v>
+        <v>47.09610152244568</v>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
@@ -1090,12 +1083,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Berdasarkan referensi yang tersedia, **tidak ditemukan ketentuan spesifik** mengenai bentuk bahasa (misalnya wajib bahasa Indonesia atau boleh bahasa asing) yang harus digunakan dalam pembuatan Perjanjian Kerja Waktu Tertentu (PKWT), baik untuk pekerja Warga Negara Indonesia maupun lainnya.
-Referensi yang tersedia hanya mengatur bahwa PKWT harus dibuat secara **tertulis** (PP No. 35 Tahun 2021 Pasal 18 ayat 2) dan memuat isi tertentu seperti nama, alamat, jabatan, upah, serta jangka waktu (PP No. 35 Tahun 2021 Pasal 6 dan Pasal 13). Ketentuan mengenai bahasa yang digunakan dalam perjanjian kerja tidak tercantum dalam pasal-pasal yang disediakan.</t>
+          <t>Istilah "PKWT" dalam pertanyaan Anda merujuk pada Perjanjian Kerja Waktu Tertentu sebagaimana diatur dalam Peraturan Pemerintah Nomor 35 Tahun 2021. Berdasarkan ketentuan tersebut, Perjanjian Kerja Waktu Tertentu wajib dibuat dalam bentuk tertulis. Ketentuan ini berlaku tanpa membedakan kewarganegaraan pekerja, sehingga berlaku pula bagi pekerja yang merupakan warga negara Indonesia.
+Dasar hukumnya adalah Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 18 ayat (2) yang menyatakan bahwa Perjanjian Kerja Waktu Tertentu atau Perjanjian Kerja Waktu Tidak Tertentu harus dibuat secara tertulis. Selain itu, isi Perjanjian Kerja Waktu Tertentu juga diatur secara rinci dalam Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 13 yang memuat unsur-unsur wajib seperti nama dan alamat perusahaan, data diri pekerja, jabatan, tempat pekerjaan, besaran dan cara pembayaran upah, hak dan kewajiban, serta jangka waktu berlakunya perjanjian.</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.5961143044630687</v>
+        <v>0.6549318275849025</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1103,22 +1096,22 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="I6" t="n">
-        <v>0.6629842519760132</v>
+        <v>0.4551010727882385</v>
       </c>
       <c r="J6" t="n">
-        <v>0.5</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>tertulis; bahasa Indonesia; bahasa asing</t>
+          <t>tertulis</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>huruf latin; penafsiran; bahasa Indonesia berlaku</t>
+          <t>huruf latin; bahasa Indonesia; bahasa asing; penafsiran; bahasa Indonesia berlaku</t>
         </is>
       </c>
       <c r="M6" t="n">
@@ -1158,13 +1151,13 @@
         <v>1</v>
       </c>
       <c r="Y6" t="n">
-        <v>93</v>
+        <v>127</v>
       </c>
       <c r="Z6" t="n">
         <v>1</v>
       </c>
       <c r="AA6" t="n">
-        <v>23.19345831871033</v>
+        <v>30.96747088432312</v>
       </c>
       <c r="AB6" t="inlineStr">
         <is>
@@ -1210,14 +1203,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Berdasarkan referensi yang tersedia, syarat pokok perusahaan alih daya adalah:
-1.  **Bentuk Badan Usaha:** Perusahaan Alih Daya harus berbentuk **badan hukum** (PP No. 35 Tahun 2021 Pasal 20 ayat 1; PM No. 7 Tahun 2026 Pasal 1 ayat 3).
-2.  **Perizinan Berusaha:** Perusahaan wajib memenuhi perizinan berusaha yang diterbitkan oleh Pemerintah Pusat sesuai dengan norma, standar, prosedur, dan kriteria yang ditetapkan (PP No. 35 Tahun 2021 Pasal 20 ayat 1).
-3.  **Jangka Waktu Usaha:** Kegiatan usaha harus dijalankan paling lambat **1 (satu) tahun** sejak perizinan berusaha diterbitkan (PM No. 7 Tahun 2026 Pasal 6 ayat c).</t>
+          <t>Istilah "perusahaan alih daya" dalam pertanyaan tersebut merujuk pada Perusahaan Alih Daya sebagaimana diatur dalam peraturan perundang-undangan ketenagakerjaan. Berdasarkan dokumen yang tersedia, syarat pokok terkait bentuk badan usaha dan perizinan adalah sebagai berikut:
+Peraturan Pemerintah No. 35 Tahun 2021, Pasal 20 ayat (1) dan ayat (2) serta Peraturan Menteri Ketenagakerjaan No. 7 Tahun 2026, Pasal 1 ayat (3) dan Pasal 6 ayat (a) menetapkan bahwa Perusahaan Alih Daya wajib berbentuk badan hukum dan wajib memenuhi perizinan berusaha yang diterbitkan oleh Pemerintah Pusat. Syarat dan tata cara memperoleh perizinan tersebut dilaksanakan sesuai dengan ketentuan peraturan perundang-undangan mengenai norma, standar, prosedur, dan kriteria perizinan berusaha yang ditetapkan oleh Pemerintah Pusat. Selain itu, Perusahaan Alih Daya juga diwajibkan untuk mencatatkan Perjanjian Alih Daya kepada Dinas dan menjalankan kegiatan usaha paling lambat satu tahun sejak perizinan berusaha diterbitkan.</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.9297636111577352</v>
+        <v>0.9311560173829397</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1228,7 +1219,7 @@
         <v>0.95</v>
       </c>
       <c r="I7" t="n">
-        <v>0.6428685188293457</v>
+        <v>0.6521512269973755</v>
       </c>
       <c r="J7" t="n">
         <v>1</v>
@@ -1276,13 +1267,13 @@
         <v>1</v>
       </c>
       <c r="Y7" t="n">
-        <v>96</v>
+        <v>134</v>
       </c>
       <c r="Z7" t="n">
         <v>1</v>
       </c>
       <c r="AA7" t="n">
-        <v>27.51719379425049</v>
+        <v>32.7417516708374</v>
       </c>
       <c r="AB7" t="inlineStr">
         <is>
@@ -1328,15 +1319,13 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Berdasarkan referensi yang tersedia, pihak yang bertanggung jawab atas perlindungan upah, kesejahteraan, syarat kerja, dan perselisihan pekerja dalam hubungan kerja alih daya adalah **Perusahaan Alih Daya**.
-Dasar hukumnya adalah:
-*   **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 18 ayat (3)**: Pelindungan Pekerja/Buruh, Upah, kesejahteraan, syarat kerja, dan perselisihan yang timbul dilaksanakan sesuai dengan ketentuan peraturan perundang-undangan dan menjadi tanggung jawab Perusahaan Alih Daya.
-*   **Peraturan Menteri Ketenagakerjaan Nomor 7 Tahun 2026 Pasal 4 ayat (2)**: Pelindungan dan hak pekerja/buruh alih daya dilaksanakan sekurang-kurangnya sesuai dengan ketentuan peraturan perundang-undangan dan menjadi tanggung jawab Perusahaan Alih Daya.
-*   **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 19 ayat (3)**: Dalam hal Pekerja/Buruh tidak memperoleh jaminan atas kelangsungan bekerja, Perusahaan Alih Daya bertanggung jawab atas pemenuhan hak Pekerja/Buruh.</t>
+          <t>Dalam hubungan kerja alih daya, pihak yang bertanggung jawab atas perlindungan upah, kesejahteraan, syarat kerja, dan perselisihan pekerja adalah Perusahaan Alih Daya.
+Hal ini diatur secara tegas dalam Peraturan Pemerintah Nomor 35 Tahun 2021 tentang Perjanjian Kerja Waktu Tertentu, Alih Daya, Waktu Kerja dan Waktu Istirahat, dan Pemutusan Hubungan Kerja. Berdasarkan Pasal 18 ayat (3) dari peraturan tersebut, pelindungan pekerja/buruh, upah, kesejahteraan, syarat kerja, dan perselisihan yang timbul dilaksanakan sesuai dengan ketentuan peraturan perundang-undangan dan menjadi tanggung jawab Perusahaan Alih Daya. Ketentuan ini juga diperkuat dalam Pasal 19 ayat (3) yang menyatakan bahwa dalam hal pekerja/buruh tidak memperoleh jaminan atas kelangsungan bekerja, Perusahaan Alih Daya bertanggung jawab atas pemenuhan hak pekerja/buruh.
+Meskipun dalam konteks penyediaan jasa pekerja/buruh (bukan alih daya murni) terdapat ketentuan dalam Undang-Undang Nomor 13 Tahun 2003 Pasal 66 ayat (2) huruf c yang menyatakan tanggung jawab serupa bagi perusahaan penyedia jasa pekerja/buruh, namun untuk skenario spesifik alih daya, tanggung jawab utama secara eksplisit berada pada Perusahaan Alih Daya sebagaimana diatur dalam Peraturan Pemerintah Nomor 35 Tahun 2021.</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.9159844358762106</v>
+        <v>0.9314830627044043</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1344,10 +1333,10 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="I8" t="n">
-        <v>0.7176740169525146</v>
+        <v>0.7543315291404724</v>
       </c>
       <c r="J8" t="n">
         <v>0.8333333333333334</v>
@@ -1399,13 +1388,13 @@
         <v>1</v>
       </c>
       <c r="Y8" t="n">
-        <v>124</v>
+        <v>170</v>
       </c>
       <c r="Z8" t="n">
         <v>1</v>
       </c>
       <c r="AA8" t="n">
-        <v>34.01590514183044</v>
+        <v>42.59892749786377</v>
       </c>
       <c r="AB8" t="inlineStr">
         <is>
@@ -1451,13 +1440,14 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Berdasarkan **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 21 ayat (2)**, terdapat dua pola waktu kerja sebagai berikut:
-1.  **Untuk 6 hari kerja dalam seminggu:** 7 (tujuh) jam per hari dan 40 (empat puluh) jam per minggu.
-2.  **Untuk 5 hari kerja dalam seminggu:** 8 (delapan) jam per hari dan 40 (empat puluh) jam per minggu.</t>
+          <t>Berdasarkan Peraturan Pemerintah Nomor 35 Tahun 2021, terdapat dua pola waktu kerja yang diatur dalam Pasal 21 ayat (2) untuk pekerja/buruh, yaitu:
+1. Pola kerja enam hari dalam seminggu dengan ketentuan waktu kerja 7 (tujuh) jam per hari dan total 40 (empat puluh) jam per minggu.
+2. Pola kerja lima hari dalam seminggu dengan ketentuan waktu kerja 8 (delapan) jam per hari dan total 40 (empat puluh) jam per minggu.
+Ketentuan ini berlaku umum bagi setiap pengusaha, kecuali bagi sektor usaha atau pekerjaan tertentu yang diatur lebih lanjut dalam Pasal 23 dan Pasal 26.</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.9788179874420168</v>
+        <v>0.9747076630592347</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1468,7 +1458,7 @@
         <v>1</v>
       </c>
       <c r="I9" t="n">
-        <v>0.8587865829467773</v>
+        <v>0.8313844203948975</v>
       </c>
       <c r="J9" t="n">
         <v>1</v>
@@ -1516,13 +1506,13 @@
         <v>1</v>
       </c>
       <c r="Y9" t="n">
-        <v>56</v>
+        <v>94</v>
       </c>
       <c r="Z9" t="n">
         <v>1</v>
       </c>
       <c r="AA9" t="n">
-        <v>16.22343039512634</v>
+        <v>23.17125368118286</v>
       </c>
       <c r="AB9" t="inlineStr">
         <is>
@@ -1568,14 +1558,13 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Sebelum pengusaha mempekerjakan pekerja melebihi waktu kerja normal, syarat utamanya adalah adanya **persetujuan pekerja/buruh yang bersangkutan**.
-Dasar hukumnya adalah:
-*   **PP Nomor 35 Tahun 2021 Pasal 52 ayat 2**: Pengusaha dilarang mempekerjakan pekerja/buruh melebihi waktu kerja sebagaimana dimaksud dalam Pasal 51 ayat (2) kecuali dengan persetujuan pekerja/buruh.
-*   **UU No. 13 Tahun 2003 Pasal 78 ayat (1)**: Pengusaha yang mempekerjakan pekerja/buruh melebihi waktu kerja harus memenuhi syarat adanya persetujuan pekerja/buruh yang bersangkutan.</t>
+          <t>Syarat utama yang harus dipenuhi sebelum pengusaha mempekerjakan pekerja melebihi waktu kerja normal adalah adanya persetujuan tertulis dari pekerja/buruh yang bersangkutan. Ketentuan ini diatur dalam Undang-Undang Nomor 13 Tahun 2003 tentang Ketenagakerjaan Pasal 78 ayat (1) huruf a.
+Selain persetujuan pekerja, pengusaha juga wajib membatasi waktu kerja lembur maksimal 3 (tiga) jam dalam 1 (satu) hari dan 14 (empat belas) jam dalam 1 (satu) minggu sesuai Pasal 78 ayat (1) huruf b Undang-Undang Nomor 13 Tahun 2003. Perlu dicatat bahwa batasan waktu kerja lembur tersebut tidak berlaku bagi sektor usaha atau pekerjaan tertentu sebagaimana dimaksud dalam Pasal 78 ayat (3) Undang-Undang Nomor 13 Tahun 2003.
+Aturan terbaru yang lebih spesifik mengenai hal ini terdapat dalam Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 27 ayat (1) yang mewajibkan pembayaran upah kerja lembur bagi pekerja yang melebihi waktu kerja, dengan pengecualian bagi pekerja dalam golongan jabatan tertentu yang memiliki tanggung jawab sebagai pemikir, perencana, pelaksana, dan pengendali jalannya perusahaan dengan waktu kerja tidak terbatas dan mendapat upah lebih tinggi.</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.7361297393412818</v>
+        <v>0.816637122091793</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1583,22 +1572,22 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>0.6</v>
+        <v>0.85</v>
       </c>
       <c r="I10" t="n">
-        <v>0.8011823892593384</v>
+        <v>0.7545649409294128</v>
       </c>
       <c r="J10" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>persetujuan pekerja; melebihi waktu kerja</t>
+          <t>lembur; persetujuan pekerja; melebihi waktu kerja</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>lembur; perintah kerja lembur</t>
+          <t>perintah kerja lembur</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -1638,13 +1627,13 @@
         <v>1</v>
       </c>
       <c r="Y10" t="n">
-        <v>72</v>
+        <v>167</v>
       </c>
       <c r="Z10" t="n">
         <v>1</v>
       </c>
       <c r="AA10" t="n">
-        <v>20.82744526863098</v>
+        <v>42.02114582061768</v>
       </c>
       <c r="AB10" t="inlineStr">
         <is>
@@ -1690,16 +1679,16 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Berdasarkan referensi yang tersedia, jika pekerja melanggar ketentuan perjanjian kerja atau peraturan perusahaan setelah diberi surat peringatan pertama, kedua, dan ketiga secara berturut-turut, maka pekerja berhak atas:
-1.  **Uang pesangon** sebesar 0,5 kali ketentuan Pasal 40 ayat (2) (sesuai PP No. 35 Tahun 2021 Pasal 52 ayat 1 huruf a).
-2.  **Uang penghargaan masa kerja** sebesar 1 kali ketentuan Pasal 40 ayat (3) (sesuai PP No. 35 Tahun 2021 Pasal 52 ayat 1 huruf b).
-3.  **Uang penggantian hak** sesuai ketentuan Pasal 40 ayat (4) (sesuai PP No. 35 Tahun 2021 Pasal 52 ayat 1 huruf c).
-Dasar hukumnya adalah **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 52 ayat (1)**.
-*Catatan: Ketentuan ini berlaku untuk Perjanjian Kerja Waktu Tertentu (PKWT). Untuk Perjanjian Kerja Waktu Tidak Tertentu (PKWTT), dasar hukumnya adalah Undang-Undang No. 13 Tahun 2003 Pasal 161 yang memberikan hak atas uang pesangon 1 kali ketentuan Pasal 156 ayat (2), uang penghargaan masa kerja 1 kali ketentuan Pasal 156 ayat (3), dan uang penggantian hak.*</t>
+          <t>Istilah "pelanggaran" dalam pertanyaan Anda merujuk pada pelanggaran ketentuan yang diatur dalam perjanjian kerja, peraturan perusahaan, atau perjanjian kerja bersama sebagaimana dimaksud dalam Pasal 161 ayat (1) Undang-Undang Nomor 13 Tahun 2003 tentang Ketenagakerjaan. Berdasarkan aturan terbaru yang lebih spesifik, yaitu Peraturan Pemerintah Nomor 35 Tahun 2021, hak yang diterima pekerja dalam kondisi tersebut diatur dalam Pasal 52 ayat (1).
+Dalam kondisi di mana pekerja melakukan pelanggaran ketentuan perjanjian kerja, peraturan perusahaan, atau perjanjian kerja bersama dan sebelumnya telah diberikan surat peringatan pertama, kedua, dan ketiga secara berturut-turut, pekerja berhak atas:
+1. Uang pesangon sebesar 0,5 (nol koma lima) kali ketentuan Pasal 40 ayat (2);
+2. Uang penghargaan masa kerja sebesar 1 (satu) kali ketentuan Pasal 40 ayat (3); dan
+3. Uang penggantian hak sesuai ketentuan Pasal 40 ayat (4).
+Perlu dicatat bahwa ketentuan ini berlaku untuk Perjanjian Kerja Waktu Tertentu (PKWT) sebagaimana diatur dalam Peraturan Pemerintah Nomor 35 Tahun 2021. Jika konteksnya adalah Perjanjian Kerja Waktu Tidak Tertentu (PKWTT) berdasarkan Undang-Undang Nomor 13 Tahun 2003, maka hak yang diterima pekerja adalah uang pesangon sebesar 1 (satu) kali ketentuan Pasal 156 ayat (2), uang penghargaan masa kerja sebesar 1 (satu) kali ketentuan Pasal 156 ayat (3), dan uang penggantian hak sesuai ketentuan Pasal 156 ayat (4). Namun, mengingat adanya aturan baru yang lebih spesifik mengenai hak akibat PHK, maka ketentuan dalam Peraturan Pemerintah Nomor 35 Tahun 2021 menjadi acuan utama.</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0.8868805615107219</v>
+        <v>0.8690293098290762</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1710,7 +1699,7 @@
         <v>0.95</v>
       </c>
       <c r="I11" t="n">
-        <v>0.7680926322937012</v>
+        <v>0.6513065099716187</v>
       </c>
       <c r="J11" t="n">
         <v>0.6666666666666666</v>
@@ -1762,13 +1751,13 @@
         <v>1</v>
       </c>
       <c r="Y11" t="n">
-        <v>165</v>
+        <v>230</v>
       </c>
       <c r="Z11" t="n">
-        <v>1</v>
+        <v>0.9666666666666667</v>
       </c>
       <c r="AA11" t="n">
-        <v>44.57093548774719</v>
+        <v>57.71416640281677</v>
       </c>
       <c r="AB11" t="inlineStr">
         <is>
@@ -1814,15 +1803,15 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Berdasarkan referensi yang tersedia, jika pekerja di-PHK karena pelanggaran bersifat mendesak, ia **tidak berhak** atas uang pesangon dan uang penghargaan masa kerja (UPMK).
-Menurut **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 52 ayat (2)**, dalam hal pengusaha melakukan PHK karena alasan pelanggaran bersifat mendesak, pekerja/buruh hanya berhak atas:
-1.  Uang penggantian hak sesuai ketentuan Pasal 40 ayat (4).
-2.  Uang pisah yang besarannya diatur dalam Perjanjian Kerja, Peraturan Perusahaan, atau Perjanjian Kerja Bersama.
-Sementara itu, hak atas uang pesangon dan UPMK hanya diberikan jika PHK dilakukan karena pelanggaran ketentuan yang telah diberikan surat peringatan pertama, kedua, dan ketiga secara berturut-turut (**PP Nomor 35 Tahun 2021 Pasal 52 ayat (1)**).</t>
+          <t>Istilah "di-PHK karena pelanggaran bersifat mendesak" dalam konteks hukum ketenagakerjaan merujuk pada Pemutusan Hubungan Kerja karena alasan pelanggaran yang diatur dalam Perjanjian Kerja, Peraturan Perusahaan, atau Perjanjian Kerja Bersama sebagaimana dimaksud dalam Pasal 52 ayat (2) Peraturan Pemerintah Nomor 35 Tahun 2021.
+Berdasarkan ketentuan tersebut, pekerja **tidak berhak** atas uang pesangon dan uang penghargaan masa kerja. Hak yang diterima pekerja hanya terbatas pada uang penggantian hak sesuai ketentuan Pasal 40 ayat (4).
+Dasar hukumnya adalah:
+Peraturan Pemerintah Nomor 35 Tahun 2021, Pasal 52 ayat (2) yang menyatakan bahwa pengusaha dapat melakukan Pemutusan Hubungan Kerja terhadap Pekerja/Buruh karena alasan Pekerja/Buruh melakukan pelanggaran bersifat mendesak yang diatur dalam Perjanjian Kerja, Peraturan Perusahaan, atau Perjanjian Kerja Bersama maka Pekerja/Buruh berhak atas: a. uang penggantian hak sesuai ketentuan Pasal 40 ayat (4); dan b. uang pisah yang besarannya diatur dalam Perjanjian Kerja, Peraturan Perusahaan, atau Perjanjian Kerja Bersama.
+Sedangkan ketentuan mengenai uang pesangon dan uang penghargaan masa kerja untuk kasus pelanggaran mendesak tidak diatur dalam ayat tersebut, sehingga hak atas kedua komponen tersebut tidak timbul dalam kondisi ini. Ketentuan ini berbeda dengan pelanggaran biasa yang memerlukan Surat Peringatan (SP) bertingkat (SP 1, SP 2, SP 3) yang diatur dalam Pasal 52 ayat (1) dan Pasal 161 Undang-Undang Nomor 13 Tahun 2003, di mana pekerja tetap berhak atas uang pesangon dan uang penghargaan masa kerja.</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.8965328709284466</v>
+        <v>0.8872310147682827</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -1833,7 +1822,7 @@
         <v>0.95</v>
       </c>
       <c r="I12" t="n">
-        <v>0.7991080284118652</v>
+        <v>0.7370956540107727</v>
       </c>
       <c r="J12" t="n">
         <v>0.6</v>
@@ -1885,13 +1874,13 @@
         <v>1</v>
       </c>
       <c r="Y12" t="n">
-        <v>109</v>
+        <v>220</v>
       </c>
       <c r="Z12" t="n">
         <v>1</v>
       </c>
       <c r="AA12" t="n">
-        <v>28.02168560028076</v>
+        <v>53.58318257331848</v>
       </c>
       <c r="AB12" t="inlineStr">
         <is>
@@ -1937,20 +1926,16 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Berdasarkan referensi yang tersedia, pekerja yang mengundurkan diri atas kemauan sendiri dan memenuhi syarat berhak atas:
-1.  **Uang Penggantian Hak:** Sesuai ketentuan Pasal 40 ayat (4) PP Nomor 35 Tahun 2021 (merujuk pada hak yang sama dalam Pasal 156 ayat (4) UU No. 13 Tahun 2003).
-2.  **Uang Pisah:** Besarnya dan pelaksanaannya diatur dalam Perjanjian Kerja, Peraturan Perusahaan, atau Perjanjian Kerja Bersama.
-**Dasar Hukum:**
-*   **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 50 ayat (1)** dan **Pasal 36 huruf i**.
-*   **Undang-Undang Nomor 13 Tahun 2003 Pasal 162 ayat (1) dan (2)**.
-**Syarat Pengunduran Diri (sesuai PP No. 35 Tahun 2021 Pasal 36 huruf i):**
-1.  Mengajukan permohonan pengunduran diri secara tertulis selambat-lambatnya 30 (tiga puluh) hari sebelum tanggal mulai pengunduran diri.
-2.  Tidak terikat dalam ikatan dinas.
-3.  Tetap melaksanakan kewajibannya sampai tanggal mulai pengunduran diri.</t>
+          <t>Istilah "mengundurkan diri atas kemauan sendiri" dalam konteks hukum ketenagakerjaan merujuk pada pemutusan hubungan kerja karena alasan pengunduran diri yang diajukan oleh pekerja/buruh. Berdasarkan peraturan terbaru yang berlaku, yaitu Peraturan Pemerintah Nomor 35 Tahun 2021, hak pekerja yang mengundurkan diri atas kemauan sendiri dan memenuhi syarat sebagaimana dimaksud dalam Pasal 36 huruf i adalah berhak atas uang penggantian hak sesuai ketentuan Pasal 40 ayat (4) dan uang pisah yang besarnya diatur dalam Perjanjian Kerja, Peraturan Perusahaan, atau Perjanjian Kerja Bersama.
+Syarat pengunduran diri yang harus dipenuhi menurut Pasal 36 ayat (1) huruf i Peraturan Pemerintah Nomor 35 Tahun 2021 adalah:
+1. Mengajukan permohonan pengunduran diri secara tertulis selambat-lambatnya 30 (tiga puluh) hari sebelum tanggal mulai pengunduran diri.
+2. Tidak terikat dalam ikatan dinas.
+3. Tetap melaksanakan kewajibannya sampai tanggal mulai pengunduran diri.
+Peraturan Pemerintah Nomor 35 Tahun 2021 ini merupakan aturan yang lebih baru dan spesifik dibandingkan Undang-Undang Nomor 13 Tahun 2003, sehingga ketentuan dalam peraturan ini yang menjadi acuan utama. Dalam hal ini, pekerja yang mengundurkan diri atas kemauan sendiri tidak berhak atas uang pesangon, namun tetap berhak atas uang penggantian hak dan uang pisah jika memenuhi syarat-syarat tersebut.</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0.9322046665350597</v>
+        <v>0.9380271432797115</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1961,7 +1946,7 @@
         <v>0.95</v>
       </c>
       <c r="I13" t="n">
-        <v>0.7369199991226196</v>
+        <v>0.7757365107536316</v>
       </c>
       <c r="J13" t="n">
         <v>1</v>
@@ -2009,13 +1994,13 @@
         <v>1</v>
       </c>
       <c r="Y13" t="n">
-        <v>137</v>
+        <v>190</v>
       </c>
       <c r="Z13" t="n">
         <v>1</v>
       </c>
       <c r="AA13" t="n">
-        <v>40.18789720535278</v>
+        <v>47.3691999912262</v>
       </c>
       <c r="AB13" t="inlineStr">
         <is>
@@ -2061,37 +2046,36 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Menurut **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 40 ayat (4)**, komponen yang termasuk dalam uang penggantian hak adalah:
-1.  **Cuti tahunan** yang belum diambil dan belum gugur.
-2.  **Biaya atau ongkos pulang** untuk Pekerja/Buruh.
-*(Catatan: Referensi yang tersedia tidak menyebutkan komponen lain di luar kedua poin tersebut).*</t>
+          <t>Menurut Peraturan Pemerintah Nomor 35 Tahun 2021, istilah "uang penggantian hak" merujuk pada komponen kompensasi yang wajib dibayarkan oleh pengusaha kepada pekerja/buruh dalam berbagai skenario Pemutusan Hubungan Kerja. Komponen-komponen tersebut secara spesifik diatur dalam Pasal 40 ayat (4) yang menyebutkan bahwa uang penggantian hak meliputi cuti tahunan yang belum diambil dan belum gugur serta biaya atau ongkos pulang untuk pekerja/buruh yang dipindahkan.
+Selain komponen yang disebutkan secara eksplisit dalam Pasal 40 ayat (4), terdapat komponen lain yang dapat dikategorikan sebagai bagian dari hak penggantian atau kompensasi tambahan tergantung pada alasan PHK yang terjadi. Dalam kasus PHK karena pelanggaran berat (pelanggaran bersifat mendesak) sebagaimana diatur dalam Pasal 52 ayat (2), pekerja/buruh berhak atas uang penggantian hak sesuai ketentuan Pasal 40 ayat (4) dan uang pisah yang besaran dan syaratnya diatur dalam Perjanjian Kerja, Peraturan Perusahaan, atau Perjanjian Kerja Bersama.
+Sementara itu, dalam skenario PHK karena alasan pengambilalihan perusahaan (Pasal 42 ayat 1 dan 2) atau karena sakit berkepanjangan/cacat akibat kecelakaan kerja (Pasal 41 dan Pasal 55), pekerja/buruh tetap berhak atas uang penggantian hak sesuai ketentuan Pasal 40 ayat (4). Perlu dicatat bahwa dalam skenario khusus bagi pengusaha pada usaha mikro dan usaha kecil yang melakukan PHK berdasarkan kesepakatan, sebagaimana diatur dalam Pasal 59, pembayaran uang penggantian hak dapat dilakukan berdasarkan kesepakatan antara pengusaha dan pekerja/buruh.</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.8188177343777249</v>
+        <v>0.8947867844785964</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>excellent</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
       <c r="I14" t="n">
-        <v>0.6635468006134033</v>
+        <v>0.7509595155715942</v>
       </c>
       <c r="J14" t="n">
-        <v>0.4285714285714285</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>uang penggantian hak; cuti tahunan; ongkos pulang</t>
+          <t>uang penggantian hak; cuti tahunan; ongkos pulang; perjanjian kerja; peraturan perusahaan</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>pekerja dan keluarga; perjanjian kerja; peraturan perusahaan; PKB</t>
+          <t>pekerja dan keluarga; PKB</t>
         </is>
       </c>
       <c r="M14" t="n">
@@ -2131,13 +2115,13 @@
         <v>1</v>
       </c>
       <c r="Y14" t="n">
-        <v>48</v>
+        <v>214</v>
       </c>
       <c r="Z14" t="n">
         <v>1</v>
       </c>
       <c r="AA14" t="n">
-        <v>14.29284286499023</v>
+        <v>51.57540655136108</v>
       </c>
       <c r="AB14" t="inlineStr">
         <is>
@@ -2183,16 +2167,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Berdasarkan referensi yang tersedia, komponen uang yang wajib dibayarkan pengusaha ketika terjadi Pemutusan Hubungan Kerja (PHK) secara umum adalah:
-1.  **Uang Pesangon**
-2.  **Uang Penghargaan Masa Kerja**
-3.  **Uang Penggantian Hak**
-Dasar hukumnya adalah **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 40 ayat (1)** dan **Undang-Undang Nomor 13 Tahun 2003 Pasal 156 ayat (1)** yang menyatakan bahwa pengusaha wajib membayar ketiga komponen tersebut.
-*Catatan: Untuk usaha mikro dan usaha kecil, pembayaran ketiga komponen tersebut dapat ditentukan berdasarkan kesepakatan antara pengusaha dan pekerja sesuai **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 59**.*</t>
+          <t>Dalam konteks Pemutusan Hubungan Kerja (PHK) secara umum, istilah yang digunakan dalam peraturan adalah "uang pesangon", "uang penghargaan masa kerja", dan "uang penggantian hak". Berdasarkan Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 40 ayat (1), pengusaha wajib membayar ketiga komponen tersebut. Namun, terdapat perbedaan ketentuan berdasarkan jenis usaha dan jenis PHK.
+Untuk usaha mikro dan usaha kecil, sesuai Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 59, besaran pembayaran uang pesangon, uang penghargaan masa kerja, dan/atau uang pisah ditentukan berdasarkan kesepakatan antara pengusaha dan pekerja/buruh.
+Sedangkan untuk usaha selain usaha mikro dan usaha kecil, sesuai Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 40 ayat (1), komponen yang wajib dibayarkan adalah:
+1. Uang pesangon, yang perhitungannya diatur secara rinci dalam Pasal 40 ayat (2) berdasarkan masa kerja (mulai dari kurang dari 1 tahun hingga 8 tahun atau lebih).
+2. Uang penghargaan masa kerja, yang perhitungannya diatur dalam Pasal 40 ayat (3) untuk masa kerja 3 tahun atau lebih.
+3. Uang penggantian hak, yang meliputi cuti tahunan yang belum diambil dan belum gugur serta biaya atau ongkos pulang untuk pekerja/buruh dan keluarganya ke tempat dimana pekerja/buruh diterima bekerja, sebagaimana diatur dalam Pasal 40 ayat (4).
+Selain komponen di atas, jika terjadi PHK dan upah pekerja/buruh yang dilaporkan tidak sesuai dengan upah yang sebenarnya sehingga terdapat kekurangan pembayaran manfaat uang tunai, pengusaha wajib membayar kekurangan manfaat uang tunai tersebut secara sekaligus sesuai Peraturan Pemerintah Nomor 37 Tahun 2021 Pasal 23.</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.8664051770766577</v>
+        <v>0.864962592768669</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -2203,7 +2188,7 @@
         <v>0.95</v>
       </c>
       <c r="I15" t="n">
-        <v>0.7138122916221619</v>
+        <v>0.7077506184577942</v>
       </c>
       <c r="J15" t="n">
         <v>1</v>
@@ -2251,13 +2236,13 @@
         <v>1</v>
       </c>
       <c r="Y15" t="n">
-        <v>91</v>
+        <v>236</v>
       </c>
       <c r="Z15" t="n">
-        <v>1</v>
+        <v>0.9466666666666667</v>
       </c>
       <c r="AA15" t="n">
-        <v>25.62117075920105</v>
+        <v>53.95512056350708</v>
       </c>
       <c r="AB15" t="inlineStr">
         <is>
@@ -2303,26 +2288,30 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Dasar perhitungan upah untuk menghitung pesangon dan uang penghargaan masa kerja adalah **upah pokok** serta **segala macam bentuk tunjangan yang bersifat tetap** yang diberikan kepada pekerja/buruh dan keluarganya, termasuk harga pembelian dari catu yang diberikan secara cuma-cuma (jika catu harus dibayar dengan subsidi, maka dihitung sebagai selisih antara harga pembelian dan harga yang dibayar pekerja).
-Aturan ini diatur dalam:
-*   **Pasal 157 ayat (1) UU No. 13 Tahun 2003** (untuk pekerja tetap).
-*   **Pasal 40 ayat (1) PP No. 35 Tahun 2021** (untuk pekerja kontrak).
-Selain itu, jika upah dibayarkan secara harian, bulanan, satuan hasil, borongan, atau tergantung cuaca, maka perhitungan upah sebulan disesuaikan dengan ketentuan rata-rata penghasilan selama 12 bulan terakhir atau ketentuan upah minimum yang berlaku (Pasal 157 ayat (2), (3), dan (4) UU No. 13 Tahun 2003 / Pasal 40 ayat (1) PP No. 35 Tahun 2021).</t>
+          <t>Dasar perhitungan upah untuk menghitung uang pesangon dan uang penghargaan masa kerja adalah upah pokok serta segala macam bentuk tunjangan yang bersifat tetap yang diberikan kepada pekerja/buruh dan keluarganya, termasuk harga pembelian dari catu yang diberikan secara cuma-cuma atau selisih harga pembelian dengan harga yang harus dibayar oleh pekerja/buruh jika catu tersebut disubsidi.
+Sesuai dengan **Undang-Undang Nomor 13 Tahun 2003 tentang Ketenagakerjaan Pasal 157 ayat (1)**, komponen upah yang digunakan terdiri atas:
+a. Upah pokok;
+b. Segala macam bentuk tunjangan yang bersifat tetap yang diberikan kepada pekerja/buruh dan keluarganya, termasuk harga pembelian dari catu yang diberikan kepada pekerja/buruh secara cuma-cuma, yang apabila catu harus dibayar pekerja/buruh dengan subsidi, maka sebagai upah dianggap selisih antara harga pembelian dengan harga yang harus dibayar oleh pekerja/buruh.
+Selain itu, ketentuan perhitungan upah sebulan juga diatur sebagai berikut:
+1. Dalam hal penghasilan dibayarkan atas dasar perhitungan harian, maka penghasilan sebulan adalah sama dengan 30 kali penghasilan sehari (**Pasal 157 ayat (2)**).
+2. Dalam hal upah dibayarkan atas dasar perhitungan satuan hasil, potongan/borongan atau komisi, maka penghasilan sehari adalah sama dengan pendapatan rata-rata per hari selama 12 (dua belas) bulan terakhir, dengan ketentuan tidak boleh kurang dari ketentuan upah minimum provinsi atau kabupaten/kota (**Pasal 157 ayat (3)**).
+3. Dalam hal pekerjaan tergantung pada keadaan cuaca dan upahnya didasarkan pada upah borongan, maka perhitungan upah sebulan dihitung dari upah rata-rata 12 (dua belas) bulan terakhir (**Pasal 157 ayat (4)**).
+Peraturan Pemerintah Nomor 35 Tahun 2021 juga mengadopsi ketentuan serupa untuk Perjanjian Kerja Waktu Tertentu (PKWT), di mana uang pesangon dan uang penghargaan masa kerja dihitung berdasarkan ketentuan upah yang sama sebagaimana diatur dalam **Pasal 157 ayat (1) Undang-Undang Nomor 13 Tahun 2003**, sebagaimana dirujuk dalam **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 40 ayat (2) dan ayat (3)**.</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.8424351239204406</v>
+        <v>0.8528445161660513</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>excellent</t>
         </is>
       </c>
       <c r="H16" t="n">
         <v>0.95</v>
       </c>
       <c r="I16" t="n">
-        <v>0.7662341594696045</v>
+        <v>0.8514078855514526</v>
       </c>
       <c r="J16" t="n">
         <v>0.8</v>
@@ -2374,13 +2363,13 @@
         <v>1</v>
       </c>
       <c r="Y16" t="n">
-        <v>140</v>
+        <v>291</v>
       </c>
       <c r="Z16" t="n">
-        <v>1</v>
+        <v>0.7633333333333333</v>
       </c>
       <c r="AA16" t="n">
-        <v>38.46526765823364</v>
+        <v>71.64906573295593</v>
       </c>
       <c r="AB16" t="inlineStr">
         <is>
@@ -2426,24 +2415,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Berdasarkan referensi yang tersedia, berikut adalah jawaban atas kasus tersebut:
-**1. Langkah yang Harus Diupayakan Sebelum PHK**
-Sebelum melakukan Pemutusan Hubungan Kerja (PHK), pengusaha wajib memberikan **Surat Peringatan (SP) berturut-turut sebanyak tiga kali (SP1, SP2, dan SP3)** kepada pekerja yang bersangkutan.
-*   **Dasar Hukum:** PP Nomor 35 Tahun 2021 Pasal 52 ayat (1) dan UU No. 13 Tahun 2003 Pasal 161 ayat (1).
-*   **Catatan:** Surat peringatan tersebut berlaku untuk jangka waktu paling lama 6 bulan, kecuali ditentukan lain dalam Perjanjian Kerja, Peraturan Perusahaan, atau Perjanjian Kerja Bersama.
-**2. Hak Uang yang Menjadi Dasar (Jika PHK karena Pelanggaran Berulang)**
-Jika pekerja melakukan pelanggaran ketentuan yang diatur dalam Perjanjian Kerja, Peraturan Perusahaan, atau Perjanjian Kerja Bersama setelah menerima SP1, SP2, dan SP3 secara berturut-turut, pekerja berhak atas:
-*   **Uang Pesangon:** 0,5 (nol koma lima) kali ketentuan Pasal 40 ayat (2).
-*   **Uang Penghargaan Masa Kerja:** 1 (satu) kali ketentuan Pasal 40 ayat (3).
-*   **Uang Penggantian Hak:** Sesuai ketentuan Pasal 40 ayat (4).
-*   **Dasar Hukum:** PP Nomor 35 Tahun 2021 Pasal 52 ayat (1).
-**3. Penyelesaian Sengketa Jika Bipartit/Mediasi Gagal**
-Jika terjadi perbedaan pendapat mengenai PHK tersebut, penyelesaian harus dilakukan melalui **perundingan bipartit** antara Pengusaha dengan Pekerja/Buruh dan/atau Serikat Pekerja/Serikat Buruh. Jika perundingan bipartit tidak mencapai kesepakatan, penyelesaian tahap berikutnya dilakukan melalui **mekanisme penyelesaian perselisihan hubungan industrial** sesuai ketentuan peraturan perundang-undangan.
-*   **Dasar Hukum:** PP Nomor 35 Tahun 2021 Pasal 39 ayat (2) dan ayat (3).</t>
+          <t>Istilah "pelanggaran berulang" dalam konteks pertanyaan Anda merujuk pada pelanggaran ketentuan yang diatur dalam Perjanjian Kerja, Peraturan Perusahaan, atau Perjanjian Kerja Bersama yang telah diberikan Surat Peringatan (SP) pertama, kedua, dan ketiga secara berturut-turut. Berdasarkan peraturan terbaru, yaitu Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 52 ayat (1), jika pengusaha melakukan Pemutusan Hubungan Kerja (PHK) karena alasan tersebut, pekerja/buruh berhak atas uang pesangon sebesar 0,5 (nol koma lima) kali ketentuan Pasal 40 ayat (2), uang penghargaan masa kerja sebesar 1 (satu) kali ketentuan Pasal 40 ayat (3), dan uang penggantian hak sesuai ketentuan Pasal 40 ayat (4).
+Sebelum melakukan PHK, pengusaha wajib memberikan Surat Peringatan pertama, kedua, dan ketiga secara berturut-turut kepada pekerja/buruh yang bersangkutan. Jika pekerja menolak surat pemberitahuan PHK, pengusaha harus membuat surat penolakan disertai alasan paling lama 7 (tujuh) hari kerja setelah diterimanya surat pemberitahuan sebagaimana diatur dalam Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 39 ayat (1). Selanjutnya, penyelesaian sengketa harus dilakukan melalui perundingan bipartit antara Pengusaha dengan Pekerja/Buruh dan/atau Serikat Pekerja/Serikat Buruh. Dalam hal perundingan bipartit tidak mencapai kesepakatan, penyelesaian dilakukan melalui mekanisme penyelesaian perselisihan hubungan industrial sesuai ketentuan peraturan perundang-undangan.</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0.7477272827307383</v>
+        <v>0.7152532309293748</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -2451,22 +2428,22 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
       <c r="I17" t="n">
-        <v>0.788404107093811</v>
+        <v>0.6016882061958313</v>
       </c>
       <c r="J17" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.5</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>perundingan; SP1; SP2; SP3; uang penggantian hak; bipartit; 30 hari kerja; mediasi</t>
+          <t>perundingan; SP1; SP2; SP3; uang penggantian hak; bipartit</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>mencegah PHK; setengah kali pesangon; satu kali UPMK; Pengadilan Hubungan Industrial</t>
+          <t>mencegah PHK; setengah kali pesangon; satu kali UPMK; 30 hari kerja; mediasi; Pengadilan Hubungan Industrial</t>
         </is>
       </c>
       <c r="M17" t="n">
@@ -2506,13 +2483,13 @@
         <v>1</v>
       </c>
       <c r="Y17" t="n">
-        <v>236</v>
+        <v>186</v>
       </c>
       <c r="Z17" t="n">
-        <v>0.9466666666666667</v>
+        <v>1</v>
       </c>
       <c r="AA17" t="n">
-        <v>66.88468241691589</v>
+        <v>47.20666074752808</v>
       </c>
       <c r="AB17" t="inlineStr">
         <is>
@@ -2558,31 +2535,30 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Berdasarkan referensi yang tersedia, berikut adalah pembedaan hak uang dari pengusaha saat PHK dengan manfaat JKP dari program jaminan sosial:
-**1. Hak Uang dari Pengusaha (Saat PHK)**
-Hak ini bersifat wajib bagi pengusaha untuk dipenuhi secara sekaligus kepada pekerja yang mengalami PHK, kecuali pengusaha tersebut berstatus usaha mikro.
-*   **Dasar Hukum:** PP Nomor 37 Tahun 2021 Pasal 37 ayat (1).
-*   **Komponen:** Manfaat uang tunai yang dihitung sesuai ketentuan Pasal 21 ayat (1) (biasanya mencakup uang pesangon, uang penghargaan masa kerja, dan uang penggantian hak).
-*   **Kewajiban:** Pengusaha wajib membayar sekaligus, kecuali untuk usaha mikro.
+          <t>Istilah "PKWTT" dalam pertanyaan Anda merujuk pada pekerja dengan Perjanjian Kerja Waktu Tidak Tertentu, dan "menuntut hak PHK" mengacu pada hak atas uang pesangon atau uang pengganti pesangon yang diatur dalam peraturan perundang-undangan ketenagakerjaan, berbeda dengan manfaat JKP yang merupakan jaminan sosial.
+Berdasarkan konteks tersebut, berikut adalah pembedahan hak dan manfaatnya:
+**1. Hak Uang dari Pengusaha (Uang Pesangon/Uang Pengganti Pesangon)**
+Hak ini timbul karena adanya Pemutusan Hubungan Kerja (PHK) dan menjadi kewajiban pengusaha untuk dibayarkan secara sekaligus kepada pekerja. Hak ini diatur dalam **Peraturan Pemerintah Nomor 37 Tahun 2021, Pasal 21 ayat (1)**.
+Komponen hak uang dari pengusaha ini terdiri dari:
+*   Uang pesangon (jika PHK karena alasan tertentu yang mewajibkan pesangon).
+*   Uang penghargaan masa kerja.
+*   Uang penggantian hak.
+*   *Catatan:* Jika pengusaha tidak mengikutsertakan pekerja dalam program JKP, maka pengusaha wajib memenuhi hak uang tunai sesuai perhitungan Pasal 21 ayat (1) tersebut secara sekaligus.
 **2. Manfaat JKP dari Program Jaminan Sosial**
-Manfaat ini diberikan oleh BPJS Ketenagakerjaan kepada pekerja/buruh yang telah terdaftar dan membayar iuran serta mengalami PHK.
-*   **Dasar Hukum:** PP Nomor 37 Tahun 2021 Pasal 1 ayat (1) dan Pasal 18.
-*   **Komponen Manfaat:**
-    1.  Uang tunai.
-    2.  Akses informasi pasar kerja.
-    3.  Pelatihan kerja.
-*   **Syarat Kepesertaan:** Pekerja harus telah terdaftar dan membayar iuran dengan masa iuran akumulasi minimal 12 bulan dalam 24 bulan kalender (PP Nomor 6 Tahun 2025 Pasal 19 ayat (2) dan (3)).
-*   **Skema Uang Tunai JKP:**
-    *   Dibayarkan dalam bentuk uang tunai.
-    *   Jumlah pembayaran dibatasi maksimal 6 kali dengan durasi masing-masing 3 bulan (total maksimal 18 bulan), kecuali untuk pekerja yang telah mencapai usia pensiun, meninggal dunia, atau cacat total tetap (PP Nomor 37 Tahun 2021 Pasal 21).
-    *   Pembayaran dilakukan oleh BPJS Ketenagakerjaan, bukan oleh pengusaha.
-**Catatan Penting:**
-*   **Naturalisasi Dasar Hukum:** PP Nomor 35 Tahun 2021 Pasal 52 ayat (2) tidak ditemukan dalam referensi yang diberikan. Referensi yang tersedia hanya mencakup PP Nomor 37 Tahun 2021 dan PP Nomor 6 Tahun 2025.
-*   **Hubungan Kedua Hak:** Kedua hak ini dapat dituntut secara bersamaan karena berasal dari sumber yang berbeda (pengusaha vs. jaminan sosial). Namun, jika pekerja tidak memenuhi syarat kepesertaan JKP (misalnya masa iuran belum cukup), maka pekerja hanya berhak atas hak uang dari pengusaha, bukan manfaat JKP.</t>
+Manfaat JKP adalah jaminan sosial yang diberikan kepada pekerja/buruh yang mengalami PHK, terlepas dari apakah pekerja tersebut terdaftar dalam program JKP atau tidak (namun bagi yang tidak terdaftar, penggantian kewajiban ada pada pengusaha). Manfaat ini diatur dalam **Peraturan Pemerintah Nomor 37 Tahun 2021, Pasal 18** dan **Peraturan Menteri Ketenagakerjaan Nomor 7 Tahun 2025, Pasal 2**.
+Komponen manfaat JKP terdiri dari tiga bagian utama:
+*   **Uang Tunai:** Dibayarkan secara sekaligus.
+*   **Akses Informasi Pasar Kerja:** Layanan untuk mencari pekerjaan baru.
+*   **Pelatihan Kerja:** Program peningkatan kompetensi.
+**Skema dan Ketentuan Uang Tunai JKP:**
+*   **Sumber Dana:** Dana iuran peserta berasal dari anggaran pendapatan dan belanja negara (APBN) dan dibayarkan oleh pemerintah, bukan oleh pengusaha secara langsung dari iuran pekerja (sesuai **Peraturan Menteri Ketenagakerjaan Nomor 7 Tahun 2025, Pasal 1 ayat (1)**).
+*   **Syarat Penerima:** Pekerja/buruh yang mempunyai hubungan kerja dengan pengusaha dan telah terdaftar serta membayar iuran (sesuai **Peraturan Pemerintah Nomor 37 Tahun 2021, Pasal 1 ayat (6)**).
+*   **Syarat Masa Iuran:** Peserta berhak mendapatkan manfaat JKP jika telah memenuhi syarat masa iuran. Berdasarkan **Peraturan Pemerintah Nomor 6 Tahun 2025, Pasal 19 ayat (2)**, yang dimaksud "bersedia untuk bekerja kembali" adalah bekerja sebagai pekerja penerima upah atau berusaha mandiri atau wirausaha. Syarat masa iuran 12 (dua belas) bulan dimaknai untuk jumlah bulan iuran JKP yang dibayarkan oleh peserta secara akumulasi jumlah bulan iuran dalam 24 (dua puluh empat) bulan kalender.
+*   **Pengecualian:** Kewajiban pemenuhan hak uang tunai oleh pengusaha (sesuai Pasal</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.7382594025135041</v>
+        <v>0.7181985915342967</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -2593,7 +2569,7 @@
         <v>0.85</v>
       </c>
       <c r="I18" t="n">
-        <v>0.7717293500900269</v>
+        <v>0.6542128324508667</v>
       </c>
       <c r="J18" t="n">
         <v>0.8333333333333334</v>
@@ -2645,13 +2621,13 @@
         <v>1</v>
       </c>
       <c r="Y18" t="n">
-        <v>320</v>
+        <v>393</v>
       </c>
       <c r="Z18" t="n">
-        <v>0.6666666666666667</v>
+        <v>0.4233333333333333</v>
       </c>
       <c r="AA18" t="n">
-        <v>83.43450665473938</v>
+        <v>104.8532993793488</v>
       </c>
       <c r="AB18" t="inlineStr">
         <is>
@@ -2697,61 +2673,39 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Berdasarkan referensi yang tersedia, berikut adalah kewajiban dan bentuk dukungan dalam program pemagangan untuk peserta penyandang disabilitas:
-**1. Kewajiban Penyelenggara Pemagangan (Sesuai Permen No. 6 Tahun 2020 Pasal 16)**
-Penyelenggara wajib:
-*   Membimbing peserta sesuai program pemagangan.
-*   Memenuhi hak peserta sesuai Perjanjian Pemagangan.
-*   Menyediakan Alat Pelindung Diri (APD) sesuai persyaratan K3.
-*   Memberikan uang saku kepada peserta.
-*   Mengikutsertakan peserta dalam program jaminan sosial.
-*   Mengevaluasi peserta pemagangan.
-*   Memberikan sertifikat pemagangan atau surat keterangan telah mengikuti pemagangan.
-**2. Bentuk Dukungan dan Kebutuhan Khusus Peserta (Sesuai Permen No. 6 Tahun 2020 Pasal 24)**
-Penyelenggaraan harus memperhatikan kebutuhan khusus peserta, yang mencakup:
-*   **Masa Orientasi/Adaptasi:** Memberikan kesempatan untuk masa orientasi atau adaptasi di awal masa kerja untuk menentukan apa yang diperlukan, termasuk penyelenggaraan pelatihan atau magang.
-*   **Fleksibilitas Tempat Kerja:** Menyediakan tempat bekerja yang fleksibel dengan menyesuaikan ragam disabilitas tanpa mengurangi target tugas kerja.
-*   **Waktu Istirahat:** Menyediakan waktu istirahat.
-*   **Jadwal Kerja Fleksibel:** Menyediakan jadwal kerja yang fleksibel dengan tetap memenuhi alokasi waktu kerja.
-*   **Asistensi:** Memberikan asistensi dalam pelaksanaan pekerjaan dengan memperhatikan kebutuhan khusus.
-*   **Cuti Khusus:** Memberikan izin atau cuti khusus untuk pengobatan.
-**3. Peran Unit Layanan Disabilitas Bidang Ketenagakerjaan (ULD Ketenagakerjaan) (Sesuai Permen No. 21 Tahun 2020 Pasal 18)**
-ULD Ketenagakerjaan bertugas:
-*   Merencanakan penghormatan, pelindungan, dan pemenuhan hak atas pekerjaan penyandang disabilitas.
-*   Memberikan informasi kepada pemerintah, pemerintah daerah, dan perusahaan swasta mengenai proses rekrutmen, penerimaan, pelatihan kerja, penempatan kerja, keberlanjutan kerja, dan pengembangan karier yang adil dan tanpa diskriminasi.
-*   Menyediakan pendampingan kepada tenaga kerja penyandang disabilitas.
-*   Menyediakan pendampingan kepada pemberi kerja yang menerima tenaga kerja penyandang disabilitas.
-*   Mengoordinasikan ULD Ketenagakerjaan, pemberi kerja, dan tenaga kerja dalam pemenuhan dan penyediaan alat bantu kerja untuk penyandang disabilitas.
-**Dasar Hukum:**
-*   Peraturan Menteri Ketenagakerjaan No. 6 Tahun 2020 Pasal 16 dan Pasal 24.
-*   Peraturan Menteri Ketenagakerjaan No. 21 Tahun 2020 Pasal 18.</t>
+          <t>Berdasarkan konteks pertanyaan mengenai program pemagangan untuk peserta penyandang disabilitas, berikut adalah rincian kewajiban dan bentuk dukungan yang harus diperhatikan:
+Pertama, mengenai definisi istilah, istilah "pelanggaran berat" dalam konteks ini dipetakan ke dalam konsep "Diskriminasi" sebagaimana diatur dalam Pasal 5 ayat (1) huruf d Peraturan Pemerintah Nomor 60 Tahun 2020, yang didefinisikan sebagai setiap pembedaan, pengecualian, pembatasan, pelecehan, atau pengucilan atas dasar disabilitas yang bermaksud atau berdampak pada pembatasan atau peniadaan pengakuan, penikmatan, atau pelaksanaan hak Penyandang Disabilitas.
+Kedua, dari sisi kewajiban penyelenggara pemagangan, sesuai dengan Pasal 16 Peraturan Menteri Ketenagakerjaan Nomor 6 Tahun 2020, penyelenggara pemagangan wajib melakukan tujuh hal, yaitu: membimbing peserta pemagangan sesuai dengan program pemagangan; memenuhi hak peserta pemagangan sesuai dengan perjanjian pemagangan; menyediakan alat pelindung diri sesuai dengan persyaratan keselamatan dan kesehatan kerja; memberikan uang saku kepada peserta pemagangan; mengikutsertakan peserta pemagangan dalam program jaminan sosial; mengevaluasi peserta pemagangan; serta memberikan sertifikat pemagangan atau surat keterangan telah mengikuti pemagangan.
+Ketiga, terkait kebutuhan khusus peserta penyandang disabilitas, Pasal 24 Peraturan Menteri Ketenagakerjaan Nomor 6 Tahun 2020 secara tegas menyatakan bahwa penyelenggaraan pemagangan bagi peserta pemagangan penyandang disabilitas harus dilaksanakan dengan memperhatikan kebutuhan khusus peserta pemagangan tersebut.
+Keempat, mengenai bentuk dukungan yang dapat diberikan pemberi kerja dalam penempatan tenaga kerja penyandang disabilitas, Pasal 48 ayat (1) Undang-Undang Nomor 8 Tahun 2016 tentang Penyandang Disabilitas memberikan opsi fleksibilitas kepada pemberi kerja, yaitu: memberikan kesempatan untuk masa orientasi atau adaptasi di awal masa kerja untuk menentukan apa yang diperlukan, termasuk penyelenggaraan pelatihan atau magang; menyediakan tempat bekerja yang fleksibel dengan menyesuaikan kepada ragam disabilitas tanpa mengurangi target tugas kerja; menyediakan waktu istirahat; menyediakan jadwal kerja yang fleksibel dengan tetap memenuhi alokasi waktu kerja; memberikan asistensi dalam pelaksanaan pekerjaan dengan memperhatikan kebutuhan khusus penyandang disabilitas; dan memberikan izin atau cuti khusus untuk pengobatan.
+Kelima, peran Unit Layanan Disabilitas Bidang Ketenagakerjaan (ULD Ketenagakerjaan) dalam mendukung program ini diatur dalam Pasal 18 Peraturan Pemerintah Nomor 60 Tahun 2020, yang mencakup tugas untuk merencanakan penghormatan, pelindungan, dan pemenuhan hak atas pekerjaan penyandang disabilitas; memberikan informasi kepada pemerintah, pemerintah daerah, dan perusahaan swasta mengenai proses rekrutmen, penerimaan, pelatihan kerja, penempatan kerja, keberlanjutan kerja, dan pengembangan karier yang adil dan tanpa diskriminasi kepada penyandang disabilitas; menyediakan pendampingan kepada tenaga kerja penyandang disabilitas; menyediakan pendampingan kepada pemberi kerja yang menerima tenaga kerja penyandang disabilitas; serta mengoordinasikan ULD Ketenagakerjaan, pemberi kerja, dan tenaga kerja dalam pemenuhan dan penyediaan alat bantu kerja untuk penyandang disabilitas.</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>0.8650565798282623</v>
+        <v>0.8153615871429444</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>excellent</t>
+          <t>good</t>
         </is>
       </c>
       <c r="H19" t="n">
         <v>0.95</v>
       </c>
       <c r="I19" t="n">
-        <v>0.8537105321884155</v>
+        <v>0.6250772476196289</v>
       </c>
       <c r="J19" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.75</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>pemagangan; penyandang disabilitas; kebutuhan khusus; K3; uang saku; jaminan sosial; sertifikat; alat pelindung diri; ULD Ketenagakerjaan; alat bantu kerja</t>
+          <t>pemagangan; penyandang disabilitas; kebutuhan khusus; uang saku; jaminan sosial; sertifikat; alat pelindung diri; ULD Ketenagakerjaan; alat bantu kerja</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>bimbingan; tenaga pendamping</t>
+          <t>bimbingan; K3; tenaga pendamping</t>
         </is>
       </c>
       <c r="M19" t="n">
@@ -2791,13 +2745,13 @@
         <v>1</v>
       </c>
       <c r="Y19" t="n">
-        <v>310</v>
+        <v>397</v>
       </c>
       <c r="Z19" t="n">
-        <v>0.7</v>
+        <v>0.41</v>
       </c>
       <c r="AA19" t="n">
-        <v>88.86415815353394</v>
+        <v>96.15785145759583</v>
       </c>
       <c r="AB19" t="inlineStr">
         <is>
@@ -2843,31 +2797,14 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Berdasarkan referensi yang tersedia, berikut adalah jawaban atas pertanyaan Anda:
-**1. Dasar Penempatan**
-Penempatan Calon Pekerja Migran Indonesia (CPMI) oleh Badan Pelindungan Pekerja Migran Indonesia (BP2MI) didasarkan pada dua hal:
-*   Kebutuhan pemerintah; dan
-*   Permintaan dari pemerintah negara Pemberi Kerja atau permintaan Pemberi Kerja berbadan hukum di negara tujuan penempatan.
-*(Dasar hukum: PP Nomor 10 Tahun 2020 Pasal 2)*
-**2. Isi Minimum Perjanjian Tertulis**
-Perjanjian tertulis antara BP2MI dan CPMI (Perjanjian Penempatan) harus memuat rincian dari surat permintaan yang telah diverifikasi, yaitu:
-*   Identitas pemberi kerja;
-*   Jumlah penempatan;
-*   Jenis pekerjaan;
-*   Upah atau gaji;
-*   Kualifikasi jabatan;
-*   Masa berlaku Perjanjian Kerja;
-*   Fasilitas tempat kerja; dan
-*   Jaminan sosial dan/atau asuransi.
-*(Dasar hukum: PP Nomor 10 Tahun 2020 Pasal 7 ayat 2)*
-**3. Dokumen dan Hubungan Kerja yang Wajib Ada**
-*   **Dokumen Wajib:** CPMI wajib memiliki surat permintaan dari Pemberi Kerja yang telah diverifikasi oleh Atase Ketenagakerjaan (atau pejabat dinas luar negeri jika Atase belum ada).
-*   **Hubungan Kerja:** Terjadi hubungan kerja antara CPMI dengan Pemberi Kerja melalui Perjanjian Kerja yang memuat syarat kerja, hak, kewajiban, serta jaminan keamanan dan keselamatan selama bekerja.
-*(Dasar hukum: PP Nomor 10 Tahun 2020 Pasal 7 ayat 1 &amp; 2; PP Nomor 10 Tahun 2020 Pasal 1 bagian 1 ayat 3 &amp; 5)*</t>
+          <t>Berdasarkan konteks pertanyaan mengenai penempatan Calon Pekerja Migran Indonesia melalui Badan Pelindungan Pekerja Migran Indonesia (BP2MI) atas permintaan Pemberi Kerja berbadan hukum, berikut adalah penjelasan hukumnya:
+Pertama, mengenai dasar penempatan, hal tersebut diatur dalam Peraturan Pemerintah Nomor 10 Tahun 2020 Pasal 2 ayat (2) yang menyatakan bahwa penempatan oleh BP2MI didasarkan pada permintaan dari pemerintah negara Pemberi Kerja atau permintaan Pemberi Kerja berbadan hukum di negara tujuan penempatan.
+Kedua, mengenai isi minimum perjanjian tertulis antara BP2MI dan Calon Pekerja Migran Indonesia, isi tersebut harus memuat identitas pemberi kerja, jumlah penempatan, jenis pekerjaan, upah atau gaji, kualifikasi jabatan, masa berlaku Perjanjian Kerja, fasilitas tempat kerja, dan jaminan sosial serta asuransi sebagaimana diatur dalam Peraturan Pemerintah Nomor 10 Tahun 2020 Pasal 7 ayat (2).
+Ketiga, mengenai dokumen dan hubungan kerja yang wajib ada, Calon Pekerja Migran Indonesia harus memiliki surat permintaan dari Pemberi Kerja yang telah diverifikasi oleh Atase Ketenagakerjaan atau pejabat dinas luar negeri yang ditunjuk jika Atase belum ada di negara tujuan, serta wajib menandatangani Perjanjian Kerja dengan Pemberi Kerja yang memuat syarat kerja, hak, kewajiban, dan jaminan keamanan serta keselamatan selama bekerja sesuai dengan ketentuan peraturan perundang-undangan.</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>0.7188415389794571</v>
+        <v>0.7312327282245344</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -2875,22 +2812,22 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>0.75</v>
+        <v>0.85</v>
       </c>
       <c r="I20" t="n">
-        <v>0.664071798324585</v>
+        <v>0.6902694702148438</v>
       </c>
       <c r="J20" t="n">
-        <v>0.4615384615384616</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>BP2MI; pekerja migran; permintaan pemberi kerja berbadan hukum; perjanjian tertulis; perjanjian penempatan; perjanjian kerja</t>
+          <t>BP2MI; pekerja migran; permintaan pemberi kerja berbadan hukum; perjanjian tertulis; perjanjian kerja</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>hak dan kewajiban; mekanisme pelindungan; penyelesaian sengketa; sertifikat kompetensi; paspor; visa kerja; pekerjaan upah perintah</t>
+          <t>hak dan kewajiban; mekanisme pelindungan; penyelesaian sengketa; sertifikat kompetensi; paspor; visa kerja; perjanjian penempatan; pekerjaan upah perintah</t>
         </is>
       </c>
       <c r="M20" t="n">
@@ -2930,13 +2867,13 @@
         <v>1</v>
       </c>
       <c r="Y20" t="n">
-        <v>213</v>
+        <v>188</v>
       </c>
       <c r="Z20" t="n">
         <v>1</v>
       </c>
       <c r="AA20" t="n">
-        <v>57.62241983413696</v>
+        <v>43.0357608795166</v>
       </c>
       <c r="AB20" t="inlineStr">
         <is>
@@ -2982,22 +2919,17 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Berdasarkan referensi yang tersedia, berikut adalah penjelasan tindakan kepatuhan dan konsekuensi hukumnya:
-**1. Tindakan Pelaporan dan Kebijakan Pencegahan**
-*   **Pelaporan:** Pengusaha wajib segera melaporkan temuan peredaran narkotika kepada Kepolisian Negara Republik Indonesia dan instansi ketenagakerjaan Kabupaten/Kota melalui mekanisme Panitia Pembina Keselamatan dan Kesehatan Kerja (P2K3) atau Pelayanan Kesehatan Kerja (Pasal 8 ayat 1 dan 2).
-*   **Kebijakan Pencegahan:** Pengusaha wajib menetapkan kebijakan tertulis yang memuat komitmen pencegahan dan pembentukan unit penanganan, serta melibatkan pekerja/buruh, serikat pekerja/buruh, atau pihak ketiga ahli dalam pelaksanaannya (Pasal 2 ayat 1-3 dan Pasal 4 ayat 1-4).
-**2. Hak K3 Peserta Pemagangan**
-*   Referensi yang tersedia **tidak mengatur secara spesifik** mengenai hak Keselamatan dan Kesehatan Kerja (K3) khusus untuk peserta pemagangan.
-*   Namun, berdasarkan Pasal 2 ayat (3), upaya pencegahan dan penanggulangan wajib dilakukan dengan melibatkan "pekerja/buruh". Peserta pemagangan secara hukum tidak dikategorikan sebagai pekerja/buruh (mereka adalah peserta pelatihan), sehingga keterlibatan mereka dalam mekanisme pelaporan dan program pencegahan harus disesuaikan dengan definisi "tempat kerja" dan prinsip non-diskriminasi yang berlaku umum, meskipun detail teknisnya tidak tercantum dalam referensi ini.
-**3. Konsekuensi Jika Pekerja Belum Diikutsertakan dalam JKK/JKM**
-*   Referensi yang tersedia **tidak mencantumkan** konsekuensi hukum atau sanksi spesifik bagi pengusaha yang tidak mengikutsertakan pekerja dalam Jaminan Kecelakaan Kerja (JKK) atau Jaminan Kematian (JKM).
-*   Referensi hanya mengatur bahwa ketentuan perawatan dan rehabilitasi akibat penyalahgunaan zat diatur dalam Perjanjian Kerja, Peraturan Perusahaan, atau Perjanjian Kerja Bersama (Pasal 7 ayat 1), namun tidak menyebutkan kewajiban mutlak JKK/JKM atau sanksinya dalam dokumen ini.
-**Catatan Tambahan:**
-Referensi yang tersedia belum cukup untuk menjawab secara lengkap mengenai konsekuensi hukum tidak adanya JKK/JKM dan hak spesifik peserta pemagangan, karena referensi hanya memuat regulasi Pencegahan dan Penanggulangan Penyalahgunaan Narkotika (PER.11/MEN/VI/2005). Untuk aspek JKK/JKM dan regulasi pemagangan, diperlukan referensi lain seperti UU Ketenagakerjaan atau Peraturan Pemerintah terkait Jaminan Sosial dan Pemagangan.</t>
+          <t>Istilah "pemagangan" dalam konteks pertanyaan ini dipetakan ke dalam istilah resmi "pekerja/buruh" sebagaimana didefinisikan dalam Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 1 ayat (7), yang mencakup setiap orang yang bekerja dengan menerima upah atau imbalan dalam bentuk lain.
+Berdasarkan Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, berikut adalah tindakan kepatuhan yang harus dilakukan:
+1. **Pelaporan Segera**
+   Apabila ditemukan indikasi peredaran narkotika, psikotropika, dan zat adiktif lainnya di tempat kerja, pengusaha wajib segera melaporkan kepada Kepolisian Negara Republik Indonesia sesuai dengan ketentuan Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 8 ayat (1). Laporan tersebut juga harus disampaikan kepada instansi yang bertanggung jawab di bidang ketenagakerjaan Kabupaten/Kota melalui mekanisme pelaporan Panitia Pembina Keselamatan dan Kesehatan Kerja (P2K3) atau Pelayanan Kesehatan Kerja sesuai dengan Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 8 ayat (2).
+2. **Penetapan Kebijakan dan Program Pencegahan**
+   Pengusaha wajib melakukan upaya aktif pencegahan dan penanggulangan penyalahgunaan dan peredaran gelap narkotika, psikotropika, dan zat adiktif lainnya di tempat kerja sesuai dengan Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 2 ayat (1). Upaya ini meliputi penetapan kebijakan dan penyusunan serta pelaksanaan program sesuai dengan Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 2 ayat (2).
+   Proses penetapan kebijakan harus melalui konsultasi antara pengusaha dengan pekerja/buruh dan atau serikat pekerja/serikat buruh sesuai dengan Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 4 ayat (1). Kebijakan tersebut harus dinyatakan secara tertulis dan sekurang-kurangnya memuat komitmen pengusaha dalam upaya pencegahan dan penanggulangan serta komitmen pembentukan unit yang menangani program pencegahan dan penanggulangan sesuai dengan Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 4 ayat (2). Unit tersebut dapat merupakan unit tersendiri atau terintegrasi dengan P2K3 atau Pelayanan Kesehatan Kerja sesuai dengan Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 4 ayat (3). Pelaksanaan upaya pencegahan dan penanggulangan harus dilakukan dengan melibatkan pekerja/buruh, serikat pekerja/serikat buruh, pihak ketiga, atau ahli di bidang narkotika, psikotropika, dan zat adiktif lainnya sesuai dengan Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/200</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0.7755328321139018</v>
+        <v>0.7291302879515149</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -3008,19 +2940,19 @@
         <v>0.85</v>
       </c>
       <c r="I21" t="n">
-        <v>0.7204411029815674</v>
+        <v>0.5601701736450195</v>
       </c>
       <c r="J21" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>narkotika; tempat kerja; kebijakan tertulis; instansi ketenagakerjaan; pemagangan; fasilitas K3; JKK; JKM</t>
+          <t>narkotika; psikotropika; zat adiktif; tempat kerja; pemagangan; fasilitas K3</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>psikotropika; zat adiktif; konsultasi pekerja; lapor Kepolisian; alat pelindung diri; pemberi kerja wajib membayar hak pekerja</t>
+          <t>kebijakan tertulis; konsultasi pekerja; lapor Kepolisian; instansi ketenagakerjaan; alat pelindung diri; JKK; JKM; pemberi kerja wajib membayar hak pekerja</t>
         </is>
       </c>
       <c r="M21" t="n">
@@ -3060,13 +2992,13 @@
         <v>1</v>
       </c>
       <c r="Y21" t="n">
-        <v>296</v>
+        <v>324</v>
       </c>
       <c r="Z21" t="n">
-        <v>0.7466666666666666</v>
+        <v>0.6533333333333333</v>
       </c>
       <c r="AA21" t="n">
-        <v>79.33536076545715</v>
+        <v>101.6953108310699</v>
       </c>
       <c r="AB21" t="inlineStr">
         <is>
@@ -3137,13 +3069,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.845</v>
+        <v>0.9100000000000001</v>
       </c>
       <c r="C2" t="n">
         <v>0.95</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -3156,16 +3088,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.7520683497190476</v>
+        <v>0.6996643304824829</v>
       </c>
       <c r="C3" t="n">
-        <v>0.7659493088722229</v>
+        <v>0.7160898447036743</v>
       </c>
       <c r="D3" t="n">
-        <v>0.6428685188293457</v>
+        <v>0.4551010727882385</v>
       </c>
       <c r="E3" t="n">
-        <v>0.8587865829467773</v>
+        <v>0.8514078855514526</v>
       </c>
     </row>
     <row r="4">
@@ -3175,13 +3107,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.7664102564102565</v>
+        <v>0.7430402930402932</v>
       </c>
       <c r="C4" t="n">
-        <v>0.8166666666666667</v>
+        <v>0.8</v>
       </c>
       <c r="D4" t="n">
-        <v>0.4285714285714285</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="E4" t="n">
         <v>1</v>
@@ -3327,13 +3259,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.953</v>
+        <v>0.9031666666666667</v>
       </c>
       <c r="C12" t="n">
         <v>1</v>
       </c>
       <c r="D12" t="n">
-        <v>0.6666666666666667</v>
+        <v>0.41</v>
       </c>
       <c r="E12" t="n">
         <v>1</v>
@@ -3384,16 +3316,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.8474470290146338</v>
+        <v>0.8485825982903213</v>
       </c>
       <c r="C15" t="n">
-        <v>0.8715443336764972</v>
+        <v>0.8687926161686581</v>
       </c>
       <c r="D15" t="n">
-        <v>0.5961143044630687</v>
+        <v>0.6549318275849025</v>
       </c>
       <c r="E15" t="n">
-        <v>0.9788179874420168</v>
+        <v>0.9747076630592347</v>
       </c>
     </row>
     <row r="16">
@@ -3403,16 +3335,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>41.96127111911774</v>
+        <v>54.90808475017548</v>
       </c>
       <c r="C16" t="n">
-        <v>39.32658243179321</v>
+        <v>47.28793036937714</v>
       </c>
       <c r="D16" t="n">
-        <v>14.29284286499023</v>
+        <v>23.17125368118286</v>
       </c>
       <c r="E16" t="n">
-        <v>88.86415815353394</v>
+        <v>104.8532993793488</v>
       </c>
     </row>
     <row r="17">
@@ -3422,16 +3354,16 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>151.85</v>
+        <v>217.3</v>
       </c>
       <c r="C17" t="n">
-        <v>138.5</v>
+        <v>189</v>
       </c>
       <c r="D17" t="n">
-        <v>48</v>
+        <v>94</v>
       </c>
       <c r="E17" t="n">
-        <v>320</v>
+        <v>397</v>
       </c>
     </row>
   </sheetData>
@@ -3510,13 +3442,13 @@
         <v>2</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9228740235169729</v>
+        <v>0.931319540043672</v>
       </c>
       <c r="D2" t="n">
-        <v>0.95</v>
+        <v>0.975</v>
       </c>
       <c r="E2" t="n">
-        <v>0.6802712678909302</v>
+        <v>0.703241378068924</v>
       </c>
       <c r="F2" t="n">
         <v>0.9166666666666667</v>
@@ -3531,7 +3463,7 @@
         <v>1</v>
       </c>
       <c r="J2" t="n">
-        <v>30.76654946804047</v>
+        <v>37.67033958435059</v>
       </c>
     </row>
     <row r="3">
@@ -3544,16 +3476,16 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>0.8650565798282623</v>
+        <v>0.8153615871429444</v>
       </c>
       <c r="D3" t="n">
         <v>0.95</v>
       </c>
       <c r="E3" t="n">
-        <v>0.8537105321884155</v>
+        <v>0.6250772476196289</v>
       </c>
       <c r="F3" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.75</v>
       </c>
       <c r="G3" t="n">
         <v>0.6</v>
@@ -3565,7 +3497,7 @@
         <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>88.86415815353394</v>
+        <v>96.15785145759583</v>
       </c>
     </row>
     <row r="4">
@@ -3578,16 +3510,16 @@
         <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>0.7755328321139018</v>
+        <v>0.7291302879515149</v>
       </c>
       <c r="D4" t="n">
         <v>0.85</v>
       </c>
       <c r="E4" t="n">
-        <v>0.7204411029815674</v>
+        <v>0.5601701736450195</v>
       </c>
       <c r="F4" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="G4" t="n">
         <v>0.4285714285714285</v>
@@ -3599,7 +3531,7 @@
         <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>79.33536076545715</v>
+        <v>101.6953108310699</v>
       </c>
     </row>
     <row r="5">
@@ -3612,16 +3544,16 @@
         <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>0.7361297393412818</v>
+        <v>0.816637122091793</v>
       </c>
       <c r="D5" t="n">
-        <v>0.6</v>
+        <v>0.85</v>
       </c>
       <c r="E5" t="n">
-        <v>0.8011823892593384</v>
+        <v>0.7545649409294128</v>
       </c>
       <c r="F5" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="G5" t="n">
         <v>1</v>
@@ -3633,7 +3565,7 @@
         <v>1</v>
       </c>
       <c r="J5" t="n">
-        <v>20.82744526863098</v>
+        <v>42.02114582061768</v>
       </c>
     </row>
     <row r="6">
@@ -3646,16 +3578,16 @@
         <v>6</v>
       </c>
       <c r="C6" t="n">
-        <v>0.873879355724842</v>
+        <v>0.8844802268817311</v>
       </c>
       <c r="D6" t="n">
-        <v>0.9333333333333332</v>
+        <v>0.9499999999999998</v>
       </c>
       <c r="E6" t="n">
-        <v>0.741285651922226</v>
+        <v>0.7457094490528107</v>
       </c>
       <c r="F6" t="n">
-        <v>0.7492063492063492</v>
+        <v>0.7968253968253968</v>
       </c>
       <c r="G6" t="n">
         <v>1</v>
@@ -3667,7 +3599,7 @@
         <v>1</v>
       </c>
       <c r="J6" t="n">
-        <v>31.85996659596761</v>
+        <v>55.97435696919759</v>
       </c>
     </row>
     <row r="7">
@@ -3680,13 +3612,13 @@
         <v>1</v>
       </c>
       <c r="C7" t="n">
-        <v>0.7382594025135041</v>
+        <v>0.7181985915342967</v>
       </c>
       <c r="D7" t="n">
         <v>0.85</v>
       </c>
       <c r="E7" t="n">
-        <v>0.7717293500900269</v>
+        <v>0.6542128324508667</v>
       </c>
       <c r="F7" t="n">
         <v>0.8333333333333334</v>
@@ -3701,7 +3633,7 @@
         <v>1</v>
       </c>
       <c r="J7" t="n">
-        <v>83.43450665473938</v>
+        <v>104.8532993793488</v>
       </c>
     </row>
     <row r="8">
@@ -3714,16 +3646,16 @@
         <v>1</v>
       </c>
       <c r="C8" t="n">
-        <v>0.7477272827307383</v>
+        <v>0.7152532309293748</v>
       </c>
       <c r="D8" t="n">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
       <c r="E8" t="n">
-        <v>0.788404107093811</v>
+        <v>0.6016882061958313</v>
       </c>
       <c r="F8" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.5</v>
       </c>
       <c r="G8" t="n">
         <v>0.2</v>
@@ -3735,7 +3667,7 @@
         <v>1</v>
       </c>
       <c r="J8" t="n">
-        <v>66.88468241691589</v>
+        <v>47.20666074752808</v>
       </c>
     </row>
     <row r="9">
@@ -3748,16 +3680,16 @@
         <v>4</v>
       </c>
       <c r="C9" t="n">
-        <v>0.8440627957383793</v>
+        <v>0.8489274720946949</v>
       </c>
       <c r="D9" t="n">
-        <v>0.6375</v>
+        <v>0.825</v>
       </c>
       <c r="E9" t="n">
-        <v>0.7659741938114166</v>
+        <v>0.6834053695201874</v>
       </c>
       <c r="F9" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.7</v>
       </c>
       <c r="G9" t="n">
         <v>1</v>
@@ -3769,7 +3701,7 @@
         <v>1</v>
       </c>
       <c r="J9" t="n">
-        <v>39.14067429304123</v>
+        <v>45.43437242507935</v>
       </c>
     </row>
     <row r="10">
@@ -3782,13 +3714,13 @@
         <v>1</v>
       </c>
       <c r="C10" t="n">
-        <v>0.9232998530069988</v>
+        <v>0.9059004251162213</v>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="E10" t="n">
-        <v>0.7108879089355469</v>
+        <v>0.6615583896636963</v>
       </c>
       <c r="F10" t="n">
         <v>0.8</v>
@@ -3803,7 +3735,7 @@
         <v>1</v>
       </c>
       <c r="J10" t="n">
-        <v>16.77782320976257</v>
+        <v>47.09610152244568</v>
       </c>
     </row>
     <row r="11">
@@ -3816,16 +3748,16 @@
         <v>1</v>
       </c>
       <c r="C11" t="n">
-        <v>0.7188415389794571</v>
+        <v>0.7312327282245344</v>
       </c>
       <c r="D11" t="n">
-        <v>0.75</v>
+        <v>0.85</v>
       </c>
       <c r="E11" t="n">
-        <v>0.664071798324585</v>
+        <v>0.6902694702148438</v>
       </c>
       <c r="F11" t="n">
-        <v>0.4615384615384616</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="G11" t="n">
         <v>0.3333333333333333</v>
@@ -3837,7 +3769,7 @@
         <v>1</v>
       </c>
       <c r="J11" t="n">
-        <v>57.62241983413696</v>
+        <v>43.0357608795166</v>
       </c>
     </row>
     <row r="12">
@@ -3850,13 +3782,13 @@
         <v>1</v>
       </c>
       <c r="C12" t="n">
-        <v>0.9788179874420168</v>
+        <v>0.9747076630592347</v>
       </c>
       <c r="D12" t="n">
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>0.8587865829467773</v>
+        <v>0.8313844203948975</v>
       </c>
       <c r="F12" t="n">
         <v>1</v>
@@ -3871,7 +3803,7 @@
         <v>1</v>
       </c>
       <c r="J12" t="n">
-        <v>16.22343039512634</v>
+        <v>23.17125368118286</v>
       </c>
     </row>
   </sheetData>
@@ -3968,8 +3900,8 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Berdasarkan referensi yang tersedia, **tidak ditemukan ketentuan spesifik** mengenai bentuk bahasa (misalnya wajib bahasa Indonesia atau boleh bahasa asing) yang harus digunakan dalam pembuatan Perjanjian Kerja Waktu Tertentu (PKWT), baik untuk pekerja Warga Negara Indonesia maupun lainnya.
-Referensi yang tersedia hanya mengatur bahwa PKWT harus dibuat secara **tertulis** (PP No. 35 Tahun 2021 Pasal 18 ayat 2) dan memuat isi tertentu seperti nama, alamat, jabatan, upah, serta jangka waktu (PP No. 35 Tahun 2021 Pasal 6 dan Pasal 13). Ketentuan mengenai bahasa yang digunakan dalam perjanjian kerja tidak tercantum dalam pasal-pasal yang disediakan.</t>
+          <t>Istilah "PKWT" dalam pertanyaan Anda merujuk pada Perjanjian Kerja Waktu Tertentu sebagaimana diatur dalam Peraturan Pemerintah Nomor 35 Tahun 2021. Berdasarkan ketentuan tersebut, Perjanjian Kerja Waktu Tertentu wajib dibuat dalam bentuk tertulis. Ketentuan ini berlaku tanpa membedakan kewarganegaraan pekerja, sehingga berlaku pula bagi pekerja yang merupakan warga negara Indonesia.
+Dasar hukumnya adalah Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 18 ayat (2) yang menyatakan bahwa Perjanjian Kerja Waktu Tertentu atau Perjanjian Kerja Waktu Tidak Tertentu harus dibuat secara tertulis. Selain itu, isi Perjanjian Kerja Waktu Tertentu juga diatur secara rinci dalam Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 13 yang memuat unsur-unsur wajib seperti nama dan alamat perusahaan, data diri pekerja, jabatan, tempat pekerjaan, besaran dan cara pembayaran upah, hak dan kewajiban, serta jangka waktu berlakunya perjanjian.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -3978,10 +3910,10 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.5961143044630687</v>
+        <v>0.6549318275849025</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -3990,7 +3922,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>huruf latin; penafsiran; bahasa Indonesia berlaku</t>
+          <t>huruf latin; bahasa Indonesia; bahasa asing; penafsiran; bahasa Indonesia berlaku</t>
         </is>
       </c>
       <c r="J2" t="n">
@@ -4008,54 +3940,35 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Q19</t>
+          <t>Q16</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Pekerja migran Indonesia</t>
+          <t>PHK dan perselisihan hubungan industrial</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Calon pekerja migran akan ditempatkan melalui BP2MI berdasarkan permintaan pemberi kerja berbadan hukum di negara tujuan. Jelaskan dasar penempatannya, isi minimum perjanjian tertulis antar pihak penempatan, dan dokumen/hubungan kerja yang wajib ada bagi pekerja migran.</t>
+          <t>Perusahaan ingin mem-PHK pekerja karena pelanggaran aturan perusahaan setelah SP1, SP2, dan SP3, tetapi pekerja menolak. Jelaskan urutan langkah yang tepat: apa yang harus diupayakan sebelum PHK, hak uang apa yang menjadi dasar bila PHK karena pelanggaran berulang, dan ke mana sengketa dibawa jika bipartit/mediasi gagal?</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Berdasarkan referensi yang tersedia, berikut adalah jawaban atas pertanyaan Anda:
-**1. Dasar Penempatan**
-Penempatan Calon Pekerja Migran Indonesia (CPMI) oleh Badan Pelindungan Pekerja Migran Indonesia (BP2MI) didasarkan pada dua hal:
-*   Kebutuhan pemerintah; dan
-*   Permintaan dari pemerintah negara Pemberi Kerja atau permintaan Pemberi Kerja berbadan hukum di negara tujuan penempatan.
-*(Dasar hukum: PP Nomor 10 Tahun 2020 Pasal 2)*
-**2. Isi Minimum Perjanjian Tertulis**
-Perjanjian tertulis antara BP2MI dan CPMI (Perjanjian Penempatan) harus memuat rincian dari surat permintaan yang telah diverifikasi, yaitu:
-*   Identitas pemberi kerja;
-*   Jumlah penempatan;
-*   Jenis pekerjaan;
-*   Upah atau gaji;
-*   Kualifikasi jabatan;
-*   Masa berlaku Perjanjian Kerja;
-*   Fasilitas tempat kerja; dan
-*   Jaminan sosial dan/atau asuransi.
-*(Dasar hukum: PP Nomor 10 Tahun 2020 Pasal 7 ayat 2)*
-**3. Dokumen dan Hubungan Kerja yang Wajib Ada**
-*   **Dokumen Wajib:** CPMI wajib memiliki surat permintaan dari Pemberi Kerja yang telah diverifikasi oleh Atase Ketenagakerjaan (atau pejabat dinas luar negeri jika Atase belum ada).
-*   **Hubungan Kerja:** Terjadi hubungan kerja antara CPMI dengan Pemberi Kerja melalui Perjanjian Kerja yang memuat syarat kerja, hak, kewajiban, serta jaminan keamanan dan keselamatan selama bekerja.
-*(Dasar hukum: PP Nomor 10 Tahun 2020 Pasal 7 ayat 1 &amp; 2; PP Nomor 10 Tahun 2020 Pasal 1 bagian 1 ayat 3 &amp; 5)*</t>
+          <t>Istilah "pelanggaran berulang" dalam konteks pertanyaan Anda merujuk pada pelanggaran ketentuan yang diatur dalam Perjanjian Kerja, Peraturan Perusahaan, atau Perjanjian Kerja Bersama yang telah diberikan Surat Peringatan (SP) pertama, kedua, dan ketiga secara berturut-turut. Berdasarkan peraturan terbaru, yaitu Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 52 ayat (1), jika pengusaha melakukan Pemutusan Hubungan Kerja (PHK) karena alasan tersebut, pekerja/buruh berhak atas uang pesangon sebesar 0,5 (nol koma lima) kali ketentuan Pasal 40 ayat (2), uang penghargaan masa kerja sebesar 1 (satu) kali ketentuan Pasal 40 ayat (3), dan uang penggantian hak sesuai ketentuan Pasal 40 ayat (4).
+Sebelum melakukan PHK, pengusaha wajib memberikan Surat Peringatan pertama, kedua, dan ketiga secara berturut-turut kepada pekerja/buruh yang bersangkutan. Jika pekerja menolak surat pemberitahuan PHK, pengusaha harus membuat surat penolakan disertai alasan paling lama 7 (tujuh) hari kerja setelah diterimanya surat pemberitahuan sebagaimana diatur dalam Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 39 ayat (1). Selanjutnya, penyelesaian sengketa harus dilakukan melalui perundingan bipartit antara Pengusaha dengan Pekerja/Buruh dan/atau Serikat Pekerja/Serikat Buruh. Dalam hal perundingan bipartit tidak mencapai kesepakatan, penyelesaian dilakukan melalui mekanisme penyelesaian perselisihan hubungan industrial sesuai ketentuan peraturan perundang-undangan.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Penempatan PMI oleh BP2MI dapat didasarkan pada kebutuhan pemerintah atau permintaan dari pemerintah negara pemberi kerja atau pemberi kerja berbadan hukum di negara tujuan. Penempatan itu dilakukan atas dasar perjanjian tertulis. Perjanjian tertulis disusun berdasarkan prinsip persamaan kedudukan, saling menguntungkan, dan memperhatikan hukum nasional serta internasional, dan paling sedikit memuat identitas para pihak, hak dan kewajiban, syarat dan prosedur penempatan, mekanisme pelindungan PMI, pemantauan dan evaluasi, penyelesaian sengketa, perubahan perjanjian, serta jangka waktu dan pengakhiran. Dari sisi calon PMI, dokumen wajib mencakup antara lain sertifikat kompetensi, surat keterangan sehat, paspor, visa kerja, perjanjian penempatan, dan perjanjian kerja. Hubungan kerja dengan pemberi kerja didasarkan pada perjanjian kerja yang memuat unsur pekerjaan, upah, dan perintah, serta terjadi setelah perjanjian kerja disepakati dan ditandatangani.</t>
+          <t>Sebelum PHK, para pihak harus mengupayakan agar PHK tidak terjadi dan merundingkan maksud PHK. Untuk pelanggaran ketentuan perjanjian kerja, peraturan perusahaan, atau PKB yang telah didahului SP1, SP2, dan SP3 berturut-turut, dasar haknya adalah 0,5 kali uang pesangon, 1 kali uang penghargaan masa kerja, dan uang penggantian hak. Jika pekerja menolak, perselisihan wajib lebih dulu diupayakan melalui perundingan bipartit paling lama 30 hari kerja. Bila gagal, perselisihan dicatatkan ke instansi ketenagakerjaan dengan bukti bipartit; jika konsiliasi atau mediasi tidak mencapai kesepakatan, salah satu pihak dapat mengajukan gugatan ke Pengadilan Hubungan Industrial.</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.7188415389794571</v>
+        <v>0.7152532309293748</v>
       </c>
       <c r="G3" t="n">
-        <v>0.75</v>
+        <v>0.95</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -4064,55 +3977,71 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>hak dan kewajiban; mekanisme pelindungan; penyelesaian sengketa; sertifikat kompetensi; paspor; visa kerja; pekerjaan upah perintah</t>
+          <t>mencegah PHK; setengah kali pesangon; satu kali UPMK; 30 hari kerja; mediasi; Pengadilan Hubungan Industrial</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K3" t="n">
         <v>1</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Peraturan Pemerintah No. 10 Tahun 2020, Pasal 3 | PP_10_2020.pdf | Pasal 3</t>
+          <t>Undang-Undang No. 13 Tahun 2003, Pasal 1 | UU_Nomor_13_Tahun_2003.pdf | Pasal 1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Q09</t>
+          <t>Q17</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Lembur</t>
+          <t>PHK dan Jaminan Kehilangan Pekerjaan</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Apa syarat utama yang harus ada sebelum pengusaha mempekerjakan pekerja melebihi waktu kerja normal?</t>
+          <t>Seorang pekerja PKWTT terkena PHK dan ingin menuntut hak PHK sekaligus manfaat JKP. Bedakan hak uang dari pengusaha saat PHK dengan manfaat JKP dari program jaminan sosial, termasuk komponen manfaat JKP dan skema uang tunainya.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Sebelum pengusaha mempekerjakan pekerja melebihi waktu kerja normal, syarat utamanya adalah adanya **persetujuan pekerja/buruh yang bersangkutan**.
-Dasar hukumnya adalah:
-*   **PP Nomor 35 Tahun 2021 Pasal 52 ayat 2**: Pengusaha dilarang mempekerjakan pekerja/buruh melebihi waktu kerja sebagaimana dimaksud dalam Pasal 51 ayat (2) kecuali dengan persetujuan pekerja/buruh.
-*   **UU No. 13 Tahun 2003 Pasal 78 ayat (1)**: Pengusaha yang mempekerjakan pekerja/buruh melebihi waktu kerja harus memenuhi syarat adanya persetujuan pekerja/buruh yang bersangkutan.</t>
+          <t>Istilah "PKWTT" dalam pertanyaan Anda merujuk pada pekerja dengan Perjanjian Kerja Waktu Tidak Tertentu, dan "menuntut hak PHK" mengacu pada hak atas uang pesangon atau uang pengganti pesangon yang diatur dalam peraturan perundang-undangan ketenagakerjaan, berbeda dengan manfaat JKP yang merupakan jaminan sosial.
+Berdasarkan konteks tersebut, berikut adalah pembedahan hak dan manfaatnya:
+**1. Hak Uang dari Pengusaha (Uang Pesangon/Uang Pengganti Pesangon)**
+Hak ini timbul karena adanya Pemutusan Hubungan Kerja (PHK) dan menjadi kewajiban pengusaha untuk dibayarkan secara sekaligus kepada pekerja. Hak ini diatur dalam **Peraturan Pemerintah Nomor 37 Tahun 2021, Pasal 21 ayat (1)**.
+Komponen hak uang dari pengusaha ini terdiri dari:
+*   Uang pesangon (jika PHK karena alasan tertentu yang mewajibkan pesangon).
+*   Uang penghargaan masa kerja.
+*   Uang penggantian hak.
+*   *Catatan:* Jika pengusaha tidak mengikutsertakan pekerja dalam program JKP, maka pengusaha wajib memenuhi hak uang tunai sesuai perhitungan Pasal 21 ayat (1) tersebut secara sekaligus.
+**2. Manfaat JKP dari Program Jaminan Sosial**
+Manfaat JKP adalah jaminan sosial yang diberikan kepada pekerja/buruh yang mengalami PHK, terlepas dari apakah pekerja tersebut terdaftar dalam program JKP atau tidak (namun bagi yang tidak terdaftar, penggantian kewajiban ada pada pengusaha). Manfaat ini diatur dalam **Peraturan Pemerintah Nomor 37 Tahun 2021, Pasal 18** dan **Peraturan Menteri Ketenagakerjaan Nomor 7 Tahun 2025, Pasal 2**.
+Komponen manfaat JKP terdiri dari tiga bagian utama:
+*   **Uang Tunai:** Dibayarkan secara sekaligus.
+*   **Akses Informasi Pasar Kerja:** Layanan untuk mencari pekerjaan baru.
+*   **Pelatihan Kerja:** Program peningkatan kompetensi.
+**Skema dan Ketentuan Uang Tunai JKP:**
+*   **Sumber Dana:** Dana iuran peserta berasal dari anggaran pendapatan dan belanja negara (APBN) dan dibayarkan oleh pemerintah, bukan oleh pengusaha secara langsung dari iuran pekerja (sesuai **Peraturan Menteri Ketenagakerjaan Nomor 7 Tahun 2025, Pasal 1 ayat (1)**).
+*   **Syarat Penerima:** Pekerja/buruh yang mempunyai hubungan kerja dengan pengusaha dan telah terdaftar serta membayar iuran (sesuai **Peraturan Pemerintah Nomor 37 Tahun 2021, Pasal 1 ayat (6)**).
+*   **Syarat Masa Iuran:** Peserta berhak mendapatkan manfaat JKP jika telah memenuhi syarat masa iuran. Berdasarkan **Peraturan Pemerintah Nomor 6 Tahun 2025, Pasal 19 ayat (2)**, yang dimaksud "bersedia untuk bekerja kembali" adalah bekerja sebagai pekerja penerima upah atau berusaha mandiri atau wirausaha. Syarat masa iuran 12 (dua belas) bulan dimaknai untuk jumlah bulan iuran JKP yang dibayarkan oleh peserta secara akumulasi jumlah bulan iuran dalam 24 (dua puluh empat) bulan kalender.
+*   **Pengecualian:** Kewajiban pemenuhan hak uang tunai oleh pengusaha (sesuai Pasal</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Pengusaha yang mempekerjakan pekerja melebihi waktu kerja harus memenuhi syarat adanya persetujuan pekerja yang bersangkutan dan adanya perintah kerja lembur dari pengusaha.</t>
+          <t>Hak uang akibat PHK dari pengusaha mengacu pada kewajiban pembayaran uang pesangon dan/atau uang penghargaan masa kerja serta uang penggantian hak. Itu berbeda dari JKP, karena JKP adalah program yang wajib diikuti oleh pengusaha untuk mempertahankan derajat kehidupan layak saat pekerja kehilangan pekerjaan. Manfaat JKP terdiri dari uang tunai, akses informasi pasar kerja, dan pelatihan kerja. Uang tunai JKP diberikan paling banyak 6 bulan upah: 45% dari upah untuk 3 bulan pertama dan 25% dari upah untuk 3 bulan berikutnya, dengan dasar upah terakhir yang dilaporkan dan batas atas yang berlaku.</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.7361297393412818</v>
+        <v>0.7181985915342967</v>
       </c>
       <c r="G4" t="n">
-        <v>0.6</v>
+        <v>0.85</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -4121,69 +4050,55 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>lembur; perintah kerja lembur</t>
+          <t>kehilangan pekerjaan; 45 persen</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Undang-Undang No. 13 Tahun 2003, Pasal 78 | UU_Nomor_13_Tahun_2003.pdf | Pasal 78</t>
+          <t>Peraturan Pemerintah No. 37 Tahun 2021, Pasal 1 | pp_Nomor_37_Tahun_2021.pdf | Pasal 1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Q17</t>
+          <t>Q20</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>PHK dan Jaminan Kehilangan Pekerjaan</t>
+          <t>K3, narkotika, dan jaminan sosial</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Seorang pekerja PKWTT terkena PHK dan ingin menuntut hak PHK sekaligus manfaat JKP. Bedakan hak uang dari pengusaha saat PHK dengan manfaat JKP dari program jaminan sosial, termasuk komponen manfaat JKP dan skema uang tunainya.</t>
+          <t>Perusahaan menemukan indikasi peredaran narkotika di tempat kerja dan pada saat yang sama menjalankan pemagangan. Jelaskan tindakan kepatuhan yang perlu dilakukan terkait pelaporan/kebijakan pencegahan narkotika, hak K3 peserta pemagangan, dan konsekuensi bila pekerja belum diikutsertakan dalam JKK/JKM.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Berdasarkan referensi yang tersedia, berikut adalah pembedaan hak uang dari pengusaha saat PHK dengan manfaat JKP dari program jaminan sosial:
-**1. Hak Uang dari Pengusaha (Saat PHK)**
-Hak ini bersifat wajib bagi pengusaha untuk dipenuhi secara sekaligus kepada pekerja yang mengalami PHK, kecuali pengusaha tersebut berstatus usaha mikro.
-*   **Dasar Hukum:** PP Nomor 37 Tahun 2021 Pasal 37 ayat (1).
-*   **Komponen:** Manfaat uang tunai yang dihitung sesuai ketentuan Pasal 21 ayat (1) (biasanya mencakup uang pesangon, uang penghargaan masa kerja, dan uang penggantian hak).
-*   **Kewajiban:** Pengusaha wajib membayar sekaligus, kecuali untuk usaha mikro.
-**2. Manfaat JKP dari Program Jaminan Sosial**
-Manfaat ini diberikan oleh BPJS Ketenagakerjaan kepada pekerja/buruh yang telah terdaftar dan membayar iuran serta mengalami PHK.
-*   **Dasar Hukum:** PP Nomor 37 Tahun 2021 Pasal 1 ayat (1) dan Pasal 18.
-*   **Komponen Manfaat:**
-    1.  Uang tunai.
-    2.  Akses informasi pasar kerja.
-    3.  Pelatihan kerja.
-*   **Syarat Kepesertaan:** Pekerja harus telah terdaftar dan membayar iuran dengan masa iuran akumulasi minimal 12 bulan dalam 24 bulan kalender (PP Nomor 6 Tahun 2025 Pasal 19 ayat (2) dan (3)).
-*   **Skema Uang Tunai JKP:**
-    *   Dibayarkan dalam bentuk uang tunai.
-    *   Jumlah pembayaran dibatasi maksimal 6 kali dengan durasi masing-masing 3 bulan (total maksimal 18 bulan), kecuali untuk pekerja yang telah mencapai usia pensiun, meninggal dunia, atau cacat total tetap (PP Nomor 37 Tahun 2021 Pasal 21).
-    *   Pembayaran dilakukan oleh BPJS Ketenagakerjaan, bukan oleh pengusaha.
-**Catatan Penting:**
-*   **Naturalisasi Dasar Hukum:** PP Nomor 35 Tahun 2021 Pasal 52 ayat (2) tidak ditemukan dalam referensi yang diberikan. Referensi yang tersedia hanya mencakup PP Nomor 37 Tahun 2021 dan PP Nomor 6 Tahun 2025.
-*   **Hubungan Kedua Hak:** Kedua hak ini dapat dituntut secara bersamaan karena berasal dari sumber yang berbeda (pengusaha vs. jaminan sosial). Namun, jika pekerja tidak memenuhi syarat kepesertaan JKP (misalnya masa iuran belum cukup), maka pekerja hanya berhak atas hak uang dari pengusaha, bukan manfaat JKP.</t>
+          <t>Istilah "pemagangan" dalam konteks pertanyaan ini dipetakan ke dalam istilah resmi "pekerja/buruh" sebagaimana didefinisikan dalam Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 1 ayat (7), yang mencakup setiap orang yang bekerja dengan menerima upah atau imbalan dalam bentuk lain.
+Berdasarkan Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, berikut adalah tindakan kepatuhan yang harus dilakukan:
+1. **Pelaporan Segera**
+   Apabila ditemukan indikasi peredaran narkotika, psikotropika, dan zat adiktif lainnya di tempat kerja, pengusaha wajib segera melaporkan kepada Kepolisian Negara Republik Indonesia sesuai dengan ketentuan Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 8 ayat (1). Laporan tersebut juga harus disampaikan kepada instansi yang bertanggung jawab di bidang ketenagakerjaan Kabupaten/Kota melalui mekanisme pelaporan Panitia Pembina Keselamatan dan Kesehatan Kerja (P2K3) atau Pelayanan Kesehatan Kerja sesuai dengan Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 8 ayat (2).
+2. **Penetapan Kebijakan dan Program Pencegahan**
+   Pengusaha wajib melakukan upaya aktif pencegahan dan penanggulangan penyalahgunaan dan peredaran gelap narkotika, psikotropika, dan zat adiktif lainnya di tempat kerja sesuai dengan Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 2 ayat (1). Upaya ini meliputi penetapan kebijakan dan penyusunan serta pelaksanaan program sesuai dengan Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 2 ayat (2).
+   Proses penetapan kebijakan harus melalui konsultasi antara pengusaha dengan pekerja/buruh dan atau serikat pekerja/serikat buruh sesuai dengan Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 4 ayat (1). Kebijakan tersebut harus dinyatakan secara tertulis dan sekurang-kurangnya memuat komitmen pengusaha dalam upaya pencegahan dan penanggulangan serta komitmen pembentukan unit yang menangani program pencegahan dan penanggulangan sesuai dengan Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 4 ayat (2). Unit tersebut dapat merupakan unit tersendiri atau terintegrasi dengan P2K3 atau Pelayanan Kesehatan Kerja sesuai dengan Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 4 ayat (3). Pelaksanaan upaya pencegahan dan penanggulangan harus dilakukan dengan melibatkan pekerja/buruh, serikat pekerja/serikat buruh, pihak ketiga, atau ahli di bidang narkotika, psikotropika, dan zat adiktif lainnya sesuai dengan Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/200</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Hak uang akibat PHK dari pengusaha mengacu pada kewajiban pembayaran uang pesangon dan/atau uang penghargaan masa kerja serta uang penggantian hak. Itu berbeda dari JKP, karena JKP adalah program yang wajib diikuti oleh pengusaha untuk mempertahankan derajat kehidupan layak saat pekerja kehilangan pekerjaan. Manfaat JKP terdiri dari uang tunai, akses informasi pasar kerja, dan pelatihan kerja. Uang tunai JKP diberikan paling banyak 6 bulan upah: 45% dari upah untuk 3 bulan pertama dan 25% dari upah untuk 3 bulan berikutnya, dengan dasar upah terakhir yang dilaporkan dan batas atas yang berlaku.</t>
+          <t>Untuk pencegahan dan penanggulangan narkotika di tempat kerja, pengusaha wajib melakukan upaya aktif, antara lain penetapan kebijakan, penyusunan dan pelaksanaan program, serta konsultasi/koordinasi dengan pihak terkait. Bila ditemukan seseorang memiliki atau mengedarkan narkotika, psikotropika, atau zat adiktif lainnya di tempat kerja, pengusaha atau pekerja harus segera melaporkan kepada Kepolisian dan laporan juga disampaikan kepada instansi ketenagakerjaan. Dalam pemagangan, peserta berhak memperoleh fasilitas K3, dan penyelenggara wajib menyediakan alat pelindung diri sesuai persyaratan K3. Jika pemberi kerja belum mengikutsertakan pekerjanya dalam program JKK atau JKM dan terjadi risiko, pemberi kerja wajib membayar hak pekerja sesuai ketentuan program tersebut.</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.7382594025135041</v>
+        <v>0.7291302879515149</v>
       </c>
       <c r="G5" t="n">
         <v>0.85</v>
@@ -4195,62 +4110,52 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>kehilangan pekerjaan; 45 persen</t>
+          <t>kebijakan tertulis; konsultasi pekerja; lapor Kepolisian; instansi ketenagakerjaan; alat pelindung diri; JKK; JKM; pemberi kerja wajib membayar hak pekerja</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K5" t="n">
         <v>1</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Peraturan Pemerintah No. 37 Tahun 2021, Pasal 1 | pp_Nomor_37_Tahun_2021.pdf | Pasal 1</t>
+          <t>Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 8 | PER-11-MEN-VI-2005.pdf | Pasal 8</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Q16</t>
+          <t>Q19</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>PHK dan perselisihan hubungan industrial</t>
+          <t>Pekerja migran Indonesia</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Perusahaan ingin mem-PHK pekerja karena pelanggaran aturan perusahaan setelah SP1, SP2, dan SP3, tetapi pekerja menolak. Jelaskan urutan langkah yang tepat: apa yang harus diupayakan sebelum PHK, hak uang apa yang menjadi dasar bila PHK karena pelanggaran berulang, dan ke mana sengketa dibawa jika bipartit/mediasi gagal?</t>
+          <t>Calon pekerja migran akan ditempatkan melalui BP2MI berdasarkan permintaan pemberi kerja berbadan hukum di negara tujuan. Jelaskan dasar penempatannya, isi minimum perjanjian tertulis antar pihak penempatan, dan dokumen/hubungan kerja yang wajib ada bagi pekerja migran.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Berdasarkan referensi yang tersedia, berikut adalah jawaban atas kasus tersebut:
-**1. Langkah yang Harus Diupayakan Sebelum PHK**
-Sebelum melakukan Pemutusan Hubungan Kerja (PHK), pengusaha wajib memberikan **Surat Peringatan (SP) berturut-turut sebanyak tiga kali (SP1, SP2, dan SP3)** kepada pekerja yang bersangkutan.
-*   **Dasar Hukum:** PP Nomor 35 Tahun 2021 Pasal 52 ayat (1) dan UU No. 13 Tahun 2003 Pasal 161 ayat (1).
-*   **Catatan:** Surat peringatan tersebut berlaku untuk jangka waktu paling lama 6 bulan, kecuali ditentukan lain dalam Perjanjian Kerja, Peraturan Perusahaan, atau Perjanjian Kerja Bersama.
-**2. Hak Uang yang Menjadi Dasar (Jika PHK karena Pelanggaran Berulang)**
-Jika pekerja melakukan pelanggaran ketentuan yang diatur dalam Perjanjian Kerja, Peraturan Perusahaan, atau Perjanjian Kerja Bersama setelah menerima SP1, SP2, dan SP3 secara berturut-turut, pekerja berhak atas:
-*   **Uang Pesangon:** 0,5 (nol koma lima) kali ketentuan Pasal 40 ayat (2).
-*   **Uang Penghargaan Masa Kerja:** 1 (satu) kali ketentuan Pasal 40 ayat (3).
-*   **Uang Penggantian Hak:** Sesuai ketentuan Pasal 40 ayat (4).
-*   **Dasar Hukum:** PP Nomor 35 Tahun 2021 Pasal 52 ayat (1).
-**3. Penyelesaian Sengketa Jika Bipartit/Mediasi Gagal**
-Jika terjadi perbedaan pendapat mengenai PHK tersebut, penyelesaian harus dilakukan melalui **perundingan bipartit** antara Pengusaha dengan Pekerja/Buruh dan/atau Serikat Pekerja/Serikat Buruh. Jika perundingan bipartit tidak mencapai kesepakatan, penyelesaian tahap berikutnya dilakukan melalui **mekanisme penyelesaian perselisihan hubungan industrial** sesuai ketentuan peraturan perundang-undangan.
-*   **Dasar Hukum:** PP Nomor 35 Tahun 2021 Pasal 39 ayat (2) dan ayat (3).</t>
+          <t>Berdasarkan konteks pertanyaan mengenai penempatan Calon Pekerja Migran Indonesia melalui Badan Pelindungan Pekerja Migran Indonesia (BP2MI) atas permintaan Pemberi Kerja berbadan hukum, berikut adalah penjelasan hukumnya:
+Pertama, mengenai dasar penempatan, hal tersebut diatur dalam Peraturan Pemerintah Nomor 10 Tahun 2020 Pasal 2 ayat (2) yang menyatakan bahwa penempatan oleh BP2MI didasarkan pada permintaan dari pemerintah negara Pemberi Kerja atau permintaan Pemberi Kerja berbadan hukum di negara tujuan penempatan.
+Kedua, mengenai isi minimum perjanjian tertulis antara BP2MI dan Calon Pekerja Migran Indonesia, isi tersebut harus memuat identitas pemberi kerja, jumlah penempatan, jenis pekerjaan, upah atau gaji, kualifikasi jabatan, masa berlaku Perjanjian Kerja, fasilitas tempat kerja, dan jaminan sosial serta asuransi sebagaimana diatur dalam Peraturan Pemerintah Nomor 10 Tahun 2020 Pasal 7 ayat (2).
+Ketiga, mengenai dokumen dan hubungan kerja yang wajib ada, Calon Pekerja Migran Indonesia harus memiliki surat permintaan dari Pemberi Kerja yang telah diverifikasi oleh Atase Ketenagakerjaan atau pejabat dinas luar negeri yang ditunjuk jika Atase belum ada di negara tujuan, serta wajib menandatangani Perjanjian Kerja dengan Pemberi Kerja yang memuat syarat kerja, hak, kewajiban, dan jaminan keamanan serta keselamatan selama bekerja sesuai dengan ketentuan peraturan perundang-undangan.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Sebelum PHK, para pihak harus mengupayakan agar PHK tidak terjadi dan merundingkan maksud PHK. Untuk pelanggaran ketentuan perjanjian kerja, peraturan perusahaan, atau PKB yang telah didahului SP1, SP2, dan SP3 berturut-turut, dasar haknya adalah 0,5 kali uang pesangon, 1 kali uang penghargaan masa kerja, dan uang penggantian hak. Jika pekerja menolak, perselisihan wajib lebih dulu diupayakan melalui perundingan bipartit paling lama 30 hari kerja. Bila gagal, perselisihan dicatatkan ke instansi ketenagakerjaan dengan bukti bipartit; jika konsiliasi atau mediasi tidak mencapai kesepakatan, salah satu pihak dapat mengajukan gugatan ke Pengadilan Hubungan Industrial.</t>
+          <t>Penempatan PMI oleh BP2MI dapat didasarkan pada kebutuhan pemerintah atau permintaan dari pemerintah negara pemberi kerja atau pemberi kerja berbadan hukum di negara tujuan. Penempatan itu dilakukan atas dasar perjanjian tertulis. Perjanjian tertulis disusun berdasarkan prinsip persamaan kedudukan, saling menguntungkan, dan memperhatikan hukum nasional serta internasional, dan paling sedikit memuat identitas para pihak, hak dan kewajiban, syarat dan prosedur penempatan, mekanisme pelindungan PMI, pemantauan dan evaluasi, penyelesaian sengketa, perubahan perjanjian, serta jangka waktu dan pengakhiran. Dari sisi calon PMI, dokumen wajib mencakup antara lain sertifikat kompetensi, surat keterangan sehat, paspor, visa kerja, perjanjian penempatan, dan perjanjian kerja. Hubungan kerja dengan pemberi kerja didasarkan pada perjanjian kerja yang memuat unsur pekerjaan, upah, dan perintah, serta terjadi setelah perjanjian kerja disepakati dan ditandatangani.</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.7477272827307383</v>
+        <v>0.7312327282245344</v>
       </c>
       <c r="G6" t="n">
         <v>0.85</v>
@@ -4262,63 +4167,57 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>mencegah PHK; setengah kali pesangon; satu kali UPMK; Pengadilan Hubungan Industrial</t>
+          <t>hak dan kewajiban; mekanisme pelindungan; penyelesaian sengketa; sertifikat kompetensi; paspor; visa kerja; perjanjian penempatan; pekerjaan upah perintah</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K6" t="n">
         <v>1</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Undang-Undang No. 13 Tahun 2003, Pasal 1 | UU_Nomor_13_Tahun_2003.pdf | Pasal 1</t>
+          <t>Peraturan Pemerintah No. 10 Tahun 2020, Pasal 3 | PP_10_2020.pdf | Pasal 3</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Q20</t>
+          <t>Q18</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>K3, narkotika, dan jaminan sosial</t>
+          <t>Disabilitas dan pemagangan</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Perusahaan menemukan indikasi peredaran narkotika di tempat kerja dan pada saat yang sama menjalankan pemagangan. Jelaskan tindakan kepatuhan yang perlu dilakukan terkait pelaporan/kebijakan pencegahan narkotika, hak K3 peserta pemagangan, dan konsekuensi bila pekerja belum diikutsertakan dalam JKK/JKM.</t>
+          <t>Jika pemberi kerja membuka program pemagangan untuk peserta penyandang disabilitas, apa saja kewajiban dan bentuk dukungan yang harus diperhatikan dari sisi hak peserta, kewajiban penyelenggara, kebutuhan khusus peserta, dan peran ULD Ketenagakerjaan?</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Berdasarkan referensi yang tersedia, berikut adalah penjelasan tindakan kepatuhan dan konsekuensi hukumnya:
-**1. Tindakan Pelaporan dan Kebijakan Pencegahan**
-*   **Pelaporan:** Pengusaha wajib segera melaporkan temuan peredaran narkotika kepada Kepolisian Negara Republik Indonesia dan instansi ketenagakerjaan Kabupaten/Kota melalui mekanisme Panitia Pembina Keselamatan dan Kesehatan Kerja (P2K3) atau Pelayanan Kesehatan Kerja (Pasal 8 ayat 1 dan 2).
-*   **Kebijakan Pencegahan:** Pengusaha wajib menetapkan kebijakan tertulis yang memuat komitmen pencegahan dan pembentukan unit penanganan, serta melibatkan pekerja/buruh, serikat pekerja/buruh, atau pihak ketiga ahli dalam pelaksanaannya (Pasal 2 ayat 1-3 dan Pasal 4 ayat 1-4).
-**2. Hak K3 Peserta Pemagangan**
-*   Referensi yang tersedia **tidak mengatur secara spesifik** mengenai hak Keselamatan dan Kesehatan Kerja (K3) khusus untuk peserta pemagangan.
-*   Namun, berdasarkan Pasal 2 ayat (3), upaya pencegahan dan penanggulangan wajib dilakukan dengan melibatkan "pekerja/buruh". Peserta pemagangan secara hukum tidak dikategorikan sebagai pekerja/buruh (mereka adalah peserta pelatihan), sehingga keterlibatan mereka dalam mekanisme pelaporan dan program pencegahan harus disesuaikan dengan definisi "tempat kerja" dan prinsip non-diskriminasi yang berlaku umum, meskipun detail teknisnya tidak tercantum dalam referensi ini.
-**3. Konsekuensi Jika Pekerja Belum Diikutsertakan dalam JKK/JKM**
-*   Referensi yang tersedia **tidak mencantumkan** konsekuensi hukum atau sanksi spesifik bagi pengusaha yang tidak mengikutsertakan pekerja dalam Jaminan Kecelakaan Kerja (JKK) atau Jaminan Kematian (JKM).
-*   Referensi hanya mengatur bahwa ketentuan perawatan dan rehabilitasi akibat penyalahgunaan zat diatur dalam Perjanjian Kerja, Peraturan Perusahaan, atau Perjanjian Kerja Bersama (Pasal 7 ayat 1), namun tidak menyebutkan kewajiban mutlak JKK/JKM atau sanksinya dalam dokumen ini.
-**Catatan Tambahan:**
-Referensi yang tersedia belum cukup untuk menjawab secara lengkap mengenai konsekuensi hukum tidak adanya JKK/JKM dan hak spesifik peserta pemagangan, karena referensi hanya memuat regulasi Pencegahan dan Penanggulangan Penyalahgunaan Narkotika (PER.11/MEN/VI/2005). Untuk aspek JKK/JKM dan regulasi pemagangan, diperlukan referensi lain seperti UU Ketenagakerjaan atau Peraturan Pemerintah terkait Jaminan Sosial dan Pemagangan.</t>
+          <t>Berdasarkan konteks pertanyaan mengenai program pemagangan untuk peserta penyandang disabilitas, berikut adalah rincian kewajiban dan bentuk dukungan yang harus diperhatikan:
+Pertama, mengenai definisi istilah, istilah "pelanggaran berat" dalam konteks ini dipetakan ke dalam konsep "Diskriminasi" sebagaimana diatur dalam Pasal 5 ayat (1) huruf d Peraturan Pemerintah Nomor 60 Tahun 2020, yang didefinisikan sebagai setiap pembedaan, pengecualian, pembatasan, pelecehan, atau pengucilan atas dasar disabilitas yang bermaksud atau berdampak pada pembatasan atau peniadaan pengakuan, penikmatan, atau pelaksanaan hak Penyandang Disabilitas.
+Kedua, dari sisi kewajiban penyelenggara pemagangan, sesuai dengan Pasal 16 Peraturan Menteri Ketenagakerjaan Nomor 6 Tahun 2020, penyelenggara pemagangan wajib melakukan tujuh hal, yaitu: membimbing peserta pemagangan sesuai dengan program pemagangan; memenuhi hak peserta pemagangan sesuai dengan perjanjian pemagangan; menyediakan alat pelindung diri sesuai dengan persyaratan keselamatan dan kesehatan kerja; memberikan uang saku kepada peserta pemagangan; mengikutsertakan peserta pemagangan dalam program jaminan sosial; mengevaluasi peserta pemagangan; serta memberikan sertifikat pemagangan atau surat keterangan telah mengikuti pemagangan.
+Ketiga, terkait kebutuhan khusus peserta penyandang disabilitas, Pasal 24 Peraturan Menteri Ketenagakerjaan Nomor 6 Tahun 2020 secara tegas menyatakan bahwa penyelenggaraan pemagangan bagi peserta pemagangan penyandang disabilitas harus dilaksanakan dengan memperhatikan kebutuhan khusus peserta pemagangan tersebut.
+Keempat, mengenai bentuk dukungan yang dapat diberikan pemberi kerja dalam penempatan tenaga kerja penyandang disabilitas, Pasal 48 ayat (1) Undang-Undang Nomor 8 Tahun 2016 tentang Penyandang Disabilitas memberikan opsi fleksibilitas kepada pemberi kerja, yaitu: memberikan kesempatan untuk masa orientasi atau adaptasi di awal masa kerja untuk menentukan apa yang diperlukan, termasuk penyelenggaraan pelatihan atau magang; menyediakan tempat bekerja yang fleksibel dengan menyesuaikan kepada ragam disabilitas tanpa mengurangi target tugas kerja; menyediakan waktu istirahat; menyediakan jadwal kerja yang fleksibel dengan tetap memenuhi alokasi waktu kerja; memberikan asistensi dalam pelaksanaan pekerjaan dengan memperhatikan kebutuhan khusus penyandang disabilitas; dan memberikan izin atau cuti khusus untuk pengobatan.
+Kelima, peran Unit Layanan Disabilitas Bidang Ketenagakerjaan (ULD Ketenagakerjaan) dalam mendukung program ini diatur dalam Pasal 18 Peraturan Pemerintah Nomor 60 Tahun 2020, yang mencakup tugas untuk merencanakan penghormatan, pelindungan, dan pemenuhan hak atas pekerjaan penyandang disabilitas; memberikan informasi kepada pemerintah, pemerintah daerah, dan perusahaan swasta mengenai proses rekrutmen, penerimaan, pelatihan kerja, penempatan kerja, keberlanjutan kerja, dan pengembangan karier yang adil dan tanpa diskriminasi kepada penyandang disabilitas; menyediakan pendampingan kepada tenaga kerja penyandang disabilitas; menyediakan pendampingan kepada pemberi kerja yang menerima tenaga kerja penyandang disabilitas; serta mengoordinasikan ULD Ketenagakerjaan, pemberi kerja, dan tenaga kerja dalam pemenuhan dan penyediaan alat bantu kerja untuk penyandang disabilitas.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Untuk pencegahan dan penanggulangan narkotika di tempat kerja, pengusaha wajib melakukan upaya aktif, antara lain penetapan kebijakan, penyusunan dan pelaksanaan program, serta konsultasi/koordinasi dengan pihak terkait. Bila ditemukan seseorang memiliki atau mengedarkan narkotika, psikotropika, atau zat adiktif lainnya di tempat kerja, pengusaha atau pekerja harus segera melaporkan kepada Kepolisian dan laporan juga disampaikan kepada instansi ketenagakerjaan. Dalam pemagangan, peserta berhak memperoleh fasilitas K3, dan penyelenggara wajib menyediakan alat pelindung diri sesuai persyaratan K3. Jika pemberi kerja belum mengikutsertakan pekerjanya dalam program JKK atau JKM dan terjadi risiko, pemberi kerja wajib membayar hak pekerja sesuai ketentuan program tersebut.</t>
+          <t>Peserta pemagangan berhak memperoleh bimbingan, pemenuhan hak sesuai perjanjian pemagangan, fasilitas K3, uang saku, kepesertaan jaminan sosial, serta sertifikat atau surat keterangan. Penyelenggara wajib membimbing peserta, memenuhi hak peserta, menyediakan alat pelindung diri sesuai K3, memberi uang saku, mengikutsertakan peserta dalam jaminan sosial, mengevaluasi, dan memberikan sertifikat atau surat keterangan. Untuk peserta penyandang disabilitas, penyelenggaraan pemagangan harus memperhatikan kebutuhan khusus peserta. ULD Ketenagakerjaan dapat mendukung melalui tenaga pendamping yang mendampingi tenaga kerja penyandang disabilitas dan pemberi kerja, termasuk penyuluhan, bimbingan jabatan, konsultasi pelatihan/penempatan/pemberdayaan, pemenuhan dan pelindungan hak, serta penyediaan alat bantu kerja.</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.7755328321139018</v>
+        <v>0.8153615871429444</v>
       </c>
       <c r="G7" t="n">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -4327,52 +4226,51 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>psikotropika; zat adiktif; konsultasi pekerja; lapor Kepolisian; alat pelindung diri; pemberi kerja wajib membayar hak pekerja</t>
+          <t>bimbingan; K3; tenaga pendamping</t>
         </is>
       </c>
       <c r="J7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K7" t="n">
         <v>1</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Peraturan Menteri Ketenagakerjaan No. PER.11/MEN/VI/2005 Tahun 2005, Pasal 8 | PER-11-MEN-VI-2005.pdf | Pasal 8</t>
+          <t>Peraturan Menteri Ketenagakerjaan No. 21 Tahun 2020, Pasal 1 bagian 1 | permen_Nomor_21_Tahun_2020.pdf | Pasal 1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Q13</t>
+          <t>Q09</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PHK</t>
+          <t>Lembur</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Dalam PHK, komponen apa saja yang termasuk uang penggantian hak menurut PP 35 Tahun 2021?</t>
+          <t>Apa syarat utama yang harus ada sebelum pengusaha mempekerjakan pekerja melebihi waktu kerja normal?</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Menurut **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 40 ayat (4)**, komponen yang termasuk dalam uang penggantian hak adalah:
-1.  **Cuti tahunan** yang belum diambil dan belum gugur.
-2.  **Biaya atau ongkos pulang** untuk Pekerja/Buruh.
-*(Catatan: Referensi yang tersedia tidak menyebutkan komponen lain di luar kedua poin tersebut).*</t>
+          <t>Syarat utama yang harus dipenuhi sebelum pengusaha mempekerjakan pekerja melebihi waktu kerja normal adalah adanya persetujuan tertulis dari pekerja/buruh yang bersangkutan. Ketentuan ini diatur dalam Undang-Undang Nomor 13 Tahun 2003 tentang Ketenagakerjaan Pasal 78 ayat (1) huruf a.
+Selain persetujuan pekerja, pengusaha juga wajib membatasi waktu kerja lembur maksimal 3 (tiga) jam dalam 1 (satu) hari dan 14 (empat belas) jam dalam 1 (satu) minggu sesuai Pasal 78 ayat (1) huruf b Undang-Undang Nomor 13 Tahun 2003. Perlu dicatat bahwa batasan waktu kerja lembur tersebut tidak berlaku bagi sektor usaha atau pekerjaan tertentu sebagaimana dimaksud dalam Pasal 78 ayat (3) Undang-Undang Nomor 13 Tahun 2003.
+Aturan terbaru yang lebih spesifik mengenai hal ini terdapat dalam Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 27 ayat (1) yang mewajibkan pembayaran upah kerja lembur bagi pekerja yang melebihi waktu kerja, dengan pengecualian bagi pekerja dalam golongan jabatan tertentu yang memiliki tanggung jawab sebagai pemikir, perencana, pelaksana, dan pengendali jalannya perusahaan dengan waktu kerja tidak terbatas dan mendapat upah lebih tinggi.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Uang penggantian hak meliputi cuti tahunan yang belum diambil dan belum gugur, biaya atau ongkos pulang untuk pekerja dan keluarganya ke tempat pekerja diterima bekerja, serta hal lain yang ditetapkan dalam perjanjian kerja, peraturan perusahaan, atau perjanjian kerja bersama.</t>
+          <t>Pengusaha yang mempekerjakan pekerja melebihi waktu kerja harus memenuhi syarat adanya persetujuan pekerja yang bersangkutan dan adanya perintah kerja lembur dari pengusaha.</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.8188177343777249</v>
+        <v>0.816637122091793</v>
       </c>
       <c r="G8" t="n">
         <v>0.85</v>
@@ -4384,18 +4282,18 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>pekerja dan keluarga; perjanjian kerja; peraturan perusahaan; PKB</t>
+          <t>perintah kerja lembur</t>
         </is>
       </c>
       <c r="J8" t="n">
+        <v>7</v>
+      </c>
+      <c r="K8" t="n">
         <v>2</v>
       </c>
-      <c r="K8" t="n">
-        <v>1</v>
-      </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 59 | PP Nomor 35 Tahun 2021.pdf | Pasal 59</t>
+          <t>Undang-Undang No. 13 Tahun 2003, Pasal 78 | UU_Nomor_13_Tahun_2003.pdf | Pasal 78</t>
         </is>
       </c>
     </row>
@@ -4417,11 +4315,15 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Dasar perhitungan upah untuk menghitung pesangon dan uang penghargaan masa kerja adalah **upah pokok** serta **segala macam bentuk tunjangan yang bersifat tetap** yang diberikan kepada pekerja/buruh dan keluarganya, termasuk harga pembelian dari catu yang diberikan secara cuma-cuma (jika catu harus dibayar dengan subsidi, maka dihitung sebagai selisih antara harga pembelian dan harga yang dibayar pekerja).
-Aturan ini diatur dalam:
-*   **Pasal 157 ayat (1) UU No. 13 Tahun 2003** (untuk pekerja tetap).
-*   **Pasal 40 ayat (1) PP No. 35 Tahun 2021** (untuk pekerja kontrak).
-Selain itu, jika upah dibayarkan secara harian, bulanan, satuan hasil, borongan, atau tergantung cuaca, maka perhitungan upah sebulan disesuaikan dengan ketentuan rata-rata penghasilan selama 12 bulan terakhir atau ketentuan upah minimum yang berlaku (Pasal 157 ayat (2), (3), dan (4) UU No. 13 Tahun 2003 / Pasal 40 ayat (1) PP No. 35 Tahun 2021).</t>
+          <t>Dasar perhitungan upah untuk menghitung uang pesangon dan uang penghargaan masa kerja adalah upah pokok serta segala macam bentuk tunjangan yang bersifat tetap yang diberikan kepada pekerja/buruh dan keluarganya, termasuk harga pembelian dari catu yang diberikan secara cuma-cuma atau selisih harga pembelian dengan harga yang harus dibayar oleh pekerja/buruh jika catu tersebut disubsidi.
+Sesuai dengan **Undang-Undang Nomor 13 Tahun 2003 tentang Ketenagakerjaan Pasal 157 ayat (1)**, komponen upah yang digunakan terdiri atas:
+a. Upah pokok;
+b. Segala macam bentuk tunjangan yang bersifat tetap yang diberikan kepada pekerja/buruh dan keluarganya, termasuk harga pembelian dari catu yang diberikan kepada pekerja/buruh secara cuma-cuma, yang apabila catu harus dibayar pekerja/buruh dengan subsidi, maka sebagai upah dianggap selisih antara harga pembelian dengan harga yang harus dibayar oleh pekerja/buruh.
+Selain itu, ketentuan perhitungan upah sebulan juga diatur sebagai berikut:
+1. Dalam hal penghasilan dibayarkan atas dasar perhitungan harian, maka penghasilan sebulan adalah sama dengan 30 kali penghasilan sehari (**Pasal 157 ayat (2)**).
+2. Dalam hal upah dibayarkan atas dasar perhitungan satuan hasil, potongan/borongan atau komisi, maka penghasilan sehari adalah sama dengan pendapatan rata-rata per hari selama 12 (dua belas) bulan terakhir, dengan ketentuan tidak boleh kurang dari ketentuan upah minimum provinsi atau kabupaten/kota (**Pasal 157 ayat (3)**).
+3. Dalam hal pekerjaan tergantung pada keadaan cuaca dan upahnya didasarkan pada upah borongan, maka perhitungan upah sebulan dihitung dari upah rata-rata 12 (dua belas) bulan terakhir (**Pasal 157 ayat (4)**).
+Peraturan Pemerintah Nomor 35 Tahun 2021 juga mengadopsi ketentuan serupa untuk Perjanjian Kerja Waktu Tertentu (PKWT), di mana uang pesangon dan uang penghargaan masa kerja dihitung berdasarkan ketentuan upah yang sama sebagaimana diatur dalam **Pasal 157 ayat (1) Undang-Undang Nomor 13 Tahun 2003**, sebagaimana dirujuk dalam **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 40 ayat (2) dan ayat (3)**.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -4430,14 +4332,14 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.8424351239204406</v>
+        <v>0.8528445161660513</v>
       </c>
       <c r="G9" t="n">
         <v>0.95</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>excellent</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -4460,58 +4362,37 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Q18</t>
+          <t>Q14</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Disabilitas dan pemagangan</t>
+          <t>PHK</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Jika pemberi kerja membuka program pemagangan untuk peserta penyandang disabilitas, apa saja kewajiban dan bentuk dukungan yang harus diperhatikan dari sisi hak peserta, kewajiban penyelenggara, kebutuhan khusus peserta, dan peran ULD Ketenagakerjaan?</t>
+          <t>Apa saja komponen uang yang wajib dibayarkan pengusaha ketika terjadi PHK secara umum?</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Berdasarkan referensi yang tersedia, berikut adalah kewajiban dan bentuk dukungan dalam program pemagangan untuk peserta penyandang disabilitas:
-**1. Kewajiban Penyelenggara Pemagangan (Sesuai Permen No. 6 Tahun 2020 Pasal 16)**
-Penyelenggara wajib:
-*   Membimbing peserta sesuai program pemagangan.
-*   Memenuhi hak peserta sesuai Perjanjian Pemagangan.
-*   Menyediakan Alat Pelindung Diri (APD) sesuai persyaratan K3.
-*   Memberikan uang saku kepada peserta.
-*   Mengikutsertakan peserta dalam program jaminan sosial.
-*   Mengevaluasi peserta pemagangan.
-*   Memberikan sertifikat pemagangan atau surat keterangan telah mengikuti pemagangan.
-**2. Bentuk Dukungan dan Kebutuhan Khusus Peserta (Sesuai Permen No. 6 Tahun 2020 Pasal 24)**
-Penyelenggaraan harus memperhatikan kebutuhan khusus peserta, yang mencakup:
-*   **Masa Orientasi/Adaptasi:** Memberikan kesempatan untuk masa orientasi atau adaptasi di awal masa kerja untuk menentukan apa yang diperlukan, termasuk penyelenggaraan pelatihan atau magang.
-*   **Fleksibilitas Tempat Kerja:** Menyediakan tempat bekerja yang fleksibel dengan menyesuaikan ragam disabilitas tanpa mengurangi target tugas kerja.
-*   **Waktu Istirahat:** Menyediakan waktu istirahat.
-*   **Jadwal Kerja Fleksibel:** Menyediakan jadwal kerja yang fleksibel dengan tetap memenuhi alokasi waktu kerja.
-*   **Asistensi:** Memberikan asistensi dalam pelaksanaan pekerjaan dengan memperhatikan kebutuhan khusus.
-*   **Cuti Khusus:** Memberikan izin atau cuti khusus untuk pengobatan.
-**3. Peran Unit Layanan Disabilitas Bidang Ketenagakerjaan (ULD Ketenagakerjaan) (Sesuai Permen No. 21 Tahun 2020 Pasal 18)**
-ULD Ketenagakerjaan bertugas:
-*   Merencanakan penghormatan, pelindungan, dan pemenuhan hak atas pekerjaan penyandang disabilitas.
-*   Memberikan informasi kepada pemerintah, pemerintah daerah, dan perusahaan swasta mengenai proses rekrutmen, penerimaan, pelatihan kerja, penempatan kerja, keberlanjutan kerja, dan pengembangan karier yang adil dan tanpa diskriminasi.
-*   Menyediakan pendampingan kepada tenaga kerja penyandang disabilitas.
-*   Menyediakan pendampingan kepada pemberi kerja yang menerima tenaga kerja penyandang disabilitas.
-*   Mengoordinasikan ULD Ketenagakerjaan, pemberi kerja, dan tenaga kerja dalam pemenuhan dan penyediaan alat bantu kerja untuk penyandang disabilitas.
-**Dasar Hukum:**
-*   Peraturan Menteri Ketenagakerjaan No. 6 Tahun 2020 Pasal 16 dan Pasal 24.
-*   Peraturan Menteri Ketenagakerjaan No. 21 Tahun 2020 Pasal 18.</t>
+          <t>Dalam konteks Pemutusan Hubungan Kerja (PHK) secara umum, istilah yang digunakan dalam peraturan adalah "uang pesangon", "uang penghargaan masa kerja", dan "uang penggantian hak". Berdasarkan Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 40 ayat (1), pengusaha wajib membayar ketiga komponen tersebut. Namun, terdapat perbedaan ketentuan berdasarkan jenis usaha dan jenis PHK.
+Untuk usaha mikro dan usaha kecil, sesuai Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 59, besaran pembayaran uang pesangon, uang penghargaan masa kerja, dan/atau uang pisah ditentukan berdasarkan kesepakatan antara pengusaha dan pekerja/buruh.
+Sedangkan untuk usaha selain usaha mikro dan usaha kecil, sesuai Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 40 ayat (1), komponen yang wajib dibayarkan adalah:
+1. Uang pesangon, yang perhitungannya diatur secara rinci dalam Pasal 40 ayat (2) berdasarkan masa kerja (mulai dari kurang dari 1 tahun hingga 8 tahun atau lebih).
+2. Uang penghargaan masa kerja, yang perhitungannya diatur dalam Pasal 40 ayat (3) untuk masa kerja 3 tahun atau lebih.
+3. Uang penggantian hak, yang meliputi cuti tahunan yang belum diambil dan belum gugur serta biaya atau ongkos pulang untuk pekerja/buruh dan keluarganya ke tempat dimana pekerja/buruh diterima bekerja, sebagaimana diatur dalam Pasal 40 ayat (4).
+Selain komponen di atas, jika terjadi PHK dan upah pekerja/buruh yang dilaporkan tidak sesuai dengan upah yang sebenarnya sehingga terdapat kekurangan pembayaran manfaat uang tunai, pengusaha wajib membayar kekurangan manfaat uang tunai tersebut secara sekaligus sesuai Peraturan Pemerintah Nomor 37 Tahun 2021 Pasal 23.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Peserta pemagangan berhak memperoleh bimbingan, pemenuhan hak sesuai perjanjian pemagangan, fasilitas K3, uang saku, kepesertaan jaminan sosial, serta sertifikat atau surat keterangan. Penyelenggara wajib membimbing peserta, memenuhi hak peserta, menyediakan alat pelindung diri sesuai K3, memberi uang saku, mengikutsertakan peserta dalam jaminan sosial, mengevaluasi, dan memberikan sertifikat atau surat keterangan. Untuk peserta penyandang disabilitas, penyelenggaraan pemagangan harus memperhatikan kebutuhan khusus peserta. ULD Ketenagakerjaan dapat mendukung melalui tenaga pendamping yang mendampingi tenaga kerja penyandang disabilitas dan pemberi kerja, termasuk penyuluhan, bimbingan jabatan, konsultasi pelatihan/penempatan/pemberdayaan, pemenuhan dan pelindungan hak, serta penyediaan alat bantu kerja.</t>
+          <t>Ketika terjadi PHK, pengusaha wajib membayar uang pesangon, uang penghargaan masa kerja, dan uang penggantian hak yang seharusnya diterima pekerja. Besaran detailnya bergantung pada alasan PHK dan masa kerja.</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.8650565798282623</v>
+        <v>0.864962592768669</v>
       </c>
       <c r="G10" t="n">
         <v>0.95</v>
@@ -4521,138 +4402,140 @@
           <t>excellent</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>bimbingan; tenaga pendamping</t>
-        </is>
-      </c>
+      <c r="I10" t="inlineStr"/>
       <c r="J10" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K10" t="n">
         <v>1</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Peraturan Menteri Ketenagakerjaan No. 21 Tahun 2020, Pasal 1 bagian 1 | permen_Nomor_21_Tahun_2020.pdf | Pasal 1</t>
+          <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 59 | PP Nomor 35 Tahun 2021.pdf | Pasal 59</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Q14</t>
+          <t>Q01</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>PHK</t>
+          <t>PKWT</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Apa saja komponen uang yang wajib dibayarkan pengusaha ketika terjadi PHK secara umum?</t>
+          <t>Jika pekerja PKWT bekerja selama 6 bulan lalu kontraknya berakhir sesuai jangka waktu, hak kompensasi apa yang perlu diberikan pengusaha dan bagaimana rumus umumnya?</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Berdasarkan referensi yang tersedia, komponen uang yang wajib dibayarkan pengusaha ketika terjadi Pemutusan Hubungan Kerja (PHK) secara umum adalah:
-1.  **Uang Pesangon**
-2.  **Uang Penghargaan Masa Kerja**
-3.  **Uang Penggantian Hak**
-Dasar hukumnya adalah **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 40 ayat (1)** dan **Undang-Undang Nomor 13 Tahun 2003 Pasal 156 ayat (1)** yang menyatakan bahwa pengusaha wajib membayar ketiga komponen tersebut.
-*Catatan: Untuk usaha mikro dan usaha kecil, pembayaran ketiga komponen tersebut dapat ditentukan berdasarkan kesepakatan antara pengusaha dan pekerja sesuai **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 59**.*</t>
+          <t>Istilah "kompensasi" dalam konteks pertanyaan Anda merujuk pada Uang Kompensasi sebagaimana diatur dalam Peraturan Pemerintah Nomor 35 Tahun 2021. Berdasarkan dokumen tersebut, jika Perjanjian Kerja Waktu Tertentu (PKWT) berakhir sesuai jangka waktu yang diperjanjikan, pengusaha wajib memberikan Uang Kompensasi kepada pekerja yang telah memiliki masa kerja paling sedikit satu bulan secara terus menerus.
+Sesuai dengan Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 15 ayat (1), (2), dan (4), kewajiban pembayaran Uang Kompensasi berlaku bagi pekerja PKWT yang hubungan kerjanya berakhir pada saat jangka waktu PKWT selesai.
+Untuk kasus pekerja yang bekerja selama 6 bulan, perhitungan besaran Uang Kompensanya diatur dalam Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 16 ayat (1) huruf b. Rumus umum perhitungannya adalah:
+**Masa Kerja (dalam bulan) x 1 (satu) bulan Upah**
+Karena masa kerja 6 bulan berada dalam kategori "satu bulan atau lebih tetapi kurang dari 12 bulan", maka pekerja berhak mendapatkan Uang Kompensasi sebesar 6 bulan upah. Dasar perhitungan upah tersebut terdiri dari Upah Pokok dan Tunjangan Tetap sesuai Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 16 ayat (2).</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Ketika terjadi PHK, pengusaha wajib membayar uang pesangon, uang penghargaan masa kerja, dan uang penggantian hak yang seharusnya diterima pekerja. Besaran detailnya bergantung pada alasan PHK dan masa kerja.</t>
+          <t>Pekerja PKWT berhak memperoleh uang kompensasi saat hubungan kerja berakhir karena jangka waktu selesai. Untuk masa kerja 12 bulan secara terus menerus kompensasinya 1 bulan upah. Untuk masa kerja kurang dari 12 bulan atau lebih dari 12 bulan, nilainya dihitung proporsional berdasarkan masa kerja dibagi 12 dikali 1 bulan upah. Jadi masa kerja 6 bulan dihitung 6 per 12 dikali 1 bulan upah.</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0.8664051770766577</v>
+        <v>0.8685559225082399</v>
       </c>
       <c r="G11" t="n">
-        <v>0.95</v>
+        <v>0.6</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
           <t>excellent</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>proporsional</t>
+        </is>
+      </c>
       <c r="J11" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K11" t="n">
         <v>1</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 59 | PP Nomor 35 Tahun 2021.pdf | Pasal 59</t>
+          <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 15 | PP Nomor 35 Tahun 2021.pdf | Pasal 15</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Q03</t>
+          <t>Q10</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PKWT</t>
+          <t>PHK</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Untuk pekerjaan yang diperkirakan selesai dalam waktu tertentu, berapa batas maksimal jangka waktu PKWT beserta perpanjangannya?</t>
+          <t>Jika pekerja melanggar ketentuan perjanjian kerja atau peraturan perusahaan setelah diberi surat peringatan pertama, kedua, dan ketiga, hak PHK apa yang menjadi dasar jawabannya?</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Batas maksimal jangka waktu Perjanjian Kerja Waktu Tertentu (PKWT) untuk pekerjaan yang diperkirakan selesai dalam waktu tertentu adalah **3 (tiga) tahun**, dengan ketentuan dapat diperpanjang **1 (satu) kali** untuk jangka waktu paling lama **1 (satu) tahun**.
-Dasar hukumnya adalah:
-*   **Pasal 4 ayat (1) huruf a PP Nomor 35 Tahun 2021**: PKWT dapat dibuat untuk pekerjaan yang diperkirakan penyelesaiannya dalam waktu yang tidak terlalu lama.
-*   **Pasal 8 ayat (1) PP Nomor 35 Tahun 2021**: Jangka waktu PKWT berdasarkan jangka waktu dapat dibuat untuk paling lama 5 (lima) tahun.
-*   **Pasal 59 ayat (1) huruf b UU Nomor 13 Tahun 2003**: Pekerjaan yang diperkirakan penyelesaiannya dalam waktu yang tidak terlalu lama paling lama 3 (tiga) tahun.
-*   **Pasal 59 ayat (4) UU Nomor 13 Tahun 2003**: PKWT dapat diperpanjang 1 (satu) kali untuk jangka waktu paling lama 1 (satu) tahun.
-*Catatan: Terdapat perbedaan regulasi antara PP Nomor 35 Tahun 2021 (maksimal 5 tahun) dan UU Nomor 13 Tahun 2003 (maksimal 3 tahun + 1 tahun perpanjangan). Berdasarkan referensi yang diberikan, kedua aturan tersebut berlaku.*</t>
+          <t>Istilah "pelanggaran" dalam pertanyaan Anda merujuk pada pelanggaran ketentuan yang diatur dalam perjanjian kerja, peraturan perusahaan, atau perjanjian kerja bersama sebagaimana dimaksud dalam Pasal 161 ayat (1) Undang-Undang Nomor 13 Tahun 2003 tentang Ketenagakerjaan. Berdasarkan aturan terbaru yang lebih spesifik, yaitu Peraturan Pemerintah Nomor 35 Tahun 2021, hak yang diterima pekerja dalam kondisi tersebut diatur dalam Pasal 52 ayat (1).
+Dalam kondisi di mana pekerja melakukan pelanggaran ketentuan perjanjian kerja, peraturan perusahaan, atau perjanjian kerja bersama dan sebelumnya telah diberikan surat peringatan pertama, kedua, dan ketiga secara berturut-turut, pekerja berhak atas:
+1. Uang pesangon sebesar 0,5 (nol koma lima) kali ketentuan Pasal 40 ayat (2);
+2. Uang penghargaan masa kerja sebesar 1 (satu) kali ketentuan Pasal 40 ayat (3); dan
+3. Uang penggantian hak sesuai ketentuan Pasal 40 ayat (4).
+Perlu dicatat bahwa ketentuan ini berlaku untuk Perjanjian Kerja Waktu Tertentu (PKWT) sebagaimana diatur dalam Peraturan Pemerintah Nomor 35 Tahun 2021. Jika konteksnya adalah Perjanjian Kerja Waktu Tidak Tertentu (PKWTT) berdasarkan Undang-Undang Nomor 13 Tahun 2003, maka hak yang diterima pekerja adalah uang pesangon sebesar 1 (satu) kali ketentuan Pasal 156 ayat (2), uang penghargaan masa kerja sebesar 1 (satu) kali ketentuan Pasal 156 ayat (3), dan uang penggantian hak sesuai ketentuan Pasal 156 ayat (4). Namun, mengingat adanya aturan baru yang lebih spesifik mengenai hak akibat PHK, maka ketentuan dalam Peraturan Pemerintah Nomor 35 Tahun 2021 menjadi acuan utama.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>PKWT berdasarkan jangka waktu untuk pekerjaan yang diperkirakan selesai dalam waktu tertentu dapat dibuat paling lama 5 tahun termasuk perpanjangannya.</t>
+          <t>Untuk PHK karena pekerja melakukan pelanggaran setelah diberikan surat peringatan pertama, kedua, dan ketiga, pekerja berhak atas uang pesangon sebesar setengah kali ketentuan pesangon, uang penghargaan masa kerja sebesar satu kali ketentuan, dan uang penggantian hak.</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.8766834902763367</v>
+        <v>0.8690293098290762</v>
       </c>
       <c r="G12" t="n">
-        <v>0.6</v>
+        <v>0.95</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
           <t>excellent</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>setengah kali pesangon; satu kali uang penghargaan masa kerja</t>
+        </is>
+      </c>
       <c r="J12" t="n">
         <v>2</v>
       </c>
       <c r="K12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 9 | PP Nomor 35 Tahun 2021.pdf | Pasal 9</t>
+          <t>Undang-Undang No. 13 Tahun 2003, Pasal 161 | UU_Nomor_13_Tahun_2003.pdf | Pasal 161</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Q10</t>
+          <t>Q11</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -4662,26 +4545,25 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Jika pekerja melanggar ketentuan perjanjian kerja atau peraturan perusahaan setelah diberi surat peringatan pertama, kedua, dan ketiga, hak PHK apa yang menjadi dasar jawabannya?</t>
+          <t>Jika pekerja di-PHK karena pelanggaran bersifat mendesak, apakah ia tetap mendapat pesangon dan UPMK?</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Berdasarkan referensi yang tersedia, jika pekerja melanggar ketentuan perjanjian kerja atau peraturan perusahaan setelah diberi surat peringatan pertama, kedua, dan ketiga secara berturut-turut, maka pekerja berhak atas:
-1.  **Uang pesangon** sebesar 0,5 kali ketentuan Pasal 40 ayat (2) (sesuai PP No. 35 Tahun 2021 Pasal 52 ayat 1 huruf a).
-2.  **Uang penghargaan masa kerja** sebesar 1 kali ketentuan Pasal 40 ayat (3) (sesuai PP No. 35 Tahun 2021 Pasal 52 ayat 1 huruf b).
-3.  **Uang penggantian hak** sesuai ketentuan Pasal 40 ayat (4) (sesuai PP No. 35 Tahun 2021 Pasal 52 ayat 1 huruf c).
-Dasar hukumnya adalah **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 52 ayat (1)**.
-*Catatan: Ketentuan ini berlaku untuk Perjanjian Kerja Waktu Tertentu (PKWT). Untuk Perjanjian Kerja Waktu Tidak Tertentu (PKWTT), dasar hukumnya adalah Undang-Undang No. 13 Tahun 2003 Pasal 161 yang memberikan hak atas uang pesangon 1 kali ketentuan Pasal 156 ayat (2), uang penghargaan masa kerja 1 kali ketentuan Pasal 156 ayat (3), dan uang penggantian hak.*</t>
+          <t>Istilah "di-PHK karena pelanggaran bersifat mendesak" dalam konteks hukum ketenagakerjaan merujuk pada Pemutusan Hubungan Kerja karena alasan pelanggaran yang diatur dalam Perjanjian Kerja, Peraturan Perusahaan, atau Perjanjian Kerja Bersama sebagaimana dimaksud dalam Pasal 52 ayat (2) Peraturan Pemerintah Nomor 35 Tahun 2021.
+Berdasarkan ketentuan tersebut, pekerja **tidak berhak** atas uang pesangon dan uang penghargaan masa kerja. Hak yang diterima pekerja hanya terbatas pada uang penggantian hak sesuai ketentuan Pasal 40 ayat (4).
+Dasar hukumnya adalah:
+Peraturan Pemerintah Nomor 35 Tahun 2021, Pasal 52 ayat (2) yang menyatakan bahwa pengusaha dapat melakukan Pemutusan Hubungan Kerja terhadap Pekerja/Buruh karena alasan Pekerja/Buruh melakukan pelanggaran bersifat mendesak yang diatur dalam Perjanjian Kerja, Peraturan Perusahaan, atau Perjanjian Kerja Bersama maka Pekerja/Buruh berhak atas: a. uang penggantian hak sesuai ketentuan Pasal 40 ayat (4); dan b. uang pisah yang besarannya diatur dalam Perjanjian Kerja, Peraturan Perusahaan, atau Perjanjian Kerja Bersama.
+Sedangkan ketentuan mengenai uang pesangon dan uang penghargaan masa kerja untuk kasus pelanggaran mendesak tidak diatur dalam ayat tersebut, sehingga hak atas kedua komponen tersebut tidak timbul dalam kondisi ini. Ketentuan ini berbeda dengan pelanggaran biasa yang memerlukan Surat Peringatan (SP) bertingkat (SP 1, SP 2, SP 3) yang diatur dalam Pasal 52 ayat (1) dan Pasal 161 Undang-Undang Nomor 13 Tahun 2003, di mana pekerja tetap berhak atas uang pesangon dan uang penghargaan masa kerja.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Untuk PHK karena pekerja melakukan pelanggaran setelah diberikan surat peringatan pertama, kedua, dan ketiga, pekerja berhak atas uang pesangon sebesar setengah kali ketentuan pesangon, uang penghargaan masa kerja sebesar satu kali ketentuan, dan uang penggantian hak.</t>
+          <t>Jika PHK terjadi karena pekerja melakukan pelanggaran bersifat mendesak yang diatur dalam perjanjian kerja, peraturan perusahaan, atau perjanjian kerja bersama, pekerja berhak atas uang penggantian hak dan uang pisah yang besarannya diatur dalam perjanjian kerja, peraturan perusahaan, atau perjanjian kerja bersama. Ketentuan ini tidak memberikan uang pesangon dan uang penghargaan masa kerja.</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0.8868805615107219</v>
+        <v>0.8872310147682827</v>
       </c>
       <c r="G13" t="n">
         <v>0.95</v>
@@ -4693,25 +4575,25 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>setengah kali pesangon; satu kali uang penghargaan masa kerja</t>
+          <t>tidak pesangon; tidak UPMK</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Undang-Undang No. 13 Tahun 2003, Pasal 161 | UU_Nomor_13_Tahun_2003.pdf | Pasal 161</t>
+          <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 52 | PP Nomor 35 Tahun 2021.pdf | Pasal 52</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Q11</t>
+          <t>Q13</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -4721,25 +4603,23 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Jika pekerja di-PHK karena pelanggaran bersifat mendesak, apakah ia tetap mendapat pesangon dan UPMK?</t>
+          <t>Dalam PHK, komponen apa saja yang termasuk uang penggantian hak menurut PP 35 Tahun 2021?</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Berdasarkan referensi yang tersedia, jika pekerja di-PHK karena pelanggaran bersifat mendesak, ia **tidak berhak** atas uang pesangon dan uang penghargaan masa kerja (UPMK).
-Menurut **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 52 ayat (2)**, dalam hal pengusaha melakukan PHK karena alasan pelanggaran bersifat mendesak, pekerja/buruh hanya berhak atas:
-1.  Uang penggantian hak sesuai ketentuan Pasal 40 ayat (4).
-2.  Uang pisah yang besarannya diatur dalam Perjanjian Kerja, Peraturan Perusahaan, atau Perjanjian Kerja Bersama.
-Sementara itu, hak atas uang pesangon dan UPMK hanya diberikan jika PHK dilakukan karena pelanggaran ketentuan yang telah diberikan surat peringatan pertama, kedua, dan ketiga secara berturut-turut (**PP Nomor 35 Tahun 2021 Pasal 52 ayat (1)**).</t>
+          <t>Menurut Peraturan Pemerintah Nomor 35 Tahun 2021, istilah "uang penggantian hak" merujuk pada komponen kompensasi yang wajib dibayarkan oleh pengusaha kepada pekerja/buruh dalam berbagai skenario Pemutusan Hubungan Kerja. Komponen-komponen tersebut secara spesifik diatur dalam Pasal 40 ayat (4) yang menyebutkan bahwa uang penggantian hak meliputi cuti tahunan yang belum diambil dan belum gugur serta biaya atau ongkos pulang untuk pekerja/buruh yang dipindahkan.
+Selain komponen yang disebutkan secara eksplisit dalam Pasal 40 ayat (4), terdapat komponen lain yang dapat dikategorikan sebagai bagian dari hak penggantian atau kompensasi tambahan tergantung pada alasan PHK yang terjadi. Dalam kasus PHK karena pelanggaran berat (pelanggaran bersifat mendesak) sebagaimana diatur dalam Pasal 52 ayat (2), pekerja/buruh berhak atas uang penggantian hak sesuai ketentuan Pasal 40 ayat (4) dan uang pisah yang besaran dan syaratnya diatur dalam Perjanjian Kerja, Peraturan Perusahaan, atau Perjanjian Kerja Bersama.
+Sementara itu, dalam skenario PHK karena alasan pengambilalihan perusahaan (Pasal 42 ayat 1 dan 2) atau karena sakit berkepanjangan/cacat akibat kecelakaan kerja (Pasal 41 dan Pasal 55), pekerja/buruh tetap berhak atas uang penggantian hak sesuai ketentuan Pasal 40 ayat (4). Perlu dicatat bahwa dalam skenario khusus bagi pengusaha pada usaha mikro dan usaha kecil yang melakukan PHK berdasarkan kesepakatan, sebagaimana diatur dalam Pasal 59, pembayaran uang penggantian hak dapat dilakukan berdasarkan kesepakatan antara pengusaha dan pekerja/buruh.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Jika PHK terjadi karena pekerja melakukan pelanggaran bersifat mendesak yang diatur dalam perjanjian kerja, peraturan perusahaan, atau perjanjian kerja bersama, pekerja berhak atas uang penggantian hak dan uang pisah yang besarannya diatur dalam perjanjian kerja, peraturan perusahaan, atau perjanjian kerja bersama. Ketentuan ini tidak memberikan uang pesangon dan uang penghargaan masa kerja.</t>
+          <t>Uang penggantian hak meliputi cuti tahunan yang belum diambil dan belum gugur, biaya atau ongkos pulang untuk pekerja dan keluarganya ke tempat pekerja diterima bekerja, serta hal lain yang ditetapkan dalam perjanjian kerja, peraturan perusahaan, atau perjanjian kerja bersama.</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.8965328709284466</v>
+        <v>0.8947867844785964</v>
       </c>
       <c r="G14" t="n">
         <v>0.95</v>
@@ -4751,53 +4631,52 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>tidak pesangon; tidak UPMK</t>
+          <t>pekerja dan keluarga; PKB</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K14" t="n">
         <v>1</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 52 | PP Nomor 35 Tahun 2021.pdf | Pasal 52</t>
+          <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 59 | PP Nomor 35 Tahun 2021.pdf | Pasal 59</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Q07</t>
+          <t>Q04</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Alih daya</t>
+          <t>PKWT harian</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Dalam hubungan kerja alih daya, siapa pihak yang bertanggung jawab atas perlindungan upah, kesejahteraan, syarat kerja, dan perselisihan pekerja?</t>
+          <t>Pekerja harian lepas bekerja 23 hari dalam sebulan selama 3 bulan berturut-turut. Bagaimana status hubungan kerjanya menurut aturan PKWT harian?</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Berdasarkan referensi yang tersedia, pihak yang bertanggung jawab atas perlindungan upah, kesejahteraan, syarat kerja, dan perselisihan pekerja dalam hubungan kerja alih daya adalah **Perusahaan Alih Daya**.
-Dasar hukumnya adalah:
-*   **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 18 ayat (3)**: Pelindungan Pekerja/Buruh, Upah, kesejahteraan, syarat kerja, dan perselisihan yang timbul dilaksanakan sesuai dengan ketentuan peraturan perundang-undangan dan menjadi tanggung jawab Perusahaan Alih Daya.
-*   **Peraturan Menteri Ketenagakerjaan Nomor 7 Tahun 2026 Pasal 4 ayat (2)**: Pelindungan dan hak pekerja/buruh alih daya dilaksanakan sekurang-kurangnya sesuai dengan ketentuan peraturan perundang-undangan dan menjadi tanggung jawab Perusahaan Alih Daya.
-*   **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 19 ayat (3)**: Dalam hal Pekerja/Buruh tidak memperoleh jaminan atas kelangsungan bekerja, Perusahaan Alih Daya bertanggung jawab atas pemenuhan hak Pekerja/Buruh.</t>
+          <t>Istilah "pekerja harian lepas" dalam pertanyaan Anda dipetakan ke dalam istilah resmi "Perjanjian Kerja Harian" sebagaimana diatur dalam Peraturan Pemerintah Nomor 35 Tahun 2021.
+Berdasarkan **Peraturan Pemerintah Nomor 35 Tahun 2021 tentang Perjanjian Kerja Waktu Tertentu, Alih Daya, Waktu Kerja dan Waktu Istirahat, dan Pemutusan Hubungan Kerja**, khususnya **Pasal 10 ayat (3)** dan **ayat (4)**, status hubungan kerja Anda berubah secara otomatis.
+Aturan tersebut menyatakan bahwa Perjanjian Kerja Harian hanya berlaku jika pekerja bekerja kurang dari 21 hari dalam satu bulan. Namun, dalam kasus Anda, pekerja telah bekerja selama 23 hari dalam sebulan selama 3 bulan berturut-turut. Oleh karena itu, Perjanjian Kerja Harian menjadi tidak berlaku dan hubungan kerja antara pengusaha dengan pekerja demi hukum berubah menjadi **Perjanjian Kerja Waktu Tidak Tertentu (PKWTT)** berdasarkan **Pasal 10 ayat (4)**.
+Konsekuensi hukumnya adalah hubungan kerja yang semula bersifat harian dan tidak tetap, kini beralih menjadi hubungan kerja yang bersifat tetap (PKWTT) sesuai dengan ketentuan dalam **Pasal 10 ayat (1)** yang menyebutkan bahwa pekerjaan dengan sifat tidak tetap dapat dilakukan dengan Perjanjian Kerja Harian, namun ketentuan pada ayat (4) mengoreksi status tersebut jika batas waktu kerja harian tercapai.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Perlindungan pekerja, upah, kesejahteraan, syarat kerja, dan perselisihan yang timbul menjadi tanggung jawab perusahaan alih daya sebagai pemberi kerja pekerja alih daya.</t>
+          <t>PKWT harian hanya dapat dibuat untuk pekerjaan tertentu yang berubah dalam waktu dan volume pekerjaan serta upah berdasarkan kehadiran, dengan ketentuan pekerja bekerja kurang dari 21 hari dalam 1 bulan. Jika pekerja bekerja 21 hari atau lebih selama 3 bulan berturut-turut atau lebih, perjanjian kerja harian menjadi PKWTT.</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.9159844358762106</v>
+        <v>0.9059004251162213</v>
       </c>
       <c r="G15" t="n">
         <v>0.95</v>
@@ -4809,7 +4688,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>perlindungan pekerja</t>
+          <t>menjadi PKWTT</t>
         </is>
       </c>
       <c r="J15" t="n">
@@ -4820,39 +4699,40 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 18 | PP Nomor 35 Tahun 2021.pdf | Pasal 18</t>
+          <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 10 | PP Nomor 35 Tahun 2021.pdf | Pasal 10</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Q04</t>
+          <t>Q02</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PKWT harian</t>
+          <t>PKWT</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Pekerja harian lepas bekerja 23 hari dalam sebulan selama 3 bulan berturut-turut. Bagaimana status hubungan kerjanya menurut aturan PKWT harian?</t>
+          <t>Apakah masa percobaan boleh diterapkan kepada pekerja PKWT, dan apa akibat hukumnya bila tetap dicantumkan?</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Berdasarkan **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 10 ayat (4)**, hubungan kerja pekerja harian tersebut **demi hukum berubah menjadi Perjanjian Kerja Waktu Tidak Tertentu (PKWTT)**.
-Hal ini terjadi karena pekerja telah bekerja selama **23 hari** (melebihi batas 21 hari) dalam **3 bulan berturut-turut**, sehingga Perjanjian Kerja Harian yang semula berlaku menjadi tidak berlaku.</t>
+          <t>Istilah "PKWT" dalam pertanyaan Anda merujuk pada Perjanjian Kerja Waktu Tertentu sebagaimana diatur dalam peraturan perundang-undangan ketenagakerjaan. Berdasarkan regulasi yang berlaku, masa percobaan kerja tidak boleh diterapkan kepada pekerja yang diikat dengan Perjanjian Kerja Waktu Tertentu.
+Hal ini diatur secara tegas dalam Peraturan Pemerintah Nomor 35 Tahun 2021 tentang Perjanjian Kerja Waktu Tertentu, Alih Daya, Waktu Kerja dan Waktu Istirahat, dan Pemutusan Hubungan Kerja Pasal 12 ayat (1) yang menyatakan bahwa PKWT tidak dapat mensyaratkan adanya masa percobaan kerja. Ketentuan yang sama juga terdapat dalam Undang-Undang Nomor 13 Tahun 2003 tentang Ketenagakerjaan Pasal 58 ayat (1).
+Akibat hukum jika pihak pengusaha tetap mencantumkan masa percobaan dalam Perjanjian Kerja Waktu Tertentu adalah masa percobaan kerja tersebut batal demi hukum. Meskipun masa percobaan tersebut dicantumkan, masa kerja pekerja tetap dihitung sejak terjadinya hubungan kerja berdasarkan Perjanjian Kerja Waktu Tertentu tersebut, tanpa adanya pengurangan atau pemotongan masa kerja akibat masa percobaan yang tidak sah. Ketentuan ini ditegaskan kembali dalam Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 12 ayat (2) dan Undang-Undang Nomor 13 Tahun 2003 Pasal 58 ayat (2).</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>PKWT harian hanya dapat dibuat untuk pekerjaan tertentu yang berubah dalam waktu dan volume pekerjaan serta upah berdasarkan kehadiran, dengan ketentuan pekerja bekerja kurang dari 21 hari dalam 1 bulan. Jika pekerja bekerja 21 hari atau lebih selama 3 bulan berturut-turut atau lebih, perjanjian kerja harian menjadi PKWTT.</t>
+          <t>Masa percobaan tidak boleh disyaratkan dalam PKWT. Jika masa percobaan tetap dicantumkan, masa percobaan tersebut batal demi hukum dan masa kerja pekerja tetap dihitung.</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.9232998530069988</v>
+        <v>0.9286643606424333</v>
       </c>
       <c r="G16" t="n">
         <v>1</v>
@@ -4864,7 +4744,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>menjadi PKWTT</t>
+          <t>masa kerja tetap dihitung</t>
         </is>
       </c>
       <c r="J16" t="n">
@@ -4875,7 +4755,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 10 | PP Nomor 35 Tahun 2021.pdf | Pasal 10</t>
+          <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 12 | PP Nomor 35 Tahun 2021.pdf | Pasal 12</t>
         </is>
       </c>
     </row>
@@ -4897,10 +4777,8 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Berdasarkan referensi yang tersedia, syarat pokok perusahaan alih daya adalah:
-1.  **Bentuk Badan Usaha:** Perusahaan Alih Daya harus berbentuk **badan hukum** (PP No. 35 Tahun 2021 Pasal 20 ayat 1; PM No. 7 Tahun 2026 Pasal 1 ayat 3).
-2.  **Perizinan Berusaha:** Perusahaan wajib memenuhi perizinan berusaha yang diterbitkan oleh Pemerintah Pusat sesuai dengan norma, standar, prosedur, dan kriteria yang ditetapkan (PP No. 35 Tahun 2021 Pasal 20 ayat 1).
-3.  **Jangka Waktu Usaha:** Kegiatan usaha harus dijalankan paling lambat **1 (satu) tahun** sejak perizinan berusaha diterbitkan (PM No. 7 Tahun 2026 Pasal 6 ayat c).</t>
+          <t>Istilah "perusahaan alih daya" dalam pertanyaan tersebut merujuk pada Perusahaan Alih Daya sebagaimana diatur dalam peraturan perundang-undangan ketenagakerjaan. Berdasarkan dokumen yang tersedia, syarat pokok terkait bentuk badan usaha dan perizinan adalah sebagai berikut:
+Peraturan Pemerintah No. 35 Tahun 2021, Pasal 20 ayat (1) dan ayat (2) serta Peraturan Menteri Ketenagakerjaan No. 7 Tahun 2026, Pasal 1 ayat (3) dan Pasal 6 ayat (a) menetapkan bahwa Perusahaan Alih Daya wajib berbentuk badan hukum dan wajib memenuhi perizinan berusaha yang diterbitkan oleh Pemerintah Pusat. Syarat dan tata cara memperoleh perizinan tersebut dilaksanakan sesuai dengan ketentuan peraturan perundang-undangan mengenai norma, standar, prosedur, dan kriteria perizinan berusaha yang ditetapkan oleh Pemerintah Pusat. Selain itu, Perusahaan Alih Daya juga diwajibkan untuk mencatatkan Perjanjian Alih Daya kepada Dinas dan menjalankan kegiatan usaha paling lambat satu tahun sejak perizinan berusaha diterbitkan.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -4909,7 +4787,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0.9297636111577352</v>
+        <v>0.9311560173829397</v>
       </c>
       <c r="G17" t="n">
         <v>0.95</v>
@@ -4935,43 +4813,36 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Q01</t>
+          <t>Q07</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PKWT</t>
+          <t>Alih daya</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Jika pekerja PKWT bekerja selama 6 bulan lalu kontraknya berakhir sesuai jangka waktu, hak kompensasi apa yang perlu diberikan pengusaha dan bagaimana rumus umumnya?</t>
+          <t>Dalam hubungan kerja alih daya, siapa pihak yang bertanggung jawab atas perlindungan upah, kesejahteraan, syarat kerja, dan perselisihan pekerja?</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Berdasarkan referensi yang tersedia, pengusaha wajib memberikan **Uang Kompensasi** kepada pekerja PKWT yang telah bekerja selama 6 bulan sesuai jangka waktu kontrak.
-**Dasar Hukum:**
-*   **PP Nomor 35 Tahun 2021 Pasal 15 ayat (1):** Pengusaha wajib memberikan uang kompensasi kepada pekerja/buruh yang hubungan kerjanya berdasarkan PKWT.
-*   **PP Nomor 35 Tahun 2021 Pasal 15 ayat (3):** Uang kompensasi diberikan kepada pekerja/buruh yang telah mempunyai masa kerja paling sedikit 1 (satu) bulan secara terus menerus.
-*   **PP Nomor 35 Tahun 2021 Pasal 16 ayat (1) huruf b:** Untuk PKWT selama 1 (satu) bulan atau lebih tetapi kurang dari 12 (dua belas) bulan, dihitung secara proporsional.
-**Rumus Umum:**
-Uang Kompensasi = (Masa Kerja / 12) x 1 Bulan Upah
-*(Di mana "1 Bulan Upah" terdiri dari Upah Pokok dan Tunjangan Tetap sesuai Pasal 16 ayat (2)).*
-**Perhitungan untuk kasus 6 bulan:**
-Uang Kompensasi = (6 / 12) x 1 Bulan Upah = **0,5 (satu setengah) Bulan Upah**.</t>
+          <t>Dalam hubungan kerja alih daya, pihak yang bertanggung jawab atas perlindungan upah, kesejahteraan, syarat kerja, dan perselisihan pekerja adalah Perusahaan Alih Daya.
+Hal ini diatur secara tegas dalam Peraturan Pemerintah Nomor 35 Tahun 2021 tentang Perjanjian Kerja Waktu Tertentu, Alih Daya, Waktu Kerja dan Waktu Istirahat, dan Pemutusan Hubungan Kerja. Berdasarkan Pasal 18 ayat (3) dari peraturan tersebut, pelindungan pekerja/buruh, upah, kesejahteraan, syarat kerja, dan perselisihan yang timbul dilaksanakan sesuai dengan ketentuan peraturan perundang-undangan dan menjadi tanggung jawab Perusahaan Alih Daya. Ketentuan ini juga diperkuat dalam Pasal 19 ayat (3) yang menyatakan bahwa dalam hal pekerja/buruh tidak memperoleh jaminan atas kelangsungan bekerja, Perusahaan Alih Daya bertanggung jawab atas pemenuhan hak pekerja/buruh.
+Meskipun dalam konteks penyediaan jasa pekerja/buruh (bukan alih daya murni) terdapat ketentuan dalam Undang-Undang Nomor 13 Tahun 2003 Pasal 66 ayat (2) huruf c yang menyatakan tanggung jawab serupa bagi perusahaan penyedia jasa pekerja/buruh, namun untuk skenario spesifik alih daya, tanggung jawab utama secara eksplisit berada pada Perusahaan Alih Daya sebagaimana diatur dalam Peraturan Pemerintah Nomor 35 Tahun 2021.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Pekerja PKWT berhak memperoleh uang kompensasi saat hubungan kerja berakhir karena jangka waktu selesai. Untuk masa kerja 12 bulan secara terus menerus kompensasinya 1 bulan upah. Untuk masa kerja kurang dari 12 bulan atau lebih dari 12 bulan, nilainya dihitung proporsional berdasarkan masa kerja dibagi 12 dikali 1 bulan upah. Jadi masa kerja 6 bulan dihitung 6 per 12 dikali 1 bulan upah.</t>
+          <t>Perlindungan pekerja, upah, kesejahteraan, syarat kerja, dan perselisihan yang timbul menjadi tanggung jawab perusahaan alih daya sebagai pemberi kerja pekerja alih daya.</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.9298496687412263</v>
+        <v>0.9314830627044043</v>
       </c>
       <c r="G18" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -4980,7 +4851,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>berakhir</t>
+          <t>perlindungan pekerja</t>
         </is>
       </c>
       <c r="J18" t="n">
@@ -4991,7 +4862,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 15 | PP Nomor 35 Tahun 2021.pdf | Pasal 15</t>
+          <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 18 | PP Nomor 35 Tahun 2021.pdf | Pasal 18</t>
         </is>
       </c>
     </row>
@@ -5013,16 +4884,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Berdasarkan referensi yang tersedia, pekerja yang mengundurkan diri atas kemauan sendiri dan memenuhi syarat berhak atas:
-1.  **Uang Penggantian Hak:** Sesuai ketentuan Pasal 40 ayat (4) PP Nomor 35 Tahun 2021 (merujuk pada hak yang sama dalam Pasal 156 ayat (4) UU No. 13 Tahun 2003).
-2.  **Uang Pisah:** Besarnya dan pelaksanaannya diatur dalam Perjanjian Kerja, Peraturan Perusahaan, atau Perjanjian Kerja Bersama.
-**Dasar Hukum:**
-*   **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 50 ayat (1)** dan **Pasal 36 huruf i**.
-*   **Undang-Undang Nomor 13 Tahun 2003 Pasal 162 ayat (1) dan (2)**.
-**Syarat Pengunduran Diri (sesuai PP No. 35 Tahun 2021 Pasal 36 huruf i):**
-1.  Mengajukan permohonan pengunduran diri secara tertulis selambat-lambatnya 30 (tiga puluh) hari sebelum tanggal mulai pengunduran diri.
-2.  Tidak terikat dalam ikatan dinas.
-3.  Tetap melaksanakan kewajibannya sampai tanggal mulai pengunduran diri.</t>
+          <t>Istilah "mengundurkan diri atas kemauan sendiri" dalam konteks hukum ketenagakerjaan merujuk pada pemutusan hubungan kerja karena alasan pengunduran diri yang diajukan oleh pekerja/buruh. Berdasarkan peraturan terbaru yang berlaku, yaitu Peraturan Pemerintah Nomor 35 Tahun 2021, hak pekerja yang mengundurkan diri atas kemauan sendiri dan memenuhi syarat sebagaimana dimaksud dalam Pasal 36 huruf i adalah berhak atas uang penggantian hak sesuai ketentuan Pasal 40 ayat (4) dan uang pisah yang besarnya diatur dalam Perjanjian Kerja, Peraturan Perusahaan, atau Perjanjian Kerja Bersama.
+Syarat pengunduran diri yang harus dipenuhi menurut Pasal 36 ayat (1) huruf i Peraturan Pemerintah Nomor 35 Tahun 2021 adalah:
+1. Mengajukan permohonan pengunduran diri secara tertulis selambat-lambatnya 30 (tiga puluh) hari sebelum tanggal mulai pengunduran diri.
+2. Tidak terikat dalam ikatan dinas.
+3. Tetap melaksanakan kewajibannya sampai tanggal mulai pengunduran diri.
+Peraturan Pemerintah Nomor 35 Tahun 2021 ini merupakan aturan yang lebih baru dan spesifik dibandingkan Undang-Undang Nomor 13 Tahun 2003, sehingga ketentuan dalam peraturan ini yang menjadi acuan utama. Dalam hal ini, pekerja yang mengundurkan diri atas kemauan sendiri tidak berhak atas uang pesangon, namun tetap berhak atas uang penggantian hak dan uang pisah jika memenuhi syarat-syarat tersebut.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -5031,7 +4898,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>0.9322046665350597</v>
+        <v>0.9380271432797115</v>
       </c>
       <c r="G19" t="n">
         <v>0.95</v>
@@ -5057,7 +4924,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Q02</t>
+          <t>Q03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -5067,28 +4934,24 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Apakah masa percobaan boleh diterapkan kepada pekerja PKWT, dan apa akibat hukumnya bila tetap dicantumkan?</t>
+          <t>Untuk pekerjaan yang diperkirakan selesai dalam waktu tertentu, berapa batas maksimal jangka waktu PKWT beserta perpanjangannya?</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Berdasarkan referensi yang tersedia, masa percobaan **tidak boleh** diterapkan kepada pekerja Perjanjian Kerja Waktu Tertentu (PKWT).
-Dasar hukumnya adalah:
-1.  **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 12 ayat (1)**: PKWT tidak dapat mensyaratkan adanya masa percobaan kerja.
-2.  **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 12 ayat (2)**: Dalam hal disyaratkan masa percobaan kerja, maka masa percobaan kerja yang disyaratkan tersebut **batal demi hukum** dan masa kerja tetap dihitung.
-3.  **Undang-Undang Nomor 13 Tahun 2003 Pasal 58 ayat (1)**: Perjanjian kerja untuk waktu tertentu tidak dapat mensyaratkan adanya masa percobaan kerja.
-4.  **Undang-Undang Nomor 13 Tahun 2003 Pasal 58 ayat (2)**: Dalam hal disyaratkan masa percobaan kerja, masa percobaan kerja yang disyaratkan **batal demi hukum**.
-**Kesimpulan:**
-Masa percobaan dalam PKWT adalah **ilegal**. Jika tetap dicantumkan dalam perjanjian, masa percobaan tersebut dianggap tidak berlaku (batal demi hukum), dan masa kerja pekerja dihitung sejak awal perjanjian tanpa pengurangan waktu.</t>
+          <t>Berdasarkan konteks pertanyaan mengenai batas maksimal jangka waktu Perjanjian Kerja Waktu Tertentu (PKWT) untuk pekerjaan yang diperkirakan selesai dalam waktu tertentu, terdapat perbedaan ketentuan antara peraturan lama dan peraturan terbaru yang lebih spesifik.
+Istilah "pekerjaan yang diperkirakan selesai dalam waktu tertentu" dalam pertanyaan tersebut merujuk pada "pekerjaan yang diperkirakan penyelesaiannya dalam waktu yang tidak terlalu lama" sebagaimana diatur dalam **Undang-Undang Nomor 13 Tahun 2003 Pasal 59 ayat (1) huruf b**. Berdasarkan aturan lama ini, PKWT untuk jenis pekerjaan tersebut dapat diadakan untuk paling lama 2 (dua) tahun dan hanya boleh diperpanjang 1 (satu) kali untuk jangka waktu paling lama 1 (satu) tahun.
+Namun, **Peraturan Pemerintah Nomor 35 Tahun 2021** merupakan aturan terbaru yang lebih spesifik dan mengoreksi ketentuan lama tersebut. Dalam **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 8 ayat (1)**, dinyatakan secara tegas bahwa PKWT berdasarkan jangka waktu dapat dibuat untuk paling lama 5 (lima) tahun. Ayat (2) dari pasal yang sama mengatur bahwa jika pekerjaan belum selesai saat jangka waktu berakhir, perpanjangan dapat dilakukan dengan kesepakatan, dengan ketentuan jangka waktu keseluruhan PKWT beserta perpanjangannya tidak lebih dari 5 (lima) tahun.
+Oleh karena itu, berdasarkan aturan terbaru yang berlaku, batas maksimal jangka waktu PKWT beserta perpanjangannya untuk pekerjaan yang diperkirakan selesai dalam waktu tertentu adalah 5 (lima) tahun. Ketentuan lama mengenai batas 2 tahun dan perpanjangan 1 tahun yang tercantum dalam **Undang-Undang Nomor 13 Tahun 2003 Pasal 59 ayat (4)** telah digantikan oleh ketentuan baru dalam **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 8 ayat (1) dan ayat (2)**.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Masa percobaan tidak boleh disyaratkan dalam PKWT. Jika masa percobaan tetap dicantumkan, masa percobaan tersebut batal demi hukum dan masa kerja pekerja tetap dihitung.</t>
+          <t>PKWT berdasarkan jangka waktu untuk pekerjaan yang diperkirakan selesai dalam waktu tertentu dapat dibuat paling lama 5 tahun termasuk perpanjangannya.</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>0.9736037194728853</v>
+        <v>0.9435577776432038</v>
       </c>
       <c r="G20" t="n">
         <v>1</v>
@@ -5100,14 +4963,14 @@
       </c>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K20" t="n">
         <v>1</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 12 | PP Nomor 35 Tahun 2021.pdf | Pasal 12</t>
+          <t>Peraturan Pemerintah No. 35 Tahun 2021, Pasal 9 | PP Nomor 35 Tahun 2021.pdf | Pasal 9</t>
         </is>
       </c>
     </row>
@@ -5129,9 +4992,10 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Berdasarkan **Peraturan Pemerintah Nomor 35 Tahun 2021 Pasal 21 ayat (2)**, terdapat dua pola waktu kerja sebagai berikut:
-1.  **Untuk 6 hari kerja dalam seminggu:** 7 (tujuh) jam per hari dan 40 (empat puluh) jam per minggu.
-2.  **Untuk 5 hari kerja dalam seminggu:** 8 (delapan) jam per hari dan 40 (empat puluh) jam per minggu.</t>
+          <t>Berdasarkan Peraturan Pemerintah Nomor 35 Tahun 2021, terdapat dua pola waktu kerja yang diatur dalam Pasal 21 ayat (2) untuk pekerja/buruh, yaitu:
+1. Pola kerja enam hari dalam seminggu dengan ketentuan waktu kerja 7 (tujuh) jam per hari dan total 40 (empat puluh) jam per minggu.
+2. Pola kerja lima hari dalam seminggu dengan ketentuan waktu kerja 8 (delapan) jam per hari dan total 40 (empat puluh) jam per minggu.
+Ketentuan ini berlaku umum bagi setiap pengusaha, kecuali bagi sektor usaha atau pekerjaan tertentu yang diatur lebih lanjut dalam Pasal 23 dan Pasal 26.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -5140,7 +5004,7 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0.9788179874420168</v>
+        <v>0.9747076630592347</v>
       </c>
       <c r="G21" t="n">
         <v>1</v>

</xml_diff>